<commit_message>
Update BSPI15 through October 9, 2026
Append all 17 audited October 9 closes, regenerate index and benchmark data, and extend the cumulative formula review workbook. Preserve prior canonical rows and source receipts.

Validation: strict Marketstack audit, calculation reconciliation, type checking, production build, desktop/mobile preview and holdings CSV checks passed. Repository lint retains seven pre-existing errors in unrelated output scripts.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R24ceb2a81c6d4761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R5d1dee8bb64a4437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Ree3b62dcade14420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R9948895027ae4fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rfb28306d0b70413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2497a28ca6684504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R7dd283648d654d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R789b5fb55ae14fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Rd082d43da1ea4808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R1900fc3138224dcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -220,7 +220,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -248,7 +248,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -267,7 +267,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H95" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H110" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -283,7 +283,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:L107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:L124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -303,7 +303,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1148,6 +1148,85 @@
         <x:v>-3.513362421883326</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="40" customHeight="1">
+      <x:c r="A12" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="n">
+        <x:f>B11*(1+SUM('Returns and Contributions'!F96:F110))</x:f>
+        <x:v>988.7186891541369</x:v>
+      </x:c>
+      <x:c r="C12" s="18" t="n">
+        <x:f>B12/B11-1</x:f>
+        <x:v>0.012160564720784528</x:v>
+      </x:c>
+      <x:c r="D12" s="18" t="n">
+        <x:f>B12/$B$6-1</x:f>
+        <x:v>-0.011281310845863146</x:v>
+      </x:c>
+      <x:c r="E12" s="17" t="n">
+        <x:f>1000*'Prices'!H123/'Prices'!I123</x:f>
+        <x:v>1018.9253174546237</x:v>
+      </x:c>
+      <x:c r="F12" s="18" t="n">
+        <x:f>E12/E11-1</x:f>
+        <x:v>0.005946923259191994</x:v>
+      </x:c>
+      <x:c r="G12" s="18" t="n">
+        <x:f>E12/1000-1</x:f>
+        <x:v>0.01892531745462378</x:v>
+      </x:c>
+      <x:c r="H12" s="17" t="n">
+        <x:f>1000*'Prices'!H124/'Prices'!I124</x:f>
+        <x:v>1018.4050923332402</x:v>
+      </x:c>
+      <x:c r="I12" s="18" t="n">
+        <x:f>H12/H11-1</x:f>
+        <x:v>0.006355604029189443</x:v>
+      </x:c>
+      <x:c r="J12" s="18" t="n">
+        <x:f>H12/1000-1</x:f>
+        <x:v>0.01840509233324017</x:v>
+      </x:c>
+      <x:c r="K12" s="22" t="n">
+        <x:f>(C12-F12)*100</x:f>
+        <x:v>0.6213641461592534</x:v>
+      </x:c>
+      <x:c r="L12" s="22" t="n">
+        <x:f>(C12-I12)*100</x:f>
+        <x:v>0.5804960691595085</x:v>
+      </x:c>
+      <x:c r="M12" s="20" t="n">
+        <x:f>SUM('Returns and Contributions'!G96:G110)</x:f>
+        <x:v>0.9999999999999999</x:v>
+      </x:c>
+      <x:c r="N12" s="26" t="n">
+        <x:f>SUM('Returns and Contributions'!F96:F110)-C12</x:f>
+        <x:v>-8.500145032286355e-17</x:v>
+      </x:c>
+      <x:c r="O12" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P12" s="11" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I108:I124,"Mismatch")=0,"Passed","Failed")</x:f>
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="Q12" s="27" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+      <x:c r="R12" s="26" t="n">
+        <x:f>B12-1000*('Prices'!H108/'Prices'!H6+'Prices'!H109/'Prices'!H7+'Prices'!H110/'Prices'!H8+'Prices'!H111/'Prices'!H9+'Prices'!H112/'Prices'!H10+'Prices'!H113/'Prices'!H11+'Prices'!H114/'Prices'!H12+'Prices'!H115/'Prices'!H13+'Prices'!H116/'Prices'!H14+'Prices'!H117/'Prices'!H15+'Prices'!H118/'Prices'!H16+'Prices'!H119/'Prices'!H17+'Prices'!H120/'Prices'!H18+'Prices'!H121/'Prices'!H19+'Prices'!H122/'Prices'!H20)/15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="22" t="n">
+        <x:f>(D12-G12)*100</x:f>
+        <x:v>-3.0206628300486926</x:v>
+      </x:c>
+      <x:c r="T12" s="22" t="n">
+        <x:f>(D12-J12)*100</x:f>
+        <x:v>-2.9686403179103316</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1155,7 +1234,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc22099783ddb40ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13ccdd623eb14f54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4889,6 +4968,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="108" ht="27" customHeight="1">
+      <x:c r="A108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B108" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C108" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D108" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E108" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F108" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G108" s="15" t="n">
+        <x:f>H91</x:f>
+        <x:v>6019</x:v>
+      </x:c>
+      <x:c r="H108" s="30" t="n">
+        <x:v>6103</x:v>
+      </x:c>
+      <x:c r="I108" s="30" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K108" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="27" customHeight="1">
+      <x:c r="A109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B109" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C109" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D109" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E109" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F109" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G109" s="29" t="n">
+        <x:f>H92</x:f>
+        <x:v>4789</x:v>
+      </x:c>
+      <x:c r="H109" s="31" t="n">
+        <x:v>4783</x:v>
+      </x:c>
+      <x:c r="I109" s="31" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K109" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="27" customHeight="1">
+      <x:c r="A110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B110" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C110" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D110" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E110" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F110" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G110" s="15" t="n">
+        <x:f>H93</x:f>
+        <x:v>26.86</x:v>
+      </x:c>
+      <x:c r="H110" s="30" t="n">
+        <x:v>27.04</x:v>
+      </x:c>
+      <x:c r="I110" s="30" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K110" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="27" customHeight="1">
+      <x:c r="A111" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B111" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C111" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D111" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E111" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F111" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G111" s="29" t="n">
+        <x:f>H94</x:f>
+        <x:v>398.72</x:v>
+      </x:c>
+      <x:c r="H111" s="31" t="n">
+        <x:v>402.68</x:v>
+      </x:c>
+      <x:c r="I111" s="31" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J111" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K111" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="27" customHeight="1">
+      <x:c r="A112" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B112" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C112" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D112" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E112" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F112" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G112" s="15" t="n">
+        <x:f>H95</x:f>
+        <x:v>4795</x:v>
+      </x:c>
+      <x:c r="H112" s="30" t="n">
+        <x:v>4859</x:v>
+      </x:c>
+      <x:c r="I112" s="30" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J112" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K112" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="27" customHeight="1">
+      <x:c r="A113" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B113" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C113" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D113" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E113" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F113" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G113" s="29" t="n">
+        <x:f>H96</x:f>
+        <x:v>49.85</x:v>
+      </x:c>
+      <x:c r="H113" s="31" t="n">
+        <x:v>50.59</x:v>
+      </x:c>
+      <x:c r="I113" s="31" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J113" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K113" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="27" customHeight="1">
+      <x:c r="A114" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B114" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C114" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D114" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E114" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F114" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G114" s="15" t="n">
+        <x:f>H97</x:f>
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="H114" s="30" t="n">
+        <x:v>80540</x:v>
+      </x:c>
+      <x:c r="I114" s="30" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J114" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K114" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="27" customHeight="1">
+      <x:c r="A115" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B115" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C115" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D115" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E115" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F115" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G115" s="29" t="n">
+        <x:f>H98</x:f>
+        <x:v>60.91</x:v>
+      </x:c>
+      <x:c r="H115" s="31" t="n">
+        <x:v>62.92</x:v>
+      </x:c>
+      <x:c r="I115" s="31" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J115" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K115" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="27" customHeight="1">
+      <x:c r="A116" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B116" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C116" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D116" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E116" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F116" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G116" s="15" t="n">
+        <x:f>H99</x:f>
+        <x:v>39.53</x:v>
+      </x:c>
+      <x:c r="H116" s="30" t="n">
+        <x:v>39.9</x:v>
+      </x:c>
+      <x:c r="I116" s="30" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J116" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K116" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="27" customHeight="1">
+      <x:c r="A117" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B117" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C117" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D117" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E117" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F117" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G117" s="29" t="n">
+        <x:f>H100</x:f>
+        <x:v>15.61</x:v>
+      </x:c>
+      <x:c r="H117" s="31" t="n">
+        <x:v>16.01</x:v>
+      </x:c>
+      <x:c r="I117" s="31" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J117" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K117" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="27" customHeight="1">
+      <x:c r="A118" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B118" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C118" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D118" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E118" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F118" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G118" s="15" t="n">
+        <x:f>H101</x:f>
+        <x:v>434.14</x:v>
+      </x:c>
+      <x:c r="H118" s="30" t="n">
+        <x:v>432.59</x:v>
+      </x:c>
+      <x:c r="I118" s="30" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J118" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K118" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="27" customHeight="1">
+      <x:c r="A119" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B119" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C119" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D119" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E119" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F119" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G119" s="29" t="n">
+        <x:f>H102</x:f>
+        <x:v>264.25</x:v>
+      </x:c>
+      <x:c r="H119" s="31" t="n">
+        <x:v>272.1</x:v>
+      </x:c>
+      <x:c r="I119" s="31" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J119" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K119" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="27" customHeight="1">
+      <x:c r="A120" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B120" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C120" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D120" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E120" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F120" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G120" s="15" t="n">
+        <x:f>H103</x:f>
+        <x:v>231.07</x:v>
+      </x:c>
+      <x:c r="H120" s="30" t="n">
+        <x:v>227.52</x:v>
+      </x:c>
+      <x:c r="I120" s="30" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J120" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K120" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="27" customHeight="1">
+      <x:c r="A121" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B121" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C121" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D121" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E121" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F121" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G121" s="29" t="n">
+        <x:f>H104</x:f>
+        <x:v>5716</x:v>
+      </x:c>
+      <x:c r="H121" s="31" t="n">
+        <x:v>5773</x:v>
+      </x:c>
+      <x:c r="I121" s="31" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J121" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K121" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="27" customHeight="1">
+      <x:c r="A122" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B122" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C122" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D122" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E122" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F122" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G122" s="15" t="n">
+        <x:f>H105</x:f>
+        <x:v>101.25</x:v>
+      </x:c>
+      <x:c r="H122" s="30" t="n">
+        <x:v>104.15</x:v>
+      </x:c>
+      <x:c r="I122" s="30" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J122" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K122" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="27" customHeight="1">
+      <x:c r="A123" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B123" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C123" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D123" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E123" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F123" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G123" s="29" t="n">
+        <x:f>H106</x:f>
+        <x:v>7765.36</x:v>
+      </x:c>
+      <x:c r="H123" s="31" t="n">
+        <x:v>7811.54</x:v>
+      </x:c>
+      <x:c r="I123" s="31" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J123" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K123" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="27" customHeight="1">
+      <x:c r="A124" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B124" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C124" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D124" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E124" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F124" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G124" s="15" t="n">
+        <x:f>H107</x:f>
+        <x:v>27193.3398</x:v>
+      </x:c>
+      <x:c r="H124" s="30" t="n">
+        <x:v>27366.1699</x:v>
+      </x:c>
+      <x:c r="I124" s="30" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J124" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="K124" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -4896,7 +5587,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f923e4047314d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df7227d44c64258"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7685,6 +8376,471 @@
         <x:v>0.022520702888305433</x:v>
       </x:c>
     </x:row>
+    <x:row r="96" ht="27" customHeight="1">
+      <x:c r="A96" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B96" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C96" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D96" s="18" t="n">
+        <x:f>G81</x:f>
+        <x:v>0.06704430190053146</x:v>
+      </x:c>
+      <x:c r="E96" s="20" t="n">
+        <x:f>'Prices'!H108/'Prices'!G108-1</x:f>
+        <x:v>0.01395580661239415</x:v>
+      </x:c>
+      <x:c r="F96" s="18" t="n">
+        <x:f>D96*E96</x:f>
+        <x:v>0.0009356573117867866</x:v>
+      </x:c>
+      <x:c r="G96" s="18" t="n">
+        <x:f>D96*(1+E96)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06716321657035833</x:v>
+      </x:c>
+      <x:c r="H96" s="20" t="n">
+        <x:f>'Prices'!H108/'Prices'!I108-1</x:f>
+        <x:v>-0.0039170882976986565</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="27" customHeight="1">
+      <x:c r="A97" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B97" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C97" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D97" s="19" t="n">
+        <x:f>G82</x:f>
+        <x:v>0.06839009650574954</x:v>
+      </x:c>
+      <x:c r="E97" s="21" t="n">
+        <x:f>'Prices'!H109/'Prices'!G109-1</x:f>
+        <x:v>-0.0012528711630820366</x:v>
+      </x:c>
+      <x:c r="F97" s="19" t="n">
+        <x:f>D97*E97</x:f>
+        <x:v>-0.00008568397975245115</x:v>
+      </x:c>
+      <x:c r="G97" s="19" t="n">
+        <x:f>D97*(1+E97)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06748377175200419</x:v>
+      </x:c>
+      <x:c r="H97" s="21" t="n">
+        <x:f>'Prices'!H109/'Prices'!I109-1</x:f>
+        <x:v>0.0008369951872777559</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="27" customHeight="1">
+      <x:c r="A98" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B98" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C98" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D98" s="18" t="n">
+        <x:f>G83</x:f>
+        <x:v>0.06495826385486109</x:v>
+      </x:c>
+      <x:c r="E98" s="20" t="n">
+        <x:f>'Prices'!H110/'Prices'!G110-1</x:f>
+        <x:v>0.006701414743112366</x:v>
+      </x:c>
+      <x:c r="F98" s="18" t="n">
+        <x:f>D98*E98</x:f>
+        <x:v>0.00043531226708394923</x:v>
+      </x:c>
+      <x:c r="G98" s="18" t="n">
+        <x:f>D98*(1+E98)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06460790748154129</x:v>
+      </x:c>
+      <x:c r="H98" s="20" t="n">
+        <x:f>'Prices'!H110/'Prices'!I110-1</x:f>
+        <x:v>-0.04181431608788089</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="27" customHeight="1">
+      <x:c r="A99" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B99" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C99" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D99" s="19" t="n">
+        <x:f>G84</x:f>
+        <x:v>0.06544543980878394</x:v>
+      </x:c>
+      <x:c r="E99" s="21" t="n">
+        <x:f>'Prices'!H111/'Prices'!G111-1</x:f>
+        <x:v>0.009931781701444597</x:v>
+      </x:c>
+      <x:c r="F99" s="19" t="n">
+        <x:f>D99*E99</x:f>
+        <x:v>0.0006499898215358742</x:v>
+      </x:c>
+      <x:c r="G99" s="19" t="n">
+        <x:f>D99*(1+E99)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06530132859755601</x:v>
+      </x:c>
+      <x:c r="H99" s="21" t="n">
+        <x:f>'Prices'!H111/'Prices'!I111-1</x:f>
+        <x:v>-0.031530339835012855</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="27" customHeight="1">
+      <x:c r="A100" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B100" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C100" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D100" s="18" t="n">
+        <x:f>G85</x:f>
+        <x:v>0.06577804119401282</x:v>
+      </x:c>
+      <x:c r="E100" s="20" t="n">
+        <x:f>'Prices'!H112/'Prices'!G112-1</x:f>
+        <x:v>0.013347236704901011</x:v>
+      </x:c>
+      <x:c r="F100" s="18" t="n">
+        <x:f>D100*E100</x:f>
+        <x:v>0.0008779550858012186</x:v>
+      </x:c>
+      <x:c r="G100" s="18" t="n">
+        <x:f>D100*(1+E100)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06585516034029819</x:v>
+      </x:c>
+      <x:c r="H100" s="20" t="n">
+        <x:f>'Prices'!H112/'Prices'!I112-1</x:f>
+        <x:v>-0.023316582914572836</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="27" customHeight="1">
+      <x:c r="A101" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B101" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C101" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D101" s="19" t="n">
+        <x:f>G86</x:f>
+        <x:v>0.06555158767168619</x:v>
+      </x:c>
+      <x:c r="E101" s="21" t="n">
+        <x:f>'Prices'!H113/'Prices'!G113-1</x:f>
+        <x:v>0.014844533600802512</x:v>
+      </x:c>
+      <x:c r="F101" s="19" t="n">
+        <x:f>D101*E101</x:f>
+        <x:v>0.0009730827457782973</x:v>
+      </x:c>
+      <x:c r="G101" s="19" t="n">
+        <x:f>D101*(1+E101)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06572541228754158</x:v>
+      </x:c>
+      <x:c r="H101" s="21" t="n">
+        <x:f>'Prices'!H113/'Prices'!I113-1</x:f>
+        <x:v>-0.025240847784200326</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="27" customHeight="1">
+      <x:c r="A102" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B102" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C102" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D102" s="18" t="n">
+        <x:f>G87</x:f>
+        <x:v>0.06723870923431403</x:v>
+      </x:c>
+      <x:c r="E102" s="20" t="n">
+        <x:f>'Prices'!H114/'Prices'!G114-1</x:f>
+        <x:v>0.006750000000000034</x:v>
+      </x:c>
+      <x:c r="F102" s="18" t="n">
+        <x:f>D102*E102</x:f>
+        <x:v>0.000453861287331622</x:v>
+      </x:c>
+      <x:c r="G102" s="18" t="n">
+        <x:f>D102*(1+E102)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06687928070021122</x:v>
+      </x:c>
+      <x:c r="H102" s="20" t="n">
+        <x:f>'Prices'!H114/'Prices'!I114-1</x:f>
+        <x:v>-0.00812807881773403</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="27" customHeight="1">
+      <x:c r="A103" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B103" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C103" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D103" s="19" t="n">
+        <x:f>G88</x:f>
+        <x:v>0.06681038936280935</x:v>
+      </x:c>
+      <x:c r="E103" s="21" t="n">
+        <x:f>'Prices'!H115/'Prices'!G115-1</x:f>
+        <x:v>0.03299950747003777</x:v>
+      </x:c>
+      <x:c r="F103" s="19" t="n">
+        <x:f>D103*E103</x:f>
+        <x:v>0.002204709942854159</x:v>
+      </x:c>
+      <x:c r="G103" s="19" t="n">
+        <x:f>D103*(1+E103)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.0681859200123076</x:v>
+      </x:c>
+      <x:c r="H103" s="21" t="n">
+        <x:f>'Prices'!H115/'Prices'!I115-1</x:f>
+        <x:v>0.011250401800064314</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="27" customHeight="1">
+      <x:c r="A104" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B104" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C104" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D104" s="18" t="n">
+        <x:f>G89</x:f>
+        <x:v>0.06600967381142453</x:v>
+      </x:c>
+      <x:c r="E104" s="20" t="n">
+        <x:f>'Prices'!H116/'Prices'!G116-1</x:f>
+        <x:v>0.009359979762205928</x:v>
+      </x:c>
+      <x:c r="F104" s="18" t="n">
+        <x:f>D104*E104</x:f>
+        <x:v>0.0006178492109847482</x:v>
+      </x:c>
+      <x:c r="G104" s="18" t="n">
+        <x:f>D104*(1+E104)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06582702917376473</x:v>
+      </x:c>
+      <x:c r="H104" s="20" t="n">
+        <x:f>'Prices'!H116/'Prices'!I116-1</x:f>
+        <x:v>-0.023733790066063132</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="27" customHeight="1">
+      <x:c r="A105" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B105" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C105" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D105" s="19" t="n">
+        <x:f>G90</x:f>
+        <x:v>0.06687634619678949</x:v>
+      </x:c>
+      <x:c r="E105" s="21" t="n">
+        <x:f>'Prices'!H117/'Prices'!G117-1</x:f>
+        <x:v>0.02562459961563124</x:v>
+      </x:c>
+      <x:c r="F105" s="19" t="n">
+        <x:f>D105*E105</x:f>
+        <x:v>0.0017136795950490737</x:v>
+      </x:c>
+      <x:c r="G105" s="19" t="n">
+        <x:f>D105*(1+E105)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.0677659535280945</x:v>
+      </x:c>
+      <x:c r="H105" s="21" t="n">
+        <x:f>'Prices'!H117/'Prices'!I117-1</x:f>
+        <x:v>0.005021971123666091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="27" customHeight="1">
+      <x:c r="A106" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B106" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C106" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D106" s="18" t="n">
+        <x:f>G91</x:f>
+        <x:v>0.0669654840668773</x:v>
+      </x:c>
+      <x:c r="E106" s="20" t="n">
+        <x:f>'Prices'!H118/'Prices'!G118-1</x:f>
+        <x:v>-0.0035702768692127407</x:v>
+      </x:c>
+      <x:c r="F106" s="18" t="n">
+        <x:f>D106*E106</x:f>
+        <x:v>-0.00023908531879960636</x:v>
+      </x:c>
+      <x:c r="G106" s="18" t="n">
+        <x:f>D106*(1+E106)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06592471696077676</x:v>
+      </x:c>
+      <x:c r="H106" s="20" t="n">
+        <x:f>'Prices'!H118/'Prices'!I118-1</x:f>
+        <x:v>-0.02228500395524924</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="27" customHeight="1">
+      <x:c r="A107" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B107" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C107" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D107" s="19" t="n">
+        <x:f>G92</x:f>
+        <x:v>0.06632712890362265</x:v>
+      </x:c>
+      <x:c r="E107" s="21" t="n">
+        <x:f>'Prices'!H119/'Prices'!G119-1</x:f>
+        <x:v>0.0297067171239358</x:v>
+      </x:c>
+      <x:c r="F107" s="19" t="n">
+        <x:f>D107*E107</x:f>
+        <x:v>0.001970361255982744</x:v>
+      </x:c>
+      <x:c r="G107" s="19" t="n">
+        <x:f>D107*(1+E107)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06747693255412099</x:v>
+      </x:c>
+      <x:c r="H107" s="21" t="n">
+        <x:f>'Prices'!H119/'Prices'!I119-1</x:f>
+        <x:v>0.000735564545789158</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="27" customHeight="1">
+      <x:c r="A108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B108" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C108" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D108" s="18" t="n">
+        <x:f>G93</x:f>
+        <x:v>0.06593043718765222</x:v>
+      </x:c>
+      <x:c r="E108" s="20" t="n">
+        <x:f>'Prices'!H120/'Prices'!G120-1</x:f>
+        <x:v>-0.015363309819535154</x:v>
+      </x:c>
+      <x:c r="F108" s="18" t="n">
+        <x:f>D108*E108</x:f>
+        <x:v>-0.001012909733051303</x:v>
+      </x:c>
+      <x:c r="G108" s="18" t="n">
+        <x:f>D108*(1+E108)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.06413757828285784</x:v>
+      </x:c>
+      <x:c r="H108" s="20" t="n">
+        <x:f>'Prices'!H120/'Prices'!I120-1</x:f>
+        <x:v>-0.048789665119779224</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="27" customHeight="1">
+      <x:c r="A109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B109" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C109" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D109" s="19" t="n">
+        <x:f>G94</x:f>
+        <x:v>0.06688983348989865</x:v>
+      </x:c>
+      <x:c r="E109" s="21" t="n">
+        <x:f>'Prices'!H121/'Prices'!G121-1</x:f>
+        <x:v>0.009972008397480803</x:v>
+      </x:c>
+      <x:c r="F109" s="19" t="n">
+        <x:f>D109*E109</x:f>
+        <x:v>0.0006670259812673619</x:v>
+      </x:c>
+      <x:c r="G109" s="19" t="n">
+        <x:f>D109*(1+E109)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.066745200145001</x:v>
+      </x:c>
+      <x:c r="H109" s="21" t="n">
+        <x:f>'Prices'!H121/'Prices'!I121-1</x:f>
+        <x:v>-0.010116598079561001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="27" customHeight="1">
+      <x:c r="A110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B110" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C110" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D110" s="18" t="n">
+        <x:f>G95</x:f>
+        <x:v>0.06978426681098678</x:v>
+      </x:c>
+      <x:c r="E110" s="20" t="n">
+        <x:f>'Prices'!H122/'Prices'!G122-1</x:f>
+        <x:v>0.028641975308641987</x:v>
+      </x:c>
+      <x:c r="F110" s="18" t="n">
+        <x:f>D110*E110</x:f>
+        <x:v>0.0019987592469319676</x:v>
+      </x:c>
+      <x:c r="G110" s="18" t="n">
+        <x:f>D110*(1+E110)/(1+SUM($F$96:$F$110))</x:f>
+        <x:v>0.07092059161356565</x:v>
+      </x:c>
+      <x:c r="H110" s="20" t="n">
+        <x:f>'Prices'!H122/'Prices'!I122-1</x:f>
+        <x:v>0.05180771561300768</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -7692,7 +8848,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R613e34d01b3142e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8241eecc35d8410a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11607,6 +12763,635 @@
         <x:v>46304.492743877316</x:v>
       </x:c>
     </x:row>
+    <x:row r="108" ht="50" customHeight="1">
+      <x:c r="A108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B108" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C108" s="15" t="n">
+        <x:v>6103</x:v>
+      </x:c>
+      <x:c r="D108" s="15" t="n">
+        <x:v>6103</x:v>
+      </x:c>
+      <x:c r="E108" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F108" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G108" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H108" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I108" s="11" t="str">
+        <x:f>IF(AND(G108=H108,C108&gt;0,ABS(C108-'Prices'!H108)&lt;=MAX(0.01,'Prices'!H108*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J108" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K108" s="34" t="str"/>
+      <x:c r="L108" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="50" customHeight="1">
+      <x:c r="A109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B109" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C109" s="29" t="n">
+        <x:v>4783</x:v>
+      </x:c>
+      <x:c r="D109" s="29" t="n">
+        <x:v>4783</x:v>
+      </x:c>
+      <x:c r="E109" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F109" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G109" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H109" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I109" s="12" t="str">
+        <x:f>IF(AND(G109=H109,C109&gt;0,ABS(C109-'Prices'!H109)&lt;=MAX(0.01,'Prices'!H109*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J109" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K109" s="36" t="str"/>
+      <x:c r="L109" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="50" customHeight="1">
+      <x:c r="A110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B110" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C110" s="15" t="n">
+        <x:v>27.04</x:v>
+      </x:c>
+      <x:c r="D110" s="15" t="n">
+        <x:v>27.04</x:v>
+      </x:c>
+      <x:c r="E110" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F110" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G110" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H110" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I110" s="11" t="str">
+        <x:f>IF(AND(G110=H110,C110&gt;0,ABS(C110-'Prices'!H110)&lt;=MAX(0.01,'Prices'!H110*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J110" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K110" s="34" t="str"/>
+      <x:c r="L110" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="50" customHeight="1">
+      <x:c r="A111" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B111" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C111" s="29" t="n">
+        <x:v>402.68</x:v>
+      </x:c>
+      <x:c r="D111" s="29" t="n">
+        <x:v>402.68</x:v>
+      </x:c>
+      <x:c r="E111" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F111" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G111" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H111" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I111" s="12" t="str">
+        <x:f>IF(AND(G111=H111,C111&gt;0,ABS(C111-'Prices'!H111)&lt;=MAX(0.01,'Prices'!H111*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J111" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K111" s="36" t="str"/>
+      <x:c r="L111" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="50" customHeight="1">
+      <x:c r="A112" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B112" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C112" s="15" t="n">
+        <x:v>4859</x:v>
+      </x:c>
+      <x:c r="D112" s="15" t="n">
+        <x:v>4859</x:v>
+      </x:c>
+      <x:c r="E112" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F112" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G112" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H112" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I112" s="11" t="str">
+        <x:f>IF(AND(G112=H112,C112&gt;0,ABS(C112-'Prices'!H112)&lt;=MAX(0.01,'Prices'!H112*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J112" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K112" s="34" t="str"/>
+      <x:c r="L112" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="50" customHeight="1">
+      <x:c r="A113" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B113" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C113" s="29" t="n">
+        <x:v>50.59</x:v>
+      </x:c>
+      <x:c r="D113" s="29" t="n">
+        <x:v>50.59</x:v>
+      </x:c>
+      <x:c r="E113" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F113" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G113" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H113" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I113" s="12" t="str">
+        <x:f>IF(AND(G113=H113,C113&gt;0,ABS(C113-'Prices'!H113)&lt;=MAX(0.01,'Prices'!H113*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J113" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K113" s="36" t="str"/>
+      <x:c r="L113" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="50" customHeight="1">
+      <x:c r="A114" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B114" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C114" s="15" t="n">
+        <x:v>80540</x:v>
+      </x:c>
+      <x:c r="D114" s="15" t="n">
+        <x:v>80540</x:v>
+      </x:c>
+      <x:c r="E114" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F114" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G114" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H114" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I114" s="11" t="str">
+        <x:f>IF(AND(G114=H114,C114&gt;0,ABS(C114-'Prices'!H114)&lt;=MAX(0.01,'Prices'!H114*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J114" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K114" s="34" t="str"/>
+      <x:c r="L114" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="50" customHeight="1">
+      <x:c r="A115" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B115" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C115" s="29" t="n">
+        <x:v>62.92</x:v>
+      </x:c>
+      <x:c r="D115" s="29" t="n">
+        <x:v>62.92</x:v>
+      </x:c>
+      <x:c r="E115" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F115" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G115" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H115" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I115" s="12" t="str">
+        <x:f>IF(AND(G115=H115,C115&gt;0,ABS(C115-'Prices'!H115)&lt;=MAX(0.01,'Prices'!H115*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J115" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K115" s="36" t="str"/>
+      <x:c r="L115" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="50" customHeight="1">
+      <x:c r="A116" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B116" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C116" s="15" t="n">
+        <x:v>39.9</x:v>
+      </x:c>
+      <x:c r="D116" s="15" t="n">
+        <x:v>39.9</x:v>
+      </x:c>
+      <x:c r="E116" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F116" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G116" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H116" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I116" s="11" t="str">
+        <x:f>IF(AND(G116=H116,C116&gt;0,ABS(C116-'Prices'!H116)&lt;=MAX(0.01,'Prices'!H116*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J116" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K116" s="34" t="str"/>
+      <x:c r="L116" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="50" customHeight="1">
+      <x:c r="A117" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B117" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C117" s="29" t="n">
+        <x:v>16.01</x:v>
+      </x:c>
+      <x:c r="D117" s="29" t="n">
+        <x:v>16.01</x:v>
+      </x:c>
+      <x:c r="E117" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F117" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G117" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H117" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I117" s="12" t="str">
+        <x:f>IF(AND(G117=H117,C117&gt;0,ABS(C117-'Prices'!H117)&lt;=MAX(0.01,'Prices'!H117*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J117" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K117" s="36" t="str"/>
+      <x:c r="L117" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="50" customHeight="1">
+      <x:c r="A118" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B118" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C118" s="15" t="n">
+        <x:v>432.59</x:v>
+      </x:c>
+      <x:c r="D118" s="15" t="n">
+        <x:v>432.59</x:v>
+      </x:c>
+      <x:c r="E118" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F118" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G118" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H118" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I118" s="11" t="str">
+        <x:f>IF(AND(G118=H118,C118&gt;0,ABS(C118-'Prices'!H118)&lt;=MAX(0.01,'Prices'!H118*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J118" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K118" s="34" t="str"/>
+      <x:c r="L118" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="50" customHeight="1">
+      <x:c r="A119" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B119" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C119" s="29" t="n">
+        <x:v>272.1</x:v>
+      </x:c>
+      <x:c r="D119" s="29" t="n">
+        <x:v>272.1</x:v>
+      </x:c>
+      <x:c r="E119" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F119" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G119" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H119" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I119" s="12" t="str">
+        <x:f>IF(AND(G119=H119,C119&gt;0,ABS(C119-'Prices'!H119)&lt;=MAX(0.01,'Prices'!H119*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J119" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K119" s="36" t="str"/>
+      <x:c r="L119" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="50" customHeight="1">
+      <x:c r="A120" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B120" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C120" s="15" t="n">
+        <x:v>227.52</x:v>
+      </x:c>
+      <x:c r="D120" s="15" t="n">
+        <x:v>227.52</x:v>
+      </x:c>
+      <x:c r="E120" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F120" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G120" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H120" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I120" s="11" t="str">
+        <x:f>IF(AND(G120=H120,C120&gt;0,ABS(C120-'Prices'!H120)&lt;=MAX(0.01,'Prices'!H120*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J120" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K120" s="34" t="str"/>
+      <x:c r="L120" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="50" customHeight="1">
+      <x:c r="A121" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B121" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C121" s="29" t="n">
+        <x:v>5773</x:v>
+      </x:c>
+      <x:c r="D121" s="29" t="n">
+        <x:v>5773</x:v>
+      </x:c>
+      <x:c r="E121" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F121" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G121" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H121" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I121" s="12" t="str">
+        <x:f>IF(AND(G121=H121,C121&gt;0,ABS(C121-'Prices'!H121)&lt;=MAX(0.01,'Prices'!H121*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J121" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K121" s="36" t="str"/>
+      <x:c r="L121" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="50" customHeight="1">
+      <x:c r="A122" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B122" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C122" s="15" t="n">
+        <x:v>104.15</x:v>
+      </x:c>
+      <x:c r="D122" s="15" t="n">
+        <x:v>104.15</x:v>
+      </x:c>
+      <x:c r="E122" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F122" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G122" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H122" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I122" s="11" t="str">
+        <x:f>IF(AND(G122=H122,C122&gt;0,ABS(C122-'Prices'!H122)&lt;=MAX(0.01,'Prices'!H122*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J122" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K122" s="34" t="str"/>
+      <x:c r="L122" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="50" customHeight="1">
+      <x:c r="A123" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B123" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C123" s="29" t="n">
+        <x:v>7811.54</x:v>
+      </x:c>
+      <x:c r="D123" s="29" t="n">
+        <x:v>7811.54</x:v>
+      </x:c>
+      <x:c r="E123" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F123" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G123" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H123" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I123" s="12" t="str">
+        <x:f>IF(AND(G123=H123,C123&gt;0,ABS(C123-'Prices'!H123)&lt;=MAX(0.01,'Prices'!H123*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J123" s="36" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K123" s="36" t="str"/>
+      <x:c r="L123" s="37" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="50" customHeight="1">
+      <x:c r="A124" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B124" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C124" s="15" t="n">
+        <x:v>27366.1699</x:v>
+      </x:c>
+      <x:c r="D124" s="15" t="n">
+        <x:v>27366.1699</x:v>
+      </x:c>
+      <x:c r="E124" s="15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F124" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G124" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H124" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I124" s="11" t="str">
+        <x:f>IF(AND(G124=H124,C124&gt;0,ABS(C124-'Prices'!H124)&lt;=MAX(0.01,'Prices'!H124*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J124" s="34" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-10T11-34-55-985Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K124" s="34" t="str"/>
+      <x:c r="L124" s="35" t="n">
+        <x:v>46305.48259241898</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -11614,7 +13399,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R224fe760f8dd4437"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2454f733afb4461"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14661,6 +16446,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="108" ht="27" customHeight="1">
+      <x:c r="A108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B108" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C108" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D108" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E108" s="17" t="n">
+        <x:f>'Source Audit'!E108</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F108" s="38" t="n">
+        <x:f>'Source Audit'!F108</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G108" s="11" t="str">
+        <x:f>IF(AND(E108=0,F108=1,'Source Audit'!G108='Source Audit'!H108),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H108" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="27" customHeight="1">
+      <x:c r="A109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B109" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C109" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D109" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E109" s="16" t="n">
+        <x:f>'Source Audit'!E109</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F109" s="39" t="n">
+        <x:f>'Source Audit'!F109</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G109" s="12" t="str">
+        <x:f>IF(AND(E109=0,F109=1,'Source Audit'!G109='Source Audit'!H109),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H109" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="27" customHeight="1">
+      <x:c r="A110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B110" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C110" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D110" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E110" s="17" t="n">
+        <x:f>'Source Audit'!E110</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F110" s="38" t="n">
+        <x:f>'Source Audit'!F110</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G110" s="11" t="str">
+        <x:f>IF(AND(E110=0,F110=1,'Source Audit'!G110='Source Audit'!H110),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H110" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="27" customHeight="1">
+      <x:c r="A111" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B111" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C111" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D111" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E111" s="16" t="n">
+        <x:f>'Source Audit'!E111</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F111" s="39" t="n">
+        <x:f>'Source Audit'!F111</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G111" s="12" t="str">
+        <x:f>IF(AND(E111=0,F111=1,'Source Audit'!G111='Source Audit'!H111),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H111" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="27" customHeight="1">
+      <x:c r="A112" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B112" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C112" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D112" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E112" s="17" t="n">
+        <x:f>'Source Audit'!E112</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F112" s="38" t="n">
+        <x:f>'Source Audit'!F112</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G112" s="11" t="str">
+        <x:f>IF(AND(E112=0,F112=1,'Source Audit'!G112='Source Audit'!H112),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H112" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="27" customHeight="1">
+      <x:c r="A113" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B113" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C113" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D113" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E113" s="16" t="n">
+        <x:f>'Source Audit'!E113</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F113" s="39" t="n">
+        <x:f>'Source Audit'!F113</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G113" s="12" t="str">
+        <x:f>IF(AND(E113=0,F113=1,'Source Audit'!G113='Source Audit'!H113),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H113" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="27" customHeight="1">
+      <x:c r="A114" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B114" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C114" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D114" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E114" s="17" t="n">
+        <x:f>'Source Audit'!E114</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F114" s="38" t="n">
+        <x:f>'Source Audit'!F114</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G114" s="11" t="str">
+        <x:f>IF(AND(E114=0,F114=1,'Source Audit'!G114='Source Audit'!H114),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H114" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="27" customHeight="1">
+      <x:c r="A115" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B115" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C115" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D115" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E115" s="16" t="n">
+        <x:f>'Source Audit'!E115</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F115" s="39" t="n">
+        <x:f>'Source Audit'!F115</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G115" s="12" t="str">
+        <x:f>IF(AND(E115=0,F115=1,'Source Audit'!G115='Source Audit'!H115),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H115" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="27" customHeight="1">
+      <x:c r="A116" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B116" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C116" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D116" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E116" s="17" t="n">
+        <x:f>'Source Audit'!E116</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F116" s="38" t="n">
+        <x:f>'Source Audit'!F116</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G116" s="11" t="str">
+        <x:f>IF(AND(E116=0,F116=1,'Source Audit'!G116='Source Audit'!H116),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H116" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="27" customHeight="1">
+      <x:c r="A117" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B117" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C117" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D117" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E117" s="16" t="n">
+        <x:f>'Source Audit'!E117</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F117" s="39" t="n">
+        <x:f>'Source Audit'!F117</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G117" s="12" t="str">
+        <x:f>IF(AND(E117=0,F117=1,'Source Audit'!G117='Source Audit'!H117),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H117" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="27" customHeight="1">
+      <x:c r="A118" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B118" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C118" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D118" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E118" s="17" t="n">
+        <x:f>'Source Audit'!E118</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F118" s="38" t="n">
+        <x:f>'Source Audit'!F118</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G118" s="11" t="str">
+        <x:f>IF(AND(E118=0,F118=1,'Source Audit'!G118='Source Audit'!H118),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H118" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="27" customHeight="1">
+      <x:c r="A119" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B119" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C119" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D119" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E119" s="16" t="n">
+        <x:f>'Source Audit'!E119</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F119" s="39" t="n">
+        <x:f>'Source Audit'!F119</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G119" s="12" t="str">
+        <x:f>IF(AND(E119=0,F119=1,'Source Audit'!G119='Source Audit'!H119),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H119" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="27" customHeight="1">
+      <x:c r="A120" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B120" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C120" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D120" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E120" s="17" t="n">
+        <x:f>'Source Audit'!E120</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F120" s="38" t="n">
+        <x:f>'Source Audit'!F120</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G120" s="11" t="str">
+        <x:f>IF(AND(E120=0,F120=1,'Source Audit'!G120='Source Audit'!H120),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H120" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="27" customHeight="1">
+      <x:c r="A121" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B121" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C121" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D121" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E121" s="16" t="n">
+        <x:f>'Source Audit'!E121</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F121" s="39" t="n">
+        <x:f>'Source Audit'!F121</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G121" s="12" t="str">
+        <x:f>IF(AND(E121=0,F121=1,'Source Audit'!G121='Source Audit'!H121),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H121" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="27" customHeight="1">
+      <x:c r="A122" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B122" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C122" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D122" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E122" s="17" t="n">
+        <x:f>'Source Audit'!E122</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F122" s="38" t="n">
+        <x:f>'Source Audit'!F122</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G122" s="11" t="str">
+        <x:f>IF(AND(E122=0,F122=1,'Source Audit'!G122='Source Audit'!H122),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H122" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="27" customHeight="1">
+      <x:c r="A123" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B123" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C123" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D123" s="9" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E123" s="16" t="n">
+        <x:f>'Source Audit'!E123</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F123" s="39" t="n">
+        <x:f>'Source Audit'!F123</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G123" s="12" t="str">
+        <x:f>IF(AND(E123=0,F123=1,'Source Audit'!G123='Source Audit'!H123),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H123" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="27" customHeight="1">
+      <x:c r="A124" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="B124" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C124" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D124" s="8" t="n">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="E124" s="17" t="n">
+        <x:f>'Source Audit'!E124</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F124" s="38" t="n">
+        <x:f>'Source Audit'!F124</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G124" s="11" t="str">
+        <x:f>IF(AND(E124=0,F124=1,'Source Audit'!G124='Source Audit'!H124),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H124" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -14668,7 +16946,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cecb59157ad45b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda79b6ca9b38422b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 through October 14 and improve mobile date labels
Append audited October 14 closes and extend the cumulative five-sheet review workbook and website series to ten trading dates. Preserve earlier history and record the approved Ouster provider MIC exception in the immutable audit trail. Space chart date labels evenly to avoid mobile overlaps.

Validation: 17 requested prices and 138 historical comparisons passed; workbook formulas and website data reconcile; type checking, production build, desktop/mobile and holdings CSV checks passed. Repository lint retains seven pre-existing errors and eight warnings in unrelated files.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6bed6836b4884a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R4083a1d2648d40aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R83bb3fca3278439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R7461f72ebf834d65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Ra84706d725144868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5159a61a9d084f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rfb55181f591a49d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R03cc6846f4a04ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R83c25ceea5464faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rfb1cf0dac3474941"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K158" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H140" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H155" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M158" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H158" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1392,6 +1392,85 @@
         <x:v>-4.474388089849435</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="40" customHeight="1">
+      <x:c r="A15" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B15" s="18" t="n">
+        <x:f>B14*(1+SUM('Returns and Contributions'!F141:F155))</x:f>
+        <x:v>946.463158801601</x:v>
+      </x:c>
+      <x:c r="C15" s="21" t="n">
+        <x:f>B15/B14-1</x:f>
+        <x:v>-0.021885438336927132</x:v>
+      </x:c>
+      <x:c r="D15" s="21" t="n">
+        <x:f>B15/$B$6-1</x:f>
+        <x:v>-0.053536841198398966</x:v>
+      </x:c>
+      <x:c r="E15" s="18" t="n">
+        <x:f>1000*'Prices'!H174/'Prices'!I174</x:f>
+        <x:v>1006.8467152332566</x:v>
+      </x:c>
+      <x:c r="F15" s="21" t="n">
+        <x:f>E15/E14-1</x:f>
+        <x:v>-0.01108328155327365</x:v>
+      </x:c>
+      <x:c r="G15" s="21" t="n">
+        <x:f>E15/1000-1</x:f>
+        <x:v>0.0068467152332567505</x:v>
+      </x:c>
+      <x:c r="H15" s="18" t="n">
+        <x:f>1000*'Prices'!H175/'Prices'!I175</x:f>
+        <x:v>993.3488653969291</x:v>
+      </x:c>
+      <x:c r="I15" s="21" t="n">
+        <x:f>H15/H14-1</x:f>
+        <x:v>-0.01880255249624141</x:v>
+      </x:c>
+      <x:c r="J15" s="21" t="n">
+        <x:f>H15/1000-1</x:f>
+        <x:v>-0.006651134603070874</x:v>
+      </x:c>
+      <x:c r="K15" s="25" t="n">
+        <x:f>(C15-F15)*100</x:f>
+        <x:v>-1.0802156783653483</x:v>
+      </x:c>
+      <x:c r="L15" s="25" t="n">
+        <x:f>(C15-I15)*100</x:f>
+        <x:v>-0.3082885840685723</x:v>
+      </x:c>
+      <x:c r="M15" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G141:G155)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N15" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F141:F155)-C15</x:f>
+        <x:v>1.734723475976807e-17</x:v>
+      </x:c>
+      <x:c r="O15" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P15" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I159:I175,"Mismatch")=0,IF(COUNTIF('Source Audit'!I159:I175,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q15" s="30" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="R15" s="27" t="n">
+        <x:f>B15-1000*('Prices'!H159/'Prices'!H6+'Prices'!H160/'Prices'!H7+'Prices'!H161/'Prices'!H8+'Prices'!H162/'Prices'!H9+'Prices'!H163/'Prices'!H10+'Prices'!H164/'Prices'!H11+'Prices'!H165/'Prices'!H12+'Prices'!H166/'Prices'!H13+'Prices'!H167/'Prices'!H14+'Prices'!H168/'Prices'!H15+'Prices'!H169/'Prices'!H16+'Prices'!H170/'Prices'!H17+'Prices'!H171/'Prices'!H18+'Prices'!H172/'Prices'!H19+'Prices'!H173/'Prices'!H20)/15</x:f>
+        <x:v>-1.1368683772161603e-13</x:v>
+      </x:c>
+      <x:c r="S15" s="25" t="n">
+        <x:f>(D15-G15)*100</x:f>
+        <x:v>-6.038355643165572</x:v>
+      </x:c>
+      <x:c r="T15" s="25" t="n">
+        <x:f>(D15-J15)*100</x:f>
+        <x:v>-4.688570659532809</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1399,7 +1478,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60caaa334d1b4fff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cb04974e0404d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6969,6 +7048,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="159" ht="27" customHeight="1">
+      <x:c r="A159" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B159" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C159" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D159" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E159" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F159" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G159" s="33" t="n">
+        <x:f>H142</x:f>
+        <x:v>6192</x:v>
+      </x:c>
+      <x:c r="H159" s="35" t="n">
+        <x:v>6250</x:v>
+      </x:c>
+      <x:c r="I159" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J159" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K159" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="27" customHeight="1">
+      <x:c r="A160" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B160" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C160" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D160" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E160" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F160" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G160" s="17" t="n">
+        <x:f>H143</x:f>
+        <x:v>4840</x:v>
+      </x:c>
+      <x:c r="H160" s="34" t="n">
+        <x:v>4712</x:v>
+      </x:c>
+      <x:c r="I160" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J160" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K160" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="27" customHeight="1">
+      <x:c r="A161" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B161" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C161" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D161" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E161" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F161" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G161" s="33" t="n">
+        <x:f>H144</x:f>
+        <x:v>25.88</x:v>
+      </x:c>
+      <x:c r="H161" s="35" t="n">
+        <x:v>25.22</x:v>
+      </x:c>
+      <x:c r="I161" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J161" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K161" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="27" customHeight="1">
+      <x:c r="A162" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B162" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C162" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D162" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E162" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F162" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G162" s="17" t="n">
+        <x:f>H145</x:f>
+        <x:v>380.29</x:v>
+      </x:c>
+      <x:c r="H162" s="34" t="n">
+        <x:v>359.44</x:v>
+      </x:c>
+      <x:c r="I162" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J162" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K162" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="27" customHeight="1">
+      <x:c r="A163" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B163" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C163" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D163" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E163" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F163" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G163" s="33" t="n">
+        <x:f>H146</x:f>
+        <x:v>4862</x:v>
+      </x:c>
+      <x:c r="H163" s="35" t="n">
+        <x:v>4826</x:v>
+      </x:c>
+      <x:c r="I163" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J163" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K163" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="27" customHeight="1">
+      <x:c r="A164" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B164" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C164" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D164" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E164" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F164" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G164" s="17" t="n">
+        <x:f>H147</x:f>
+        <x:v>50.89</x:v>
+      </x:c>
+      <x:c r="H164" s="34" t="n">
+        <x:v>49.33</x:v>
+      </x:c>
+      <x:c r="I164" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J164" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K164" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="27" customHeight="1">
+      <x:c r="A165" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B165" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C165" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D165" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E165" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F165" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G165" s="33" t="n">
+        <x:f>H148</x:f>
+        <x:v>79770</x:v>
+      </x:c>
+      <x:c r="H165" s="35" t="n">
+        <x:v>80330</x:v>
+      </x:c>
+      <x:c r="I165" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J165" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K165" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="27" customHeight="1">
+      <x:c r="A166" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B166" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C166" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D166" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E166" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F166" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G166" s="17" t="n">
+        <x:f>H149</x:f>
+        <x:v>60.01</x:v>
+      </x:c>
+      <x:c r="H166" s="34" t="n">
+        <x:v>57.27</x:v>
+      </x:c>
+      <x:c r="I166" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J166" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K166" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="27" customHeight="1">
+      <x:c r="A167" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B167" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C167" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D167" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E167" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F167" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G167" s="33" t="n">
+        <x:f>H150</x:f>
+        <x:v>35.33</x:v>
+      </x:c>
+      <x:c r="H167" s="35" t="n">
+        <x:v>31.87</x:v>
+      </x:c>
+      <x:c r="I167" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J167" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K167" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="27" customHeight="1">
+      <x:c r="A168" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B168" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C168" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D168" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E168" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F168" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G168" s="17" t="n">
+        <x:f>H151</x:f>
+        <x:v>14.46</x:v>
+      </x:c>
+      <x:c r="H168" s="34" t="n">
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="I168" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J168" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K168" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="27" customHeight="1">
+      <x:c r="A169" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B169" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C169" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D169" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E169" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F169" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G169" s="33" t="n">
+        <x:f>H152</x:f>
+        <x:v>432.29</x:v>
+      </x:c>
+      <x:c r="H169" s="35" t="n">
+        <x:v>423.42</x:v>
+      </x:c>
+      <x:c r="I169" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J169" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K169" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="27" customHeight="1">
+      <x:c r="A170" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B170" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C170" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D170" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E170" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F170" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G170" s="17" t="n">
+        <x:f>H153</x:f>
+        <x:v>274.5</x:v>
+      </x:c>
+      <x:c r="H170" s="34" t="n">
+        <x:v>275.05</x:v>
+      </x:c>
+      <x:c r="I170" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J170" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K170" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="27" customHeight="1">
+      <x:c r="A171" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B171" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C171" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D171" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E171" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F171" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G171" s="33" t="n">
+        <x:f>H154</x:f>
+        <x:v>226.32</x:v>
+      </x:c>
+      <x:c r="H171" s="35" t="n">
+        <x:v>220.83</x:v>
+      </x:c>
+      <x:c r="I171" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J171" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K171" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="27" customHeight="1">
+      <x:c r="A172" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B172" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C172" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D172" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E172" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F172" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G172" s="17" t="n">
+        <x:f>H155</x:f>
+        <x:v>5806</x:v>
+      </x:c>
+      <x:c r="H172" s="34" t="n">
+        <x:v>5864</x:v>
+      </x:c>
+      <x:c r="I172" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J172" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K172" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="27" customHeight="1">
+      <x:c r="A173" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B173" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C173" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D173" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E173" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F173" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G173" s="33" t="n">
+        <x:f>H156</x:f>
+        <x:v>104.4</x:v>
+      </x:c>
+      <x:c r="H173" s="35" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="I173" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J173" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K173" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="27" customHeight="1">
+      <x:c r="A174" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B174" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C174" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D174" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E174" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F174" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G174" s="17" t="n">
+        <x:f>H157</x:f>
+        <x:v>7805.45</x:v>
+      </x:c>
+      <x:c r="H174" s="34" t="n">
+        <x:v>7718.94</x:v>
+      </x:c>
+      <x:c r="I174" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J174" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K174" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="27" customHeight="1">
+      <x:c r="A175" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B175" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C175" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D175" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E175" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F175" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G175" s="33" t="n">
+        <x:f>H158</x:f>
+        <x:v>27204.3809</x:v>
+      </x:c>
+      <x:c r="H175" s="35" t="n">
+        <x:v>26692.8691</x:v>
+      </x:c>
+      <x:c r="I175" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J175" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="K175" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -6976,7 +7667,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0df629115b0c4f8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108966b65d134973"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11160,6 +11851,471 @@
         <x:v>0.054332458089275004</x:v>
       </x:c>
     </x:row>
+    <x:row r="141" ht="27" customHeight="1">
+      <x:c r="A141" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B141" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C141" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D141" s="21" t="n">
+        <x:f>G126</x:f>
+        <x:v>0.06962702178517538</x:v>
+      </x:c>
+      <x:c r="E141" s="23" t="n">
+        <x:f>'Prices'!H159/'Prices'!G159-1</x:f>
+        <x:v>0.009366925064599574</x:v>
+      </x:c>
+      <x:c r="F141" s="21" t="n">
+        <x:f>D141*E141</x:f>
+        <x:v>0.0006521910955329798</x:v>
+      </x:c>
+      <x:c r="G141" s="21" t="n">
+        <x:f>D141*(1+E141)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.07185171925179573</x:v>
+      </x:c>
+      <x:c r="H141" s="23" t="n">
+        <x:f>'Prices'!H159/'Prices'!I159-1</x:f>
+        <x:v>0.02007507752570592</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="27" customHeight="1">
+      <x:c r="A142" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B142" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C142" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D142" s="20" t="n">
+        <x:f>G127</x:f>
+        <x:v>0.06977552018846739</x:v>
+      </x:c>
+      <x:c r="E142" s="22" t="n">
+        <x:f>'Prices'!H160/'Prices'!G160-1</x:f>
+        <x:v>-0.026446280991735516</x:v>
+      </x:c>
+      <x:c r="F142" s="20" t="n">
+        <x:f>D142*E142</x:f>
+        <x:v>-0.0018453030132487228</x:v>
+      </x:c>
+      <x:c r="G142" s="20" t="n">
+        <x:f>D142*(1+E142)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.069450164467154</x:v>
+      </x:c>
+      <x:c r="H142" s="22" t="n">
+        <x:f>'Prices'!H160/'Prices'!I160-1</x:f>
+        <x:v>-0.014019669386901024</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="27" customHeight="1">
+      <x:c r="A143" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B143" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C143" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D143" s="21" t="n">
+        <x:f>G128</x:f>
+        <x:v>0.06318325772838658</x:v>
+      </x:c>
+      <x:c r="E143" s="23" t="n">
+        <x:f>'Prices'!H161/'Prices'!G161-1</x:f>
+        <x:v>-0.025502318392581103</x:v>
+      </x:c>
+      <x:c r="F143" s="21" t="n">
+        <x:f>D143*E143</x:f>
+        <x:v>-0.0016113195556698252</x:v>
+      </x:c>
+      <x:c r="G143" s="21" t="n">
+        <x:f>D143*(1+E143)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06294961815927468</x:v>
+      </x:c>
+      <x:c r="H143" s="23" t="n">
+        <x:f>'Prices'!H161/'Prices'!I161-1</x:f>
+        <x:v>-0.10630758327427359</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="27" customHeight="1">
+      <x:c r="A144" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B144" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C144" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D144" s="20" t="n">
+        <x:f>G129</x:f>
+        <x:v>0.06301379230687061</x:v>
+      </x:c>
+      <x:c r="E144" s="22" t="n">
+        <x:f>'Prices'!H162/'Prices'!G162-1</x:f>
+        <x:v>-0.05482657971548033</x:v>
+      </x:c>
+      <x:c r="F144" s="20" t="n">
+        <x:f>D144*E144</x:f>
+        <x:v>-0.0034548307070873625</x:v>
+      </x:c>
+      <x:c r="G144" s="20" t="n">
+        <x:f>D144*(1+E144)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06089160097822906</x:v>
+      </x:c>
+      <x:c r="H144" s="22" t="n">
+        <x:f>'Prices'!H162/'Prices'!I162-1</x:f>
+        <x:v>-0.13552514490487988</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="27" customHeight="1">
+      <x:c r="A145" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B145" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C145" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D145" s="21" t="n">
+        <x:f>G130</x:f>
+        <x:v>0.06733124132181952</x:v>
+      </x:c>
+      <x:c r="E145" s="23" t="n">
+        <x:f>'Prices'!H163/'Prices'!G163-1</x:f>
+        <x:v>-0.00740436034553682</x:v>
+      </x:c>
+      <x:c r="F145" s="21" t="n">
+        <x:f>D145*E145</x:f>
+        <x:v>-0.0004985447732590506</x:v>
+      </x:c>
+      <x:c r="G145" s="21" t="n">
+        <x:f>D145*(1+E145)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.0683280866761925</x:v>
+      </x:c>
+      <x:c r="H145" s="23" t="n">
+        <x:f>'Prices'!H163/'Prices'!I163-1</x:f>
+        <x:v>-0.029949748743718585</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="27" customHeight="1">
+      <x:c r="A146" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B146" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C146" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D146" s="20" t="n">
+        <x:f>G131</x:f>
+        <x:v>0.06755536500106327</x:v>
+      </x:c>
+      <x:c r="E146" s="22" t="n">
+        <x:f>'Prices'!H164/'Prices'!G164-1</x:f>
+        <x:v>-0.030654352525054107</x:v>
+      </x:c>
+      <x:c r="F146" s="20" t="n">
+        <x:f>D146*E146</x:f>
+        <x:v>-0.0020708659737012957</x:v>
+      </x:c>
+      <x:c r="G146" s="20" t="n">
+        <x:f>D146*(1+E146)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06694972306313456</x:v>
+      </x:c>
+      <x:c r="H146" s="22" t="n">
+        <x:f>'Prices'!H164/'Prices'!I164-1</x:f>
+        <x:v>-0.049518304431599214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="27" customHeight="1">
+      <x:c r="A147" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B147" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C147" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D147" s="21" t="n">
+        <x:f>G132</x:f>
+        <x:v>0.06768279963748645</x:v>
+      </x:c>
+      <x:c r="E147" s="23" t="n">
+        <x:f>'Prices'!H165/'Prices'!G165-1</x:f>
+        <x:v>0.007020183026200222</x:v>
+      </x:c>
+      <x:c r="F147" s="21" t="n">
+        <x:f>D147*E147</x:f>
+        <x:v>0.0004751456411807929</x:v>
+      </x:c>
+      <x:c r="G147" s="21" t="n">
+        <x:f>D147*(1+E147)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.0696829880160248</x:v>
+      </x:c>
+      <x:c r="H147" s="23" t="n">
+        <x:f>'Prices'!H165/'Prices'!I165-1</x:f>
+        <x:v>-0.010714285714285676</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="27" customHeight="1">
+      <x:c r="A148" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B148" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C148" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D148" s="20" t="n">
+        <x:f>G133</x:f>
+        <x:v>0.06644898809792142</x:v>
+      </x:c>
+      <x:c r="E148" s="22" t="n">
+        <x:f>'Prices'!H166/'Prices'!G166-1</x:f>
+        <x:v>-0.04565905682386262</x:v>
+      </x:c>
+      <x:c r="F148" s="20" t="n">
+        <x:f>D148*E148</x:f>
+        <x:v>-0.003033998123451165</x:v>
+      </x:c>
+      <x:c r="G148" s="20" t="n">
+        <x:f>D148*(1+E148)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06483390848066585</x:v>
+      </x:c>
+      <x:c r="H148" s="22" t="n">
+        <x:f>'Prices'!H166/'Prices'!I166-1</x:f>
+        <x:v>-0.07955641272902592</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="27" customHeight="1">
+      <x:c r="A149" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B149" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C149" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D149" s="21" t="n">
+        <x:f>G134</x:f>
+        <x:v>0.05955712864994033</x:v>
+      </x:c>
+      <x:c r="E149" s="23" t="n">
+        <x:f>'Prices'!H167/'Prices'!G167-1</x:f>
+        <x:v>-0.09793376733654113</x:v>
+      </x:c>
+      <x:c r="F149" s="21" t="n">
+        <x:f>D149*E149</x:f>
+        <x:v>-0.005832653980435705</x:v>
+      </x:c>
+      <x:c r="G149" s="21" t="n">
+        <x:f>D149*(1+E149)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.05492656665713855</x:v>
+      </x:c>
+      <x:c r="H149" s="23" t="n">
+        <x:f>'Prices'!H167/'Prices'!I167-1</x:f>
+        <x:v>-0.22021042329336915</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="27" customHeight="1">
+      <x:c r="A150" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B150" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C150" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D150" s="20" t="n">
+        <x:f>G135</x:f>
+        <x:v>0.06253847243338254</x:v>
+      </x:c>
+      <x:c r="E150" s="22" t="n">
+        <x:f>'Prices'!H168/'Prices'!G168-1</x:f>
+        <x:v>-0.03596127247579539</x:v>
+      </x:c>
+      <x:c r="F150" s="20" t="n">
+        <x:f>D150*E150</x:f>
+        <x:v>-0.002248963047396888</x:v>
+      </x:c>
+      <x:c r="G150" s="20" t="n">
+        <x:f>D150*(1+E150)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06163849486452419</x:v>
+      </x:c>
+      <x:c r="H150" s="22" t="n">
+        <x:f>'Prices'!H168/'Prices'!I168-1</x:f>
+        <x:v>-0.12492153170119269</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="27" customHeight="1">
+      <x:c r="A151" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B151" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C151" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D151" s="21" t="n">
+        <x:f>G136</x:f>
+        <x:v>0.06731405319872744</x:v>
+      </x:c>
+      <x:c r="E151" s="23" t="n">
+        <x:f>'Prices'!H169/'Prices'!G169-1</x:f>
+        <x:v>-0.020518633324851376</x:v>
+      </x:c>
+      <x:c r="F151" s="21" t="n">
+        <x:f>D151*E151</x:f>
+        <x:v>-0.001381192375194227</x:v>
+      </x:c>
+      <x:c r="G151" s="21" t="n">
+        <x:f>D151*(1+E151)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.0674081170118034</x:v>
+      </x:c>
+      <x:c r="H151" s="23" t="n">
+        <x:f>'Prices'!H169/'Prices'!I169-1</x:f>
+        <x:v>-0.04301050966210862</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="27" customHeight="1">
+      <x:c r="A152" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B152" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C152" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D152" s="20" t="n">
+        <x:f>G137</x:f>
+        <x:v>0.06955492601360354</x:v>
+      </x:c>
+      <x:c r="E152" s="22" t="n">
+        <x:f>'Prices'!H170/'Prices'!G170-1</x:f>
+        <x:v>0.002003642987249643</x:v>
+      </x:c>
+      <x:c r="F152" s="20" t="n">
+        <x:f>D152*E152</x:f>
+        <x:v>0.0001393632397358245</x:v>
+      </x:c>
+      <x:c r="G152" s="20" t="n">
+        <x:f>D152*(1+E152)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.07125370788350113</x:v>
+      </x:c>
+      <x:c r="H152" s="22" t="n">
+        <x:f>'Prices'!H170/'Prices'!I170-1</x:f>
+        <x:v>0.011585141596175186</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="27" customHeight="1">
+      <x:c r="A153" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B153" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C153" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D153" s="21" t="n">
+        <x:f>G138</x:f>
+        <x:v>0.06518905229836365</x:v>
+      </x:c>
+      <x:c r="E153" s="23" t="n">
+        <x:f>'Prices'!H171/'Prices'!G171-1</x:f>
+        <x:v>-0.024257688229056162</x:v>
+      </x:c>
+      <x:c r="F153" s="21" t="n">
+        <x:f>D153*E153</x:f>
+        <x:v>-0.0015813357066013424</x:v>
+      </x:c>
+      <x:c r="G153" s="21" t="n">
+        <x:f>D153*(1+E153)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.06503094738065356</x:v>
+      </x:c>
+      <x:c r="H153" s="23" t="n">
+        <x:f>'Prices'!H171/'Prices'!I171-1</x:f>
+        <x:v>-0.07675906183368864</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="27" customHeight="1">
+      <x:c r="A154" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B154" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C154" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D154" s="20" t="n">
+        <x:f>G139</x:f>
+        <x:v>0.06858896792539093</x:v>
+      </x:c>
+      <x:c r="E154" s="22" t="n">
+        <x:f>'Prices'!H172/'Prices'!G172-1</x:f>
+        <x:v>0.009989665862900399</x:v>
+      </x:c>
+      <x:c r="F154" s="20" t="n">
+        <x:f>D154*E154</x:f>
+        <x:v>0.0006851808714558482</x:v>
+      </x:c>
+      <x:c r="G154" s="20" t="n">
+        <x:f>D154*(1+E154)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.07082416673059343</x:v>
+      </x:c>
+      <x:c r="H154" s="22" t="n">
+        <x:f>'Prices'!H172/'Prices'!I172-1</x:f>
+        <x:v>0.005486968449931462</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="27" customHeight="1">
+      <x:c r="A155" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B155" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C155" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D155" s="21" t="n">
+        <x:f>G140</x:f>
+        <x:v>0.07263941341340083</x:v>
+      </x:c>
+      <x:c r="E155" s="23" t="n">
+        <x:f>'Prices'!H173/'Prices'!G173-1</x:f>
+        <x:v>-0.003831417624521105</x:v>
+      </x:c>
+      <x:c r="F155" s="21" t="n">
+        <x:f>D155*E155</x:f>
+        <x:v>-0.0002783119287869787</x:v>
+      </x:c>
+      <x:c r="G155" s="21" t="n">
+        <x:f>D155*(1+E155)/(1+SUM($F$141:$F$155))</x:f>
+        <x:v>0.07398019037931446</x:v>
+      </x:c>
+      <x:c r="H155" s="23" t="n">
+        <x:f>'Prices'!H173/'Prices'!I173-1</x:f>
+        <x:v>0.05029287012724715</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -11167,7 +12323,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20a5b59a3f8e4605"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5615d0c33874d17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17158,6 +18314,654 @@
       </x:c>
       <x:c r="M158" s="14" t="str"/>
     </x:row>
+    <x:row r="159" ht="50" customHeight="1">
+      <x:c r="A159" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B159" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C159" s="33" t="n">
+        <x:v>6250</x:v>
+      </x:c>
+      <x:c r="D159" s="33" t="n">
+        <x:v>6250</x:v>
+      </x:c>
+      <x:c r="E159" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F159" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G159" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H159" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I159" s="32" t="str">
+        <x:f>IF(AND(G159=H159,C159&gt;0,ABS(C159-'Prices'!H159)&lt;=MAX(0.01,'Prices'!H159*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J159" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K159" s="16" t="str"/>
+      <x:c r="L159" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M159" s="16" t="str"/>
+    </x:row>
+    <x:row r="160" ht="50" customHeight="1">
+      <x:c r="A160" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B160" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C160" s="17" t="n">
+        <x:v>4712</x:v>
+      </x:c>
+      <x:c r="D160" s="17" t="n">
+        <x:v>4712</x:v>
+      </x:c>
+      <x:c r="E160" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F160" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G160" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H160" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I160" s="31" t="str">
+        <x:f>IF(AND(G160=H160,C160&gt;0,ABS(C160-'Prices'!H160)&lt;=MAX(0.01,'Prices'!H160*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J160" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K160" s="14" t="str"/>
+      <x:c r="L160" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M160" s="14" t="str"/>
+    </x:row>
+    <x:row r="161" ht="50" customHeight="1">
+      <x:c r="A161" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B161" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C161" s="33" t="n">
+        <x:v>25.22</x:v>
+      </x:c>
+      <x:c r="D161" s="33" t="n">
+        <x:v>25.22</x:v>
+      </x:c>
+      <x:c r="E161" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F161" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G161" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H161" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I161" s="32" t="str">
+        <x:f>IF(AND(G161=H161,C161&gt;0,ABS(C161-'Prices'!H161)&lt;=MAX(0.01,'Prices'!H161*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J161" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K161" s="16" t="str"/>
+      <x:c r="L161" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M161" s="16" t="str"/>
+    </x:row>
+    <x:row r="162" ht="50" customHeight="1">
+      <x:c r="A162" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B162" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C162" s="17" t="n">
+        <x:v>359.44</x:v>
+      </x:c>
+      <x:c r="D162" s="17" t="n">
+        <x:v>359.44</x:v>
+      </x:c>
+      <x:c r="E162" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F162" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G162" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H162" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I162" s="31" t="str">
+        <x:f>IF(AND(G162=H162,C162&gt;0,ABS(C162-'Prices'!H162)&lt;=MAX(0.01,'Prices'!H162*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J162" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K162" s="14" t="str"/>
+      <x:c r="L162" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M162" s="14" t="str"/>
+    </x:row>
+    <x:row r="163" ht="50" customHeight="1">
+      <x:c r="A163" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B163" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C163" s="33" t="n">
+        <x:v>4826</x:v>
+      </x:c>
+      <x:c r="D163" s="33" t="n">
+        <x:v>4826</x:v>
+      </x:c>
+      <x:c r="E163" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F163" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G163" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H163" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I163" s="32" t="str">
+        <x:f>IF(AND(G163=H163,C163&gt;0,ABS(C163-'Prices'!H163)&lt;=MAX(0.01,'Prices'!H163*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J163" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K163" s="16" t="str"/>
+      <x:c r="L163" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M163" s="16" t="str"/>
+    </x:row>
+    <x:row r="164" ht="50" customHeight="1">
+      <x:c r="A164" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B164" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C164" s="17" t="n">
+        <x:v>49.33</x:v>
+      </x:c>
+      <x:c r="D164" s="17" t="n">
+        <x:v>49.33</x:v>
+      </x:c>
+      <x:c r="E164" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F164" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G164" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H164" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I164" s="31" t="str">
+        <x:f>IF(AND(G164=H164,C164&gt;0,ABS(C164-'Prices'!H164)&lt;=MAX(0.01,'Prices'!H164*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J164" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K164" s="14" t="str"/>
+      <x:c r="L164" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M164" s="14" t="str"/>
+    </x:row>
+    <x:row r="165" ht="50" customHeight="1">
+      <x:c r="A165" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B165" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C165" s="33" t="n">
+        <x:v>80330</x:v>
+      </x:c>
+      <x:c r="D165" s="33" t="n">
+        <x:v>80330</x:v>
+      </x:c>
+      <x:c r="E165" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F165" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G165" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H165" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I165" s="32" t="str">
+        <x:f>IF(AND(G165=H165,C165&gt;0,ABS(C165-'Prices'!H165)&lt;=MAX(0.01,'Prices'!H165*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J165" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K165" s="16" t="str"/>
+      <x:c r="L165" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M165" s="16" t="str"/>
+    </x:row>
+    <x:row r="166" ht="50" customHeight="1">
+      <x:c r="A166" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B166" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C166" s="17" t="n">
+        <x:v>57.27</x:v>
+      </x:c>
+      <x:c r="D166" s="17" t="n">
+        <x:v>57.27</x:v>
+      </x:c>
+      <x:c r="E166" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F166" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G166" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H166" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I166" s="31" t="str">
+        <x:f>IF(AND(G166=H166,C166&gt;0,ABS(C166-'Prices'!H166)&lt;=MAX(0.01,'Prices'!H166*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J166" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K166" s="14" t="str"/>
+      <x:c r="L166" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M166" s="14" t="str"/>
+    </x:row>
+    <x:row r="167" ht="50" customHeight="1">
+      <x:c r="A167" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B167" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C167" s="33" t="n">
+        <x:v>31.87</x:v>
+      </x:c>
+      <x:c r="D167" s="33" t="n">
+        <x:v>31.87</x:v>
+      </x:c>
+      <x:c r="E167" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F167" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G167" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H167" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I167" s="32" t="str">
+        <x:f>IF(AND(OR(G167=H167,AND(B167="OUST",G167="XNAS",H167="XNYS",LEFT(M167,34)="ouster-marketstack-legacy-nyse-tag")),C167&gt;0,ABS(C167-'Prices'!H167)&lt;=MAX(0.01,'Prices'!H167*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J167" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K167" s="16" t="str"/>
+      <x:c r="L167" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M167" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="50" customHeight="1">
+      <x:c r="A168" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B168" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C168" s="17" t="n">
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="D168" s="17" t="n">
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="E168" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F168" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G168" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H168" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I168" s="31" t="str">
+        <x:f>IF(AND(G168=H168,C168&gt;0,ABS(C168-'Prices'!H168)&lt;=MAX(0.01,'Prices'!H168*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J168" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K168" s="14" t="str"/>
+      <x:c r="L168" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M168" s="14" t="str"/>
+    </x:row>
+    <x:row r="169" ht="50" customHeight="1">
+      <x:c r="A169" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B169" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C169" s="33" t="n">
+        <x:v>423.42</x:v>
+      </x:c>
+      <x:c r="D169" s="33" t="n">
+        <x:v>423.42</x:v>
+      </x:c>
+      <x:c r="E169" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F169" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G169" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H169" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I169" s="32" t="str">
+        <x:f>IF(AND(G169=H169,C169&gt;0,ABS(C169-'Prices'!H169)&lt;=MAX(0.01,'Prices'!H169*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J169" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K169" s="16" t="str"/>
+      <x:c r="L169" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M169" s="16" t="str"/>
+    </x:row>
+    <x:row r="170" ht="50" customHeight="1">
+      <x:c r="A170" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B170" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C170" s="17" t="n">
+        <x:v>275.05</x:v>
+      </x:c>
+      <x:c r="D170" s="17" t="n">
+        <x:v>275.05</x:v>
+      </x:c>
+      <x:c r="E170" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F170" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G170" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H170" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I170" s="31" t="str">
+        <x:f>IF(AND(G170=H170,C170&gt;0,ABS(C170-'Prices'!H170)&lt;=MAX(0.01,'Prices'!H170*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J170" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K170" s="14" t="str"/>
+      <x:c r="L170" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M170" s="14" t="str"/>
+    </x:row>
+    <x:row r="171" ht="50" customHeight="1">
+      <x:c r="A171" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B171" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C171" s="33" t="n">
+        <x:v>220.83</x:v>
+      </x:c>
+      <x:c r="D171" s="33" t="n">
+        <x:v>220.83</x:v>
+      </x:c>
+      <x:c r="E171" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F171" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G171" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H171" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I171" s="32" t="str">
+        <x:f>IF(AND(G171=H171,C171&gt;0,ABS(C171-'Prices'!H171)&lt;=MAX(0.01,'Prices'!H171*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J171" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K171" s="16" t="str"/>
+      <x:c r="L171" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M171" s="16" t="str"/>
+    </x:row>
+    <x:row r="172" ht="50" customHeight="1">
+      <x:c r="A172" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B172" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C172" s="17" t="n">
+        <x:v>5864</x:v>
+      </x:c>
+      <x:c r="D172" s="17" t="n">
+        <x:v>5864</x:v>
+      </x:c>
+      <x:c r="E172" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F172" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G172" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H172" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I172" s="31" t="str">
+        <x:f>IF(AND(G172=H172,C172&gt;0,ABS(C172-'Prices'!H172)&lt;=MAX(0.01,'Prices'!H172*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J172" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K172" s="14" t="str"/>
+      <x:c r="L172" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M172" s="14" t="str"/>
+    </x:row>
+    <x:row r="173" ht="50" customHeight="1">
+      <x:c r="A173" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B173" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C173" s="33" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="D173" s="33" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="E173" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F173" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G173" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H173" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I173" s="32" t="str">
+        <x:f>IF(AND(G173=H173,C173&gt;0,ABS(C173-'Prices'!H173)&lt;=MAX(0.01,'Prices'!H173*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J173" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K173" s="16" t="str"/>
+      <x:c r="L173" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M173" s="16" t="str"/>
+    </x:row>
+    <x:row r="174" ht="50" customHeight="1">
+      <x:c r="A174" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B174" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C174" s="17" t="n">
+        <x:v>7718.94</x:v>
+      </x:c>
+      <x:c r="D174" s="17" t="n">
+        <x:v>7718.94</x:v>
+      </x:c>
+      <x:c r="E174" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F174" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G174" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H174" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I174" s="31" t="str">
+        <x:f>IF(AND(G174=H174,C174&gt;0,ABS(C174-'Prices'!H174)&lt;=MAX(0.01,'Prices'!H174*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J174" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K174" s="14" t="str"/>
+      <x:c r="L174" s="38" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M174" s="14" t="str"/>
+    </x:row>
+    <x:row r="175" ht="50" customHeight="1">
+      <x:c r="A175" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B175" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C175" s="33" t="n">
+        <x:v>26692.8691</x:v>
+      </x:c>
+      <x:c r="D175" s="33" t="n">
+        <x:v>26692.8691</x:v>
+      </x:c>
+      <x:c r="E175" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F175" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G175" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H175" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I175" s="32" t="str">
+        <x:f>IF(AND(G175=H175,C175&gt;0,ABS(C175-'Prices'!H175)&lt;=MAX(0.01,'Prices'!H175*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J175" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-15T11-44-05-513Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K175" s="16" t="str"/>
+      <x:c r="L175" s="39" t="n">
+        <x:v>46310.48895269676</x:v>
+      </x:c>
+      <x:c r="M175" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -17165,7 +18969,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf84e84f9099640f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44772a4656af41d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21691,6 +23495,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="159" ht="27" customHeight="1">
+      <x:c r="A159" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B159" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C159" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D159" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E159" s="18" t="n">
+        <x:f>'Source Audit'!E159</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F159" s="41" t="n">
+        <x:f>'Source Audit'!F159</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G159" s="12" t="str">
+        <x:f>IF(AND(E159=0,F159=1,'Source Audit'!I159&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H159" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="27" customHeight="1">
+      <x:c r="A160" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B160" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C160" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D160" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E160" s="19" t="n">
+        <x:f>'Source Audit'!E160</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F160" s="40" t="n">
+        <x:f>'Source Audit'!F160</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G160" s="11" t="str">
+        <x:f>IF(AND(E160=0,F160=1,'Source Audit'!I160&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H160" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="27" customHeight="1">
+      <x:c r="A161" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B161" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C161" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D161" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E161" s="18" t="n">
+        <x:f>'Source Audit'!E161</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F161" s="41" t="n">
+        <x:f>'Source Audit'!F161</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G161" s="12" t="str">
+        <x:f>IF(AND(E161=0,F161=1,'Source Audit'!I161&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H161" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="27" customHeight="1">
+      <x:c r="A162" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B162" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C162" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D162" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E162" s="19" t="n">
+        <x:f>'Source Audit'!E162</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F162" s="40" t="n">
+        <x:f>'Source Audit'!F162</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G162" s="11" t="str">
+        <x:f>IF(AND(E162=0,F162=1,'Source Audit'!I162&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H162" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="27" customHeight="1">
+      <x:c r="A163" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B163" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C163" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D163" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E163" s="18" t="n">
+        <x:f>'Source Audit'!E163</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F163" s="41" t="n">
+        <x:f>'Source Audit'!F163</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G163" s="12" t="str">
+        <x:f>IF(AND(E163=0,F163=1,'Source Audit'!I163&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H163" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="27" customHeight="1">
+      <x:c r="A164" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B164" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C164" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D164" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E164" s="19" t="n">
+        <x:f>'Source Audit'!E164</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F164" s="40" t="n">
+        <x:f>'Source Audit'!F164</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G164" s="11" t="str">
+        <x:f>IF(AND(E164=0,F164=1,'Source Audit'!I164&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H164" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="27" customHeight="1">
+      <x:c r="A165" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B165" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C165" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D165" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E165" s="18" t="n">
+        <x:f>'Source Audit'!E165</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F165" s="41" t="n">
+        <x:f>'Source Audit'!F165</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G165" s="12" t="str">
+        <x:f>IF(AND(E165=0,F165=1,'Source Audit'!I165&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H165" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="27" customHeight="1">
+      <x:c r="A166" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B166" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C166" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D166" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E166" s="19" t="n">
+        <x:f>'Source Audit'!E166</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F166" s="40" t="n">
+        <x:f>'Source Audit'!F166</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G166" s="11" t="str">
+        <x:f>IF(AND(E166=0,F166=1,'Source Audit'!I166&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H166" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="44" customHeight="1">
+      <x:c r="A167" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B167" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C167" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D167" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E167" s="18" t="n">
+        <x:f>'Source Audit'!E167</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F167" s="41" t="n">
+        <x:f>'Source Audit'!F167</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G167" s="12" t="str">
+        <x:f>IF(AND(E167=0,F167=1,'Source Audit'!I167&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H167" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="27" customHeight="1">
+      <x:c r="A168" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B168" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C168" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D168" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E168" s="19" t="n">
+        <x:f>'Source Audit'!E168</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F168" s="40" t="n">
+        <x:f>'Source Audit'!F168</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G168" s="11" t="str">
+        <x:f>IF(AND(E168=0,F168=1,'Source Audit'!I168&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H168" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="27" customHeight="1">
+      <x:c r="A169" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B169" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C169" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D169" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E169" s="18" t="n">
+        <x:f>'Source Audit'!E169</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F169" s="41" t="n">
+        <x:f>'Source Audit'!F169</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G169" s="12" t="str">
+        <x:f>IF(AND(E169=0,F169=1,'Source Audit'!I169&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H169" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="27" customHeight="1">
+      <x:c r="A170" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B170" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C170" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D170" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E170" s="19" t="n">
+        <x:f>'Source Audit'!E170</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F170" s="40" t="n">
+        <x:f>'Source Audit'!F170</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G170" s="11" t="str">
+        <x:f>IF(AND(E170=0,F170=1,'Source Audit'!I170&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H170" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="27" customHeight="1">
+      <x:c r="A171" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B171" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C171" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D171" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E171" s="18" t="n">
+        <x:f>'Source Audit'!E171</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F171" s="41" t="n">
+        <x:f>'Source Audit'!F171</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G171" s="12" t="str">
+        <x:f>IF(AND(E171=0,F171=1,'Source Audit'!I171&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H171" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="27" customHeight="1">
+      <x:c r="A172" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B172" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C172" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D172" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E172" s="19" t="n">
+        <x:f>'Source Audit'!E172</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F172" s="40" t="n">
+        <x:f>'Source Audit'!F172</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G172" s="11" t="str">
+        <x:f>IF(AND(E172=0,F172=1,'Source Audit'!I172&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H172" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="27" customHeight="1">
+      <x:c r="A173" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B173" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C173" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D173" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E173" s="18" t="n">
+        <x:f>'Source Audit'!E173</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F173" s="41" t="n">
+        <x:f>'Source Audit'!F173</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G173" s="12" t="str">
+        <x:f>IF(AND(E173=0,F173=1,'Source Audit'!I173&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H173" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="27" customHeight="1">
+      <x:c r="A174" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B174" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C174" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D174" s="8" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E174" s="19" t="n">
+        <x:f>'Source Audit'!E174</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F174" s="40" t="n">
+        <x:f>'Source Audit'!F174</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G174" s="11" t="str">
+        <x:f>IF(AND(E174=0,F174=1,'Source Audit'!I174&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H174" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="27" customHeight="1">
+      <x:c r="A175" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="B175" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C175" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D175" s="9" t="n">
+        <x:v>46309</x:v>
+      </x:c>
+      <x:c r="E175" s="18" t="n">
+        <x:f>'Source Audit'!E175</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F175" s="41" t="n">
+        <x:f>'Source Audit'!F175</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G175" s="12" t="str">
+        <x:f>IF(AND(E175=0,F175=1,'Source Audit'!I175&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H175" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -21698,7 +23995,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb09f9bf442494a14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9504609bb517475f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 through October 15 and keep chart dates readable
Append audited October 15 closes and extend the cumulative five-sheet workbook and website series to eleven trading dates. Preserve prior canonical prices and immutable receipts, including the approved Ouster provider MIC exception. Enforce a minimum gap between visible chart date labels while retaining every observation and hover value.

Validation: 17 current observations and 155 historical comparisons passed. Workbook formulas, benchmark levels, contributions and weights reconcile. Type checking, production build, holdings CSV, desktop/mobile interactions and label spacing at eight viewport widths passed. Repository lint retains seven pre-existing errors and eight warnings in unrelated files.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5159a61a9d084f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rfb55181f591a49d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R03cc6846f4a04ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R83c25ceea5464faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rfb1cf0dac3474941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcc846c55fced48e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R9971295716df423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R73ec215dd4ad44c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R76fb2097cdf64a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rec85d627dcf04c14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H155" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H170" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H175" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1471,6 +1471,85 @@
         <x:v>-4.688570659532809</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="40" customHeight="1">
+      <x:c r="A16" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="n">
+        <x:f>B15*(1+SUM('Returns and Contributions'!F156:F170))</x:f>
+        <x:v>917.226724411436</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="n">
+        <x:f>B16/B15-1</x:f>
+        <x:v>-0.03089019801593107</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="n">
+        <x:f>B16/$B$6-1</x:f>
+        <x:v>-0.08277327558856407</x:v>
+      </x:c>
+      <x:c r="E16" s="19" t="n">
+        <x:f>1000*'Prices'!H191/'Prices'!I191</x:f>
+        <x:v>1010.1233295723575</x:v>
+      </x:c>
+      <x:c r="F16" s="20" t="n">
+        <x:f>E16/E15-1</x:f>
+        <x:v>0.003254332848810826</x:v>
+      </x:c>
+      <x:c r="G16" s="20" t="n">
+        <x:f>E16/1000-1</x:f>
+        <x:v>0.010123329572357509</x:v>
+      </x:c>
+      <x:c r="H16" s="19" t="n">
+        <x:f>1000*'Prices'!H192/'Prices'!I192</x:f>
+        <x:v>994.0989622733865</x:v>
+      </x:c>
+      <x:c r="I16" s="20" t="n">
+        <x:f>H16/H15-1</x:f>
+        <x:v>0.0007551192764061465</x:v>
+      </x:c>
+      <x:c r="J16" s="20" t="n">
+        <x:f>H16/1000-1</x:f>
+        <x:v>-0.005901037726613434</x:v>
+      </x:c>
+      <x:c r="K16" s="24" t="n">
+        <x:f>(C16-F16)*100</x:f>
+        <x:v>-3.4144530864741895</x:v>
+      </x:c>
+      <x:c r="L16" s="24" t="n">
+        <x:f>(C16-I16)*100</x:f>
+        <x:v>-3.1645317292337216</x:v>
+      </x:c>
+      <x:c r="M16" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G156:G170)</x:f>
+        <x:v>0.9999999999999998</x:v>
+      </x:c>
+      <x:c r="N16" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F156:F170)-C16</x:f>
+        <x:v>-4.163336342344337e-17</x:v>
+      </x:c>
+      <x:c r="O16" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P16" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I176:I192,"Mismatch")=0,IF(COUNTIF('Source Audit'!I176:I192,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q16" s="29" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="R16" s="28" t="n">
+        <x:f>B16-1000*('Prices'!H176/'Prices'!H6+'Prices'!H177/'Prices'!H7+'Prices'!H178/'Prices'!H8+'Prices'!H179/'Prices'!H9+'Prices'!H180/'Prices'!H10+'Prices'!H181/'Prices'!H11+'Prices'!H182/'Prices'!H12+'Prices'!H183/'Prices'!H13+'Prices'!H184/'Prices'!H14+'Prices'!H185/'Prices'!H15+'Prices'!H186/'Prices'!H16+'Prices'!H187/'Prices'!H17+'Prices'!H188/'Prices'!H18+'Prices'!H189/'Prices'!H19+'Prices'!H190/'Prices'!H20)/15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S16" s="24" t="n">
+        <x:f>(D16-G16)*100</x:f>
+        <x:v>-9.289660516092157</x:v>
+      </x:c>
+      <x:c r="T16" s="24" t="n">
+        <x:f>(D16-J16)*100</x:f>
+        <x:v>-7.687223786195063</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1478,7 +1557,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cb04974e0404d92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R052644538e1b4531"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7660,6 +7739,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="176" ht="27" customHeight="1">
+      <x:c r="A176" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B176" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C176" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D176" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E176" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F176" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G176" s="17" t="n">
+        <x:f>H159</x:f>
+        <x:v>6250</x:v>
+      </x:c>
+      <x:c r="H176" s="34" t="n">
+        <x:v>5907</x:v>
+      </x:c>
+      <x:c r="I176" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J176" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K176" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="27" customHeight="1">
+      <x:c r="A177" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B177" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C177" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D177" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E177" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F177" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G177" s="33" t="n">
+        <x:f>H160</x:f>
+        <x:v>4712</x:v>
+      </x:c>
+      <x:c r="H177" s="35" t="n">
+        <x:v>4274</x:v>
+      </x:c>
+      <x:c r="I177" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J177" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K177" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="27" customHeight="1">
+      <x:c r="A178" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B178" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C178" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D178" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E178" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F178" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G178" s="17" t="n">
+        <x:f>H161</x:f>
+        <x:v>25.22</x:v>
+      </x:c>
+      <x:c r="H178" s="34" t="n">
+        <x:v>24.09</x:v>
+      </x:c>
+      <x:c r="I178" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J178" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K178" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="27" customHeight="1">
+      <x:c r="A179" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B179" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C179" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D179" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E179" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F179" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G179" s="33" t="n">
+        <x:f>H162</x:f>
+        <x:v>359.44</x:v>
+      </x:c>
+      <x:c r="H179" s="35" t="n">
+        <x:v>343.21</x:v>
+      </x:c>
+      <x:c r="I179" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J179" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K179" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="27" customHeight="1">
+      <x:c r="A180" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B180" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C180" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D180" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E180" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F180" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G180" s="17" t="n">
+        <x:f>H163</x:f>
+        <x:v>4826</x:v>
+      </x:c>
+      <x:c r="H180" s="34" t="n">
+        <x:v>4441</x:v>
+      </x:c>
+      <x:c r="I180" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J180" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K180" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="27" customHeight="1">
+      <x:c r="A181" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B181" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C181" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D181" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E181" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F181" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G181" s="33" t="n">
+        <x:f>H164</x:f>
+        <x:v>49.33</x:v>
+      </x:c>
+      <x:c r="H181" s="35" t="n">
+        <x:v>49.39</x:v>
+      </x:c>
+      <x:c r="I181" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J181" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K181" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="27" customHeight="1">
+      <x:c r="A182" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B182" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C182" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D182" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E182" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F182" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G182" s="17" t="n">
+        <x:f>H165</x:f>
+        <x:v>80330</x:v>
+      </x:c>
+      <x:c r="H182" s="34" t="n">
+        <x:v>78970</x:v>
+      </x:c>
+      <x:c r="I182" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J182" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K182" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="27" customHeight="1">
+      <x:c r="A183" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B183" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C183" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D183" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E183" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F183" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G183" s="33" t="n">
+        <x:f>H166</x:f>
+        <x:v>57.27</x:v>
+      </x:c>
+      <x:c r="H183" s="35" t="n">
+        <x:v>55.67</x:v>
+      </x:c>
+      <x:c r="I183" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J183" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K183" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="27" customHeight="1">
+      <x:c r="A184" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B184" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C184" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D184" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E184" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F184" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G184" s="17" t="n">
+        <x:f>H167</x:f>
+        <x:v>31.87</x:v>
+      </x:c>
+      <x:c r="H184" s="34" t="n">
+        <x:v>31.33</x:v>
+      </x:c>
+      <x:c r="I184" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J184" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K184" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="27" customHeight="1">
+      <x:c r="A185" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B185" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C185" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D185" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E185" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F185" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G185" s="33" t="n">
+        <x:f>H168</x:f>
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="H185" s="35" t="n">
+        <x:v>13.36</x:v>
+      </x:c>
+      <x:c r="I185" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J185" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K185" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="27" customHeight="1">
+      <x:c r="A186" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B186" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C186" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D186" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E186" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F186" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G186" s="17" t="n">
+        <x:f>H169</x:f>
+        <x:v>423.42</x:v>
+      </x:c>
+      <x:c r="H186" s="34" t="n">
+        <x:v>422.03</x:v>
+      </x:c>
+      <x:c r="I186" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J186" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K186" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="27" customHeight="1">
+      <x:c r="A187" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B187" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C187" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D187" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E187" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F187" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G187" s="33" t="n">
+        <x:f>H170</x:f>
+        <x:v>275.05</x:v>
+      </x:c>
+      <x:c r="H187" s="35" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="I187" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J187" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K187" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="27" customHeight="1">
+      <x:c r="A188" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B188" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C188" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D188" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E188" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F188" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G188" s="17" t="n">
+        <x:f>H171</x:f>
+        <x:v>220.83</x:v>
+      </x:c>
+      <x:c r="H188" s="34" t="n">
+        <x:v>231.09</x:v>
+      </x:c>
+      <x:c r="I188" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J188" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K188" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="27" customHeight="1">
+      <x:c r="A189" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B189" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C189" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D189" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E189" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F189" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G189" s="33" t="n">
+        <x:f>H172</x:f>
+        <x:v>5864</x:v>
+      </x:c>
+      <x:c r="H189" s="35" t="n">
+        <x:v>5458</x:v>
+      </x:c>
+      <x:c r="I189" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J189" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K189" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="27" customHeight="1">
+      <x:c r="A190" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B190" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C190" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D190" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E190" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F190" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G190" s="17" t="n">
+        <x:f>H173</x:f>
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="H190" s="34" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="I190" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J190" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K190" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="27" customHeight="1">
+      <x:c r="A191" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B191" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C191" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D191" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E191" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F191" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G191" s="33" t="n">
+        <x:f>H174</x:f>
+        <x:v>7718.94</x:v>
+      </x:c>
+      <x:c r="H191" s="35" t="n">
+        <x:v>7744.06</x:v>
+      </x:c>
+      <x:c r="I191" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J191" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K191" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="27" customHeight="1">
+      <x:c r="A192" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B192" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C192" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D192" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E192" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F192" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G192" s="17" t="n">
+        <x:f>H175</x:f>
+        <x:v>26692.8691</x:v>
+      </x:c>
+      <x:c r="H192" s="34" t="n">
+        <x:v>26713.0254</x:v>
+      </x:c>
+      <x:c r="I192" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J192" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="K192" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -7667,7 +8358,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108966b65d134973"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b2ba0ea84a6427d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12316,6 +13007,471 @@
         <x:v>0.05029287012724715</x:v>
       </x:c>
     </x:row>
+    <x:row r="156" ht="27" customHeight="1">
+      <x:c r="A156" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B156" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C156" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D156" s="20" t="n">
+        <x:f>G141</x:f>
+        <x:v>0.07185171925179573</x:v>
+      </x:c>
+      <x:c r="E156" s="22" t="n">
+        <x:f>'Prices'!H176/'Prices'!G176-1</x:f>
+        <x:v>-0.05488000000000004</x:v>
+      </x:c>
+      <x:c r="F156" s="20" t="n">
+        <x:f>D156*E156</x:f>
+        <x:v>-0.003943222352538553</x:v>
+      </x:c>
+      <x:c r="G156" s="20" t="n">
+        <x:f>D156*(1+E156)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.0700730678404319</x:v>
+      </x:c>
+      <x:c r="H156" s="22" t="n">
+        <x:f>'Prices'!H176/'Prices'!I176-1</x:f>
+        <x:v>-0.03590664272890487</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="27" customHeight="1">
+      <x:c r="A157" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B157" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C157" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D157" s="21" t="n">
+        <x:f>G142</x:f>
+        <x:v>0.069450164467154</x:v>
+      </x:c>
+      <x:c r="E157" s="23" t="n">
+        <x:f>'Prices'!H177/'Prices'!G177-1</x:f>
+        <x:v>-0.09295415959252973</x:v>
+      </x:c>
+      <x:c r="F157" s="21" t="n">
+        <x:f>D157*E157</x:f>
+        <x:v>-0.006455681671607271</x:v>
+      </x:c>
+      <x:c r="G157" s="21" t="n">
+        <x:f>D157*(1+E157)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06500242043427633</x:v>
+      </x:c>
+      <x:c r="H157" s="23" t="n">
+        <x:f>'Prices'!H177/'Prices'!I177-1</x:f>
+        <x:v>-0.10567064239380619</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="27" customHeight="1">
+      <x:c r="A158" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B158" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C158" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D158" s="20" t="n">
+        <x:f>G143</x:f>
+        <x:v>0.06294961815927468</x:v>
+      </x:c>
+      <x:c r="E158" s="22" t="n">
+        <x:f>'Prices'!H178/'Prices'!G178-1</x:f>
+        <x:v>-0.044805709754163314</x:v>
+      </x:c>
+      <x:c r="F158" s="20" t="n">
+        <x:f>D158*E158</x:f>
+        <x:v>-0.0028205023203798692</x:v>
+      </x:c>
+      <x:c r="G158" s="20" t="n">
+        <x:f>D158*(1+E158)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.062045720428987323</x:v>
+      </x:c>
+      <x:c r="H158" s="22" t="n">
+        <x:f>'Prices'!H178/'Prices'!I178-1</x:f>
+        <x:v>-0.14635010630758327</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="27" customHeight="1">
+      <x:c r="A159" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B159" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C159" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D159" s="21" t="n">
+        <x:f>G144</x:f>
+        <x:v>0.06089160097822906</x:v>
+      </x:c>
+      <x:c r="E159" s="23" t="n">
+        <x:f>'Prices'!H179/'Prices'!G179-1</x:f>
+        <x:v>-0.04515357222345873</x:v>
+      </x:c>
+      <x:c r="F159" s="21" t="n">
+        <x:f>D159*E159</x:f>
+        <x:v>-0.002749473302572496</x:v>
+      </x:c>
+      <x:c r="G159" s="21" t="n">
+        <x:f>D159*(1+E159)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.05999539738079375</x:v>
+      </x:c>
+      <x:c r="H159" s="23" t="n">
+        <x:f>'Prices'!H179/'Prices'!I179-1</x:f>
+        <x:v>-0.17455927270978144</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="27" customHeight="1">
+      <x:c r="A160" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B160" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C160" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D160" s="20" t="n">
+        <x:f>G145</x:f>
+        <x:v>0.0683280866761925</x:v>
+      </x:c>
+      <x:c r="E160" s="22" t="n">
+        <x:f>'Prices'!H180/'Prices'!G180-1</x:f>
+        <x:v>-0.07977621218400333</x:v>
+      </x:c>
+      <x:c r="F160" s="20" t="n">
+        <x:f>D160*E160</x:f>
+        <x:v>-0.005450955940806903</x:v>
+      </x:c>
+      <x:c r="G160" s="20" t="n">
+        <x:f>D160*(1+E160)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06488132779862156</x:v>
+      </x:c>
+      <x:c r="H160" s="22" t="n">
+        <x:f>'Prices'!H180/'Prices'!I180-1</x:f>
+        <x:v>-0.10733668341708547</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="27" customHeight="1">
+      <x:c r="A161" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B161" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C161" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D161" s="21" t="n">
+        <x:f>G146</x:f>
+        <x:v>0.06694972306313456</x:v>
+      </x:c>
+      <x:c r="E161" s="23" t="n">
+        <x:f>'Prices'!H181/'Prices'!G181-1</x:f>
+        <x:v>0.0012162983985404274</x:v>
+      </x:c>
+      <x:c r="F161" s="21" t="n">
+        <x:f>D161*E161</x:f>
+        <x:v>0.00008143084094441568</x:v>
+      </x:c>
+      <x:c r="G161" s="21" t="n">
+        <x:f>D161*(1+E161)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06916775969745159</x:v>
+      </x:c>
+      <x:c r="H161" s="23" t="n">
+        <x:f>'Prices'!H181/'Prices'!I181-1</x:f>
+        <x:v>-0.04836223506743731</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="27" customHeight="1">
+      <x:c r="A162" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B162" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C162" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D162" s="20" t="n">
+        <x:f>G147</x:f>
+        <x:v>0.0696829880160248</x:v>
+      </x:c>
+      <x:c r="E162" s="22" t="n">
+        <x:f>'Prices'!H182/'Prices'!G182-1</x:f>
+        <x:v>-0.016930163077306104</x:v>
+      </x:c>
+      <x:c r="F162" s="20" t="n">
+        <x:f>D162*E162</x:f>
+        <x:v>-0.0011797443508252668</x:v>
+      </x:c>
+      <x:c r="G162" s="20" t="n">
+        <x:f>D162*(1+E162)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.07068677205096069</x:v>
+      </x:c>
+      <x:c r="H162" s="22" t="n">
+        <x:f>'Prices'!H182/'Prices'!I182-1</x:f>
+        <x:v>-0.027463054187192082</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="27" customHeight="1">
+      <x:c r="A163" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B163" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C163" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D163" s="21" t="n">
+        <x:f>G148</x:f>
+        <x:v>0.06483390848066585</x:v>
+      </x:c>
+      <x:c r="E163" s="23" t="n">
+        <x:f>'Prices'!H183/'Prices'!G183-1</x:f>
+        <x:v>-0.02793783830976082</x:v>
+      </x:c>
+      <x:c r="F163" s="21" t="n">
+        <x:f>D163*E163</x:f>
+        <x:v>-0.0018113192521226733</x:v>
+      </x:c>
+      <x:c r="G163" s="21" t="n">
+        <x:f>D163*(1+E163)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06503142275469338</x:v>
+      </x:c>
+      <x:c r="H163" s="23" t="n">
+        <x:f>'Prices'!H183/'Prices'!I183-1</x:f>
+        <x:v>-0.10527161684345865</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="27" customHeight="1">
+      <x:c r="A164" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B164" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C164" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D164" s="20" t="n">
+        <x:f>G149</x:f>
+        <x:v>0.05492656665713855</x:v>
+      </x:c>
+      <x:c r="E164" s="22" t="n">
+        <x:f>'Prices'!H184/'Prices'!G184-1</x:f>
+        <x:v>-0.016943834326953344</x:v>
+      </x:c>
+      <x:c r="F164" s="20" t="n">
+        <x:f>D164*E164</x:f>
+        <x:v>-0.0009306666455869151</x:v>
+      </x:c>
+      <x:c r="G164" s="20" t="n">
+        <x:f>D164*(1+E164)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.05571700946683776</x:v>
+      </x:c>
+      <x:c r="H164" s="22" t="n">
+        <x:f>'Prices'!H184/'Prices'!I184-1</x:f>
+        <x:v>-0.2334230486909714</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="27" customHeight="1">
+      <x:c r="A165" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B165" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C165" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D165" s="21" t="n">
+        <x:f>G150</x:f>
+        <x:v>0.06163849486452419</x:v>
+      </x:c>
+      <x:c r="E165" s="23" t="n">
+        <x:f>'Prices'!H185/'Prices'!G185-1</x:f>
+        <x:v>-0.04160688665710188</x:v>
+      </x:c>
+      <x:c r="F165" s="21" t="n">
+        <x:f>D165*E165</x:f>
+        <x:v>-0.0025645858695426144</x:v>
+      </x:c>
+      <x:c r="G165" s="21" t="n">
+        <x:f>D165*(1+E165)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06095687905956469</x:v>
+      </x:c>
+      <x:c r="H165" s="23" t="n">
+        <x:f>'Prices'!H185/'Prices'!I185-1</x:f>
+        <x:v>-0.16133082234777152</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="27" customHeight="1">
+      <x:c r="A166" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B166" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C166" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D166" s="20" t="n">
+        <x:f>G151</x:f>
+        <x:v>0.0674081170118034</x:v>
+      </x:c>
+      <x:c r="E166" s="22" t="n">
+        <x:f>'Prices'!H186/'Prices'!G186-1</x:f>
+        <x:v>-0.0032827924991735147</x:v>
+      </x:c>
+      <x:c r="F166" s="20" t="n">
+        <x:f>D166*E166</x:f>
+        <x:v>-0.00022128686090975877</x:v>
+      </x:c>
+      <x:c r="G166" s="20" t="n">
+        <x:f>D166*(1+E166)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.06932839809621295</x:v>
+      </x:c>
+      <x:c r="H166" s="22" t="n">
+        <x:f>'Prices'!H186/'Prices'!I186-1</x:f>
+        <x:v>-0.04615210758277777</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="27" customHeight="1">
+      <x:c r="A167" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B167" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C167" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D167" s="21" t="n">
+        <x:f>G152</x:f>
+        <x:v>0.07125370788350113</x:v>
+      </x:c>
+      <x:c r="E167" s="23" t="n">
+        <x:f>'Prices'!H187/'Prices'!G187-1</x:f>
+        <x:v>-0.015997091437920496</x:v>
+      </x:c>
+      <x:c r="F167" s="21" t="n">
+        <x:f>D167*E167</x:f>
+        <x:v>-0.001139852080303244</x:v>
+      </x:c>
+      <x:c r="G167" s="21" t="n">
+        <x:f>D167*(1+E167)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.07234872215682168</x:v>
+      </x:c>
+      <x:c r="H167" s="23" t="n">
+        <x:f>'Prices'!H187/'Prices'!I187-1</x:f>
+        <x:v>-0.0045972784111806275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="27" customHeight="1">
+      <x:c r="A168" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B168" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C168" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D168" s="20" t="n">
+        <x:f>G153</x:f>
+        <x:v>0.06503094738065356</x:v>
+      </x:c>
+      <x:c r="E168" s="22" t="n">
+        <x:f>'Prices'!H188/'Prices'!G188-1</x:f>
+        <x:v>0.04646107865779103</x:v>
+      </x:c>
+      <x:c r="F168" s="20" t="n">
+        <x:f>D168*E168</x:f>
+        <x:v>0.003021407961443215</x:v>
+      </x:c>
+      <x:c r="G168" s="20" t="n">
+        <x:f>D168*(1+E168)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.07022151174487397</x:v>
+      </x:c>
+      <x:c r="H168" s="22" t="n">
+        <x:f>'Prices'!H188/'Prices'!I188-1</x:f>
+        <x:v>-0.03386429198545082</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="27" customHeight="1">
+      <x:c r="A169" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B169" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C169" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D169" s="21" t="n">
+        <x:f>G154</x:f>
+        <x:v>0.07082416673059343</x:v>
+      </x:c>
+      <x:c r="E169" s="23" t="n">
+        <x:f>'Prices'!H189/'Prices'!G189-1</x:f>
+        <x:v>-0.06923601637107779</x:v>
+      </x:c>
+      <x:c r="F169" s="21" t="n">
+        <x:f>D169*E169</x:f>
+        <x:v>-0.00490358316722731</x:v>
+      </x:c>
+      <x:c r="G169" s="21" t="n">
+        <x:f>D169*(1+E169)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.0680217901298761</x:v>
+      </x:c>
+      <x:c r="H169" s="23" t="n">
+        <x:f>'Prices'!H189/'Prices'!I189-1</x:f>
+        <x:v>-0.06412894375857336</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="27" customHeight="1">
+      <x:c r="A170" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B170" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C170" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D170" s="20" t="n">
+        <x:f>G155</x:f>
+        <x:v>0.07398019037931446</x:v>
+      </x:c>
+      <x:c r="E170" s="22" t="n">
+        <x:f>'Prices'!H190/'Prices'!G190-1</x:f>
+        <x:v>0.0024038461538462563</x:v>
+      </x:c>
+      <x:c r="F170" s="20" t="n">
+        <x:f>D170*E170</x:f>
+        <x:v>0.00017783699610412888</x:v>
+      </x:c>
+      <x:c r="G170" s="20" t="n">
+        <x:f>D170*(1+E170)/(1+SUM($F$156:$F$170))</x:f>
+        <x:v>0.07652180095959618</x:v>
+      </x:c>
+      <x:c r="H170" s="22" t="n">
+        <x:f>'Prices'!H190/'Prices'!I190-1</x:f>
+        <x:v>0.052817612603514474</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -12323,7 +13479,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5615d0c33874d17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c2b8378db54d13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18962,6 +20118,654 @@
       </x:c>
       <x:c r="M175" s="16" t="str"/>
     </x:row>
+    <x:row r="176" ht="50" customHeight="1">
+      <x:c r="A176" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B176" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C176" s="17" t="n">
+        <x:v>5907</x:v>
+      </x:c>
+      <x:c r="D176" s="17" t="n">
+        <x:v>5907</x:v>
+      </x:c>
+      <x:c r="E176" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F176" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G176" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H176" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I176" s="31" t="str">
+        <x:f>IF(AND(G176=H176,C176&gt;0,ABS(C176-'Prices'!H176)&lt;=MAX(0.01,'Prices'!H176*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J176" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K176" s="14" t="str"/>
+      <x:c r="L176" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M176" s="14" t="str"/>
+    </x:row>
+    <x:row r="177" ht="50" customHeight="1">
+      <x:c r="A177" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B177" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C177" s="33" t="n">
+        <x:v>4274</x:v>
+      </x:c>
+      <x:c r="D177" s="33" t="n">
+        <x:v>4274</x:v>
+      </x:c>
+      <x:c r="E177" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F177" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G177" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H177" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I177" s="32" t="str">
+        <x:f>IF(AND(G177=H177,C177&gt;0,ABS(C177-'Prices'!H177)&lt;=MAX(0.01,'Prices'!H177*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J177" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K177" s="16" t="str"/>
+      <x:c r="L177" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M177" s="16" t="str"/>
+    </x:row>
+    <x:row r="178" ht="50" customHeight="1">
+      <x:c r="A178" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B178" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C178" s="17" t="n">
+        <x:v>24.09</x:v>
+      </x:c>
+      <x:c r="D178" s="17" t="n">
+        <x:v>24.09</x:v>
+      </x:c>
+      <x:c r="E178" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F178" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G178" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H178" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I178" s="31" t="str">
+        <x:f>IF(AND(G178=H178,C178&gt;0,ABS(C178-'Prices'!H178)&lt;=MAX(0.01,'Prices'!H178*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J178" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K178" s="14" t="str"/>
+      <x:c r="L178" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M178" s="14" t="str"/>
+    </x:row>
+    <x:row r="179" ht="50" customHeight="1">
+      <x:c r="A179" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B179" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C179" s="33" t="n">
+        <x:v>343.21</x:v>
+      </x:c>
+      <x:c r="D179" s="33" t="n">
+        <x:v>343.21</x:v>
+      </x:c>
+      <x:c r="E179" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F179" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G179" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H179" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I179" s="32" t="str">
+        <x:f>IF(AND(G179=H179,C179&gt;0,ABS(C179-'Prices'!H179)&lt;=MAX(0.01,'Prices'!H179*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J179" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K179" s="16" t="str"/>
+      <x:c r="L179" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M179" s="16" t="str"/>
+    </x:row>
+    <x:row r="180" ht="50" customHeight="1">
+      <x:c r="A180" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B180" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C180" s="17" t="n">
+        <x:v>4441</x:v>
+      </x:c>
+      <x:c r="D180" s="17" t="n">
+        <x:v>4441</x:v>
+      </x:c>
+      <x:c r="E180" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F180" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G180" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H180" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I180" s="31" t="str">
+        <x:f>IF(AND(G180=H180,C180&gt;0,ABS(C180-'Prices'!H180)&lt;=MAX(0.01,'Prices'!H180*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J180" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K180" s="14" t="str"/>
+      <x:c r="L180" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M180" s="14" t="str"/>
+    </x:row>
+    <x:row r="181" ht="50" customHeight="1">
+      <x:c r="A181" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B181" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C181" s="33" t="n">
+        <x:v>49.39</x:v>
+      </x:c>
+      <x:c r="D181" s="33" t="n">
+        <x:v>49.39</x:v>
+      </x:c>
+      <x:c r="E181" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F181" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G181" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H181" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I181" s="32" t="str">
+        <x:f>IF(AND(G181=H181,C181&gt;0,ABS(C181-'Prices'!H181)&lt;=MAX(0.01,'Prices'!H181*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J181" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K181" s="16" t="str"/>
+      <x:c r="L181" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M181" s="16" t="str"/>
+    </x:row>
+    <x:row r="182" ht="50" customHeight="1">
+      <x:c r="A182" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B182" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C182" s="17" t="n">
+        <x:v>78970</x:v>
+      </x:c>
+      <x:c r="D182" s="17" t="n">
+        <x:v>78970</x:v>
+      </x:c>
+      <x:c r="E182" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F182" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G182" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H182" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I182" s="31" t="str">
+        <x:f>IF(AND(G182=H182,C182&gt;0,ABS(C182-'Prices'!H182)&lt;=MAX(0.01,'Prices'!H182*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J182" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K182" s="14" t="str"/>
+      <x:c r="L182" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M182" s="14" t="str"/>
+    </x:row>
+    <x:row r="183" ht="50" customHeight="1">
+      <x:c r="A183" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B183" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C183" s="33" t="n">
+        <x:v>55.67</x:v>
+      </x:c>
+      <x:c r="D183" s="33" t="n">
+        <x:v>55.67</x:v>
+      </x:c>
+      <x:c r="E183" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F183" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G183" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H183" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I183" s="32" t="str">
+        <x:f>IF(AND(G183=H183,C183&gt;0,ABS(C183-'Prices'!H183)&lt;=MAX(0.01,'Prices'!H183*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J183" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K183" s="16" t="str"/>
+      <x:c r="L183" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M183" s="16" t="str"/>
+    </x:row>
+    <x:row r="184" ht="50" customHeight="1">
+      <x:c r="A184" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B184" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C184" s="17" t="n">
+        <x:v>31.33</x:v>
+      </x:c>
+      <x:c r="D184" s="17" t="n">
+        <x:v>31.33</x:v>
+      </x:c>
+      <x:c r="E184" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F184" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G184" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H184" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I184" s="31" t="str">
+        <x:f>IF(AND(OR(G184=H184,AND(B184="OUST",G184="XNAS",H184="XNYS",LEFT(M184,34)="ouster-marketstack-legacy-nyse-tag")),C184&gt;0,ABS(C184-'Prices'!H184)&lt;=MAX(0.01,'Prices'!H184*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J184" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K184" s="14" t="str"/>
+      <x:c r="L184" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M184" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="50" customHeight="1">
+      <x:c r="A185" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B185" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C185" s="33" t="n">
+        <x:v>13.36</x:v>
+      </x:c>
+      <x:c r="D185" s="33" t="n">
+        <x:v>13.36</x:v>
+      </x:c>
+      <x:c r="E185" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F185" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G185" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H185" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I185" s="32" t="str">
+        <x:f>IF(AND(G185=H185,C185&gt;0,ABS(C185-'Prices'!H185)&lt;=MAX(0.01,'Prices'!H185*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J185" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K185" s="16" t="str"/>
+      <x:c r="L185" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M185" s="16" t="str"/>
+    </x:row>
+    <x:row r="186" ht="50" customHeight="1">
+      <x:c r="A186" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B186" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C186" s="17" t="n">
+        <x:v>422.03</x:v>
+      </x:c>
+      <x:c r="D186" s="17" t="n">
+        <x:v>422.03</x:v>
+      </x:c>
+      <x:c r="E186" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F186" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G186" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H186" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I186" s="31" t="str">
+        <x:f>IF(AND(G186=H186,C186&gt;0,ABS(C186-'Prices'!H186)&lt;=MAX(0.01,'Prices'!H186*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J186" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K186" s="14" t="str"/>
+      <x:c r="L186" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M186" s="14" t="str"/>
+    </x:row>
+    <x:row r="187" ht="50" customHeight="1">
+      <x:c r="A187" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B187" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C187" s="33" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="D187" s="33" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="E187" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F187" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G187" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H187" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I187" s="32" t="str">
+        <x:f>IF(AND(G187=H187,C187&gt;0,ABS(C187-'Prices'!H187)&lt;=MAX(0.01,'Prices'!H187*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J187" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K187" s="16" t="str"/>
+      <x:c r="L187" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M187" s="16" t="str"/>
+    </x:row>
+    <x:row r="188" ht="50" customHeight="1">
+      <x:c r="A188" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B188" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C188" s="17" t="n">
+        <x:v>231.09</x:v>
+      </x:c>
+      <x:c r="D188" s="17" t="n">
+        <x:v>231.09</x:v>
+      </x:c>
+      <x:c r="E188" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F188" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G188" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H188" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I188" s="31" t="str">
+        <x:f>IF(AND(G188=H188,C188&gt;0,ABS(C188-'Prices'!H188)&lt;=MAX(0.01,'Prices'!H188*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J188" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K188" s="14" t="str"/>
+      <x:c r="L188" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M188" s="14" t="str"/>
+    </x:row>
+    <x:row r="189" ht="50" customHeight="1">
+      <x:c r="A189" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B189" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C189" s="33" t="n">
+        <x:v>5458</x:v>
+      </x:c>
+      <x:c r="D189" s="33" t="n">
+        <x:v>5458</x:v>
+      </x:c>
+      <x:c r="E189" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F189" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G189" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H189" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I189" s="32" t="str">
+        <x:f>IF(AND(G189=H189,C189&gt;0,ABS(C189-'Prices'!H189)&lt;=MAX(0.01,'Prices'!H189*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J189" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K189" s="16" t="str"/>
+      <x:c r="L189" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M189" s="16" t="str"/>
+    </x:row>
+    <x:row r="190" ht="50" customHeight="1">
+      <x:c r="A190" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B190" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C190" s="17" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="D190" s="17" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="E190" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F190" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G190" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H190" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I190" s="31" t="str">
+        <x:f>IF(AND(G190=H190,C190&gt;0,ABS(C190-'Prices'!H190)&lt;=MAX(0.01,'Prices'!H190*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J190" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K190" s="14" t="str"/>
+      <x:c r="L190" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M190" s="14" t="str"/>
+    </x:row>
+    <x:row r="191" ht="50" customHeight="1">
+      <x:c r="A191" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B191" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C191" s="33" t="n">
+        <x:v>7744.06</x:v>
+      </x:c>
+      <x:c r="D191" s="33" t="n">
+        <x:v>7744.06</x:v>
+      </x:c>
+      <x:c r="E191" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F191" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G191" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H191" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I191" s="32" t="str">
+        <x:f>IF(AND(G191=H191,C191&gt;0,ABS(C191-'Prices'!H191)&lt;=MAX(0.01,'Prices'!H191*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J191" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K191" s="16" t="str"/>
+      <x:c r="L191" s="39" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M191" s="16" t="str"/>
+    </x:row>
+    <x:row r="192" ht="50" customHeight="1">
+      <x:c r="A192" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B192" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C192" s="17" t="n">
+        <x:v>26713.0254</x:v>
+      </x:c>
+      <x:c r="D192" s="17" t="n">
+        <x:v>26713.0254</x:v>
+      </x:c>
+      <x:c r="E192" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F192" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G192" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H192" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I192" s="31" t="str">
+        <x:f>IF(AND(G192=H192,C192&gt;0,ABS(C192-'Prices'!H192)&lt;=MAX(0.01,'Prices'!H192*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J192" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-16T11-31-06-696Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K192" s="14" t="str"/>
+      <x:c r="L192" s="38" t="n">
+        <x:v>46311.47993861111</x:v>
+      </x:c>
+      <x:c r="M192" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -18969,7 +20773,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44772a4656af41d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ffcd523d80f4ad3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23988,6 +25792,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="176" ht="27" customHeight="1">
+      <x:c r="A176" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B176" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C176" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D176" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E176" s="19" t="n">
+        <x:f>'Source Audit'!E176</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F176" s="40" t="n">
+        <x:f>'Source Audit'!F176</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G176" s="11" t="str">
+        <x:f>IF(AND(E176=0,F176=1,'Source Audit'!I176&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H176" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="27" customHeight="1">
+      <x:c r="A177" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B177" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C177" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D177" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E177" s="18" t="n">
+        <x:f>'Source Audit'!E177</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F177" s="41" t="n">
+        <x:f>'Source Audit'!F177</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G177" s="12" t="str">
+        <x:f>IF(AND(E177=0,F177=1,'Source Audit'!I177&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H177" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="27" customHeight="1">
+      <x:c r="A178" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B178" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C178" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D178" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E178" s="19" t="n">
+        <x:f>'Source Audit'!E178</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F178" s="40" t="n">
+        <x:f>'Source Audit'!F178</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G178" s="11" t="str">
+        <x:f>IF(AND(E178=0,F178=1,'Source Audit'!I178&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H178" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="27" customHeight="1">
+      <x:c r="A179" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B179" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C179" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D179" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E179" s="18" t="n">
+        <x:f>'Source Audit'!E179</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F179" s="41" t="n">
+        <x:f>'Source Audit'!F179</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G179" s="12" t="str">
+        <x:f>IF(AND(E179=0,F179=1,'Source Audit'!I179&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H179" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="27" customHeight="1">
+      <x:c r="A180" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B180" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C180" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D180" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E180" s="19" t="n">
+        <x:f>'Source Audit'!E180</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F180" s="40" t="n">
+        <x:f>'Source Audit'!F180</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G180" s="11" t="str">
+        <x:f>IF(AND(E180=0,F180=1,'Source Audit'!I180&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H180" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="27" customHeight="1">
+      <x:c r="A181" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B181" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C181" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D181" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E181" s="18" t="n">
+        <x:f>'Source Audit'!E181</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F181" s="41" t="n">
+        <x:f>'Source Audit'!F181</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G181" s="12" t="str">
+        <x:f>IF(AND(E181=0,F181=1,'Source Audit'!I181&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H181" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="27" customHeight="1">
+      <x:c r="A182" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B182" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C182" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D182" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E182" s="19" t="n">
+        <x:f>'Source Audit'!E182</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F182" s="40" t="n">
+        <x:f>'Source Audit'!F182</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G182" s="11" t="str">
+        <x:f>IF(AND(E182=0,F182=1,'Source Audit'!I182&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H182" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="27" customHeight="1">
+      <x:c r="A183" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B183" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C183" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D183" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E183" s="18" t="n">
+        <x:f>'Source Audit'!E183</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F183" s="41" t="n">
+        <x:f>'Source Audit'!F183</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G183" s="12" t="str">
+        <x:f>IF(AND(E183=0,F183=1,'Source Audit'!I183&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H183" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="44" customHeight="1">
+      <x:c r="A184" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B184" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C184" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D184" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E184" s="19" t="n">
+        <x:f>'Source Audit'!E184</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F184" s="40" t="n">
+        <x:f>'Source Audit'!F184</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G184" s="11" t="str">
+        <x:f>IF(AND(E184=0,F184=1,'Source Audit'!I184&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H184" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="27" customHeight="1">
+      <x:c r="A185" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B185" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C185" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D185" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E185" s="18" t="n">
+        <x:f>'Source Audit'!E185</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F185" s="41" t="n">
+        <x:f>'Source Audit'!F185</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G185" s="12" t="str">
+        <x:f>IF(AND(E185=0,F185=1,'Source Audit'!I185&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H185" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="27" customHeight="1">
+      <x:c r="A186" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B186" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C186" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D186" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E186" s="19" t="n">
+        <x:f>'Source Audit'!E186</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F186" s="40" t="n">
+        <x:f>'Source Audit'!F186</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G186" s="11" t="str">
+        <x:f>IF(AND(E186=0,F186=1,'Source Audit'!I186&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H186" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="27" customHeight="1">
+      <x:c r="A187" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B187" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C187" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D187" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E187" s="18" t="n">
+        <x:f>'Source Audit'!E187</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F187" s="41" t="n">
+        <x:f>'Source Audit'!F187</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G187" s="12" t="str">
+        <x:f>IF(AND(E187=0,F187=1,'Source Audit'!I187&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H187" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="27" customHeight="1">
+      <x:c r="A188" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B188" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C188" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D188" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E188" s="19" t="n">
+        <x:f>'Source Audit'!E188</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F188" s="40" t="n">
+        <x:f>'Source Audit'!F188</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G188" s="11" t="str">
+        <x:f>IF(AND(E188=0,F188=1,'Source Audit'!I188&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H188" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="27" customHeight="1">
+      <x:c r="A189" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B189" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C189" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D189" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E189" s="18" t="n">
+        <x:f>'Source Audit'!E189</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F189" s="41" t="n">
+        <x:f>'Source Audit'!F189</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G189" s="12" t="str">
+        <x:f>IF(AND(E189=0,F189=1,'Source Audit'!I189&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H189" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="27" customHeight="1">
+      <x:c r="A190" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B190" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C190" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D190" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E190" s="19" t="n">
+        <x:f>'Source Audit'!E190</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F190" s="40" t="n">
+        <x:f>'Source Audit'!F190</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G190" s="11" t="str">
+        <x:f>IF(AND(E190=0,F190=1,'Source Audit'!I190&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H190" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="27" customHeight="1">
+      <x:c r="A191" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B191" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C191" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D191" s="9" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E191" s="18" t="n">
+        <x:f>'Source Audit'!E191</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F191" s="41" t="n">
+        <x:f>'Source Audit'!F191</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G191" s="12" t="str">
+        <x:f>IF(AND(E191=0,F191=1,'Source Audit'!I191&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H191" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="27" customHeight="1">
+      <x:c r="A192" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B192" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C192" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D192" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="E192" s="19" t="n">
+        <x:f>'Source Audit'!E192</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F192" s="40" t="n">
+        <x:f>'Source Audit'!F192</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G192" s="11" t="str">
+        <x:f>IF(AND(E192=0,F192=1,'Source Audit'!I192&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H192" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -23995,7 +26292,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9504609bb517475f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9148181cba7c4308"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish BSPI15 through October 19 and enable automatic pushes
Append the verified October 16 and October 19 closes, extend the cumulative five-sheet workbook and website data to thirteen trading dates, and preserve the earlier reviewed inputs and immutable receipts. Record Inovance option-window review without a price-continuity adjustment.

Document standing authorization to push scoped BSPI15 updates after successful daily verification, retaining the strict Marketstack audit, approved Ouster exception and 7:30 AM Eastern schedule.

Validation: October 19 audit passed 17 current prices and 189 historical comparisons; workbook formulas, both index calculations, benchmarks, weights and contributions reconcile. Type checking, production build, desktop/mobile rendering and holdings CSV passed. Repository lint retains seven unrelated errors and nine warnings.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcc846c55fced48e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R9971295716df423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R73ec215dd4ad44c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R76fb2097cdf64a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rec85d627dcf04c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8b9c951c2fdb47af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R56f103054bbc4aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Rd72b86d1c85b4fe2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R5a98770ea99e44c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R257cffe0c77844d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H170" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H200" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H192" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1550,6 +1550,164 @@
         <x:v>-7.687223786195063</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="40" customHeight="1">
+      <x:c r="A17" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B17" s="18" t="n">
+        <x:f>B16*(1+SUM('Returns and Contributions'!F171:F185))</x:f>
+        <x:v>910.2086366893151</x:v>
+      </x:c>
+      <x:c r="C17" s="21" t="n">
+        <x:f>B17/B16-1</x:f>
+        <x:v>-0.007651420892281768</x:v>
+      </x:c>
+      <x:c r="D17" s="21" t="n">
+        <x:f>B17/$B$6-1</x:f>
+        <x:v>-0.08979136331068494</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="n">
+        <x:f>1000*'Prices'!H208/'Prices'!I208</x:f>
+        <x:v>999.0856263329181</x:v>
+      </x:c>
+      <x:c r="F17" s="21" t="n">
+        <x:f>E17/E16-1</x:f>
+        <x:v>-0.01092708475915738</x:v>
+      </x:c>
+      <x:c r="G17" s="21" t="n">
+        <x:f>E17/1000-1</x:f>
+        <x:v>-0.0009143736670819136</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="n">
+        <x:f>1000*'Prices'!H209/'Prices'!I209</x:f>
+        <x:v>972.7754760763983</x:v>
+      </x:c>
+      <x:c r="I17" s="21" t="n">
+        <x:f>H17/H16-1</x:f>
+        <x:v>-0.021450063832904487</x:v>
+      </x:c>
+      <x:c r="J17" s="21" t="n">
+        <x:f>H17/1000-1</x:f>
+        <x:v>-0.02722452392360175</x:v>
+      </x:c>
+      <x:c r="K17" s="25" t="n">
+        <x:f>(C17-F17)*100</x:f>
+        <x:v>0.3275663866875611</x:v>
+      </x:c>
+      <x:c r="L17" s="25" t="n">
+        <x:f>(C17-I17)*100</x:f>
+        <x:v>1.3798642940622718</x:v>
+      </x:c>
+      <x:c r="M17" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G171:G185)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N17" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F171:F185)-C17</x:f>
+        <x:v>-1.474514954580286e-17</x:v>
+      </x:c>
+      <x:c r="O17" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P17" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I193:I209,"Mismatch")=0,IF(COUNTIF('Source Audit'!I193:I209,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q17" s="30" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="R17" s="27" t="n">
+        <x:f>B17-1000*('Prices'!H193/'Prices'!H6+'Prices'!H194/'Prices'!H7+'Prices'!H195/'Prices'!H8+'Prices'!H196/'Prices'!H9+'Prices'!H197/'Prices'!H10+'Prices'!H198/'Prices'!H11+'Prices'!H199/'Prices'!H12+'Prices'!H200/'Prices'!H13+'Prices'!H201/'Prices'!H14+'Prices'!H202/'Prices'!H15+'Prices'!H203/'Prices'!H16+'Prices'!H204/'Prices'!H17+'Prices'!H205/'Prices'!H18+'Prices'!H206/'Prices'!H19+'Prices'!H207/'Prices'!H20)/15</x:f>
+        <x:v>1.1368683772161603e-13</x:v>
+      </x:c>
+      <x:c r="S17" s="25" t="n">
+        <x:f>(D17-G17)*100</x:f>
+        <x:v>-8.887698964360302</x:v>
+      </x:c>
+      <x:c r="T17" s="25" t="n">
+        <x:f>(D17-J17)*100</x:f>
+        <x:v>-6.256683938708319</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="40" customHeight="1">
+      <x:c r="A18" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="n">
+        <x:f>B17*(1+SUM('Returns and Contributions'!F186:F200))</x:f>
+        <x:v>917.7507372655805</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="n">
+        <x:f>B18/B17-1</x:f>
+        <x:v>0.0082861228428881</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="n">
+        <x:f>B18/$B$6-1</x:f>
+        <x:v>-0.08224926273441957</x:v>
+      </x:c>
+      <x:c r="E18" s="19" t="n">
+        <x:f>1000*'Prices'!H225/'Prices'!I225</x:f>
+        <x:v>1003.1670460252138</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="n">
+        <x:f>E18/E17-1</x:f>
+        <x:v>0.004085155050499889</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="n">
+        <x:f>E18/1000-1</x:f>
+        <x:v>0.003167046025213782</x:v>
+      </x:c>
+      <x:c r="H18" s="19" t="n">
+        <x:f>1000*'Prices'!H226/'Prices'!I226</x:f>
+        <x:v>983.5994480967871</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="n">
+        <x:f>H18/H17-1</x:f>
+        <x:v>0.011126896479798587</x:v>
+      </x:c>
+      <x:c r="J18" s="20" t="n">
+        <x:f>H18/1000-1</x:f>
+        <x:v>-0.01640055190321288</x:v>
+      </x:c>
+      <x:c r="K18" s="24" t="n">
+        <x:f>(C18-F18)*100</x:f>
+        <x:v>0.42009677923882105</x:v>
+      </x:c>
+      <x:c r="L18" s="24" t="n">
+        <x:f>(C18-I18)*100</x:f>
+        <x:v>-0.28407736369104875</x:v>
+      </x:c>
+      <x:c r="M18" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G186:G200)</x:f>
+        <x:v>0.9999999999999997</x:v>
+      </x:c>
+      <x:c r="N18" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F186:F200)-C18</x:f>
+        <x:v>-4.5102810375396984e-17</x:v>
+      </x:c>
+      <x:c r="O18" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P18" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I210:I226,"Mismatch")=0,IF(COUNTIF('Source Audit'!I210:I226,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q18" s="29" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="R18" s="28" t="n">
+        <x:f>B18-1000*('Prices'!H210/'Prices'!H6+'Prices'!H211/'Prices'!H7+'Prices'!H212/'Prices'!H8+'Prices'!H213/'Prices'!H9+'Prices'!H214/'Prices'!H10+'Prices'!H215/'Prices'!H11+'Prices'!H216/'Prices'!H12+'Prices'!H217/'Prices'!H13+'Prices'!H218/'Prices'!H14+'Prices'!H219/'Prices'!H15+'Prices'!H220/'Prices'!H16+'Prices'!H221/'Prices'!H17+'Prices'!H222/'Prices'!H18+'Prices'!H223/'Prices'!H19+'Prices'!H224/'Prices'!H20)/15</x:f>
+        <x:v>1.1368683772161603e-13</x:v>
+      </x:c>
+      <x:c r="S18" s="24" t="n">
+        <x:f>(D18-G18)*100</x:f>
+        <x:v>-8.541630875963335</x:v>
+      </x:c>
+      <x:c r="T18" s="24" t="n">
+        <x:f>(D18-J18)*100</x:f>
+        <x:v>-6.584871083120669</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1557,7 +1715,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R052644538e1b4531"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e89ceb4df074451"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8351,6 +8509,1230 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="193" ht="27" customHeight="1">
+      <x:c r="A193" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B193" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C193" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D193" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E193" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F193" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G193" s="33" t="n">
+        <x:f>H176</x:f>
+        <x:v>5907</x:v>
+      </x:c>
+      <x:c r="H193" s="35" t="n">
+        <x:v>5987</x:v>
+      </x:c>
+      <x:c r="I193" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J193" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K193" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="27" customHeight="1">
+      <x:c r="A194" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B194" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C194" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D194" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E194" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F194" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G194" s="17" t="n">
+        <x:f>H177</x:f>
+        <x:v>4274</x:v>
+      </x:c>
+      <x:c r="H194" s="34" t="n">
+        <x:v>4378</x:v>
+      </x:c>
+      <x:c r="I194" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J194" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K194" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="27" customHeight="1">
+      <x:c r="A195" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B195" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C195" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D195" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E195" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F195" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G195" s="33" t="n">
+        <x:f>H178</x:f>
+        <x:v>24.09</x:v>
+      </x:c>
+      <x:c r="H195" s="35" t="n">
+        <x:v>24.24</x:v>
+      </x:c>
+      <x:c r="I195" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J195" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K195" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="27" customHeight="1">
+      <x:c r="A196" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B196" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C196" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D196" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E196" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F196" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G196" s="17" t="n">
+        <x:f>H179</x:f>
+        <x:v>343.21</x:v>
+      </x:c>
+      <x:c r="H196" s="34" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="I196" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J196" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K196" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="27" customHeight="1">
+      <x:c r="A197" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B197" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C197" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D197" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E197" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F197" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G197" s="33" t="n">
+        <x:f>H180</x:f>
+        <x:v>4441</x:v>
+      </x:c>
+      <x:c r="H197" s="35" t="n">
+        <x:v>4488</x:v>
+      </x:c>
+      <x:c r="I197" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J197" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K197" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="27" customHeight="1">
+      <x:c r="A198" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B198" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C198" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D198" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E198" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F198" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G198" s="17" t="n">
+        <x:f>H181</x:f>
+        <x:v>49.39</x:v>
+      </x:c>
+      <x:c r="H198" s="34" t="n">
+        <x:v>49.7</x:v>
+      </x:c>
+      <x:c r="I198" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J198" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K198" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="27" customHeight="1">
+      <x:c r="A199" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B199" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C199" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D199" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E199" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F199" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G199" s="33" t="n">
+        <x:f>H182</x:f>
+        <x:v>78970</x:v>
+      </x:c>
+      <x:c r="H199" s="35" t="n">
+        <x:v>80760</x:v>
+      </x:c>
+      <x:c r="I199" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J199" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K199" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="27" customHeight="1">
+      <x:c r="A200" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B200" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C200" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D200" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E200" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F200" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G200" s="17" t="n">
+        <x:f>H183</x:f>
+        <x:v>55.67</x:v>
+      </x:c>
+      <x:c r="H200" s="34" t="n">
+        <x:v>53.99</x:v>
+      </x:c>
+      <x:c r="I200" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J200" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K200" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="27" customHeight="1">
+      <x:c r="A201" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B201" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C201" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D201" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E201" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F201" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G201" s="33" t="n">
+        <x:f>H184</x:f>
+        <x:v>31.33</x:v>
+      </x:c>
+      <x:c r="H201" s="35" t="n">
+        <x:v>28.43</x:v>
+      </x:c>
+      <x:c r="I201" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J201" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K201" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="27" customHeight="1">
+      <x:c r="A202" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B202" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C202" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D202" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E202" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F202" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G202" s="17" t="n">
+        <x:f>H185</x:f>
+        <x:v>13.36</x:v>
+      </x:c>
+      <x:c r="H202" s="34" t="n">
+        <x:v>12.42</x:v>
+      </x:c>
+      <x:c r="I202" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J202" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K202" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="27" customHeight="1">
+      <x:c r="A203" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B203" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C203" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D203" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E203" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F203" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G203" s="33" t="n">
+        <x:f>H186</x:f>
+        <x:v>422.03</x:v>
+      </x:c>
+      <x:c r="H203" s="35" t="n">
+        <x:v>426.23</x:v>
+      </x:c>
+      <x:c r="I203" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J203" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K203" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="27" customHeight="1">
+      <x:c r="A204" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B204" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C204" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D204" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E204" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F204" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G204" s="17" t="n">
+        <x:f>H187</x:f>
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="H204" s="34" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="I204" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J204" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K204" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="27" customHeight="1">
+      <x:c r="A205" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B205" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C205" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D205" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E205" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F205" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G205" s="33" t="n">
+        <x:f>H188</x:f>
+        <x:v>231.09</x:v>
+      </x:c>
+      <x:c r="H205" s="35" t="n">
+        <x:v>229.33</x:v>
+      </x:c>
+      <x:c r="I205" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J205" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K205" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="27" customHeight="1">
+      <x:c r="A206" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B206" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C206" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D206" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E206" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F206" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G206" s="17" t="n">
+        <x:f>H189</x:f>
+        <x:v>5458</x:v>
+      </x:c>
+      <x:c r="H206" s="34" t="n">
+        <x:v>5491</x:v>
+      </x:c>
+      <x:c r="I206" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J206" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K206" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="27" customHeight="1">
+      <x:c r="A207" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B207" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C207" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D207" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E207" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F207" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G207" s="33" t="n">
+        <x:f>H190</x:f>
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="H207" s="35" t="n">
+        <x:v>105.25</x:v>
+      </x:c>
+      <x:c r="I207" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J207" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K207" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="27" customHeight="1">
+      <x:c r="A208" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B208" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C208" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D208" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E208" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F208" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G208" s="17" t="n">
+        <x:f>H191</x:f>
+        <x:v>7744.06</x:v>
+      </x:c>
+      <x:c r="H208" s="34" t="n">
+        <x:v>7659.44</x:v>
+      </x:c>
+      <x:c r="I208" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J208" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K208" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="27" customHeight="1">
+      <x:c r="A209" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B209" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C209" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D209" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E209" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F209" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G209" s="33" t="n">
+        <x:f>H192</x:f>
+        <x:v>26713.0254</x:v>
+      </x:c>
+      <x:c r="H209" s="35" t="n">
+        <x:v>26140.0293</x:v>
+      </x:c>
+      <x:c r="I209" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J209" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="K209" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="27" customHeight="1">
+      <x:c r="A210" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B210" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C210" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D210" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E210" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F210" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G210" s="17" t="n">
+        <x:f>H193</x:f>
+        <x:v>5987</x:v>
+      </x:c>
+      <x:c r="H210" s="34" t="n">
+        <x:v>5946</x:v>
+      </x:c>
+      <x:c r="I210" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J210" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K210" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="27" customHeight="1">
+      <x:c r="A211" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B211" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C211" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D211" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E211" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F211" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G211" s="33" t="n">
+        <x:f>H194</x:f>
+        <x:v>4378</x:v>
+      </x:c>
+      <x:c r="H211" s="35" t="n">
+        <x:v>4373</x:v>
+      </x:c>
+      <x:c r="I211" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J211" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K211" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="27" customHeight="1">
+      <x:c r="A212" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B212" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C212" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D212" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E212" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F212" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G212" s="17" t="n">
+        <x:f>H195</x:f>
+        <x:v>24.24</x:v>
+      </x:c>
+      <x:c r="H212" s="34" t="n">
+        <x:v>25.38</x:v>
+      </x:c>
+      <x:c r="I212" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J212" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K212" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="27" customHeight="1">
+      <x:c r="A213" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B213" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C213" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D213" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E213" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F213" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G213" s="33" t="n">
+        <x:f>H196</x:f>
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="H213" s="35" t="n">
+        <x:v>335.53</x:v>
+      </x:c>
+      <x:c r="I213" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J213" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K213" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="27" customHeight="1">
+      <x:c r="A214" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B214" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C214" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D214" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E214" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F214" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G214" s="17" t="n">
+        <x:f>H197</x:f>
+        <x:v>4488</x:v>
+      </x:c>
+      <x:c r="H214" s="34" t="n">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="I214" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J214" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K214" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="27" customHeight="1">
+      <x:c r="A215" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B215" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C215" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D215" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E215" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F215" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G215" s="33" t="n">
+        <x:f>H198</x:f>
+        <x:v>49.7</x:v>
+      </x:c>
+      <x:c r="H215" s="35" t="n">
+        <x:v>50.79</x:v>
+      </x:c>
+      <x:c r="I215" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J215" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K215" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="27" customHeight="1">
+      <x:c r="A216" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B216" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C216" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D216" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E216" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F216" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G216" s="17" t="n">
+        <x:f>H199</x:f>
+        <x:v>80760</x:v>
+      </x:c>
+      <x:c r="H216" s="34" t="n">
+        <x:v>81410</x:v>
+      </x:c>
+      <x:c r="I216" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J216" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K216" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="27" customHeight="1">
+      <x:c r="A217" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B217" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C217" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D217" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E217" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F217" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G217" s="33" t="n">
+        <x:f>H200</x:f>
+        <x:v>53.99</x:v>
+      </x:c>
+      <x:c r="H217" s="35" t="n">
+        <x:v>55.16</x:v>
+      </x:c>
+      <x:c r="I217" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J217" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K217" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="27" customHeight="1">
+      <x:c r="A218" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B218" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C218" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D218" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E218" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F218" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G218" s="17" t="n">
+        <x:f>H201</x:f>
+        <x:v>28.43</x:v>
+      </x:c>
+      <x:c r="H218" s="34" t="n">
+        <x:v>28.86</x:v>
+      </x:c>
+      <x:c r="I218" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J218" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K218" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="27" customHeight="1">
+      <x:c r="A219" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B219" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C219" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D219" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E219" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F219" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G219" s="33" t="n">
+        <x:f>H202</x:f>
+        <x:v>12.42</x:v>
+      </x:c>
+      <x:c r="H219" s="35" t="n">
+        <x:v>12.92</x:v>
+      </x:c>
+      <x:c r="I219" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J219" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K219" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="27" customHeight="1">
+      <x:c r="A220" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B220" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C220" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D220" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E220" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F220" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G220" s="17" t="n">
+        <x:f>H203</x:f>
+        <x:v>426.23</x:v>
+      </x:c>
+      <x:c r="H220" s="34" t="n">
+        <x:v>424.47</x:v>
+      </x:c>
+      <x:c r="I220" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J220" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K220" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="27" customHeight="1">
+      <x:c r="A221" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B221" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C221" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D221" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E221" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F221" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G221" s="33" t="n">
+        <x:f>H204</x:f>
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="H221" s="35" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="I221" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J221" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K221" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="27" customHeight="1">
+      <x:c r="A222" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B222" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C222" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D222" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E222" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F222" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G222" s="17" t="n">
+        <x:f>H205</x:f>
+        <x:v>229.33</x:v>
+      </x:c>
+      <x:c r="H222" s="34" t="n">
+        <x:v>230.19</x:v>
+      </x:c>
+      <x:c r="I222" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J222" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K222" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="27" customHeight="1">
+      <x:c r="A223" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B223" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C223" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D223" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E223" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F223" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G223" s="33" t="n">
+        <x:f>H206</x:f>
+        <x:v>5491</x:v>
+      </x:c>
+      <x:c r="H223" s="35" t="n">
+        <x:v>5434</x:v>
+      </x:c>
+      <x:c r="I223" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J223" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K223" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="27" customHeight="1">
+      <x:c r="A224" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B224" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C224" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D224" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E224" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F224" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G224" s="17" t="n">
+        <x:f>H207</x:f>
+        <x:v>105.25</x:v>
+      </x:c>
+      <x:c r="H224" s="34" t="n">
+        <x:v>105.05</x:v>
+      </x:c>
+      <x:c r="I224" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J224" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K224" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="27" customHeight="1">
+      <x:c r="A225" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B225" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C225" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D225" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E225" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F225" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G225" s="33" t="n">
+        <x:f>H208</x:f>
+        <x:v>7659.44</x:v>
+      </x:c>
+      <x:c r="H225" s="35" t="n">
+        <x:v>7690.73</x:v>
+      </x:c>
+      <x:c r="I225" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J225" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K225" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="27" customHeight="1">
+      <x:c r="A226" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B226" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C226" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D226" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E226" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F226" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G226" s="17" t="n">
+        <x:f>H209</x:f>
+        <x:v>26140.0293</x:v>
+      </x:c>
+      <x:c r="H226" s="34" t="n">
+        <x:v>26430.8867</x:v>
+      </x:c>
+      <x:c r="I226" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J226" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="K226" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -8358,7 +9740,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b2ba0ea84a6427d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd822c473cbf4499d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13472,6 +14854,936 @@
         <x:v>0.052817612603514474</x:v>
       </x:c>
     </x:row>
+    <x:row r="171" ht="27" customHeight="1">
+      <x:c r="A171" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B171" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C171" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D171" s="21" t="n">
+        <x:f>G156</x:f>
+        <x:v>0.0700730678404319</x:v>
+      </x:c>
+      <x:c r="E171" s="23" t="n">
+        <x:f>'Prices'!H193/'Prices'!G193-1</x:f>
+        <x:v>0.0135432537667175</x:v>
+      </x:c>
+      <x:c r="F171" s="21" t="n">
+        <x:f>D171*E171</x:f>
+        <x:v>0.0009490173399753801</x:v>
+      </x:c>
+      <x:c r="G171" s="21" t="n">
+        <x:f>D171*(1+E171)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.0715696950402928</x:v>
+      </x:c>
+      <x:c r="H171" s="23" t="n">
+        <x:f>'Prices'!H193/'Prices'!I193-1</x:f>
+        <x:v>-0.022849681736575866</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="27" customHeight="1">
+      <x:c r="A172" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B172" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C172" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D172" s="20" t="n">
+        <x:f>G157</x:f>
+        <x:v>0.06500242043427633</x:v>
+      </x:c>
+      <x:c r="E172" s="22" t="n">
+        <x:f>'Prices'!H194/'Prices'!G194-1</x:f>
+        <x:v>0.02433317735142726</x:v>
+      </x:c>
+      <x:c r="F172" s="20" t="n">
+        <x:f>D172*E172</x:f>
+        <x:v>0.0015817154246992853</x:v>
+      </x:c>
+      <x:c r="G172" s="20" t="n">
+        <x:f>D172*(1+E172)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.06709752728103417</x:v>
+      </x:c>
+      <x:c r="H172" s="22" t="n">
+        <x:f>'Prices'!H194/'Prices'!I194-1</x:f>
+        <x:v>-0.08390876752458676</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="27" customHeight="1">
+      <x:c r="A173" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B173" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C173" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D173" s="21" t="n">
+        <x:f>G158</x:f>
+        <x:v>0.062045720428987323</x:v>
+      </x:c>
+      <x:c r="E173" s="23" t="n">
+        <x:f>'Prices'!H195/'Prices'!G195-1</x:f>
+        <x:v>0.0062266500622665255</x:v>
+      </x:c>
+      <x:c r="F173" s="21" t="n">
+        <x:f>D173*E173</x:f>
+        <x:v>0.00038633698897252533</x:v>
+      </x:c>
+      <x:c r="G173" s="21" t="n">
+        <x:f>D173*(1+E173)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.06291343458575449</x:v>
+      </x:c>
+      <x:c r="H173" s="23" t="n">
+        <x:f>'Prices'!H195/'Prices'!I195-1</x:f>
+        <x:v>-0.14103472714386966</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="27" customHeight="1">
+      <x:c r="A174" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B174" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C174" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D174" s="20" t="n">
+        <x:f>G159</x:f>
+        <x:v>0.05999539738079375</x:v>
+      </x:c>
+      <x:c r="E174" s="22" t="n">
+        <x:f>'Prices'!H196/'Prices'!G196-1</x:f>
+        <x:v>-0.05305789458349108</x:v>
+      </x:c>
+      <x:c r="F174" s="20" t="n">
+        <x:f>D174*E174</x:f>
+        <x:v>-0.0031832294697248117</x:v>
+      </x:c>
+      <x:c r="G174" s="20" t="n">
+        <x:f>D174*(1+E174)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.057250213389887915</x:v>
+      </x:c>
+      <x:c r="H174" s="22" t="n">
+        <x:f>'Prices'!H196/'Prices'!I196-1</x:f>
+        <x:v>-0.21835541980326612</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="27" customHeight="1">
+      <x:c r="A175" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B175" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C175" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D175" s="21" t="n">
+        <x:f>G160</x:f>
+        <x:v>0.06488132779862156</x:v>
+      </x:c>
+      <x:c r="E175" s="23" t="n">
+        <x:f>'Prices'!H197/'Prices'!G197-1</x:f>
+        <x:v>0.010583201981535728</x:v>
+      </x:c>
+      <x:c r="F175" s="21" t="n">
+        <x:f>D175*E175</x:f>
+        <x:v>0.0006866521969230409</x:v>
+      </x:c>
+      <x:c r="G175" s="21" t="n">
+        <x:f>D175*(1+E175)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.06607353643263218</x:v>
+      </x:c>
+      <x:c r="H175" s="23" t="n">
+        <x:f>'Prices'!H197/'Prices'!I197-1</x:f>
+        <x:v>-0.09788944723618087</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="27" customHeight="1">
+      <x:c r="A176" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B176" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C176" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D176" s="20" t="n">
+        <x:f>G161</x:f>
+        <x:v>0.06916775969745159</x:v>
+      </x:c>
+      <x:c r="E176" s="22" t="n">
+        <x:f>'Prices'!H198/'Prices'!G198-1</x:f>
+        <x:v>0.006276574205304808</x:v>
+      </x:c>
+      <x:c r="F176" s="20" t="n">
+        <x:f>D176*E176</x:f>
+        <x:v>0.0004341365763557461</x:v>
+      </x:c>
+      <x:c r="G176" s="20" t="n">
+        <x:f>D176*(1+E176)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.0701385558856654</x:v>
+      </x:c>
+      <x:c r="H176" s="22" t="n">
+        <x:f>'Prices'!H198/'Prices'!I198-1</x:f>
+        <x:v>-0.042389210019267765</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="27" customHeight="1">
+      <x:c r="A177" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B177" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C177" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D177" s="21" t="n">
+        <x:f>G162</x:f>
+        <x:v>0.07068677205096069</x:v>
+      </x:c>
+      <x:c r="E177" s="23" t="n">
+        <x:f>'Prices'!H199/'Prices'!G199-1</x:f>
+        <x:v>0.022666835507154648</x:v>
+      </x:c>
+      <x:c r="F177" s="21" t="n">
+        <x:f>D177*E177</x:f>
+        <x:v>0.0016022454346108625</x:v>
+      </x:c>
+      <x:c r="G177" s="21" t="n">
+        <x:f>D177*(1+E177)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.07284639592125083</x:v>
+      </x:c>
+      <x:c r="H177" s="23" t="n">
+        <x:f>'Prices'!H199/'Prices'!I199-1</x:f>
+        <x:v>-0.005418719211822687</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="27" customHeight="1">
+      <x:c r="A178" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B178" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C178" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D178" s="20" t="n">
+        <x:f>G163</x:f>
+        <x:v>0.06503142275469338</x:v>
+      </x:c>
+      <x:c r="E178" s="22" t="n">
+        <x:f>'Prices'!H200/'Prices'!G200-1</x:f>
+        <x:v>-0.030177833662654918</x:v>
+      </x:c>
+      <x:c r="F178" s="20" t="n">
+        <x:f>D178*E178</x:f>
+        <x:v>-0.001962507458736929</x:v>
+      </x:c>
+      <x:c r="G178" s="20" t="n">
+        <x:f>D178*(1+E178)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.06355520290326369</x:v>
+      </x:c>
+      <x:c r="H178" s="22" t="n">
+        <x:f>'Prices'!H200/'Prices'!I200-1</x:f>
+        <x:v>-0.13227258116361296</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="27" customHeight="1">
+      <x:c r="A179" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B179" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C179" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D179" s="21" t="n">
+        <x:f>G164</x:f>
+        <x:v>0.05571700946683776</x:v>
+      </x:c>
+      <x:c r="E179" s="23" t="n">
+        <x:f>'Prices'!H201/'Prices'!G201-1</x:f>
+        <x:v>-0.09256303862112991</x:v>
+      </x:c>
+      <x:c r="F179" s="21" t="n">
+        <x:f>D179*E179</x:f>
+        <x:v>-0.005157335699132765</x:v>
+      </x:c>
+      <x:c r="G179" s="21" t="n">
+        <x:f>D179*(1+E179)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.05094950991229948</x:v>
+      </x:c>
+      <x:c r="H179" s="23" t="n">
+        <x:f>'Prices'!H201/'Prices'!I201-1</x:f>
+        <x:v>-0.304379740641057</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="27" customHeight="1">
+      <x:c r="A180" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B180" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C180" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D180" s="20" t="n">
+        <x:f>G165</x:f>
+        <x:v>0.06095687905956469</x:v>
+      </x:c>
+      <x:c r="E180" s="22" t="n">
+        <x:f>'Prices'!H202/'Prices'!G202-1</x:f>
+        <x:v>-0.07035928143712566</x:v>
+      </x:c>
+      <x:c r="F180" s="20" t="n">
+        <x:f>D180*E180</x:f>
+        <x:v>-0.004288882209280745</x:v>
+      </x:c>
+      <x:c r="G180" s="20" t="n">
+        <x:f>D180*(1+E180)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.05710493071017206</x:v>
+      </x:c>
+      <x:c r="H180" s="22" t="n">
+        <x:f>'Prices'!H202/'Prices'!I202-1</x:f>
+        <x:v>-0.22033898305084743</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="27" customHeight="1">
+      <x:c r="A181" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B181" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C181" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D181" s="21" t="n">
+        <x:f>G166</x:f>
+        <x:v>0.06932839809621295</x:v>
+      </x:c>
+      <x:c r="E181" s="23" t="n">
+        <x:f>'Prices'!H203/'Prices'!G203-1</x:f>
+        <x:v>0.009951899154088784</x:v>
+      </x:c>
+      <x:c r="F181" s="21" t="n">
+        <x:f>D181*E181</x:f>
+        <x:v>0.0006899492263680321</x:v>
+      </x:c>
+      <x:c r="G181" s="21" t="n">
+        <x:f>D181*(1+E181)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.07055821794549129</x:v>
+      </x:c>
+      <x:c r="H181" s="23" t="n">
+        <x:f>'Prices'!H203/'Prices'!I203-1</x:f>
+        <x:v>-0.03665950954910158</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="27" customHeight="1">
+      <x:c r="A182" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B182" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C182" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D182" s="20" t="n">
+        <x:f>G167</x:f>
+        <x:v>0.07234872215682168</x:v>
+      </x:c>
+      <x:c r="E182" s="22" t="n">
+        <x:f>'Prices'!H204/'Prices'!G204-1</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F182" s="20" t="n">
+        <x:f>D182*E182</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G182" s="20" t="n">
+        <x:f>D182*(1+E182)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.07290656094038536</x:v>
+      </x:c>
+      <x:c r="H182" s="22" t="n">
+        <x:f>'Prices'!H204/'Prices'!I204-1</x:f>
+        <x:v>-0.0045972784111806275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="27" customHeight="1">
+      <x:c r="A183" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B183" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C183" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D183" s="21" t="n">
+        <x:f>G168</x:f>
+        <x:v>0.07022151174487397</x:v>
+      </x:c>
+      <x:c r="E183" s="23" t="n">
+        <x:f>'Prices'!H205/'Prices'!G205-1</x:f>
+        <x:v>-0.007616080315028695</x:v>
+      </x:c>
+      <x:c r="F183" s="21" t="n">
+        <x:f>D183*E183</x:f>
+        <x:v>-0.0005348126732916909</x:v>
+      </x:c>
+      <x:c r="G183" s="21" t="n">
+        <x:f>D183*(1+E183)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.07022401254833445</x:v>
+      </x:c>
+      <x:c r="H183" s="23" t="n">
+        <x:f>'Prices'!H205/'Prices'!I205-1</x:f>
+        <x:v>-0.041222459132906786</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="27" customHeight="1">
+      <x:c r="A184" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B184" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C184" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D184" s="20" t="n">
+        <x:f>G169</x:f>
+        <x:v>0.0680217901298761</x:v>
+      </x:c>
+      <x:c r="E184" s="22" t="n">
+        <x:f>'Prices'!H206/'Prices'!G206-1</x:f>
+        <x:v>0.006046170758519542</x:v>
+      </x:c>
+      <x:c r="F184" s="20" t="n">
+        <x:f>D184*E184</x:f>
+        <x:v>0.00041127135842541007</x:v>
+      </x:c>
+      <x:c r="G184" s="20" t="n">
+        <x:f>D184*(1+E184)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.06896070889710336</x:v>
+      </x:c>
+      <x:c r="H184" s="22" t="n">
+        <x:f>'Prices'!H206/'Prices'!I206-1</x:f>
+        <x:v>-0.05847050754458161</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="27" customHeight="1">
+      <x:c r="A185" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B185" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C185" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D185" s="21" t="n">
+        <x:f>G170</x:f>
+        <x:v>0.07652180095959618</x:v>
+      </x:c>
+      <x:c r="E185" s="23" t="n">
+        <x:f>'Prices'!H207/'Prices'!G207-1</x:f>
+        <x:v>0.00959232613908867</x:v>
+      </x:c>
+      <x:c r="F185" s="21" t="n">
+        <x:f>D185*E185</x:f>
+        <x:v>0.0007340220715548748</x:v>
+      </x:c>
+      <x:c r="G185" s="21" t="n">
+        <x:f>D185*(1+E185)/(1+SUM($F$171:$F$185))</x:f>
+        <x:v>0.07785149760643234</x:v>
+      </x:c>
+      <x:c r="H185" s="23" t="n">
+        <x:f>'Prices'!H207/'Prices'!I207-1</x:f>
+        <x:v>0.06291658250858423</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="27" customHeight="1">
+      <x:c r="A186" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B186" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C186" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D186" s="20" t="n">
+        <x:f>G171</x:f>
+        <x:v>0.0715696950402928</x:v>
+      </x:c>
+      <x:c r="E186" s="22" t="n">
+        <x:f>'Prices'!H210/'Prices'!G210-1</x:f>
+        <x:v>-0.00684817103724733</x:v>
+      </x:c>
+      <x:c r="F186" s="20" t="n">
+        <x:f>D186*E186</x:f>
+        <x:v>-0.0004901215127195571</x:v>
+      </x:c>
+      <x:c r="G186" s="20" t="n">
+        <x:f>D186*(1+E186)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.07049543965473073</x:v>
+      </x:c>
+      <x:c r="H186" s="22" t="n">
+        <x:f>'Prices'!H210/'Prices'!I210-1</x:f>
+        <x:v>-0.02954137424514447</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="27" customHeight="1">
+      <x:c r="A187" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B187" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C187" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D187" s="21" t="n">
+        <x:f>G172</x:f>
+        <x:v>0.06709752728103417</x:v>
+      </x:c>
+      <x:c r="E187" s="23" t="n">
+        <x:f>'Prices'!H211/'Prices'!G211-1</x:f>
+        <x:v>-0.0011420740063956547</x:v>
+      </x:c>
+      <x:c r="F187" s="21" t="n">
+        <x:f>D187*E187</x:f>
+        <x:v>-0.00007663034180109244</x:v>
+      </x:c>
+      <x:c r="G187" s="21" t="n">
+        <x:f>D187*(1+E187)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.066470117381231</x:v>
+      </x:c>
+      <x:c r="H187" s="23" t="n">
+        <x:f>'Prices'!H211/'Prices'!I211-1</x:f>
+        <x:v>-0.08495501150868379</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="27" customHeight="1">
+      <x:c r="A188" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B188" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C188" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D188" s="20" t="n">
+        <x:f>G173</x:f>
+        <x:v>0.06291343458575449</x:v>
+      </x:c>
+      <x:c r="E188" s="22" t="n">
+        <x:f>'Prices'!H212/'Prices'!G212-1</x:f>
+        <x:v>0.04702970297029707</x:v>
+      </x:c>
+      <x:c r="F188" s="20" t="n">
+        <x:f>D188*E188</x:f>
+        <x:v>0.0029588001414092486</x:v>
+      </x:c>
+      <x:c r="G188" s="20" t="n">
+        <x:f>D188*(1+E188)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06533089490653239</x:v>
+      </x:c>
+      <x:c r="H188" s="22" t="n">
+        <x:f>'Prices'!H212/'Prices'!I212-1</x:f>
+        <x:v>-0.1006378454996456</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="27" customHeight="1">
+      <x:c r="A189" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B189" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C189" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D189" s="21" t="n">
+        <x:f>G174</x:f>
+        <x:v>0.057250213389887915</x:v>
+      </x:c>
+      <x:c r="E189" s="23" t="n">
+        <x:f>'Prices'!H213/'Prices'!G213-1</x:f>
+        <x:v>0.032399999999999984</x:v>
+      </x:c>
+      <x:c r="F189" s="21" t="n">
+        <x:f>D189*E189</x:f>
+        <x:v>0.0018549069138323675</x:v>
+      </x:c>
+      <x:c r="G189" s="21" t="n">
+        <x:f>D189*(1+E189)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.058619392813888886</x:v>
+      </x:c>
+      <x:c r="H189" s="23" t="n">
+        <x:f>'Prices'!H213/'Prices'!I213-1</x:f>
+        <x:v>-0.193030135404892</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="27" customHeight="1">
+      <x:c r="A190" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B190" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C190" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D190" s="20" t="n">
+        <x:f>G175</x:f>
+        <x:v>0.06607353643263218</x:v>
+      </x:c>
+      <x:c r="E190" s="22" t="n">
+        <x:f>'Prices'!H214/'Prices'!G214-1</x:f>
+        <x:v>-0.006684491978609652</x:v>
+      </x:c>
+      <x:c r="F190" s="20" t="n">
+        <x:f>D190*E190</x:f>
+        <x:v>-0.00044166802428230245</x:v>
+      </x:c>
+      <x:c r="G190" s="20" t="n">
+        <x:f>D190*(1+E190)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06509250392467882</x:v>
+      </x:c>
+      <x:c r="H190" s="22" t="n">
+        <x:f>'Prices'!H214/'Prices'!I214-1</x:f>
+        <x:v>-0.10391959798994976</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="27" customHeight="1">
+      <x:c r="A191" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B191" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C191" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D191" s="21" t="n">
+        <x:f>G176</x:f>
+        <x:v>0.0701385558856654</x:v>
+      </x:c>
+      <x:c r="E191" s="23" t="n">
+        <x:f>'Prices'!H215/'Prices'!G215-1</x:f>
+        <x:v>0.021931589537223184</x:v>
+      </x:c>
+      <x:c r="F191" s="21" t="n">
+        <x:f>D191*E191</x:f>
+        <x:v>0.0015382500184180027</x:v>
+      </x:c>
+      <x:c r="G191" s="21" t="n">
+        <x:f>D191*(1+E191)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.07108776395929049</x:v>
+      </x:c>
+      <x:c r="H191" s="23" t="n">
+        <x:f>'Prices'!H215/'Prices'!I215-1</x:f>
+        <x:v>-0.021387283236994237</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="27" customHeight="1">
+      <x:c r="A192" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B192" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C192" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D192" s="20" t="n">
+        <x:f>G177</x:f>
+        <x:v>0.07284639592125083</x:v>
+      </x:c>
+      <x:c r="E192" s="22" t="n">
+        <x:f>'Prices'!H216/'Prices'!G216-1</x:f>
+        <x:v>0.008048538880633949</x:v>
+      </x:c>
+      <x:c r="F192" s="20" t="n">
+        <x:f>D192*E192</x:f>
+        <x:v>0.0005863070498862416</x:v>
+      </x:c>
+      <x:c r="G192" s="20" t="n">
+        <x:f>D192*(1+E192)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.07282923101638225</x:v>
+      </x:c>
+      <x:c r="H192" s="22" t="n">
+        <x:f>'Prices'!H216/'Prices'!I216-1</x:f>
+        <x:v>0.002586206896551646</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="27" customHeight="1">
+      <x:c r="A193" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B193" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C193" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D193" s="21" t="n">
+        <x:f>G178</x:f>
+        <x:v>0.06355520290326369</x:v>
+      </x:c>
+      <x:c r="E193" s="23" t="n">
+        <x:f>'Prices'!H217/'Prices'!G217-1</x:f>
+        <x:v>0.02167067975551018</x:v>
+      </x:c>
+      <x:c r="F193" s="21" t="n">
+        <x:f>D193*E193</x:f>
+        <x:v>0.0013772844489130984</x:v>
+      </x:c>
+      <x:c r="G193" s="21" t="n">
+        <x:f>D193*(1+E193)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06439887040109012</x:v>
+      </x:c>
+      <x:c r="H193" s="23" t="n">
+        <x:f>'Prices'!H217/'Prices'!I217-1</x:f>
+        <x:v>-0.11346833815493418</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="27" customHeight="1">
+      <x:c r="A194" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B194" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C194" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D194" s="20" t="n">
+        <x:f>G179</x:f>
+        <x:v>0.05094950991229948</x:v>
+      </x:c>
+      <x:c r="E194" s="22" t="n">
+        <x:f>'Prices'!H218/'Prices'!G218-1</x:f>
+        <x:v>0.01512486809708058</x:v>
+      </x:c>
+      <x:c r="F194" s="20" t="n">
+        <x:f>D194*E194</x:f>
+        <x:v>0.0007706046170344292</x:v>
+      </x:c>
+      <x:c r="G194" s="20" t="n">
+        <x:f>D194*(1+E194)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.05129507721826792</x:v>
+      </x:c>
+      <x:c r="H194" s="22" t="n">
+        <x:f>'Prices'!H218/'Prices'!I218-1</x:f>
+        <x:v>-0.293858575972596</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="27" customHeight="1">
+      <x:c r="A195" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B195" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C195" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D195" s="21" t="n">
+        <x:f>G180</x:f>
+        <x:v>0.05710493071017206</x:v>
+      </x:c>
+      <x:c r="E195" s="23" t="n">
+        <x:f>'Prices'!H219/'Prices'!G219-1</x:f>
+        <x:v>0.040257648953301084</x:v>
+      </x:c>
+      <x:c r="F195" s="21" t="n">
+        <x:f>D195*E195</x:f>
+        <x:v>0.002298910254032689</x:v>
+      </x:c>
+      <x:c r="G195" s="21" t="n">
+        <x:f>D195*(1+E195)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.058915658579842524</x:v>
+      </x:c>
+      <x:c r="H195" s="23" t="n">
+        <x:f>'Prices'!H219/'Prices'!I219-1</x:f>
+        <x:v>-0.1889516635279347</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="27" customHeight="1">
+      <x:c r="A196" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B196" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C196" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D196" s="20" t="n">
+        <x:f>G181</x:f>
+        <x:v>0.07055821794549129</x:v>
+      </x:c>
+      <x:c r="E196" s="22" t="n">
+        <x:f>'Prices'!H220/'Prices'!G220-1</x:f>
+        <x:v>-0.004129226004739195</x:v>
+      </x:c>
+      <x:c r="F196" s="20" t="n">
+        <x:f>D196*E196</x:f>
+        <x:v>-0.00029135082838857834</x:v>
+      </x:c>
+      <x:c r="G196" s="20" t="n">
+        <x:f>D196*(1+E196)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06968941208769541</x:v>
+      </x:c>
+      <x:c r="H196" s="22" t="n">
+        <x:f>'Prices'!H220/'Prices'!I220-1</x:f>
+        <x:v>-0.04063736015368957</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="27" customHeight="1">
+      <x:c r="A197" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B197" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C197" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D197" s="21" t="n">
+        <x:f>G182</x:f>
+        <x:v>0.07290656094038536</x:v>
+      </x:c>
+      <x:c r="E197" s="23" t="n">
+        <x:f>'Prices'!H221/'Prices'!G221-1</x:f>
+        <x:v>-0.016441899131719895</x:v>
+      </x:c>
+      <x:c r="F197" s="21" t="n">
+        <x:f>D197*E197</x:f>
+        <x:v>-0.0011987223210224056</x:v>
+      </x:c>
+      <x:c r="G197" s="21" t="n">
+        <x:f>D197*(1+E197)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.07111854164686994</x:v>
+      </x:c>
+      <x:c r="H197" s="23" t="n">
+        <x:f>'Prices'!H221/'Prices'!I221-1</x:f>
+        <x:v>-0.020963589554983453</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="27" customHeight="1">
+      <x:c r="A198" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B198" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C198" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D198" s="20" t="n">
+        <x:f>G183</x:f>
+        <x:v>0.07022401254833445</x:v>
+      </x:c>
+      <x:c r="E198" s="22" t="n">
+        <x:f>'Prices'!H222/'Prices'!G222-1</x:f>
+        <x:v>0.0037500545066060376</x:v>
+      </x:c>
+      <x:c r="F198" s="20" t="n">
+        <x:f>D198*E198</x:f>
+        <x:v>0.00026334387472884055</x:v>
+      </x:c>
+      <x:c r="G198" s="20" t="n">
+        <x:f>D198*(1+E198)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06990808940652919</x:v>
+      </x:c>
+      <x:c r="H198" s="22" t="n">
+        <x:f>'Prices'!H222/'Prices'!I222-1</x:f>
+        <x:v>-0.037626991094945494</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="27" customHeight="1">
+      <x:c r="A199" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B199" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C199" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D199" s="21" t="n">
+        <x:f>G184</x:f>
+        <x:v>0.06896070889710336</x:v>
+      </x:c>
+      <x:c r="E199" s="23" t="n">
+        <x:f>'Prices'!H223/'Prices'!G223-1</x:f>
+        <x:v>-0.01038062283737029</x:v>
+      </x:c>
+      <x:c r="F199" s="21" t="n">
+        <x:f>D199*E199</x:f>
+        <x:v>-0.0007158551096585157</x:v>
+      </x:c>
+      <x:c r="G199" s="21" t="n">
+        <x:f>D199*(1+E199)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.06768401571869972</x:v>
+      </x:c>
+      <x:c r="H199" s="23" t="n">
+        <x:f>'Prices'!H223/'Prices'!I223-1</x:f>
+        <x:v>-0.0682441700960219</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="27" customHeight="1">
+      <x:c r="A200" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B200" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C200" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D200" s="20" t="n">
+        <x:f>G185</x:f>
+        <x:v>0.07785149760643234</x:v>
+      </x:c>
+      <x:c r="E200" s="22" t="n">
+        <x:f>'Prices'!H224/'Prices'!G224-1</x:f>
+        <x:v>-0.0019002375296912621</x:v>
+      </x:c>
+      <x:c r="F200" s="20" t="n">
+        <x:f>D200*E200</x:f>
+        <x:v>-0.0001479363374944122</x:v>
+      </x:c>
+      <x:c r="G200" s="20" t="n">
+        <x:f>D200*(1+E200)/(1+SUM($F$186:$F$200))</x:f>
+        <x:v>0.07706499128427037</x:v>
+      </x:c>
+      <x:c r="H200" s="22" t="n">
+        <x:f>'Prices'!H224/'Prices'!I224-1</x:f>
+        <x:v>0.06089678852757019</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -13479,7 +15791,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c2b8378db54d13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d76f3a42074f3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20766,6 +23078,1302 @@
       </x:c>
       <x:c r="M192" s="14" t="str"/>
     </x:row>
+    <x:row r="193" ht="50" customHeight="1">
+      <x:c r="A193" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B193" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C193" s="33" t="n">
+        <x:v>5987</x:v>
+      </x:c>
+      <x:c r="D193" s="33" t="n">
+        <x:v>5987</x:v>
+      </x:c>
+      <x:c r="E193" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F193" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G193" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H193" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I193" s="32" t="str">
+        <x:f>IF(AND(G193=H193,C193&gt;0,ABS(C193-'Prices'!H193)&lt;=MAX(0.01,'Prices'!H193*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J193" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K193" s="16" t="str"/>
+      <x:c r="L193" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M193" s="16" t="str"/>
+    </x:row>
+    <x:row r="194" ht="50" customHeight="1">
+      <x:c r="A194" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B194" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C194" s="17" t="n">
+        <x:v>4378</x:v>
+      </x:c>
+      <x:c r="D194" s="17" t="n">
+        <x:v>4378</x:v>
+      </x:c>
+      <x:c r="E194" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F194" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G194" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H194" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I194" s="31" t="str">
+        <x:f>IF(AND(G194=H194,C194&gt;0,ABS(C194-'Prices'!H194)&lt;=MAX(0.01,'Prices'!H194*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J194" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K194" s="14" t="str"/>
+      <x:c r="L194" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M194" s="14" t="str"/>
+    </x:row>
+    <x:row r="195" ht="50" customHeight="1">
+      <x:c r="A195" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B195" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C195" s="33" t="n">
+        <x:v>24.24</x:v>
+      </x:c>
+      <x:c r="D195" s="33" t="n">
+        <x:v>24.24</x:v>
+      </x:c>
+      <x:c r="E195" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F195" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G195" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H195" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I195" s="32" t="str">
+        <x:f>IF(AND(G195=H195,C195&gt;0,ABS(C195-'Prices'!H195)&lt;=MAX(0.01,'Prices'!H195*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J195" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K195" s="16" t="str"/>
+      <x:c r="L195" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M195" s="16" t="str"/>
+    </x:row>
+    <x:row r="196" ht="50" customHeight="1">
+      <x:c r="A196" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B196" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C196" s="17" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="D196" s="17" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="E196" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F196" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G196" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H196" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I196" s="31" t="str">
+        <x:f>IF(AND(G196=H196,C196&gt;0,ABS(C196-'Prices'!H196)&lt;=MAX(0.01,'Prices'!H196*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J196" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K196" s="14" t="str"/>
+      <x:c r="L196" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M196" s="14" t="str"/>
+    </x:row>
+    <x:row r="197" ht="50" customHeight="1">
+      <x:c r="A197" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B197" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C197" s="33" t="n">
+        <x:v>4488</x:v>
+      </x:c>
+      <x:c r="D197" s="33" t="n">
+        <x:v>4488</x:v>
+      </x:c>
+      <x:c r="E197" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F197" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G197" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H197" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I197" s="32" t="str">
+        <x:f>IF(AND(G197=H197,C197&gt;0,ABS(C197-'Prices'!H197)&lt;=MAX(0.01,'Prices'!H197*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J197" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K197" s="16" t="str"/>
+      <x:c r="L197" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M197" s="16" t="str"/>
+    </x:row>
+    <x:row r="198" ht="50" customHeight="1">
+      <x:c r="A198" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B198" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C198" s="17" t="n">
+        <x:v>49.7</x:v>
+      </x:c>
+      <x:c r="D198" s="17" t="n">
+        <x:v>49.7</x:v>
+      </x:c>
+      <x:c r="E198" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F198" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G198" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H198" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I198" s="31" t="str">
+        <x:f>IF(AND(G198=H198,C198&gt;0,ABS(C198-'Prices'!H198)&lt;=MAX(0.01,'Prices'!H198*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J198" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K198" s="14" t="str"/>
+      <x:c r="L198" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M198" s="14" t="str"/>
+    </x:row>
+    <x:row r="199" ht="50" customHeight="1">
+      <x:c r="A199" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B199" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C199" s="33" t="n">
+        <x:v>80760</x:v>
+      </x:c>
+      <x:c r="D199" s="33" t="n">
+        <x:v>80760</x:v>
+      </x:c>
+      <x:c r="E199" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F199" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G199" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H199" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I199" s="32" t="str">
+        <x:f>IF(AND(G199=H199,C199&gt;0,ABS(C199-'Prices'!H199)&lt;=MAX(0.01,'Prices'!H199*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J199" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K199" s="16" t="str"/>
+      <x:c r="L199" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M199" s="16" t="str"/>
+    </x:row>
+    <x:row r="200" ht="50" customHeight="1">
+      <x:c r="A200" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B200" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C200" s="17" t="n">
+        <x:v>53.99</x:v>
+      </x:c>
+      <x:c r="D200" s="17" t="n">
+        <x:v>53.99</x:v>
+      </x:c>
+      <x:c r="E200" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F200" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G200" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H200" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I200" s="31" t="str">
+        <x:f>IF(AND(G200=H200,C200&gt;0,ABS(C200-'Prices'!H200)&lt;=MAX(0.01,'Prices'!H200*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J200" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K200" s="14" t="str"/>
+      <x:c r="L200" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M200" s="14" t="str"/>
+    </x:row>
+    <x:row r="201" ht="50" customHeight="1">
+      <x:c r="A201" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B201" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C201" s="33" t="n">
+        <x:v>28.43</x:v>
+      </x:c>
+      <x:c r="D201" s="33" t="n">
+        <x:v>28.43</x:v>
+      </x:c>
+      <x:c r="E201" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F201" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G201" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H201" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I201" s="32" t="str">
+        <x:f>IF(AND(OR(G201=H201,AND(B201="OUST",G201="XNAS",H201="XNYS",LEFT(M201,34)="ouster-marketstack-legacy-nyse-tag")),C201&gt;0,ABS(C201-'Prices'!H201)&lt;=MAX(0.01,'Prices'!H201*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J201" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K201" s="16" t="str"/>
+      <x:c r="L201" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M201" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="50" customHeight="1">
+      <x:c r="A202" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B202" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C202" s="17" t="n">
+        <x:v>12.42</x:v>
+      </x:c>
+      <x:c r="D202" s="17" t="n">
+        <x:v>12.42</x:v>
+      </x:c>
+      <x:c r="E202" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F202" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G202" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H202" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I202" s="31" t="str">
+        <x:f>IF(AND(G202=H202,C202&gt;0,ABS(C202-'Prices'!H202)&lt;=MAX(0.01,'Prices'!H202*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J202" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K202" s="14" t="str"/>
+      <x:c r="L202" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M202" s="14" t="str"/>
+    </x:row>
+    <x:row r="203" ht="50" customHeight="1">
+      <x:c r="A203" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B203" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C203" s="33" t="n">
+        <x:v>426.23</x:v>
+      </x:c>
+      <x:c r="D203" s="33" t="n">
+        <x:v>426.23</x:v>
+      </x:c>
+      <x:c r="E203" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F203" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G203" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H203" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I203" s="32" t="str">
+        <x:f>IF(AND(G203=H203,C203&gt;0,ABS(C203-'Prices'!H203)&lt;=MAX(0.01,'Prices'!H203*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J203" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K203" s="16" t="str"/>
+      <x:c r="L203" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M203" s="16" t="str"/>
+    </x:row>
+    <x:row r="204" ht="50" customHeight="1">
+      <x:c r="A204" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B204" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C204" s="17" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="D204" s="17" t="n">
+        <x:v>270.65</x:v>
+      </x:c>
+      <x:c r="E204" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F204" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G204" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H204" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I204" s="31" t="str">
+        <x:f>IF(AND(G204=H204,C204&gt;0,ABS(C204-'Prices'!H204)&lt;=MAX(0.01,'Prices'!H204*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J204" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K204" s="14" t="str"/>
+      <x:c r="L204" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M204" s="14" t="str"/>
+    </x:row>
+    <x:row r="205" ht="50" customHeight="1">
+      <x:c r="A205" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B205" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C205" s="33" t="n">
+        <x:v>229.33</x:v>
+      </x:c>
+      <x:c r="D205" s="33" t="n">
+        <x:v>229.33</x:v>
+      </x:c>
+      <x:c r="E205" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F205" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G205" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H205" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I205" s="32" t="str">
+        <x:f>IF(AND(G205=H205,C205&gt;0,ABS(C205-'Prices'!H205)&lt;=MAX(0.01,'Prices'!H205*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J205" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K205" s="16" t="str"/>
+      <x:c r="L205" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M205" s="16" t="str"/>
+    </x:row>
+    <x:row r="206" ht="50" customHeight="1">
+      <x:c r="A206" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B206" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C206" s="17" t="n">
+        <x:v>5491</x:v>
+      </x:c>
+      <x:c r="D206" s="17" t="n">
+        <x:v>5491</x:v>
+      </x:c>
+      <x:c r="E206" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F206" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G206" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H206" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I206" s="31" t="str">
+        <x:f>IF(AND(G206=H206,C206&gt;0,ABS(C206-'Prices'!H206)&lt;=MAX(0.01,'Prices'!H206*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J206" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K206" s="14" t="str"/>
+      <x:c r="L206" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M206" s="14" t="str"/>
+    </x:row>
+    <x:row r="207" ht="50" customHeight="1">
+      <x:c r="A207" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B207" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C207" s="33" t="n">
+        <x:v>105.25</x:v>
+      </x:c>
+      <x:c r="D207" s="33" t="n">
+        <x:v>105.25</x:v>
+      </x:c>
+      <x:c r="E207" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F207" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G207" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H207" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I207" s="32" t="str">
+        <x:f>IF(AND(G207=H207,C207&gt;0,ABS(C207-'Prices'!H207)&lt;=MAX(0.01,'Prices'!H207*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J207" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K207" s="16" t="str"/>
+      <x:c r="L207" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M207" s="16" t="str"/>
+    </x:row>
+    <x:row r="208" ht="50" customHeight="1">
+      <x:c r="A208" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B208" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C208" s="17" t="n">
+        <x:v>7659.44</x:v>
+      </x:c>
+      <x:c r="D208" s="17" t="n">
+        <x:v>7659.44</x:v>
+      </x:c>
+      <x:c r="E208" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F208" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G208" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H208" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I208" s="31" t="str">
+        <x:f>IF(AND(G208=H208,C208&gt;0,ABS(C208-'Prices'!H208)&lt;=MAX(0.01,'Prices'!H208*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J208" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K208" s="14" t="str"/>
+      <x:c r="L208" s="38" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M208" s="14" t="str"/>
+    </x:row>
+    <x:row r="209" ht="50" customHeight="1">
+      <x:c r="A209" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B209" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C209" s="33" t="n">
+        <x:v>26140.0293</x:v>
+      </x:c>
+      <x:c r="D209" s="33" t="n">
+        <x:v>26140.0293</x:v>
+      </x:c>
+      <x:c r="E209" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F209" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G209" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H209" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I209" s="32" t="str">
+        <x:f>IF(AND(G209=H209,C209&gt;0,ABS(C209-'Prices'!H209)&lt;=MAX(0.01,'Prices'!H209*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J209" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-17T11-45-30-161Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K209" s="16" t="str"/>
+      <x:c r="L209" s="39" t="n">
+        <x:v>46312.48993241898</x:v>
+      </x:c>
+      <x:c r="M209" s="16" t="str"/>
+    </x:row>
+    <x:row r="210" ht="50" customHeight="1">
+      <x:c r="A210" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B210" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C210" s="17" t="n">
+        <x:v>5946</x:v>
+      </x:c>
+      <x:c r="D210" s="17" t="n">
+        <x:v>5946</x:v>
+      </x:c>
+      <x:c r="E210" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F210" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G210" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H210" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I210" s="31" t="str">
+        <x:f>IF(AND(G210=H210,C210&gt;0,ABS(C210-'Prices'!H210)&lt;=MAX(0.01,'Prices'!H210*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J210" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K210" s="14" t="str"/>
+      <x:c r="L210" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M210" s="14" t="str"/>
+    </x:row>
+    <x:row r="211" ht="50" customHeight="1">
+      <x:c r="A211" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B211" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C211" s="33" t="n">
+        <x:v>4373</x:v>
+      </x:c>
+      <x:c r="D211" s="33" t="n">
+        <x:v>4373</x:v>
+      </x:c>
+      <x:c r="E211" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F211" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G211" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H211" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I211" s="32" t="str">
+        <x:f>IF(AND(G211=H211,C211&gt;0,ABS(C211-'Prices'!H211)&lt;=MAX(0.01,'Prices'!H211*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J211" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K211" s="16" t="str"/>
+      <x:c r="L211" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M211" s="16" t="str"/>
+    </x:row>
+    <x:row r="212" ht="50" customHeight="1">
+      <x:c r="A212" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B212" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C212" s="17" t="n">
+        <x:v>25.38</x:v>
+      </x:c>
+      <x:c r="D212" s="17" t="n">
+        <x:v>25.38</x:v>
+      </x:c>
+      <x:c r="E212" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F212" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G212" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H212" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I212" s="31" t="str">
+        <x:f>IF(AND(G212=H212,C212&gt;0,ABS(C212-'Prices'!H212)&lt;=MAX(0.01,'Prices'!H212*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J212" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K212" s="14" t="str"/>
+      <x:c r="L212" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M212" s="14" t="str"/>
+    </x:row>
+    <x:row r="213" ht="50" customHeight="1">
+      <x:c r="A213" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B213" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C213" s="33" t="n">
+        <x:v>335.53</x:v>
+      </x:c>
+      <x:c r="D213" s="33" t="n">
+        <x:v>335.53</x:v>
+      </x:c>
+      <x:c r="E213" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F213" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G213" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H213" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I213" s="32" t="str">
+        <x:f>IF(AND(G213=H213,C213&gt;0,ABS(C213-'Prices'!H213)&lt;=MAX(0.01,'Prices'!H213*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J213" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K213" s="16" t="str"/>
+      <x:c r="L213" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M213" s="16" t="str"/>
+    </x:row>
+    <x:row r="214" ht="50" customHeight="1">
+      <x:c r="A214" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B214" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C214" s="17" t="n">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="D214" s="17" t="n">
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="E214" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F214" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G214" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H214" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I214" s="31" t="str">
+        <x:f>IF(AND(G214=H214,C214&gt;0,ABS(C214-'Prices'!H214)&lt;=MAX(0.01,'Prices'!H214*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J214" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K214" s="14" t="str"/>
+      <x:c r="L214" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M214" s="14" t="str"/>
+    </x:row>
+    <x:row r="215" ht="50" customHeight="1">
+      <x:c r="A215" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B215" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C215" s="33" t="n">
+        <x:v>50.79</x:v>
+      </x:c>
+      <x:c r="D215" s="33" t="n">
+        <x:v>50.79</x:v>
+      </x:c>
+      <x:c r="E215" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F215" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G215" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H215" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I215" s="32" t="str">
+        <x:f>IF(AND(G215=H215,C215&gt;0,ABS(C215-'Prices'!H215)&lt;=MAX(0.01,'Prices'!H215*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J215" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K215" s="16" t="str"/>
+      <x:c r="L215" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M215" s="16" t="str"/>
+    </x:row>
+    <x:row r="216" ht="50" customHeight="1">
+      <x:c r="A216" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B216" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C216" s="17" t="n">
+        <x:v>81410</x:v>
+      </x:c>
+      <x:c r="D216" s="17" t="n">
+        <x:v>81410</x:v>
+      </x:c>
+      <x:c r="E216" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F216" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G216" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H216" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I216" s="31" t="str">
+        <x:f>IF(AND(G216=H216,C216&gt;0,ABS(C216-'Prices'!H216)&lt;=MAX(0.01,'Prices'!H216*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J216" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K216" s="14" t="str"/>
+      <x:c r="L216" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M216" s="14" t="str"/>
+    </x:row>
+    <x:row r="217" ht="50" customHeight="1">
+      <x:c r="A217" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B217" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C217" s="33" t="n">
+        <x:v>55.16</x:v>
+      </x:c>
+      <x:c r="D217" s="33" t="n">
+        <x:v>55.16</x:v>
+      </x:c>
+      <x:c r="E217" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F217" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G217" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H217" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I217" s="32" t="str">
+        <x:f>IF(AND(G217=H217,C217&gt;0,ABS(C217-'Prices'!H217)&lt;=MAX(0.01,'Prices'!H217*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J217" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K217" s="16" t="str"/>
+      <x:c r="L217" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M217" s="16" t="str"/>
+    </x:row>
+    <x:row r="218" ht="50" customHeight="1">
+      <x:c r="A218" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B218" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C218" s="17" t="n">
+        <x:v>28.86</x:v>
+      </x:c>
+      <x:c r="D218" s="17" t="n">
+        <x:v>28.86</x:v>
+      </x:c>
+      <x:c r="E218" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F218" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G218" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H218" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I218" s="31" t="str">
+        <x:f>IF(AND(OR(G218=H218,AND(B218="OUST",G218="XNAS",H218="XNYS",LEFT(M218,34)="ouster-marketstack-legacy-nyse-tag")),C218&gt;0,ABS(C218-'Prices'!H218)&lt;=MAX(0.01,'Prices'!H218*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J218" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K218" s="14" t="str"/>
+      <x:c r="L218" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M218" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="50" customHeight="1">
+      <x:c r="A219" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B219" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C219" s="33" t="n">
+        <x:v>12.92</x:v>
+      </x:c>
+      <x:c r="D219" s="33" t="n">
+        <x:v>12.92</x:v>
+      </x:c>
+      <x:c r="E219" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F219" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G219" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H219" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I219" s="32" t="str">
+        <x:f>IF(AND(G219=H219,C219&gt;0,ABS(C219-'Prices'!H219)&lt;=MAX(0.01,'Prices'!H219*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J219" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K219" s="16" t="str"/>
+      <x:c r="L219" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M219" s="16" t="str"/>
+    </x:row>
+    <x:row r="220" ht="50" customHeight="1">
+      <x:c r="A220" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B220" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C220" s="17" t="n">
+        <x:v>424.47</x:v>
+      </x:c>
+      <x:c r="D220" s="17" t="n">
+        <x:v>424.47</x:v>
+      </x:c>
+      <x:c r="E220" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F220" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G220" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H220" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I220" s="31" t="str">
+        <x:f>IF(AND(G220=H220,C220&gt;0,ABS(C220-'Prices'!H220)&lt;=MAX(0.01,'Prices'!H220*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J220" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K220" s="14" t="str"/>
+      <x:c r="L220" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M220" s="14" t="str"/>
+    </x:row>
+    <x:row r="221" ht="50" customHeight="1">
+      <x:c r="A221" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B221" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C221" s="33" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="D221" s="33" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="E221" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F221" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G221" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H221" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I221" s="32" t="str">
+        <x:f>IF(AND(G221=H221,C221&gt;0,ABS(C221-'Prices'!H221)&lt;=MAX(0.01,'Prices'!H221*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J221" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K221" s="16" t="str"/>
+      <x:c r="L221" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M221" s="16" t="str"/>
+    </x:row>
+    <x:row r="222" ht="50" customHeight="1">
+      <x:c r="A222" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B222" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C222" s="17" t="n">
+        <x:v>230.19</x:v>
+      </x:c>
+      <x:c r="D222" s="17" t="n">
+        <x:v>230.19</x:v>
+      </x:c>
+      <x:c r="E222" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F222" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G222" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H222" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I222" s="31" t="str">
+        <x:f>IF(AND(G222=H222,C222&gt;0,ABS(C222-'Prices'!H222)&lt;=MAX(0.01,'Prices'!H222*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J222" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K222" s="14" t="str"/>
+      <x:c r="L222" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M222" s="14" t="str"/>
+    </x:row>
+    <x:row r="223" ht="50" customHeight="1">
+      <x:c r="A223" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B223" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C223" s="33" t="n">
+        <x:v>5434</x:v>
+      </x:c>
+      <x:c r="D223" s="33" t="n">
+        <x:v>5434</x:v>
+      </x:c>
+      <x:c r="E223" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F223" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G223" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H223" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I223" s="32" t="str">
+        <x:f>IF(AND(G223=H223,C223&gt;0,ABS(C223-'Prices'!H223)&lt;=MAX(0.01,'Prices'!H223*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J223" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K223" s="16" t="str"/>
+      <x:c r="L223" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M223" s="16" t="str"/>
+    </x:row>
+    <x:row r="224" ht="50" customHeight="1">
+      <x:c r="A224" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B224" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C224" s="17" t="n">
+        <x:v>105.05</x:v>
+      </x:c>
+      <x:c r="D224" s="17" t="n">
+        <x:v>105.05</x:v>
+      </x:c>
+      <x:c r="E224" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F224" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G224" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H224" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I224" s="31" t="str">
+        <x:f>IF(AND(G224=H224,C224&gt;0,ABS(C224-'Prices'!H224)&lt;=MAX(0.01,'Prices'!H224*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J224" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K224" s="14" t="str"/>
+      <x:c r="L224" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M224" s="14" t="str"/>
+    </x:row>
+    <x:row r="225" ht="50" customHeight="1">
+      <x:c r="A225" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B225" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C225" s="33" t="n">
+        <x:v>7690.73</x:v>
+      </x:c>
+      <x:c r="D225" s="33" t="n">
+        <x:v>7690.73</x:v>
+      </x:c>
+      <x:c r="E225" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F225" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G225" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H225" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I225" s="32" t="str">
+        <x:f>IF(AND(G225=H225,C225&gt;0,ABS(C225-'Prices'!H225)&lt;=MAX(0.01,'Prices'!H225*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J225" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K225" s="16" t="str"/>
+      <x:c r="L225" s="39" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M225" s="16" t="str"/>
+    </x:row>
+    <x:row r="226" ht="50" customHeight="1">
+      <x:c r="A226" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B226" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C226" s="17" t="n">
+        <x:v>26430.8867</x:v>
+      </x:c>
+      <x:c r="D226" s="17" t="n">
+        <x:v>26430.8867</x:v>
+      </x:c>
+      <x:c r="E226" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F226" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G226" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H226" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I226" s="31" t="str">
+        <x:f>IF(AND(G226=H226,C226&gt;0,ABS(C226-'Prices'!H226)&lt;=MAX(0.01,'Prices'!H226*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J226" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-20T11-29-32-921Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K226" s="14" t="str"/>
+      <x:c r="L226" s="38" t="n">
+        <x:v>46315.478853252316</x:v>
+      </x:c>
+      <x:c r="M226" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -20773,7 +24381,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ffcd523d80f4ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeafd79b778c4ba1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26285,6 +29893,992 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="193" ht="27" customHeight="1">
+      <x:c r="A193" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B193" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C193" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D193" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E193" s="18" t="n">
+        <x:f>'Source Audit'!E193</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F193" s="41" t="n">
+        <x:f>'Source Audit'!F193</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G193" s="12" t="str">
+        <x:f>IF(AND(E193=0,F193=1,'Source Audit'!I193&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H193" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="27" customHeight="1">
+      <x:c r="A194" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B194" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C194" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D194" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E194" s="19" t="n">
+        <x:f>'Source Audit'!E194</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F194" s="40" t="n">
+        <x:f>'Source Audit'!F194</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G194" s="11" t="str">
+        <x:f>IF(AND(E194=0,F194=1,'Source Audit'!I194&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H194" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="27" customHeight="1">
+      <x:c r="A195" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B195" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C195" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D195" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E195" s="18" t="n">
+        <x:f>'Source Audit'!E195</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F195" s="41" t="n">
+        <x:f>'Source Audit'!F195</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G195" s="12" t="str">
+        <x:f>IF(AND(E195=0,F195=1,'Source Audit'!I195&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H195" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="27" customHeight="1">
+      <x:c r="A196" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B196" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C196" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D196" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E196" s="19" t="n">
+        <x:f>'Source Audit'!E196</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F196" s="40" t="n">
+        <x:f>'Source Audit'!F196</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G196" s="11" t="str">
+        <x:f>IF(AND(E196=0,F196=1,'Source Audit'!I196&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H196" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="27" customHeight="1">
+      <x:c r="A197" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B197" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C197" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D197" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E197" s="18" t="n">
+        <x:f>'Source Audit'!E197</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F197" s="41" t="n">
+        <x:f>'Source Audit'!F197</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G197" s="12" t="str">
+        <x:f>IF(AND(E197=0,F197=1,'Source Audit'!I197&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H197" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="27" customHeight="1">
+      <x:c r="A198" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B198" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C198" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D198" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E198" s="19" t="n">
+        <x:f>'Source Audit'!E198</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F198" s="40" t="n">
+        <x:f>'Source Audit'!F198</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G198" s="11" t="str">
+        <x:f>IF(AND(E198=0,F198=1,'Source Audit'!I198&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H198" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="27" customHeight="1">
+      <x:c r="A199" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B199" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C199" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D199" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E199" s="18" t="n">
+        <x:f>'Source Audit'!E199</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F199" s="41" t="n">
+        <x:f>'Source Audit'!F199</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G199" s="12" t="str">
+        <x:f>IF(AND(E199=0,F199=1,'Source Audit'!I199&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H199" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="27" customHeight="1">
+      <x:c r="A200" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B200" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C200" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D200" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E200" s="19" t="n">
+        <x:f>'Source Audit'!E200</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F200" s="40" t="n">
+        <x:f>'Source Audit'!F200</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G200" s="11" t="str">
+        <x:f>IF(AND(E200=0,F200=1,'Source Audit'!I200&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H200" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="44" customHeight="1">
+      <x:c r="A201" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B201" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C201" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D201" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E201" s="18" t="n">
+        <x:f>'Source Audit'!E201</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F201" s="41" t="n">
+        <x:f>'Source Audit'!F201</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G201" s="12" t="str">
+        <x:f>IF(AND(E201=0,F201=1,'Source Audit'!I201&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H201" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="27" customHeight="1">
+      <x:c r="A202" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B202" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C202" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D202" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E202" s="19" t="n">
+        <x:f>'Source Audit'!E202</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F202" s="40" t="n">
+        <x:f>'Source Audit'!F202</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G202" s="11" t="str">
+        <x:f>IF(AND(E202=0,F202=1,'Source Audit'!I202&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H202" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="27" customHeight="1">
+      <x:c r="A203" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B203" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C203" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D203" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E203" s="18" t="n">
+        <x:f>'Source Audit'!E203</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F203" s="41" t="n">
+        <x:f>'Source Audit'!F203</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G203" s="12" t="str">
+        <x:f>IF(AND(E203=0,F203=1,'Source Audit'!I203&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H203" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="27" customHeight="1">
+      <x:c r="A204" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B204" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C204" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D204" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E204" s="19" t="n">
+        <x:f>'Source Audit'!E204</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F204" s="40" t="n">
+        <x:f>'Source Audit'!F204</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G204" s="11" t="str">
+        <x:f>IF(AND(E204=0,F204=1,'Source Audit'!I204&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H204" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="27" customHeight="1">
+      <x:c r="A205" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B205" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C205" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D205" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E205" s="18" t="n">
+        <x:f>'Source Audit'!E205</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F205" s="41" t="n">
+        <x:f>'Source Audit'!F205</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G205" s="12" t="str">
+        <x:f>IF(AND(E205=0,F205=1,'Source Audit'!I205&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H205" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="27" customHeight="1">
+      <x:c r="A206" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B206" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C206" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D206" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E206" s="19" t="n">
+        <x:f>'Source Audit'!E206</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F206" s="40" t="n">
+        <x:f>'Source Audit'!F206</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G206" s="11" t="str">
+        <x:f>IF(AND(E206=0,F206=1,'Source Audit'!I206&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H206" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="27" customHeight="1">
+      <x:c r="A207" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B207" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C207" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D207" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E207" s="18" t="n">
+        <x:f>'Source Audit'!E207</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F207" s="41" t="n">
+        <x:f>'Source Audit'!F207</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G207" s="12" t="str">
+        <x:f>IF(AND(E207=0,F207=1,'Source Audit'!I207&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H207" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="27" customHeight="1">
+      <x:c r="A208" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B208" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C208" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D208" s="8" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E208" s="19" t="n">
+        <x:f>'Source Audit'!E208</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F208" s="40" t="n">
+        <x:f>'Source Audit'!F208</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G208" s="11" t="str">
+        <x:f>IF(AND(E208=0,F208=1,'Source Audit'!I208&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H208" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="27" customHeight="1">
+      <x:c r="A209" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="B209" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C209" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D209" s="9" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="E209" s="18" t="n">
+        <x:f>'Source Audit'!E209</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F209" s="41" t="n">
+        <x:f>'Source Audit'!F209</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G209" s="12" t="str">
+        <x:f>IF(AND(E209=0,F209=1,'Source Audit'!I209&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H209" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="27" customHeight="1">
+      <x:c r="A210" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B210" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C210" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D210" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E210" s="19" t="n">
+        <x:f>'Source Audit'!E210</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F210" s="40" t="n">
+        <x:f>'Source Audit'!F210</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G210" s="11" t="str">
+        <x:f>IF(AND(E210=0,F210=1,'Source Audit'!I210&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H210" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="27" customHeight="1">
+      <x:c r="A211" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B211" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C211" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D211" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E211" s="18" t="n">
+        <x:f>'Source Audit'!E211</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F211" s="41" t="n">
+        <x:f>'Source Audit'!F211</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G211" s="12" t="str">
+        <x:f>IF(AND(E211=0,F211=1,'Source Audit'!I211&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H211" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="27" customHeight="1">
+      <x:c r="A212" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B212" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C212" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D212" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E212" s="19" t="n">
+        <x:f>'Source Audit'!E212</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F212" s="40" t="n">
+        <x:f>'Source Audit'!F212</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G212" s="11" t="str">
+        <x:f>IF(AND(E212=0,F212=1,'Source Audit'!I212&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H212" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="27" customHeight="1">
+      <x:c r="A213" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B213" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C213" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D213" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E213" s="18" t="n">
+        <x:f>'Source Audit'!E213</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F213" s="41" t="n">
+        <x:f>'Source Audit'!F213</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G213" s="12" t="str">
+        <x:f>IF(AND(E213=0,F213=1,'Source Audit'!I213&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H213" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="27" customHeight="1">
+      <x:c r="A214" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B214" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C214" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D214" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E214" s="19" t="n">
+        <x:f>'Source Audit'!E214</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F214" s="40" t="n">
+        <x:f>'Source Audit'!F214</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G214" s="11" t="str">
+        <x:f>IF(AND(E214=0,F214=1,'Source Audit'!I214&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H214" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="27" customHeight="1">
+      <x:c r="A215" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B215" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C215" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D215" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E215" s="18" t="n">
+        <x:f>'Source Audit'!E215</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F215" s="41" t="n">
+        <x:f>'Source Audit'!F215</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G215" s="12" t="str">
+        <x:f>IF(AND(E215=0,F215=1,'Source Audit'!I215&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H215" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="27" customHeight="1">
+      <x:c r="A216" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B216" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C216" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D216" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E216" s="19" t="n">
+        <x:f>'Source Audit'!E216</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F216" s="40" t="n">
+        <x:f>'Source Audit'!F216</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G216" s="11" t="str">
+        <x:f>IF(AND(E216=0,F216=1,'Source Audit'!I216&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H216" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="27" customHeight="1">
+      <x:c r="A217" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B217" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C217" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D217" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E217" s="18" t="n">
+        <x:f>'Source Audit'!E217</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F217" s="41" t="n">
+        <x:f>'Source Audit'!F217</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G217" s="12" t="str">
+        <x:f>IF(AND(E217=0,F217=1,'Source Audit'!I217&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H217" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="44" customHeight="1">
+      <x:c r="A218" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B218" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C218" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D218" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E218" s="19" t="n">
+        <x:f>'Source Audit'!E218</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F218" s="40" t="n">
+        <x:f>'Source Audit'!F218</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G218" s="11" t="str">
+        <x:f>IF(AND(E218=0,F218=1,'Source Audit'!I218&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H218" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="27" customHeight="1">
+      <x:c r="A219" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B219" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C219" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D219" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E219" s="18" t="n">
+        <x:f>'Source Audit'!E219</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F219" s="41" t="n">
+        <x:f>'Source Audit'!F219</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G219" s="12" t="str">
+        <x:f>IF(AND(E219=0,F219=1,'Source Audit'!I219&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H219" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="27" customHeight="1">
+      <x:c r="A220" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B220" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C220" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D220" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E220" s="19" t="n">
+        <x:f>'Source Audit'!E220</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F220" s="40" t="n">
+        <x:f>'Source Audit'!F220</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G220" s="11" t="str">
+        <x:f>IF(AND(E220=0,F220=1,'Source Audit'!I220&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H220" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="27" customHeight="1">
+      <x:c r="A221" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B221" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C221" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D221" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E221" s="18" t="n">
+        <x:f>'Source Audit'!E221</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F221" s="41" t="n">
+        <x:f>'Source Audit'!F221</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G221" s="12" t="str">
+        <x:f>IF(AND(E221=0,F221=1,'Source Audit'!I221&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H221" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="27" customHeight="1">
+      <x:c r="A222" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B222" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C222" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D222" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E222" s="19" t="n">
+        <x:f>'Source Audit'!E222</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F222" s="40" t="n">
+        <x:f>'Source Audit'!F222</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G222" s="11" t="str">
+        <x:f>IF(AND(E222=0,F222=1,'Source Audit'!I222&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H222" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="27" customHeight="1">
+      <x:c r="A223" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B223" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C223" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D223" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E223" s="18" t="n">
+        <x:f>'Source Audit'!E223</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F223" s="41" t="n">
+        <x:f>'Source Audit'!F223</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G223" s="12" t="str">
+        <x:f>IF(AND(E223=0,F223=1,'Source Audit'!I223&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H223" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="27" customHeight="1">
+      <x:c r="A224" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B224" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C224" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D224" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E224" s="19" t="n">
+        <x:f>'Source Audit'!E224</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F224" s="40" t="n">
+        <x:f>'Source Audit'!F224</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G224" s="11" t="str">
+        <x:f>IF(AND(E224=0,F224=1,'Source Audit'!I224&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H224" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="27" customHeight="1">
+      <x:c r="A225" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B225" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C225" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D225" s="9" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E225" s="18" t="n">
+        <x:f>'Source Audit'!E225</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F225" s="41" t="n">
+        <x:f>'Source Audit'!F225</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G225" s="12" t="str">
+        <x:f>IF(AND(E225=0,F225=1,'Source Audit'!I225&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H225" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="27" customHeight="1">
+      <x:c r="A226" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="B226" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C226" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D226" s="8" t="n">
+        <x:v>46314</x:v>
+      </x:c>
+      <x:c r="E226" s="19" t="n">
+        <x:f>'Source Audit'!E226</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F226" s="40" t="n">
+        <x:f>'Source Audit'!F226</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G226" s="11" t="str">
+        <x:f>IF(AND(E226=0,F226=1,'Source Audit'!I226&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H226" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -26292,7 +30886,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9148181cba7c4308"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d397195598a4de3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 through October 20
Append the audited October 20 closes and extend the cumulative five-sheet review workbook and website data to fourteen trading dates, preserving every earlier reviewed input and immutable source receipt. Record the approved Ouster provider MIC exception separately in the audit and workbook.

Validation: 17 requested closes and 206 historical comparisons passed. Both index calculations, benchmark levels, contributions and weights reconcile. Type checking, production build, holdings CSV and desktop/mobile checks passed. Repository lint retains seven known unrelated errors and nine warnings.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8b9c951c2fdb47af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R56f103054bbc4aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Rd72b86d1c85b4fe2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R5a98770ea99e44c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R257cffe0c77844d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R832139e5204c403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R6806f08006d74911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R3a6ce0d8d7e34923"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R30d26043b4b94a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R8cc055f0b0574d4e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H200" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H215" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H226" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1708,6 +1708,85 @@
         <x:v>-6.584871083120669</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="40" customHeight="1">
+      <x:c r="A19" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B19" s="18" t="n">
+        <x:f>B18*(1+SUM('Returns and Contributions'!F201:F215))</x:f>
+        <x:v>921.489181665232</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="n">
+        <x:f>B19/B18-1</x:f>
+        <x:v>0.004073485585846637</x:v>
+      </x:c>
+      <x:c r="D19" s="21" t="n">
+        <x:f>B19/$B$6-1</x:f>
+        <x:v>-0.07851081833476803</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="n">
+        <x:f>1000*'Prices'!H242/'Prices'!I242</x:f>
+        <x:v>1006.0158221862793</x:v>
+      </x:c>
+      <x:c r="F19" s="21" t="n">
+        <x:f>E19/E18-1</x:f>
+        <x:v>0.0028397824393782134</x:v>
+      </x:c>
+      <x:c r="G19" s="21" t="n">
+        <x:f>E19/1000-1</x:f>
+        <x:v>0.006015822186279163</x:v>
+      </x:c>
+      <x:c r="H19" s="18" t="n">
+        <x:f>1000*'Prices'!H243/'Prices'!I243</x:f>
+        <x:v>983.3735478537286</x:v>
+      </x:c>
+      <x:c r="I19" s="21" t="n">
+        <x:f>H19/H18-1</x:f>
+        <x:v>-0.0002296669070886992</x:v>
+      </x:c>
+      <x:c r="J19" s="21" t="n">
+        <x:f>H19/1000-1</x:f>
+        <x:v>-0.016626452146271342</x:v>
+      </x:c>
+      <x:c r="K19" s="25" t="n">
+        <x:f>(C19-F19)*100</x:f>
+        <x:v>0.12337031464684234</x:v>
+      </x:c>
+      <x:c r="L19" s="25" t="n">
+        <x:f>(C19-I19)*100</x:f>
+        <x:v>0.4303152492935336</x:v>
+      </x:c>
+      <x:c r="M19" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G201:G215)</x:f>
+        <x:v>0.9999999999999997</x:v>
+      </x:c>
+      <x:c r="N19" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F201:F215)-C19</x:f>
+        <x:v>-8.673617379884035e-17</x:v>
+      </x:c>
+      <x:c r="O19" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P19" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I227:I243,"Mismatch")=0,IF(COUNTIF('Source Audit'!I227:I243,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q19" s="30" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="R19" s="27" t="n">
+        <x:f>B19-1000*('Prices'!H227/'Prices'!H6+'Prices'!H228/'Prices'!H7+'Prices'!H229/'Prices'!H8+'Prices'!H230/'Prices'!H9+'Prices'!H231/'Prices'!H10+'Prices'!H232/'Prices'!H11+'Prices'!H233/'Prices'!H12+'Prices'!H234/'Prices'!H13+'Prices'!H235/'Prices'!H14+'Prices'!H236/'Prices'!H15+'Prices'!H237/'Prices'!H16+'Prices'!H238/'Prices'!H17+'Prices'!H239/'Prices'!H18+'Prices'!H240/'Prices'!H19+'Prices'!H241/'Prices'!H20)/15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S19" s="25" t="n">
+        <x:f>(D19-G19)*100</x:f>
+        <x:v>-8.45266405210472</x:v>
+      </x:c>
+      <x:c r="T19" s="25" t="n">
+        <x:f>(D19-J19)*100</x:f>
+        <x:v>-6.188436618849669</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1715,7 +1794,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e89ceb4df074451"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6e9bd15ed574169"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9733,6 +9812,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="227" ht="27" customHeight="1">
+      <x:c r="A227" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C227" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D227" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E227" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F227" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G227" s="33" t="n">
+        <x:f>H210</x:f>
+        <x:v>5946</x:v>
+      </x:c>
+      <x:c r="H227" s="35" t="n">
+        <x:v>5788</x:v>
+      </x:c>
+      <x:c r="I227" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J227" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K227" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="27" customHeight="1">
+      <x:c r="A228" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B228" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C228" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D228" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E228" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F228" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G228" s="17" t="n">
+        <x:f>H211</x:f>
+        <x:v>4373</x:v>
+      </x:c>
+      <x:c r="H228" s="34" t="n">
+        <x:v>4277</x:v>
+      </x:c>
+      <x:c r="I228" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J228" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K228" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="27" customHeight="1">
+      <x:c r="A229" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B229" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C229" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D229" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E229" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F229" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G229" s="33" t="n">
+        <x:f>H212</x:f>
+        <x:v>25.38</x:v>
+      </x:c>
+      <x:c r="H229" s="35" t="n">
+        <x:v>26.3</x:v>
+      </x:c>
+      <x:c r="I229" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J229" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K229" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="27" customHeight="1">
+      <x:c r="A230" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B230" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C230" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D230" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E230" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F230" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G230" s="17" t="n">
+        <x:f>H213</x:f>
+        <x:v>335.53</x:v>
+      </x:c>
+      <x:c r="H230" s="34" t="n">
+        <x:v>336.59</x:v>
+      </x:c>
+      <x:c r="I230" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J230" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K230" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="27" customHeight="1">
+      <x:c r="A231" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B231" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C231" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D231" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E231" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F231" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G231" s="33" t="n">
+        <x:f>H214</x:f>
+        <x:v>4458</x:v>
+      </x:c>
+      <x:c r="H231" s="35" t="n">
+        <x:v>4293</x:v>
+      </x:c>
+      <x:c r="I231" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J231" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K231" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="27" customHeight="1">
+      <x:c r="A232" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B232" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C232" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D232" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E232" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F232" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G232" s="17" t="n">
+        <x:f>H215</x:f>
+        <x:v>50.79</x:v>
+      </x:c>
+      <x:c r="H232" s="34" t="n">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="I232" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J232" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K232" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="27" customHeight="1">
+      <x:c r="A233" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C233" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D233" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E233" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F233" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G233" s="33" t="n">
+        <x:f>H216</x:f>
+        <x:v>81410</x:v>
+      </x:c>
+      <x:c r="H233" s="35" t="n">
+        <x:v>80910</x:v>
+      </x:c>
+      <x:c r="I233" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J233" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K233" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="27" customHeight="1">
+      <x:c r="A234" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B234" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C234" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D234" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E234" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F234" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G234" s="17" t="n">
+        <x:f>H217</x:f>
+        <x:v>55.16</x:v>
+      </x:c>
+      <x:c r="H234" s="34" t="n">
+        <x:v>56.77</x:v>
+      </x:c>
+      <x:c r="I234" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J234" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K234" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="27" customHeight="1">
+      <x:c r="A235" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C235" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D235" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E235" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F235" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G235" s="33" t="n">
+        <x:f>H218</x:f>
+        <x:v>28.86</x:v>
+      </x:c>
+      <x:c r="H235" s="35" t="n">
+        <x:v>29.65</x:v>
+      </x:c>
+      <x:c r="I235" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J235" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K235" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="27" customHeight="1">
+      <x:c r="A236" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B236" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C236" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D236" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E236" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F236" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G236" s="17" t="n">
+        <x:f>H219</x:f>
+        <x:v>12.92</x:v>
+      </x:c>
+      <x:c r="H236" s="34" t="n">
+        <x:v>13.99</x:v>
+      </x:c>
+      <x:c r="I236" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J236" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K236" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="27" customHeight="1">
+      <x:c r="A237" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B237" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C237" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D237" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E237" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F237" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G237" s="33" t="n">
+        <x:f>H220</x:f>
+        <x:v>424.47</x:v>
+      </x:c>
+      <x:c r="H237" s="35" t="n">
+        <x:v>427.77</x:v>
+      </x:c>
+      <x:c r="I237" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J237" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K237" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="27" customHeight="1">
+      <x:c r="A238" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B238" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C238" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D238" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E238" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F238" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G238" s="17" t="n">
+        <x:f>H221</x:f>
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="H238" s="34" t="n">
+        <x:v>260.25</x:v>
+      </x:c>
+      <x:c r="I238" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J238" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K238" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="27" customHeight="1">
+      <x:c r="A239" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C239" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D239" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E239" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F239" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G239" s="33" t="n">
+        <x:f>H222</x:f>
+        <x:v>230.19</x:v>
+      </x:c>
+      <x:c r="H239" s="35" t="n">
+        <x:v>237.6</x:v>
+      </x:c>
+      <x:c r="I239" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J239" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K239" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="27" customHeight="1">
+      <x:c r="A240" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B240" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C240" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D240" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E240" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F240" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G240" s="17" t="n">
+        <x:f>H223</x:f>
+        <x:v>5434</x:v>
+      </x:c>
+      <x:c r="H240" s="34" t="n">
+        <x:v>5347</x:v>
+      </x:c>
+      <x:c r="I240" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J240" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K240" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="27" customHeight="1">
+      <x:c r="A241" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B241" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C241" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D241" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E241" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F241" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G241" s="33" t="n">
+        <x:f>H224</x:f>
+        <x:v>105.05</x:v>
+      </x:c>
+      <x:c r="H241" s="35" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="I241" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J241" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K241" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="27" customHeight="1">
+      <x:c r="A242" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B242" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C242" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D242" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E242" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F242" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G242" s="17" t="n">
+        <x:f>H225</x:f>
+        <x:v>7690.73</x:v>
+      </x:c>
+      <x:c r="H242" s="34" t="n">
+        <x:v>7712.57</x:v>
+      </x:c>
+      <x:c r="I242" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J242" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K242" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="27" customHeight="1">
+      <x:c r="A243" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B243" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C243" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D243" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E243" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F243" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G243" s="33" t="n">
+        <x:f>H226</x:f>
+        <x:v>26430.8867</x:v>
+      </x:c>
+      <x:c r="H243" s="35" t="n">
+        <x:v>26424.8164</x:v>
+      </x:c>
+      <x:c r="I243" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J243" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="K243" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -9740,7 +10431,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd822c473cbf4499d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e1fc0fa953b4a39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15784,6 +16475,471 @@
         <x:v>0.06089678852757019</x:v>
       </x:c>
     </x:row>
+    <x:row r="201" ht="27" customHeight="1">
+      <x:c r="A201" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B201" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C201" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D201" s="21" t="n">
+        <x:f>G186</x:f>
+        <x:v>0.07049543965473073</x:v>
+      </x:c>
+      <x:c r="E201" s="23" t="n">
+        <x:f>'Prices'!H227/'Prices'!G227-1</x:f>
+        <x:v>-0.026572485704675408</x:v>
+      </x:c>
+      <x:c r="F201" s="21" t="n">
+        <x:f>D201*E201</x:f>
+        <x:v>-0.0018732390624701402</x:v>
+      </x:c>
+      <x:c r="G201" s="21" t="n">
+        <x:f>D201*(1+E201)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06834380309546927</x:v>
+      </x:c>
+      <x:c r="H201" s="23" t="n">
+        <x:f>'Prices'!H227/'Prices'!I227-1</x:f>
+        <x:v>-0.05532887220499427</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="27" customHeight="1">
+      <x:c r="A202" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B202" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C202" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D202" s="20" t="n">
+        <x:f>G187</x:f>
+        <x:v>0.066470117381231</x:v>
+      </x:c>
+      <x:c r="E202" s="22" t="n">
+        <x:f>'Prices'!H228/'Prices'!G228-1</x:f>
+        <x:v>-0.021952892750971897</x:v>
+      </x:c>
+      <x:c r="F202" s="20" t="n">
+        <x:f>D202*E202</x:f>
+        <x:v>-0.0014592113580146771</x:v>
+      </x:c>
+      <x:c r="G202" s="20" t="n">
+        <x:f>D202*(1+E202)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06474715940266505</x:v>
+      </x:c>
+      <x:c r="H202" s="22" t="n">
+        <x:f>'Prices'!H228/'Prices'!I228-1</x:f>
+        <x:v>-0.10504289600334793</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="27" customHeight="1">
+      <x:c r="A203" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B203" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C203" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D203" s="21" t="n">
+        <x:f>G188</x:f>
+        <x:v>0.06533089490653239</x:v>
+      </x:c>
+      <x:c r="E203" s="23" t="n">
+        <x:f>'Prices'!H229/'Prices'!G229-1</x:f>
+        <x:v>0.03624901497241928</x:v>
+      </x:c>
+      <x:c r="F203" s="21" t="n">
+        <x:f>D203*E203</x:f>
+        <x:v>0.002368180587628443</x:v>
+      </x:c>
+      <x:c r="G203" s="21" t="n">
+        <x:f>D203*(1+E203)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06742442307861607</x:v>
+      </x:c>
+      <x:c r="H203" s="23" t="n">
+        <x:f>'Prices'!H229/'Prices'!I229-1</x:f>
+        <x:v>-0.068036853295535</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="27" customHeight="1">
+      <x:c r="A204" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B204" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C204" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D204" s="20" t="n">
+        <x:f>G189</x:f>
+        <x:v>0.058619392813888886</x:v>
+      </x:c>
+      <x:c r="E204" s="22" t="n">
+        <x:f>'Prices'!H230/'Prices'!G230-1</x:f>
+        <x:v>0.003159180997228228</x:v>
+      </x:c>
+      <x:c r="F204" s="20" t="n">
+        <x:f>D204*E204</x:f>
+        <x:v>0.00018518927184669472</x:v>
+      </x:c>
+      <x:c r="G204" s="20" t="n">
+        <x:f>D204*(1+E204)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.058566014270783055</x:v>
+      </x:c>
+      <x:c r="H204" s="22" t="n">
+        <x:f>'Prices'!H230/'Prices'!I230-1</x:f>
+        <x:v>-0.1904807715433272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="27" customHeight="1">
+      <x:c r="A205" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B205" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C205" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D205" s="21" t="n">
+        <x:f>G190</x:f>
+        <x:v>0.06509250392467882</x:v>
+      </x:c>
+      <x:c r="E205" s="23" t="n">
+        <x:f>'Prices'!H231/'Prices'!G231-1</x:f>
+        <x:v>-0.037012113055181706</x:v>
+      </x:c>
+      <x:c r="F205" s="21" t="n">
+        <x:f>D205*E205</x:f>
+        <x:v>-0.002409211114305071</x:v>
+      </x:c>
+      <x:c r="G205" s="21" t="n">
+        <x:f>D205*(1+E205)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06242898922263636</x:v>
+      </x:c>
+      <x:c r="H205" s="23" t="n">
+        <x:f>'Prices'!H231/'Prices'!I231-1</x:f>
+        <x:v>-0.1370854271356784</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="27" customHeight="1">
+      <x:c r="A206" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B206" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C206" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D206" s="20" t="n">
+        <x:f>G191</x:f>
+        <x:v>0.07108776395929049</x:v>
+      </x:c>
+      <x:c r="E206" s="22" t="n">
+        <x:f>'Prices'!H232/'Prices'!G232-1</x:f>
+        <x:v>0.00019688915140769758</x:v>
+      </x:c>
+      <x:c r="F206" s="20" t="n">
+        <x:f>D206*E206</x:f>
+        <x:v>0.000013996409521415413</x:v>
+      </x:c>
+      <x:c r="G206" s="20" t="n">
+        <x:f>D206*(1+E206)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.07081330339813344</x:v>
+      </x:c>
+      <x:c r="H206" s="22" t="n">
+        <x:f>'Prices'!H232/'Prices'!I232-1</x:f>
+        <x:v>-0.021194605009633993</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="27" customHeight="1">
+      <x:c r="A207" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B207" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C207" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D207" s="21" t="n">
+        <x:f>G192</x:f>
+        <x:v>0.07282923101638225</x:v>
+      </x:c>
+      <x:c r="E207" s="23" t="n">
+        <x:f>'Prices'!H233/'Prices'!G233-1</x:f>
+        <x:v>-0.00614175162756414</x:v>
+      </x:c>
+      <x:c r="F207" s="21" t="n">
+        <x:f>D207*E207</x:f>
+        <x:v>-0.00044729904812911047</x:v>
+      </x:c>
+      <x:c r="G207" s="21" t="n">
+        <x:f>D207*(1+E207)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.07208828139308994</x:v>
+      </x:c>
+      <x:c r="H207" s="23" t="n">
+        <x:f>'Prices'!H233/'Prices'!I233-1</x:f>
+        <x:v>-0.0035714285714285587</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="27" customHeight="1">
+      <x:c r="A208" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B208" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C208" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D208" s="20" t="n">
+        <x:f>G193</x:f>
+        <x:v>0.06439887040109012</x:v>
+      </x:c>
+      <x:c r="E208" s="22" t="n">
+        <x:f>'Prices'!H234/'Prices'!G234-1</x:f>
+        <x:v>0.02918781725888331</x:v>
+      </x:c>
+      <x:c r="F208" s="20" t="n">
+        <x:f>D208*E208</x:f>
+        <x:v>0.0018796624609455274</x:v>
+      </x:c>
+      <x:c r="G208" s="20" t="n">
+        <x:f>D208*(1+E208)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06600964353058691</x:v>
+      </x:c>
+      <x:c r="H208" s="22" t="n">
+        <x:f>'Prices'!H234/'Prices'!I234-1</x:f>
+        <x:v>-0.08759241401478612</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="27" customHeight="1">
+      <x:c r="A209" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B209" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C209" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D209" s="21" t="n">
+        <x:f>G194</x:f>
+        <x:v>0.05129507721826792</x:v>
+      </x:c>
+      <x:c r="E209" s="23" t="n">
+        <x:f>'Prices'!H235/'Prices'!G235-1</x:f>
+        <x:v>0.027373527373527384</x:v>
+      </x:c>
+      <x:c r="F209" s="21" t="n">
+        <x:f>D209*E209</x:f>
+        <x:v>0.0014041272003614577</x:v>
+      </x:c>
+      <x:c r="G209" s="21" t="n">
+        <x:f>D209*(1+E209)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.052485405874332966</x:v>
+      </x:c>
+      <x:c r="H209" s="23" t="n">
+        <x:f>'Prices'!H235/'Prices'!I235-1</x:f>
+        <x:v>-0.2745289943724003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="27" customHeight="1">
+      <x:c r="A210" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B210" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C210" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D210" s="20" t="n">
+        <x:f>G195</x:f>
+        <x:v>0.058915658579842524</x:v>
+      </x:c>
+      <x:c r="E210" s="22" t="n">
+        <x:f>'Prices'!H236/'Prices'!G236-1</x:f>
+        <x:v>0.08281733746130038</x:v>
+      </x:c>
+      <x:c r="F210" s="20" t="n">
+        <x:f>D210*E210</x:f>
+        <x:v>0.004879237978361576</x:v>
+      </x:c>
+      <x:c r="G210" s="20" t="n">
+        <x:f>D210*(1+E210)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06353608323894909</x:v>
+      </x:c>
+      <x:c r="H210" s="22" t="n">
+        <x:f>'Prices'!H236/'Prices'!I236-1</x:f>
+        <x:v>-0.12178279974890138</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="27" customHeight="1">
+      <x:c r="A211" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B211" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C211" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D211" s="21" t="n">
+        <x:f>G196</x:f>
+        <x:v>0.06968941208769541</x:v>
+      </x:c>
+      <x:c r="E211" s="23" t="n">
+        <x:f>'Prices'!H237/'Prices'!G237-1</x:f>
+        <x:v>0.0077744010177396294</x:v>
+      </x:c>
+      <x:c r="F211" s="21" t="n">
+        <x:f>D211*E211</x:f>
+        <x:v>0.0005417934362602556</x:v>
+      </x:c>
+      <x:c r="G211" s="21" t="n">
+        <x:f>D211*(1+E211)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06994628035912916</x:v>
+      </x:c>
+      <x:c r="H211" s="23" t="n">
+        <x:f>'Prices'!H237/'Prices'!I237-1</x:f>
+        <x:v>-0.033178890270087025</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="27" customHeight="1">
+      <x:c r="A212" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B212" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C212" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D212" s="20" t="n">
+        <x:f>G197</x:f>
+        <x:v>0.07111854164686994</x:v>
+      </x:c>
+      <x:c r="E212" s="22" t="n">
+        <x:f>'Prices'!H238/'Prices'!G238-1</x:f>
+        <x:v>-0.02235161532682195</x:v>
+      </x:c>
+      <x:c r="F212" s="20" t="n">
+        <x:f>D212*E212</x:f>
+        <x:v>-0.0015896142854954034</x:v>
+      </x:c>
+      <x:c r="G212" s="20" t="n">
+        <x:f>D212*(1+E212)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06924685131069515</x:v>
+      </x:c>
+      <x:c r="H212" s="22" t="n">
+        <x:f>'Prices'!H238/'Prices'!I238-1</x:f>
+        <x:v>-0.042846634792202964</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="27" customHeight="1">
+      <x:c r="A213" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B213" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C213" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D213" s="21" t="n">
+        <x:f>G198</x:f>
+        <x:v>0.06990808940652919</x:v>
+      </x:c>
+      <x:c r="E213" s="23" t="n">
+        <x:f>'Prices'!H239/'Prices'!G239-1</x:f>
+        <x:v>0.032190798905252116</x:v>
+      </x:c>
+      <x:c r="F213" s="21" t="n">
+        <x:f>D213*E213</x:f>
+        <x:v>0.002250397247935967</x:v>
+      </x:c>
+      <x:c r="G213" s="21" t="n">
+        <x:f>D213*(1+E213)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.07186574258791711</x:v>
+      </x:c>
+      <x:c r="H213" s="23" t="n">
+        <x:f>'Prices'!H239/'Prices'!I239-1</x:f>
+        <x:v>-0.006647435093440346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="27" customHeight="1">
+      <x:c r="A214" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B214" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C214" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D214" s="20" t="n">
+        <x:f>G199</x:f>
+        <x:v>0.06768401571869972</x:v>
+      </x:c>
+      <x:c r="E214" s="22" t="n">
+        <x:f>'Prices'!H240/'Prices'!G240-1</x:f>
+        <x:v>-0.01601030548398974</x:v>
+      </x:c>
+      <x:c r="F214" s="20" t="n">
+        <x:f>D214*E214</x:f>
+        <x:v>-0.001083641768039546</x:v>
+      </x:c>
+      <x:c r="G214" s="20" t="n">
+        <x:f>D214*(1+E214)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.06633017892291107</x:v>
+      </x:c>
+      <x:c r="H214" s="22" t="n">
+        <x:f>'Prices'!H240/'Prices'!I240-1</x:f>
+        <x:v>-0.08316186556927296</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="27" customHeight="1">
+      <x:c r="A215" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B215" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C215" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D215" s="21" t="n">
+        <x:f>G200</x:f>
+        <x:v>0.07706499128427037</x:v>
+      </x:c>
+      <x:c r="E215" s="23" t="n">
+        <x:f>'Prices'!H241/'Prices'!G241-1</x:f>
+        <x:v>-0.007615421227986641</x:v>
+      </x:c>
+      <x:c r="F215" s="21" t="n">
+        <x:f>D215*E215</x:f>
+        <x:v>-0.000586882370560838</x:v>
+      </x:c>
+      <x:c r="G215" s="21" t="n">
+        <x:f>D215*(1+E215)/(1+SUM($F$201:$F$215))</x:f>
+        <x:v>0.07616784031408504</x:v>
+      </x:c>
+      <x:c r="H215" s="23" t="n">
+        <x:f>'Prices'!H241/'Prices'!I241-1</x:f>
+        <x:v>0.052817612603514474</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -15791,7 +16947,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d76f3a42074f3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb785009f70a417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24374,6 +25530,654 @@
       </x:c>
       <x:c r="M226" s="14" t="str"/>
     </x:row>
+    <x:row r="227" ht="50" customHeight="1">
+      <x:c r="A227" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C227" s="33" t="n">
+        <x:v>5788</x:v>
+      </x:c>
+      <x:c r="D227" s="33" t="n">
+        <x:v>5788</x:v>
+      </x:c>
+      <x:c r="E227" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F227" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G227" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H227" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I227" s="32" t="str">
+        <x:f>IF(AND(G227=H227,C227&gt;0,ABS(C227-'Prices'!H227)&lt;=MAX(0.01,'Prices'!H227*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J227" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K227" s="16" t="str"/>
+      <x:c r="L227" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M227" s="16" t="str"/>
+    </x:row>
+    <x:row r="228" ht="50" customHeight="1">
+      <x:c r="A228" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B228" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C228" s="17" t="n">
+        <x:v>4277</x:v>
+      </x:c>
+      <x:c r="D228" s="17" t="n">
+        <x:v>4277</x:v>
+      </x:c>
+      <x:c r="E228" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F228" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G228" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H228" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I228" s="31" t="str">
+        <x:f>IF(AND(G228=H228,C228&gt;0,ABS(C228-'Prices'!H228)&lt;=MAX(0.01,'Prices'!H228*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J228" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K228" s="14" t="str"/>
+      <x:c r="L228" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M228" s="14" t="str"/>
+    </x:row>
+    <x:row r="229" ht="50" customHeight="1">
+      <x:c r="A229" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B229" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C229" s="33" t="n">
+        <x:v>26.3</x:v>
+      </x:c>
+      <x:c r="D229" s="33" t="n">
+        <x:v>26.3</x:v>
+      </x:c>
+      <x:c r="E229" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F229" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G229" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H229" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I229" s="32" t="str">
+        <x:f>IF(AND(G229=H229,C229&gt;0,ABS(C229-'Prices'!H229)&lt;=MAX(0.01,'Prices'!H229*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J229" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K229" s="16" t="str"/>
+      <x:c r="L229" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M229" s="16" t="str"/>
+    </x:row>
+    <x:row r="230" ht="50" customHeight="1">
+      <x:c r="A230" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B230" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C230" s="17" t="n">
+        <x:v>336.59</x:v>
+      </x:c>
+      <x:c r="D230" s="17" t="n">
+        <x:v>336.59</x:v>
+      </x:c>
+      <x:c r="E230" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F230" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G230" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H230" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I230" s="31" t="str">
+        <x:f>IF(AND(G230=H230,C230&gt;0,ABS(C230-'Prices'!H230)&lt;=MAX(0.01,'Prices'!H230*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J230" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K230" s="14" t="str"/>
+      <x:c r="L230" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M230" s="14" t="str"/>
+    </x:row>
+    <x:row r="231" ht="50" customHeight="1">
+      <x:c r="A231" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B231" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C231" s="33" t="n">
+        <x:v>4293</x:v>
+      </x:c>
+      <x:c r="D231" s="33" t="n">
+        <x:v>4293</x:v>
+      </x:c>
+      <x:c r="E231" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F231" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G231" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H231" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I231" s="32" t="str">
+        <x:f>IF(AND(G231=H231,C231&gt;0,ABS(C231-'Prices'!H231)&lt;=MAX(0.01,'Prices'!H231*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J231" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K231" s="16" t="str"/>
+      <x:c r="L231" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M231" s="16" t="str"/>
+    </x:row>
+    <x:row r="232" ht="50" customHeight="1">
+      <x:c r="A232" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B232" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C232" s="17" t="n">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="D232" s="17" t="n">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="E232" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F232" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G232" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H232" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I232" s="31" t="str">
+        <x:f>IF(AND(G232=H232,C232&gt;0,ABS(C232-'Prices'!H232)&lt;=MAX(0.01,'Prices'!H232*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J232" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K232" s="14" t="str"/>
+      <x:c r="L232" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M232" s="14" t="str"/>
+    </x:row>
+    <x:row r="233" ht="50" customHeight="1">
+      <x:c r="A233" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C233" s="33" t="n">
+        <x:v>80910</x:v>
+      </x:c>
+      <x:c r="D233" s="33" t="n">
+        <x:v>80910</x:v>
+      </x:c>
+      <x:c r="E233" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F233" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G233" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H233" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I233" s="32" t="str">
+        <x:f>IF(AND(G233=H233,C233&gt;0,ABS(C233-'Prices'!H233)&lt;=MAX(0.01,'Prices'!H233*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J233" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K233" s="16" t="str"/>
+      <x:c r="L233" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M233" s="16" t="str"/>
+    </x:row>
+    <x:row r="234" ht="50" customHeight="1">
+      <x:c r="A234" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B234" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C234" s="17" t="n">
+        <x:v>56.77</x:v>
+      </x:c>
+      <x:c r="D234" s="17" t="n">
+        <x:v>56.77</x:v>
+      </x:c>
+      <x:c r="E234" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F234" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G234" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H234" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I234" s="31" t="str">
+        <x:f>IF(AND(G234=H234,C234&gt;0,ABS(C234-'Prices'!H234)&lt;=MAX(0.01,'Prices'!H234*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J234" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K234" s="14" t="str"/>
+      <x:c r="L234" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M234" s="14" t="str"/>
+    </x:row>
+    <x:row r="235" ht="50" customHeight="1">
+      <x:c r="A235" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C235" s="33" t="n">
+        <x:v>29.65</x:v>
+      </x:c>
+      <x:c r="D235" s="33" t="n">
+        <x:v>29.65</x:v>
+      </x:c>
+      <x:c r="E235" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F235" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G235" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H235" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I235" s="32" t="str">
+        <x:f>IF(AND(OR(G235=H235,AND(B235="OUST",G235="XNAS",H235="XNYS",LEFT(M235,34)="ouster-marketstack-legacy-nyse-tag")),C235&gt;0,ABS(C235-'Prices'!H235)&lt;=MAX(0.01,'Prices'!H235*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J235" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K235" s="16" t="str"/>
+      <x:c r="L235" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M235" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="50" customHeight="1">
+      <x:c r="A236" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B236" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C236" s="17" t="n">
+        <x:v>13.99</x:v>
+      </x:c>
+      <x:c r="D236" s="17" t="n">
+        <x:v>13.99</x:v>
+      </x:c>
+      <x:c r="E236" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F236" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G236" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H236" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I236" s="31" t="str">
+        <x:f>IF(AND(G236=H236,C236&gt;0,ABS(C236-'Prices'!H236)&lt;=MAX(0.01,'Prices'!H236*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J236" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K236" s="14" t="str"/>
+      <x:c r="L236" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M236" s="14" t="str"/>
+    </x:row>
+    <x:row r="237" ht="50" customHeight="1">
+      <x:c r="A237" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B237" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C237" s="33" t="n">
+        <x:v>427.77</x:v>
+      </x:c>
+      <x:c r="D237" s="33" t="n">
+        <x:v>427.77</x:v>
+      </x:c>
+      <x:c r="E237" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F237" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G237" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H237" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I237" s="32" t="str">
+        <x:f>IF(AND(G237=H237,C237&gt;0,ABS(C237-'Prices'!H237)&lt;=MAX(0.01,'Prices'!H237*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J237" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K237" s="16" t="str"/>
+      <x:c r="L237" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M237" s="16" t="str"/>
+    </x:row>
+    <x:row r="238" ht="50" customHeight="1">
+      <x:c r="A238" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B238" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C238" s="17" t="n">
+        <x:v>260.25</x:v>
+      </x:c>
+      <x:c r="D238" s="17" t="n">
+        <x:v>260.25</x:v>
+      </x:c>
+      <x:c r="E238" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F238" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G238" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H238" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I238" s="31" t="str">
+        <x:f>IF(AND(G238=H238,C238&gt;0,ABS(C238-'Prices'!H238)&lt;=MAX(0.01,'Prices'!H238*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J238" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K238" s="14" t="str"/>
+      <x:c r="L238" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M238" s="14" t="str"/>
+    </x:row>
+    <x:row r="239" ht="50" customHeight="1">
+      <x:c r="A239" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C239" s="33" t="n">
+        <x:v>237.6</x:v>
+      </x:c>
+      <x:c r="D239" s="33" t="n">
+        <x:v>237.6</x:v>
+      </x:c>
+      <x:c r="E239" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F239" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G239" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H239" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I239" s="32" t="str">
+        <x:f>IF(AND(G239=H239,C239&gt;0,ABS(C239-'Prices'!H239)&lt;=MAX(0.01,'Prices'!H239*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J239" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K239" s="16" t="str"/>
+      <x:c r="L239" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M239" s="16" t="str"/>
+    </x:row>
+    <x:row r="240" ht="50" customHeight="1">
+      <x:c r="A240" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B240" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C240" s="17" t="n">
+        <x:v>5347</x:v>
+      </x:c>
+      <x:c r="D240" s="17" t="n">
+        <x:v>5347</x:v>
+      </x:c>
+      <x:c r="E240" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F240" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G240" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H240" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I240" s="31" t="str">
+        <x:f>IF(AND(G240=H240,C240&gt;0,ABS(C240-'Prices'!H240)&lt;=MAX(0.01,'Prices'!H240*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J240" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K240" s="14" t="str"/>
+      <x:c r="L240" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M240" s="14" t="str"/>
+    </x:row>
+    <x:row r="241" ht="50" customHeight="1">
+      <x:c r="A241" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B241" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C241" s="33" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="D241" s="33" t="n">
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="E241" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F241" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G241" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H241" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I241" s="32" t="str">
+        <x:f>IF(AND(G241=H241,C241&gt;0,ABS(C241-'Prices'!H241)&lt;=MAX(0.01,'Prices'!H241*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J241" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K241" s="16" t="str"/>
+      <x:c r="L241" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M241" s="16" t="str"/>
+    </x:row>
+    <x:row r="242" ht="50" customHeight="1">
+      <x:c r="A242" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B242" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C242" s="17" t="n">
+        <x:v>7712.57</x:v>
+      </x:c>
+      <x:c r="D242" s="17" t="n">
+        <x:v>7712.57</x:v>
+      </x:c>
+      <x:c r="E242" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F242" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G242" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H242" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I242" s="31" t="str">
+        <x:f>IF(AND(G242=H242,C242&gt;0,ABS(C242-'Prices'!H242)&lt;=MAX(0.01,'Prices'!H242*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J242" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K242" s="14" t="str"/>
+      <x:c r="L242" s="38" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M242" s="14" t="str"/>
+    </x:row>
+    <x:row r="243" ht="50" customHeight="1">
+      <x:c r="A243" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B243" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C243" s="33" t="n">
+        <x:v>26424.8164</x:v>
+      </x:c>
+      <x:c r="D243" s="33" t="n">
+        <x:v>26424.8164</x:v>
+      </x:c>
+      <x:c r="E243" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F243" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G243" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H243" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I243" s="32" t="str">
+        <x:f>IF(AND(G243=H243,C243&gt;0,ABS(C243-'Prices'!H243)&lt;=MAX(0.01,'Prices'!H243*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J243" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-21T11-35-39-133Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K243" s="16" t="str"/>
+      <x:c r="L243" s="39" t="n">
+        <x:v>46316.48309181713</x:v>
+      </x:c>
+      <x:c r="M243" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -24381,7 +26185,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeafd79b778c4ba1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8960b11df424cf8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30879,6 +32683,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="227" ht="27" customHeight="1">
+      <x:c r="A227" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C227" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D227" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E227" s="18" t="n">
+        <x:f>'Source Audit'!E227</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F227" s="41" t="n">
+        <x:f>'Source Audit'!F227</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G227" s="12" t="str">
+        <x:f>IF(AND(E227=0,F227=1,'Source Audit'!I227&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H227" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="27" customHeight="1">
+      <x:c r="A228" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B228" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C228" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D228" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E228" s="19" t="n">
+        <x:f>'Source Audit'!E228</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F228" s="40" t="n">
+        <x:f>'Source Audit'!F228</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G228" s="11" t="str">
+        <x:f>IF(AND(E228=0,F228=1,'Source Audit'!I228&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H228" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="27" customHeight="1">
+      <x:c r="A229" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B229" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C229" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D229" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E229" s="18" t="n">
+        <x:f>'Source Audit'!E229</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F229" s="41" t="n">
+        <x:f>'Source Audit'!F229</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G229" s="12" t="str">
+        <x:f>IF(AND(E229=0,F229=1,'Source Audit'!I229&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H229" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="27" customHeight="1">
+      <x:c r="A230" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B230" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C230" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D230" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E230" s="19" t="n">
+        <x:f>'Source Audit'!E230</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F230" s="40" t="n">
+        <x:f>'Source Audit'!F230</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G230" s="11" t="str">
+        <x:f>IF(AND(E230=0,F230=1,'Source Audit'!I230&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H230" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="27" customHeight="1">
+      <x:c r="A231" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B231" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C231" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D231" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E231" s="18" t="n">
+        <x:f>'Source Audit'!E231</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F231" s="41" t="n">
+        <x:f>'Source Audit'!F231</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G231" s="12" t="str">
+        <x:f>IF(AND(E231=0,F231=1,'Source Audit'!I231&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H231" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="27" customHeight="1">
+      <x:c r="A232" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B232" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C232" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D232" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E232" s="19" t="n">
+        <x:f>'Source Audit'!E232</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F232" s="40" t="n">
+        <x:f>'Source Audit'!F232</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G232" s="11" t="str">
+        <x:f>IF(AND(E232=0,F232=1,'Source Audit'!I232&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H232" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="27" customHeight="1">
+      <x:c r="A233" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C233" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D233" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E233" s="18" t="n">
+        <x:f>'Source Audit'!E233</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F233" s="41" t="n">
+        <x:f>'Source Audit'!F233</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G233" s="12" t="str">
+        <x:f>IF(AND(E233=0,F233=1,'Source Audit'!I233&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H233" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="27" customHeight="1">
+      <x:c r="A234" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B234" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C234" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D234" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E234" s="19" t="n">
+        <x:f>'Source Audit'!E234</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F234" s="40" t="n">
+        <x:f>'Source Audit'!F234</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G234" s="11" t="str">
+        <x:f>IF(AND(E234=0,F234=1,'Source Audit'!I234&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H234" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="44" customHeight="1">
+      <x:c r="A235" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C235" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D235" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E235" s="18" t="n">
+        <x:f>'Source Audit'!E235</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F235" s="41" t="n">
+        <x:f>'Source Audit'!F235</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G235" s="12" t="str">
+        <x:f>IF(AND(E235=0,F235=1,'Source Audit'!I235&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H235" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="27" customHeight="1">
+      <x:c r="A236" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B236" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C236" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D236" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E236" s="19" t="n">
+        <x:f>'Source Audit'!E236</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F236" s="40" t="n">
+        <x:f>'Source Audit'!F236</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G236" s="11" t="str">
+        <x:f>IF(AND(E236=0,F236=1,'Source Audit'!I236&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H236" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="27" customHeight="1">
+      <x:c r="A237" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B237" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C237" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D237" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E237" s="18" t="n">
+        <x:f>'Source Audit'!E237</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F237" s="41" t="n">
+        <x:f>'Source Audit'!F237</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G237" s="12" t="str">
+        <x:f>IF(AND(E237=0,F237=1,'Source Audit'!I237&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H237" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="27" customHeight="1">
+      <x:c r="A238" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B238" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C238" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D238" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E238" s="19" t="n">
+        <x:f>'Source Audit'!E238</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F238" s="40" t="n">
+        <x:f>'Source Audit'!F238</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G238" s="11" t="str">
+        <x:f>IF(AND(E238=0,F238=1,'Source Audit'!I238&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H238" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="27" customHeight="1">
+      <x:c r="A239" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C239" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D239" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E239" s="18" t="n">
+        <x:f>'Source Audit'!E239</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F239" s="41" t="n">
+        <x:f>'Source Audit'!F239</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G239" s="12" t="str">
+        <x:f>IF(AND(E239=0,F239=1,'Source Audit'!I239&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H239" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="27" customHeight="1">
+      <x:c r="A240" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B240" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C240" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D240" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E240" s="19" t="n">
+        <x:f>'Source Audit'!E240</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F240" s="40" t="n">
+        <x:f>'Source Audit'!F240</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G240" s="11" t="str">
+        <x:f>IF(AND(E240=0,F240=1,'Source Audit'!I240&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H240" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="27" customHeight="1">
+      <x:c r="A241" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B241" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C241" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D241" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E241" s="18" t="n">
+        <x:f>'Source Audit'!E241</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F241" s="41" t="n">
+        <x:f>'Source Audit'!F241</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G241" s="12" t="str">
+        <x:f>IF(AND(E241=0,F241=1,'Source Audit'!I241&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H241" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="27" customHeight="1">
+      <x:c r="A242" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B242" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C242" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D242" s="8" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E242" s="19" t="n">
+        <x:f>'Source Audit'!E242</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F242" s="40" t="n">
+        <x:f>'Source Audit'!F242</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G242" s="11" t="str">
+        <x:f>IF(AND(E242=0,F242=1,'Source Audit'!I242&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H242" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="27" customHeight="1">
+      <x:c r="A243" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B243" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C243" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D243" s="9" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="E243" s="18" t="n">
+        <x:f>'Source Audit'!E243</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F243" s="41" t="n">
+        <x:f>'Source Audit'!F243</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G243" s="12" t="str">
+        <x:f>IF(AND(E243=0,F243=1,'Source Audit'!I243&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H243" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -30886,7 +33183,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d397195598a4de3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R350ef78d88cd4b87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 21, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 223 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings, documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R832139e5204c403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R6806f08006d74911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R3a6ce0d8d7e34923"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R30d26043b4b94a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R8cc055f0b0574d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R455cdb640c2b4abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R3f4dc14b4e65461b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Red6d069b2aff49be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Rc5324143139c4131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rbb7e8400c1e34669"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H215" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H230" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1787,6 +1787,85 @@
         <x:v>-6.188436618849669</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="40" customHeight="1">
+      <x:c r="A20" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="n">
+        <x:f>B19*(1+SUM('Returns and Contributions'!F216:F230))</x:f>
+        <x:v>926.4814343915143</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="n">
+        <x:f>B20/B19-1</x:f>
+        <x:v>0.005417592333814225</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="n">
+        <x:f>B20/$B$6-1</x:f>
+        <x:v>-0.07351856560848569</x:v>
+      </x:c>
+      <x:c r="E20" s="19" t="n">
+        <x:f>1000*'Prices'!H259/'Prices'!I259</x:f>
+        <x:v>1011.8333778998102</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="n">
+        <x:f>E20/E19-1</x:f>
+        <x:v>0.005782767611833606</x:v>
+      </x:c>
+      <x:c r="G20" s="20" t="n">
+        <x:f>E20/1000-1</x:f>
+        <x:v>0.011833377899810316</x:v>
+      </x:c>
+      <x:c r="H20" s="19" t="n">
+        <x:f>1000*'Prices'!H260/'Prices'!I260</x:f>
+        <x:v>993.7205701557947</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="n">
+        <x:f>H20/H19-1</x:f>
+        <x:v>0.010521965253843746</x:v>
+      </x:c>
+      <x:c r="J20" s="20" t="n">
+        <x:f>H20/1000-1</x:f>
+        <x:v>-0.006279429844205264</x:v>
+      </x:c>
+      <x:c r="K20" s="24" t="n">
+        <x:f>(C20-F20)*100</x:f>
+        <x:v>-0.036517527801938066</x:v>
+      </x:c>
+      <x:c r="L20" s="24" t="n">
+        <x:f>(C20-I20)*100</x:f>
+        <x:v>-0.5104372920029521</x:v>
+      </x:c>
+      <x:c r="M20" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G216:G230)</x:f>
+        <x:v>0.9999999999999996</x:v>
+      </x:c>
+      <x:c r="N20" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F216:F230)-C20</x:f>
+        <x:v>-8.673617379884035e-17</x:v>
+      </x:c>
+      <x:c r="O20" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P20" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I244:I260,"Mismatch")=0,IF(COUNTIF('Source Audit'!I244:I260,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q20" s="29" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="R20" s="28" t="n">
+        <x:f>B20-1000*('Prices'!H244/'Prices'!H6+'Prices'!H245/'Prices'!H7+'Prices'!H246/'Prices'!H8+'Prices'!H247/'Prices'!H9+'Prices'!H248/'Prices'!H10+'Prices'!H249/'Prices'!H11+'Prices'!H250/'Prices'!H12+'Prices'!H251/'Prices'!H13+'Prices'!H252/'Prices'!H14+'Prices'!H253/'Prices'!H15+'Prices'!H254/'Prices'!H16+'Prices'!H255/'Prices'!H17+'Prices'!H256/'Prices'!H18+'Prices'!H257/'Prices'!H19+'Prices'!H258/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S20" s="24" t="n">
+        <x:f>(D20-G20)*100</x:f>
+        <x:v>-8.5351943508296</x:v>
+      </x:c>
+      <x:c r="T20" s="24" t="n">
+        <x:f>(D20-J20)*100</x:f>
+        <x:v>-6.723913576428043</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1794,7 +1873,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6e9bd15ed574169"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7472d9ca056a4bf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10424,6 +10503,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="244" ht="27" customHeight="1">
+      <x:c r="A244" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B244" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C244" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D244" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E244" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F244" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G244" s="17" t="n">
+        <x:f>H227</x:f>
+        <x:v>5788</x:v>
+      </x:c>
+      <x:c r="H244" s="34" t="n">
+        <x:v>5823</x:v>
+      </x:c>
+      <x:c r="I244" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J244" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K244" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="27" customHeight="1">
+      <x:c r="A245" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C245" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D245" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E245" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F245" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G245" s="33" t="n">
+        <x:f>H228</x:f>
+        <x:v>4277</x:v>
+      </x:c>
+      <x:c r="H245" s="35" t="n">
+        <x:v>4204</x:v>
+      </x:c>
+      <x:c r="I245" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J245" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K245" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="27" customHeight="1">
+      <x:c r="A246" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B246" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C246" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D246" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E246" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F246" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G246" s="17" t="n">
+        <x:f>H229</x:f>
+        <x:v>26.3</x:v>
+      </x:c>
+      <x:c r="H246" s="34" t="n">
+        <x:v>26.08</x:v>
+      </x:c>
+      <x:c r="I246" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J246" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K246" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="27" customHeight="1">
+      <x:c r="A247" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C247" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D247" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E247" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F247" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G247" s="33" t="n">
+        <x:f>H230</x:f>
+        <x:v>336.59</x:v>
+      </x:c>
+      <x:c r="H247" s="35" t="n">
+        <x:v>345.49</x:v>
+      </x:c>
+      <x:c r="I247" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J247" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K247" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="27" customHeight="1">
+      <x:c r="A248" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B248" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C248" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D248" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E248" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F248" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G248" s="17" t="n">
+        <x:f>H231</x:f>
+        <x:v>4293</x:v>
+      </x:c>
+      <x:c r="H248" s="34" t="n">
+        <x:v>4357</x:v>
+      </x:c>
+      <x:c r="I248" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J248" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K248" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="27" customHeight="1">
+      <x:c r="A249" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B249" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C249" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D249" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E249" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F249" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G249" s="33" t="n">
+        <x:f>H232</x:f>
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="H249" s="35" t="n">
+        <x:v>49.9</x:v>
+      </x:c>
+      <x:c r="I249" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J249" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K249" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="27" customHeight="1">
+      <x:c r="A250" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B250" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C250" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D250" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E250" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F250" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G250" s="17" t="n">
+        <x:f>H233</x:f>
+        <x:v>80910</x:v>
+      </x:c>
+      <x:c r="H250" s="34" t="n">
+        <x:v>80860</x:v>
+      </x:c>
+      <x:c r="I250" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J250" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K250" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="27" customHeight="1">
+      <x:c r="A251" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B251" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C251" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D251" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E251" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F251" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G251" s="33" t="n">
+        <x:f>H234</x:f>
+        <x:v>56.77</x:v>
+      </x:c>
+      <x:c r="H251" s="35" t="n">
+        <x:v>58.05</x:v>
+      </x:c>
+      <x:c r="I251" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J251" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K251" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="27" customHeight="1">
+      <x:c r="A252" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B252" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C252" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D252" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E252" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F252" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G252" s="17" t="n">
+        <x:f>H235</x:f>
+        <x:v>29.65</x:v>
+      </x:c>
+      <x:c r="H252" s="34" t="n">
+        <x:v>30.31</x:v>
+      </x:c>
+      <x:c r="I252" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J252" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K252" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="27" customHeight="1">
+      <x:c r="A253" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B253" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C253" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D253" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E253" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F253" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G253" s="33" t="n">
+        <x:f>H236</x:f>
+        <x:v>13.99</x:v>
+      </x:c>
+      <x:c r="H253" s="35" t="n">
+        <x:v>13.19</x:v>
+      </x:c>
+      <x:c r="I253" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J253" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K253" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="27" customHeight="1">
+      <x:c r="A254" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B254" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C254" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D254" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E254" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F254" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G254" s="17" t="n">
+        <x:f>H237</x:f>
+        <x:v>427.77</x:v>
+      </x:c>
+      <x:c r="H254" s="34" t="n">
+        <x:v>438.51</x:v>
+      </x:c>
+      <x:c r="I254" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J254" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K254" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="27" customHeight="1">
+      <x:c r="A255" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B255" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C255" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D255" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E255" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F255" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G255" s="33" t="n">
+        <x:f>H238</x:f>
+        <x:v>260.25</x:v>
+      </x:c>
+      <x:c r="H255" s="35" t="n">
+        <x:v>266.75</x:v>
+      </x:c>
+      <x:c r="I255" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J255" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K255" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="27" customHeight="1">
+      <x:c r="A256" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B256" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C256" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D256" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E256" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F256" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G256" s="17" t="n">
+        <x:f>H239</x:f>
+        <x:v>237.6</x:v>
+      </x:c>
+      <x:c r="H256" s="34" t="n">
+        <x:v>242.36</x:v>
+      </x:c>
+      <x:c r="I256" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J256" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K256" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="27" customHeight="1">
+      <x:c r="A257" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B257" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C257" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D257" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E257" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F257" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G257" s="33" t="n">
+        <x:f>H240</x:f>
+        <x:v>5347</x:v>
+      </x:c>
+      <x:c r="H257" s="35" t="n">
+        <x:v>5445</x:v>
+      </x:c>
+      <x:c r="I257" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J257" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K257" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="27" customHeight="1">
+      <x:c r="A258" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B258" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C258" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D258" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E258" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F258" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G258" s="17" t="n">
+        <x:f>H241</x:f>
+        <x:v>104.25</x:v>
+      </x:c>
+      <x:c r="H258" s="34" t="n">
+        <x:v>104.7</x:v>
+      </x:c>
+      <x:c r="I258" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J258" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K258" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="27" customHeight="1">
+      <x:c r="A259" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B259" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C259" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D259" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E259" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F259" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G259" s="33" t="n">
+        <x:f>H242</x:f>
+        <x:v>7712.57</x:v>
+      </x:c>
+      <x:c r="H259" s="35" t="n">
+        <x:v>7757.17</x:v>
+      </x:c>
+      <x:c r="I259" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J259" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K259" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="27" customHeight="1">
+      <x:c r="A260" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B260" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C260" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D260" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E260" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F260" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G260" s="17" t="n">
+        <x:f>H243</x:f>
+        <x:v>26424.8164</x:v>
+      </x:c>
+      <x:c r="H260" s="34" t="n">
+        <x:v>26702.8574</x:v>
+      </x:c>
+      <x:c r="I260" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J260" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="K260" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -10431,7 +11122,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e1fc0fa953b4a39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9694391018c4653"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16940,6 +17631,471 @@
         <x:v>0.052817612603514474</x:v>
       </x:c>
     </x:row>
+    <x:row r="216" ht="27" customHeight="1">
+      <x:c r="A216" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B216" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C216" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D216" s="20" t="n">
+        <x:f>G201</x:f>
+        <x:v>0.06834380309546927</x:v>
+      </x:c>
+      <x:c r="E216" s="22" t="n">
+        <x:f>'Prices'!H244/'Prices'!G244-1</x:f>
+        <x:v>0.006046993780234988</x:v>
+      </x:c>
+      <x:c r="F216" s="20" t="n">
+        <x:f>D216*E216</x:f>
+        <x:v>0.0004132745522359074</x:v>
+      </x:c>
+      <x:c r="G216" s="20" t="n">
+        <x:f>D216*(1+E216)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06838658699824773</x:v>
+      </x:c>
+      <x:c r="H216" s="22" t="n">
+        <x:f>'Prices'!H244/'Prices'!I244-1</x:f>
+        <x:v>-0.04961645177085039</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="27" customHeight="1">
+      <x:c r="A217" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B217" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C217" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D217" s="21" t="n">
+        <x:f>G202</x:f>
+        <x:v>0.06474715940266505</x:v>
+      </x:c>
+      <x:c r="E217" s="23" t="n">
+        <x:f>'Prices'!H245/'Prices'!G245-1</x:f>
+        <x:v>-0.017068038344634107</x:v>
+      </x:c>
+      <x:c r="F217" s="21" t="n">
+        <x:f>D217*E217</x:f>
+        <x:v>-0.0011051069993908238</x:v>
+      </x:c>
+      <x:c r="G217" s="21" t="n">
+        <x:f>D217*(1+E217)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06329912355675599</x:v>
+      </x:c>
+      <x:c r="H217" s="23" t="n">
+        <x:f>'Prices'!H245/'Prices'!I245-1</x:f>
+        <x:v>-0.12031805817116548</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="27" customHeight="1">
+      <x:c r="A218" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B218" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C218" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D218" s="20" t="n">
+        <x:f>G203</x:f>
+        <x:v>0.06742442307861607</x:v>
+      </x:c>
+      <x:c r="E218" s="22" t="n">
+        <x:f>'Prices'!H246/'Prices'!G246-1</x:f>
+        <x:v>-0.00836501901140696</x:v>
+      </x:c>
+      <x:c r="F218" s="20" t="n">
+        <x:f>D218*E218</x:f>
+        <x:v>-0.0005640065808857696</x:v>
+      </x:c>
+      <x:c r="G218" s="20" t="n">
+        <x:f>D218*(1+E218)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06650014581755159</x:v>
+      </x:c>
+      <x:c r="H218" s="22" t="n">
+        <x:f>'Prices'!H246/'Prices'!I246-1</x:f>
+        <x:v>-0.07583274273564855</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="27" customHeight="1">
+      <x:c r="A219" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B219" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C219" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D219" s="21" t="n">
+        <x:f>G204</x:f>
+        <x:v>0.058566014270783055</x:v>
+      </x:c>
+      <x:c r="E219" s="23" t="n">
+        <x:f>'Prices'!H247/'Prices'!G247-1</x:f>
+        <x:v>0.026441664933598785</x:v>
+      </x:c>
+      <x:c r="F219" s="21" t="n">
+        <x:f>D219*E219</x:f>
+        <x:v>0.0015485829258444104</x:v>
+      </x:c>
+      <x:c r="G219" s="21" t="n">
+        <x:f>D219*(1+E219)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.059790675690373725</x:v>
+      </x:c>
+      <x:c r="H219" s="23" t="n">
+        <x:f>'Prices'!H247/'Prices'!I247-1</x:f>
+        <x:v>-0.16907573534717046</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="27" customHeight="1">
+      <x:c r="A220" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B220" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C220" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D220" s="20" t="n">
+        <x:f>G205</x:f>
+        <x:v>0.06242898922263636</x:v>
+      </x:c>
+      <x:c r="E220" s="22" t="n">
+        <x:f>'Prices'!H248/'Prices'!G248-1</x:f>
+        <x:v>0.014907989750757134</x:v>
+      </x:c>
+      <x:c r="F220" s="20" t="n">
+        <x:f>D220*E220</x:f>
+        <x:v>0.0009306907314811904</x:v>
+      </x:c>
+      <x:c r="G220" s="20" t="n">
+        <x:f>D220*(1+E220)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.0630182726433547</x:v>
+      </x:c>
+      <x:c r="H220" s="22" t="n">
+        <x:f>'Prices'!H248/'Prices'!I248-1</x:f>
+        <x:v>-0.12422110552763821</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="27" customHeight="1">
+      <x:c r="A221" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B221" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C221" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D221" s="21" t="n">
+        <x:f>G206</x:f>
+        <x:v>0.07081330339813344</x:v>
+      </x:c>
+      <x:c r="E221" s="23" t="n">
+        <x:f>'Prices'!H249/'Prices'!G249-1</x:f>
+        <x:v>-0.017716535433070835</x:v>
+      </x:c>
+      <x:c r="F221" s="21" t="n">
+        <x:f>D221*E221</x:f>
+        <x:v>-0.0012545663987858263</x:v>
+      </x:c>
+      <x:c r="G221" s="21" t="n">
+        <x:f>D221*(1+E221)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06918392668849685</x:v>
+      </x:c>
+      <x:c r="H221" s="23" t="n">
+        <x:f>'Prices'!H249/'Prices'!I249-1</x:f>
+        <x:v>-0.038535645472061675</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="27" customHeight="1">
+      <x:c r="A222" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B222" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C222" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D222" s="20" t="n">
+        <x:f>G207</x:f>
+        <x:v>0.07208828139308994</x:v>
+      </x:c>
+      <x:c r="E222" s="22" t="n">
+        <x:f>'Prices'!H250/'Prices'!G250-1</x:f>
+        <x:v>-0.0006179705846002248</x:v>
+      </x:c>
+      <x:c r="F222" s="20" t="n">
+        <x:f>D222*E222</x:f>
+        <x:v>-0.000044548437395313295</x:v>
+      </x:c>
+      <x:c r="G222" s="20" t="n">
+        <x:f>D222*(1+E222)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.07165553249218956</x:v>
+      </x:c>
+      <x:c r="H222" s="22" t="n">
+        <x:f>'Prices'!H250/'Prices'!I250-1</x:f>
+        <x:v>-0.004187192118226601</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="27" customHeight="1">
+      <x:c r="A223" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B223" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C223" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D223" s="21" t="n">
+        <x:f>G208</x:f>
+        <x:v>0.06600964353058691</x:v>
+      </x:c>
+      <x:c r="E223" s="23" t="n">
+        <x:f>'Prices'!H251/'Prices'!G251-1</x:f>
+        <x:v>0.02254711995772407</x:v>
+      </x:c>
+      <x:c r="F223" s="21" t="n">
+        <x:f>D223*E223</x:f>
+        <x:v>0.0014883273510507477</x:v>
+      </x:c>
+      <x:c r="G223" s="21" t="n">
+        <x:f>D223*(1+E223)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06713426480330303</x:v>
+      </x:c>
+      <x:c r="H223" s="23" t="n">
+        <x:f>'Prices'!H251/'Prices'!I251-1</x:f>
+        <x:v>-0.06702025072324014</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="27" customHeight="1">
+      <x:c r="A224" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B224" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C224" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D224" s="20" t="n">
+        <x:f>G209</x:f>
+        <x:v>0.052485405874332966</x:v>
+      </x:c>
+      <x:c r="E224" s="22" t="n">
+        <x:f>'Prices'!H252/'Prices'!G252-1</x:f>
+        <x:v>0.022259696458684752</x:v>
+      </x:c>
+      <x:c r="F224" s="20" t="n">
+        <x:f>D224*E224</x:f>
+        <x:v>0.0011683092032735215</x:v>
+      </x:c>
+      <x:c r="G224" s="20" t="n">
+        <x:f>D224*(1+E224)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.05336460738971496</x:v>
+      </x:c>
+      <x:c r="H224" s="22" t="n">
+        <x:f>'Prices'!H252/'Prices'!I252-1</x:f>
+        <x:v>-0.25838022999755317</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="27" customHeight="1">
+      <x:c r="A225" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B225" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C225" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D225" s="21" t="n">
+        <x:f>G210</x:f>
+        <x:v>0.06353608323894909</x:v>
+      </x:c>
+      <x:c r="E225" s="23" t="n">
+        <x:f>'Prices'!H253/'Prices'!G253-1</x:f>
+        <x:v>-0.05718370264474626</x:v>
+      </x:c>
+      <x:c r="F225" s="21" t="n">
+        <x:f>D225*E225</x:f>
+        <x:v>-0.0036332284911479115</x:v>
+      </x:c>
+      <x:c r="G225" s="21" t="n">
+        <x:f>D225*(1+E225)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.059580074194596454</x:v>
+      </x:c>
+      <x:c r="H225" s="23" t="n">
+        <x:f>'Prices'!H253/'Prices'!I253-1</x:f>
+        <x:v>-0.17200251098556185</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="27" customHeight="1">
+      <x:c r="A226" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B226" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C226" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D226" s="20" t="n">
+        <x:f>G211</x:f>
+        <x:v>0.06994628035912916</x:v>
+      </x:c>
+      <x:c r="E226" s="22" t="n">
+        <x:f>'Prices'!H254/'Prices'!G254-1</x:f>
+        <x:v>0.025106949996493544</x:v>
+      </x:c>
+      <x:c r="F226" s="20" t="n">
+        <x:f>D226*E226</x:f>
+        <x:v>0.0017561377634173743</x:v>
+      </x:c>
+      <x:c r="G226" s="20" t="n">
+        <x:f>D226*(1+E226)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.07131605679994926</x:v>
+      </x:c>
+      <x:c r="H226" s="22" t="n">
+        <x:f>'Prices'!H254/'Prices'!I254-1</x:f>
+        <x:v>-0.008904961012543788</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="27" customHeight="1">
+      <x:c r="A227" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B227" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C227" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D227" s="21" t="n">
+        <x:f>G212</x:f>
+        <x:v>0.06924685131069515</x:v>
+      </x:c>
+      <x:c r="E227" s="23" t="n">
+        <x:f>'Prices'!H255/'Prices'!G255-1</x:f>
+        <x:v>0.024975984630163373</x:v>
+      </x:c>
+      <x:c r="F227" s="21" t="n">
+        <x:f>D227*E227</x:f>
+        <x:v>0.0017295082940231303</x:v>
+      </x:c>
+      <x:c r="G227" s="21" t="n">
+        <x:f>D227*(1+E227)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.07059391057596795</x:v>
+      </x:c>
+      <x:c r="H227" s="23" t="n">
+        <x:f>'Prices'!H255/'Prices'!I255-1</x:f>
+        <x:v>-0.01894078705406388</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="27" customHeight="1">
+      <x:c r="A228" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B228" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C228" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D228" s="20" t="n">
+        <x:f>G213</x:f>
+        <x:v>0.07186574258791711</x:v>
+      </x:c>
+      <x:c r="E228" s="22" t="n">
+        <x:f>'Prices'!H256/'Prices'!G256-1</x:f>
+        <x:v>0.02003367003367007</x:v>
+      </x:c>
+      <x:c r="F228" s="20" t="n">
+        <x:f>D228*E228</x:f>
+        <x:v>0.001439734573731002</x:v>
+      </x:c>
+      <x:c r="G228" s="20" t="n">
+        <x:f>D228*(1+E228)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.07291047791543871</x:v>
+      </x:c>
+      <x:c r="H228" s="22" t="n">
+        <x:f>'Prices'!H256/'Prices'!I256-1</x:f>
+        <x:v>0.013253062418997485</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="27" customHeight="1">
+      <x:c r="A229" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B229" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C229" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D229" s="21" t="n">
+        <x:f>G214</x:f>
+        <x:v>0.06633017892291107</x:v>
+      </x:c>
+      <x:c r="E229" s="23" t="n">
+        <x:f>'Prices'!H257/'Prices'!G257-1</x:f>
+        <x:v>0.018328034411819738</x:v>
+      </x:c>
+      <x:c r="F229" s="21" t="n">
+        <x:f>D229*E229</x:f>
+        <x:v>0.0012157018018412744</x:v>
+      </x:c>
+      <x:c r="G229" s="21" t="n">
+        <x:f>D229*(1+E229)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.06718191648901053</x:v>
+      </x:c>
+      <x:c r="H229" s="23" t="n">
+        <x:f>'Prices'!H257/'Prices'!I257-1</x:f>
+        <x:v>-0.06635802469135799</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="27" customHeight="1">
+      <x:c r="A230" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B230" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C230" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D230" s="20" t="n">
+        <x:f>G215</x:f>
+        <x:v>0.07616784031408504</x:v>
+      </x:c>
+      <x:c r="E230" s="22" t="n">
+        <x:f>'Prices'!H258/'Prices'!G258-1</x:f>
+        <x:v>0.004316546762589857</x:v>
+      </x:c>
+      <x:c r="F230" s="20" t="n">
+        <x:f>D230*E230</x:f>
+        <x:v>0.00032878204452122493</x:v>
+      </x:c>
+      <x:c r="G230" s="20" t="n">
+        <x:f>D230*(1+E230)/(1+SUM($F$216:$F$230))</x:f>
+        <x:v>0.07608442794504852</x:v>
+      </x:c>
+      <x:c r="H230" s="22" t="n">
+        <x:f>'Prices'!H258/'Prices'!I258-1</x:f>
+        <x:v>0.05736214906079584</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -16947,7 +18103,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb785009f70a417f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f5c3cbc5f21436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26178,6 +27334,654 @@
       </x:c>
       <x:c r="M243" s="16" t="str"/>
     </x:row>
+    <x:row r="244" ht="50" customHeight="1">
+      <x:c r="A244" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B244" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C244" s="17" t="n">
+        <x:v>5823</x:v>
+      </x:c>
+      <x:c r="D244" s="17" t="n">
+        <x:v>5823</x:v>
+      </x:c>
+      <x:c r="E244" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F244" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G244" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H244" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I244" s="31" t="str">
+        <x:f>IF(AND(G244=H244,C244&gt;0,ABS(C244-'Prices'!H244)&lt;=MAX(0.01,'Prices'!H244*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J244" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K244" s="14" t="str"/>
+      <x:c r="L244" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M244" s="14" t="str"/>
+    </x:row>
+    <x:row r="245" ht="50" customHeight="1">
+      <x:c r="A245" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C245" s="33" t="n">
+        <x:v>4204</x:v>
+      </x:c>
+      <x:c r="D245" s="33" t="n">
+        <x:v>4204</x:v>
+      </x:c>
+      <x:c r="E245" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F245" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G245" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H245" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I245" s="32" t="str">
+        <x:f>IF(AND(G245=H245,C245&gt;0,ABS(C245-'Prices'!H245)&lt;=MAX(0.01,'Prices'!H245*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J245" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K245" s="16" t="str"/>
+      <x:c r="L245" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M245" s="16" t="str"/>
+    </x:row>
+    <x:row r="246" ht="50" customHeight="1">
+      <x:c r="A246" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B246" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C246" s="17" t="n">
+        <x:v>26.08</x:v>
+      </x:c>
+      <x:c r="D246" s="17" t="n">
+        <x:v>26.08</x:v>
+      </x:c>
+      <x:c r="E246" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F246" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G246" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H246" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I246" s="31" t="str">
+        <x:f>IF(AND(G246=H246,C246&gt;0,ABS(C246-'Prices'!H246)&lt;=MAX(0.01,'Prices'!H246*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J246" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K246" s="14" t="str"/>
+      <x:c r="L246" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M246" s="14" t="str"/>
+    </x:row>
+    <x:row r="247" ht="50" customHeight="1">
+      <x:c r="A247" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C247" s="33" t="n">
+        <x:v>345.49</x:v>
+      </x:c>
+      <x:c r="D247" s="33" t="n">
+        <x:v>345.49</x:v>
+      </x:c>
+      <x:c r="E247" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F247" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G247" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H247" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I247" s="32" t="str">
+        <x:f>IF(AND(G247=H247,C247&gt;0,ABS(C247-'Prices'!H247)&lt;=MAX(0.01,'Prices'!H247*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J247" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K247" s="16" t="str"/>
+      <x:c r="L247" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M247" s="16" t="str"/>
+    </x:row>
+    <x:row r="248" ht="50" customHeight="1">
+      <x:c r="A248" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B248" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C248" s="17" t="n">
+        <x:v>4357</x:v>
+      </x:c>
+      <x:c r="D248" s="17" t="n">
+        <x:v>4357</x:v>
+      </x:c>
+      <x:c r="E248" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F248" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G248" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H248" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I248" s="31" t="str">
+        <x:f>IF(AND(G248=H248,C248&gt;0,ABS(C248-'Prices'!H248)&lt;=MAX(0.01,'Prices'!H248*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J248" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K248" s="14" t="str"/>
+      <x:c r="L248" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M248" s="14" t="str"/>
+    </x:row>
+    <x:row r="249" ht="50" customHeight="1">
+      <x:c r="A249" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B249" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C249" s="33" t="n">
+        <x:v>49.9</x:v>
+      </x:c>
+      <x:c r="D249" s="33" t="n">
+        <x:v>49.9</x:v>
+      </x:c>
+      <x:c r="E249" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F249" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G249" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H249" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I249" s="32" t="str">
+        <x:f>IF(AND(G249=H249,C249&gt;0,ABS(C249-'Prices'!H249)&lt;=MAX(0.01,'Prices'!H249*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J249" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K249" s="16" t="str"/>
+      <x:c r="L249" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M249" s="16" t="str"/>
+    </x:row>
+    <x:row r="250" ht="50" customHeight="1">
+      <x:c r="A250" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B250" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C250" s="17" t="n">
+        <x:v>80860</x:v>
+      </x:c>
+      <x:c r="D250" s="17" t="n">
+        <x:v>80860</x:v>
+      </x:c>
+      <x:c r="E250" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F250" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G250" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H250" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I250" s="31" t="str">
+        <x:f>IF(AND(G250=H250,C250&gt;0,ABS(C250-'Prices'!H250)&lt;=MAX(0.01,'Prices'!H250*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J250" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K250" s="14" t="str"/>
+      <x:c r="L250" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M250" s="14" t="str"/>
+    </x:row>
+    <x:row r="251" ht="50" customHeight="1">
+      <x:c r="A251" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B251" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C251" s="33" t="n">
+        <x:v>58.05</x:v>
+      </x:c>
+      <x:c r="D251" s="33" t="n">
+        <x:v>58.05</x:v>
+      </x:c>
+      <x:c r="E251" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F251" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G251" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H251" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I251" s="32" t="str">
+        <x:f>IF(AND(G251=H251,C251&gt;0,ABS(C251-'Prices'!H251)&lt;=MAX(0.01,'Prices'!H251*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J251" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K251" s="16" t="str"/>
+      <x:c r="L251" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M251" s="16" t="str"/>
+    </x:row>
+    <x:row r="252" ht="50" customHeight="1">
+      <x:c r="A252" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B252" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C252" s="17" t="n">
+        <x:v>30.31</x:v>
+      </x:c>
+      <x:c r="D252" s="17" t="n">
+        <x:v>30.31</x:v>
+      </x:c>
+      <x:c r="E252" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F252" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G252" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H252" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I252" s="31" t="str">
+        <x:f>IF(AND(OR(G252=H252,AND(B252="OUST",G252="XNAS",H252="XNYS",LEFT(M252,34)="ouster-marketstack-legacy-nyse-tag")),C252&gt;0,ABS(C252-'Prices'!H252)&lt;=MAX(0.01,'Prices'!H252*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J252" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K252" s="14" t="str"/>
+      <x:c r="L252" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M252" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="50" customHeight="1">
+      <x:c r="A253" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B253" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C253" s="33" t="n">
+        <x:v>13.19</x:v>
+      </x:c>
+      <x:c r="D253" s="33" t="n">
+        <x:v>13.19</x:v>
+      </x:c>
+      <x:c r="E253" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F253" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G253" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H253" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I253" s="32" t="str">
+        <x:f>IF(AND(G253=H253,C253&gt;0,ABS(C253-'Prices'!H253)&lt;=MAX(0.01,'Prices'!H253*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J253" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K253" s="16" t="str"/>
+      <x:c r="L253" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M253" s="16" t="str"/>
+    </x:row>
+    <x:row r="254" ht="50" customHeight="1">
+      <x:c r="A254" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B254" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C254" s="17" t="n">
+        <x:v>438.51</x:v>
+      </x:c>
+      <x:c r="D254" s="17" t="n">
+        <x:v>438.51</x:v>
+      </x:c>
+      <x:c r="E254" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F254" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G254" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H254" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I254" s="31" t="str">
+        <x:f>IF(AND(G254=H254,C254&gt;0,ABS(C254-'Prices'!H254)&lt;=MAX(0.01,'Prices'!H254*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J254" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K254" s="14" t="str"/>
+      <x:c r="L254" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M254" s="14" t="str"/>
+    </x:row>
+    <x:row r="255" ht="50" customHeight="1">
+      <x:c r="A255" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B255" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C255" s="33" t="n">
+        <x:v>266.75</x:v>
+      </x:c>
+      <x:c r="D255" s="33" t="n">
+        <x:v>266.75</x:v>
+      </x:c>
+      <x:c r="E255" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F255" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G255" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H255" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I255" s="32" t="str">
+        <x:f>IF(AND(G255=H255,C255&gt;0,ABS(C255-'Prices'!H255)&lt;=MAX(0.01,'Prices'!H255*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J255" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K255" s="16" t="str"/>
+      <x:c r="L255" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M255" s="16" t="str"/>
+    </x:row>
+    <x:row r="256" ht="50" customHeight="1">
+      <x:c r="A256" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B256" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C256" s="17" t="n">
+        <x:v>242.36</x:v>
+      </x:c>
+      <x:c r="D256" s="17" t="n">
+        <x:v>242.36</x:v>
+      </x:c>
+      <x:c r="E256" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F256" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G256" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H256" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I256" s="31" t="str">
+        <x:f>IF(AND(G256=H256,C256&gt;0,ABS(C256-'Prices'!H256)&lt;=MAX(0.01,'Prices'!H256*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J256" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K256" s="14" t="str"/>
+      <x:c r="L256" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M256" s="14" t="str"/>
+    </x:row>
+    <x:row r="257" ht="50" customHeight="1">
+      <x:c r="A257" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B257" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C257" s="33" t="n">
+        <x:v>5445</x:v>
+      </x:c>
+      <x:c r="D257" s="33" t="n">
+        <x:v>5445</x:v>
+      </x:c>
+      <x:c r="E257" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F257" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G257" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H257" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I257" s="32" t="str">
+        <x:f>IF(AND(G257=H257,C257&gt;0,ABS(C257-'Prices'!H257)&lt;=MAX(0.01,'Prices'!H257*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J257" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K257" s="16" t="str"/>
+      <x:c r="L257" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M257" s="16" t="str"/>
+    </x:row>
+    <x:row r="258" ht="50" customHeight="1">
+      <x:c r="A258" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B258" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C258" s="17" t="n">
+        <x:v>104.7</x:v>
+      </x:c>
+      <x:c r="D258" s="17" t="n">
+        <x:v>104.7</x:v>
+      </x:c>
+      <x:c r="E258" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F258" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G258" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H258" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I258" s="31" t="str">
+        <x:f>IF(AND(G258=H258,C258&gt;0,ABS(C258-'Prices'!H258)&lt;=MAX(0.01,'Prices'!H258*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J258" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K258" s="14" t="str"/>
+      <x:c r="L258" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M258" s="14" t="str"/>
+    </x:row>
+    <x:row r="259" ht="50" customHeight="1">
+      <x:c r="A259" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B259" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C259" s="33" t="n">
+        <x:v>7757.17</x:v>
+      </x:c>
+      <x:c r="D259" s="33" t="n">
+        <x:v>7757.17</x:v>
+      </x:c>
+      <x:c r="E259" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F259" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G259" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H259" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I259" s="32" t="str">
+        <x:f>IF(AND(G259=H259,C259&gt;0,ABS(C259-'Prices'!H259)&lt;=MAX(0.01,'Prices'!H259*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J259" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K259" s="16" t="str"/>
+      <x:c r="L259" s="39" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M259" s="16" t="str"/>
+    </x:row>
+    <x:row r="260" ht="50" customHeight="1">
+      <x:c r="A260" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B260" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C260" s="17" t="n">
+        <x:v>26702.8574</x:v>
+      </x:c>
+      <x:c r="D260" s="17" t="n">
+        <x:v>26702.8574</x:v>
+      </x:c>
+      <x:c r="E260" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F260" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G260" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H260" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I260" s="31" t="str">
+        <x:f>IF(AND(G260=H260,C260&gt;0,ABS(C260-'Prices'!H260)&lt;=MAX(0.01,'Prices'!H260*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J260" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-22T11-36-22-004Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K260" s="14" t="str"/>
+      <x:c r="L260" s="38" t="n">
+        <x:v>46317.48358800926</x:v>
+      </x:c>
+      <x:c r="M260" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -26185,7 +27989,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8960b11df424cf8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R667b5e536e664b29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33176,6 +34980,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="244" ht="27" customHeight="1">
+      <x:c r="A244" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B244" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C244" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D244" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E244" s="19" t="n">
+        <x:f>'Source Audit'!E244</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F244" s="40" t="n">
+        <x:f>'Source Audit'!F244</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G244" s="11" t="str">
+        <x:f>IF(AND(E244=0,F244=1,'Source Audit'!I244&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H244" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="27" customHeight="1">
+      <x:c r="A245" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C245" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D245" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E245" s="18" t="n">
+        <x:f>'Source Audit'!E245</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F245" s="41" t="n">
+        <x:f>'Source Audit'!F245</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G245" s="12" t="str">
+        <x:f>IF(AND(E245=0,F245=1,'Source Audit'!I245&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H245" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="27" customHeight="1">
+      <x:c r="A246" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B246" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C246" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D246" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E246" s="19" t="n">
+        <x:f>'Source Audit'!E246</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F246" s="40" t="n">
+        <x:f>'Source Audit'!F246</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G246" s="11" t="str">
+        <x:f>IF(AND(E246=0,F246=1,'Source Audit'!I246&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H246" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="27" customHeight="1">
+      <x:c r="A247" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C247" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D247" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E247" s="18" t="n">
+        <x:f>'Source Audit'!E247</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F247" s="41" t="n">
+        <x:f>'Source Audit'!F247</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G247" s="12" t="str">
+        <x:f>IF(AND(E247=0,F247=1,'Source Audit'!I247&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H247" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="27" customHeight="1">
+      <x:c r="A248" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B248" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C248" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D248" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E248" s="19" t="n">
+        <x:f>'Source Audit'!E248</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F248" s="40" t="n">
+        <x:f>'Source Audit'!F248</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G248" s="11" t="str">
+        <x:f>IF(AND(E248=0,F248=1,'Source Audit'!I248&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H248" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="27" customHeight="1">
+      <x:c r="A249" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B249" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C249" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D249" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E249" s="18" t="n">
+        <x:f>'Source Audit'!E249</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F249" s="41" t="n">
+        <x:f>'Source Audit'!F249</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G249" s="12" t="str">
+        <x:f>IF(AND(E249=0,F249=1,'Source Audit'!I249&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H249" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="27" customHeight="1">
+      <x:c r="A250" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B250" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C250" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D250" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E250" s="19" t="n">
+        <x:f>'Source Audit'!E250</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F250" s="40" t="n">
+        <x:f>'Source Audit'!F250</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G250" s="11" t="str">
+        <x:f>IF(AND(E250=0,F250=1,'Source Audit'!I250&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H250" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="27" customHeight="1">
+      <x:c r="A251" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B251" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C251" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D251" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E251" s="18" t="n">
+        <x:f>'Source Audit'!E251</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F251" s="41" t="n">
+        <x:f>'Source Audit'!F251</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G251" s="12" t="str">
+        <x:f>IF(AND(E251=0,F251=1,'Source Audit'!I251&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H251" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="44" customHeight="1">
+      <x:c r="A252" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B252" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C252" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D252" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E252" s="19" t="n">
+        <x:f>'Source Audit'!E252</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F252" s="40" t="n">
+        <x:f>'Source Audit'!F252</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G252" s="11" t="str">
+        <x:f>IF(AND(E252=0,F252=1,'Source Audit'!I252&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H252" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="27" customHeight="1">
+      <x:c r="A253" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B253" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C253" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D253" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E253" s="18" t="n">
+        <x:f>'Source Audit'!E253</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F253" s="41" t="n">
+        <x:f>'Source Audit'!F253</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G253" s="12" t="str">
+        <x:f>IF(AND(E253=0,F253=1,'Source Audit'!I253&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H253" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="27" customHeight="1">
+      <x:c r="A254" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B254" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C254" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D254" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E254" s="19" t="n">
+        <x:f>'Source Audit'!E254</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F254" s="40" t="n">
+        <x:f>'Source Audit'!F254</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G254" s="11" t="str">
+        <x:f>IF(AND(E254=0,F254=1,'Source Audit'!I254&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H254" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="27" customHeight="1">
+      <x:c r="A255" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B255" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C255" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D255" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E255" s="18" t="n">
+        <x:f>'Source Audit'!E255</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F255" s="41" t="n">
+        <x:f>'Source Audit'!F255</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G255" s="12" t="str">
+        <x:f>IF(AND(E255=0,F255=1,'Source Audit'!I255&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H255" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="27" customHeight="1">
+      <x:c r="A256" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B256" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C256" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D256" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E256" s="19" t="n">
+        <x:f>'Source Audit'!E256</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F256" s="40" t="n">
+        <x:f>'Source Audit'!F256</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G256" s="11" t="str">
+        <x:f>IF(AND(E256=0,F256=1,'Source Audit'!I256&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H256" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="27" customHeight="1">
+      <x:c r="A257" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B257" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C257" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D257" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E257" s="18" t="n">
+        <x:f>'Source Audit'!E257</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F257" s="41" t="n">
+        <x:f>'Source Audit'!F257</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G257" s="12" t="str">
+        <x:f>IF(AND(E257=0,F257=1,'Source Audit'!I257&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H257" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="27" customHeight="1">
+      <x:c r="A258" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B258" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C258" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D258" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E258" s="19" t="n">
+        <x:f>'Source Audit'!E258</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F258" s="40" t="n">
+        <x:f>'Source Audit'!F258</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G258" s="11" t="str">
+        <x:f>IF(AND(E258=0,F258=1,'Source Audit'!I258&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H258" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="27" customHeight="1">
+      <x:c r="A259" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B259" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C259" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D259" s="9" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E259" s="18" t="n">
+        <x:f>'Source Audit'!E259</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F259" s="41" t="n">
+        <x:f>'Source Audit'!F259</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G259" s="12" t="str">
+        <x:f>IF(AND(E259=0,F259=1,'Source Audit'!I259&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H259" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="27" customHeight="1">
+      <x:c r="A260" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="B260" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C260" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D260" s="8" t="n">
+        <x:v>46316</x:v>
+      </x:c>
+      <x:c r="E260" s="19" t="n">
+        <x:f>'Source Audit'!E260</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F260" s="40" t="n">
+        <x:f>'Source Audit'!F260</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G260" s="11" t="str">
+        <x:f>IF(AND(E260=0,F260=1,'Source Audit'!I260&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H260" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -33183,7 +35480,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R350ef78d88cd4b87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d5f6a12cce4bc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 22, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 240 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings, documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R455cdb640c2b4abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R3f4dc14b4e65461b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Red6d069b2aff49be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Rc5324143139c4131"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rbb7e8400c1e34669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf0a6e9c376444121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R7fe7f3ed3dcf4d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R0e52e26b416045e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R39f702099641419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Ra014eb96ff0049ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H230" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H245" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1866,6 +1866,85 @@
         <x:v>-6.723913576428043</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="40" customHeight="1">
+      <x:c r="A21" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B21" s="18" t="n">
+        <x:f>B20*(1+SUM('Returns and Contributions'!F231:F245))</x:f>
+        <x:v>891.5035175925743</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="n">
+        <x:f>B21/B20-1</x:f>
+        <x:v>-0.03775349996291344</x:v>
+      </x:c>
+      <x:c r="D21" s="21" t="n">
+        <x:f>B21/$B$6-1</x:f>
+        <x:v>-0.10849648240742571</x:v>
+      </x:c>
+      <x:c r="E21" s="18" t="n">
+        <x:f>1000*'Prices'!H276/'Prices'!I276</x:f>
+        <x:v>999.606075823882</x:v>
+      </x:c>
+      <x:c r="F21" s="21" t="n">
+        <x:f>E21/E20-1</x:f>
+        <x:v>-0.012084303940741337</x:v>
+      </x:c>
+      <x:c r="G21" s="21" t="n">
+        <x:f>E21/1000-1</x:f>
+        <x:v>-0.0003939241761180545</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="n">
+        <x:f>1000*'Prices'!H277/'Prices'!I277</x:f>
+        <x:v>967.8941172816172</x:v>
+      </x:c>
+      <x:c r="I21" s="21" t="n">
+        <x:f>H21/H20-1</x:f>
+        <x:v>-0.025989653077351904</x:v>
+      </x:c>
+      <x:c r="J21" s="21" t="n">
+        <x:f>H21/1000-1</x:f>
+        <x:v>-0.03210588271838277</x:v>
+      </x:c>
+      <x:c r="K21" s="25" t="n">
+        <x:f>(C21-F21)*100</x:f>
+        <x:v>-2.5669196022172103</x:v>
+      </x:c>
+      <x:c r="L21" s="25" t="n">
+        <x:f>(C21-I21)*100</x:f>
+        <x:v>-1.1763846885561535</x:v>
+      </x:c>
+      <x:c r="M21" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G231:G245)</x:f>
+        <x:v>0.9999999999999996</x:v>
+      </x:c>
+      <x:c r="N21" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F231:F245)-C21</x:f>
+        <x:v>-3.469446951953614e-17</x:v>
+      </x:c>
+      <x:c r="O21" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P21" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I261:I277,"Mismatch")=0,IF(COUNTIF('Source Audit'!I261:I277,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q21" s="30" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="R21" s="27" t="n">
+        <x:f>B21-1000*('Prices'!H261/'Prices'!H6+'Prices'!H262/'Prices'!H7+'Prices'!H263/'Prices'!H8+'Prices'!H264/'Prices'!H9+'Prices'!H265/'Prices'!H10+'Prices'!H266/'Prices'!H11+'Prices'!H267/'Prices'!H12+'Prices'!H268/'Prices'!H13+'Prices'!H269/'Prices'!H14+'Prices'!H270/'Prices'!H15+'Prices'!H271/'Prices'!H16+'Prices'!H272/'Prices'!H17+'Prices'!H273/'Prices'!H18+'Prices'!H274/'Prices'!H19+'Prices'!H275/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S21" s="25" t="n">
+        <x:f>(D21-G21)*100</x:f>
+        <x:v>-10.810255823130765</x:v>
+      </x:c>
+      <x:c r="T21" s="25" t="n">
+        <x:f>(D21-J21)*100</x:f>
+        <x:v>-7.639059968904293</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1873,7 +1952,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7472d9ca056a4bf2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78569524b4a745d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11115,6 +11194,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="261" ht="27" customHeight="1">
+      <x:c r="A261" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B261" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C261" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D261" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E261" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F261" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G261" s="33" t="n">
+        <x:f>H244</x:f>
+        <x:v>5823</x:v>
+      </x:c>
+      <x:c r="H261" s="35" t="n">
+        <x:v>5624</x:v>
+      </x:c>
+      <x:c r="I261" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J261" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K261" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="27" customHeight="1">
+      <x:c r="A262" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B262" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C262" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D262" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E262" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F262" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G262" s="17" t="n">
+        <x:f>H245</x:f>
+        <x:v>4204</x:v>
+      </x:c>
+      <x:c r="H262" s="34" t="n">
+        <x:v>4033</x:v>
+      </x:c>
+      <x:c r="I262" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J262" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K262" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="27" customHeight="1">
+      <x:c r="A263" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B263" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C263" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D263" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E263" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F263" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G263" s="33" t="n">
+        <x:f>H246</x:f>
+        <x:v>26.08</x:v>
+      </x:c>
+      <x:c r="H263" s="35" t="n">
+        <x:v>26.53</x:v>
+      </x:c>
+      <x:c r="I263" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J263" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K263" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="27" customHeight="1">
+      <x:c r="A264" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B264" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C264" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D264" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E264" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F264" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G264" s="17" t="n">
+        <x:f>H247</x:f>
+        <x:v>345.49</x:v>
+      </x:c>
+      <x:c r="H264" s="34" t="n">
+        <x:v>308.75</x:v>
+      </x:c>
+      <x:c r="I264" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J264" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K264" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="27" customHeight="1">
+      <x:c r="A265" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B265" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C265" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D265" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E265" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F265" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G265" s="33" t="n">
+        <x:f>H248</x:f>
+        <x:v>4357</x:v>
+      </x:c>
+      <x:c r="H265" s="35" t="n">
+        <x:v>4166</x:v>
+      </x:c>
+      <x:c r="I265" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J265" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K265" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="27" customHeight="1">
+      <x:c r="A266" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B266" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C266" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D266" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E266" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F266" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G266" s="17" t="n">
+        <x:f>H249</x:f>
+        <x:v>49.9</x:v>
+      </x:c>
+      <x:c r="H266" s="34" t="n">
+        <x:v>49.91</x:v>
+      </x:c>
+      <x:c r="I266" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J266" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K266" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="27" customHeight="1">
+      <x:c r="A267" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B267" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C267" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D267" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E267" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F267" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G267" s="33" t="n">
+        <x:f>H250</x:f>
+        <x:v>80860</x:v>
+      </x:c>
+      <x:c r="H267" s="35" t="n">
+        <x:v>80360</x:v>
+      </x:c>
+      <x:c r="I267" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J267" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K267" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="27" customHeight="1">
+      <x:c r="A268" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B268" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C268" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D268" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E268" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F268" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G268" s="17" t="n">
+        <x:f>H251</x:f>
+        <x:v>58.05</x:v>
+      </x:c>
+      <x:c r="H268" s="34" t="n">
+        <x:v>54.6</x:v>
+      </x:c>
+      <x:c r="I268" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J268" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K268" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="27" customHeight="1">
+      <x:c r="A269" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B269" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C269" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D269" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E269" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F269" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G269" s="33" t="n">
+        <x:f>H252</x:f>
+        <x:v>30.31</x:v>
+      </x:c>
+      <x:c r="H269" s="35" t="n">
+        <x:v>27.98</x:v>
+      </x:c>
+      <x:c r="I269" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J269" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K269" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="27" customHeight="1">
+      <x:c r="A270" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B270" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C270" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D270" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E270" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F270" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G270" s="17" t="n">
+        <x:f>H253</x:f>
+        <x:v>13.19</x:v>
+      </x:c>
+      <x:c r="H270" s="34" t="n">
+        <x:v>12.14</x:v>
+      </x:c>
+      <x:c r="I270" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J270" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K270" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="27" customHeight="1">
+      <x:c r="A271" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B271" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C271" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D271" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E271" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F271" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G271" s="33" t="n">
+        <x:f>H254</x:f>
+        <x:v>438.51</x:v>
+      </x:c>
+      <x:c r="H271" s="35" t="n">
+        <x:v>423.87</x:v>
+      </x:c>
+      <x:c r="I271" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J271" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K271" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="27" customHeight="1">
+      <x:c r="A272" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B272" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C272" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D272" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E272" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F272" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G272" s="17" t="n">
+        <x:f>H255</x:f>
+        <x:v>266.75</x:v>
+      </x:c>
+      <x:c r="H272" s="34" t="n">
+        <x:v>255.7</x:v>
+      </x:c>
+      <x:c r="I272" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J272" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K272" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="27" customHeight="1">
+      <x:c r="A273" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B273" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C273" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D273" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E273" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F273" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G273" s="33" t="n">
+        <x:f>H256</x:f>
+        <x:v>242.36</x:v>
+      </x:c>
+      <x:c r="H273" s="35" t="n">
+        <x:v>237.79</x:v>
+      </x:c>
+      <x:c r="I273" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J273" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K273" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="27" customHeight="1">
+      <x:c r="A274" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B274" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C274" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D274" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E274" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F274" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G274" s="17" t="n">
+        <x:f>H257</x:f>
+        <x:v>5445</x:v>
+      </x:c>
+      <x:c r="H274" s="34" t="n">
+        <x:v>5202</x:v>
+      </x:c>
+      <x:c r="I274" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J274" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K274" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="27" customHeight="1">
+      <x:c r="A275" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B275" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C275" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D275" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E275" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F275" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G275" s="33" t="n">
+        <x:f>H258</x:f>
+        <x:v>104.7</x:v>
+      </x:c>
+      <x:c r="H275" s="35" t="n">
+        <x:v>102.05</x:v>
+      </x:c>
+      <x:c r="I275" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J275" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K275" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="27" customHeight="1">
+      <x:c r="A276" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B276" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C276" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D276" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E276" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F276" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G276" s="17" t="n">
+        <x:f>H259</x:f>
+        <x:v>7757.17</x:v>
+      </x:c>
+      <x:c r="H276" s="34" t="n">
+        <x:v>7663.43</x:v>
+      </x:c>
+      <x:c r="I276" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J276" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K276" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="27" customHeight="1">
+      <x:c r="A277" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B277" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C277" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D277" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E277" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F277" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G277" s="33" t="n">
+        <x:f>H260</x:f>
+        <x:v>26702.8574</x:v>
+      </x:c>
+      <x:c r="H277" s="35" t="n">
+        <x:v>26008.8594</x:v>
+      </x:c>
+      <x:c r="I277" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J277" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="K277" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -11122,7 +11813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9694391018c4653"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R152397450ee9406f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18096,6 +18787,471 @@
         <x:v>0.05736214906079584</x:v>
       </x:c>
     </x:row>
+    <x:row r="231" ht="27" customHeight="1">
+      <x:c r="A231" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B231" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C231" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D231" s="21" t="n">
+        <x:f>G216</x:f>
+        <x:v>0.06838658699824773</x:v>
+      </x:c>
+      <x:c r="E231" s="23" t="n">
+        <x:f>'Prices'!H261/'Prices'!G261-1</x:f>
+        <x:v>-0.034174823973896595</x:v>
+      </x:c>
+      <x:c r="F231" s="21" t="n">
+        <x:f>D231*E231</x:f>
+        <x:v>-0.002337099572840682</x:v>
+      </x:c>
+      <x:c r="G231" s="21" t="n">
+        <x:f>D231*(1+E231)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.06864092249009104</x:v>
+      </x:c>
+      <x:c r="H231" s="23" t="n">
+        <x:f>'Prices'!H261/'Prices'!I261-1</x:f>
+        <x:v>-0.0820956422392688</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="27" customHeight="1">
+      <x:c r="A232" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B232" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C232" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D232" s="20" t="n">
+        <x:f>G217</x:f>
+        <x:v>0.06329912355675599</x:v>
+      </x:c>
+      <x:c r="E232" s="22" t="n">
+        <x:f>'Prices'!H262/'Prices'!G262-1</x:f>
+        <x:v>-0.04067554709800192</x:v>
+      </x:c>
+      <x:c r="F232" s="20" t="n">
+        <x:f>D232*E232</x:f>
+        <x:v>-0.002574726481495071</x:v>
+      </x:c>
+      <x:c r="G232" s="20" t="n">
+        <x:f>D232*(1+E232)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.06310690355633457</x:v>
+      </x:c>
+      <x:c r="H232" s="22" t="n">
+        <x:f>'Prices'!H262/'Prices'!I262-1</x:f>
+        <x:v>-0.15609960242728604</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="27" customHeight="1">
+      <x:c r="A233" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B233" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C233" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D233" s="21" t="n">
+        <x:f>G218</x:f>
+        <x:v>0.06650014581755159</x:v>
+      </x:c>
+      <x:c r="E233" s="23" t="n">
+        <x:f>'Prices'!H263/'Prices'!G263-1</x:f>
+        <x:v>0.01725460122699407</x:v>
+      </x:c>
+      <x:c r="F233" s="21" t="n">
+        <x:f>D233*E233</x:f>
+        <x:v>0.0011474334976188103</x:v>
+      </x:c>
+      <x:c r="G233" s="21" t="n">
+        <x:f>D233*(1+E233)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07030171511412424</x:v>
+      </x:c>
+      <x:c r="H233" s="23" t="n">
+        <x:f>'Prices'!H263/'Prices'!I263-1</x:f>
+        <x:v>-0.059886605244507396</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="27" customHeight="1">
+      <x:c r="A234" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B234" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C234" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D234" s="20" t="n">
+        <x:f>G219</x:f>
+        <x:v>0.059790675690373725</x:v>
+      </x:c>
+      <x:c r="E234" s="22" t="n">
+        <x:f>'Prices'!H264/'Prices'!G264-1</x:f>
+        <x:v>-0.1063417175605662</x:v>
+      </x:c>
+      <x:c r="F234" s="20" t="n">
+        <x:f>D234*E234</x:f>
+        <x:v>-0.006358243147021134</x:v>
+      </x:c>
+      <x:c r="G234" s="20" t="n">
+        <x:f>D234*(1+E234)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.055528840625861685</x:v>
+      </x:c>
+      <x:c r="H234" s="22" t="n">
+        <x:f>'Prices'!H264/'Prices'!I264-1</x:f>
+        <x:v>-0.2574376488131028</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="27" customHeight="1">
+      <x:c r="A235" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B235" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C235" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D235" s="21" t="n">
+        <x:f>G220</x:f>
+        <x:v>0.0630182726433547</x:v>
+      </x:c>
+      <x:c r="E235" s="23" t="n">
+        <x:f>'Prices'!H265/'Prices'!G265-1</x:f>
+        <x:v>-0.0438375028689465</x:v>
+      </x:c>
+      <x:c r="F235" s="21" t="n">
+        <x:f>D235*E235</x:f>
+        <x:v>-0.0027625637077991145</x:v>
+      </x:c>
+      <x:c r="G235" s="21" t="n">
+        <x:f>D235*(1+E235)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.06261982655508047</x:v>
+      </x:c>
+      <x:c r="H235" s="23" t="n">
+        <x:f>'Prices'!H265/'Prices'!I265-1</x:f>
+        <x:v>-0.1626130653266331</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="27" customHeight="1">
+      <x:c r="A236" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B236" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C236" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D236" s="20" t="n">
+        <x:f>G221</x:f>
+        <x:v>0.06918392668849685</x:v>
+      </x:c>
+      <x:c r="E236" s="22" t="n">
+        <x:f>'Prices'!H266/'Prices'!G266-1</x:f>
+        <x:v>0.00020040080160321772</x:v>
+      </x:c>
+      <x:c r="F236" s="20" t="n">
+        <x:f>D236*E236</x:f>
+        <x:v>0.000013864514366433017</x:v>
+      </x:c>
+      <x:c r="G236" s="20" t="n">
+        <x:f>D236*(1+E236)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07191274917622073</x:v>
+      </x:c>
+      <x:c r="H236" s="22" t="n">
+        <x:f>'Prices'!H266/'Prices'!I266-1</x:f>
+        <x:v>-0.03834296724470143</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="27" customHeight="1">
+      <x:c r="A237" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B237" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C237" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D237" s="21" t="n">
+        <x:f>G222</x:f>
+        <x:v>0.07165553249218956</x:v>
+      </x:c>
+      <x:c r="E237" s="23" t="n">
+        <x:f>'Prices'!H267/'Prices'!G267-1</x:f>
+        <x:v>-0.006183527083848617</x:v>
+      </x:c>
+      <x:c r="F237" s="21" t="n">
+        <x:f>D237*E237</x:f>
+        <x:v>-0.00044308392587304873</x:v>
+      </x:c>
+      <x:c r="G237" s="21" t="n">
+        <x:f>D237*(1+E237)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07400645111577114</x:v>
+      </x:c>
+      <x:c r="H237" s="23" t="n">
+        <x:f>'Prices'!H267/'Prices'!I267-1</x:f>
+        <x:v>-0.010344827586206917</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="27" customHeight="1">
+      <x:c r="A238" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B238" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C238" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D238" s="20" t="n">
+        <x:f>G223</x:f>
+        <x:v>0.06713426480330303</x:v>
+      </x:c>
+      <x:c r="E238" s="22" t="n">
+        <x:f>'Prices'!H268/'Prices'!G268-1</x:f>
+        <x:v>-0.05943152454780354</x:v>
+      </x:c>
+      <x:c r="F238" s="20" t="n">
+        <x:f>D238*E238</x:f>
+        <x:v>-0.003989891706656247</x:v>
+      </x:c>
+      <x:c r="G238" s="20" t="n">
+        <x:f>D238*(1+E238)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.06562182672965099</x:v>
+      </x:c>
+      <x:c r="H238" s="22" t="n">
+        <x:f>'Prices'!H268/'Prices'!I268-1</x:f>
+        <x:v>-0.12246865959498554</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="27" customHeight="1">
+      <x:c r="A239" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B239" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C239" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D239" s="21" t="n">
+        <x:f>G224</x:f>
+        <x:v>0.05336460738971496</x:v>
+      </x:c>
+      <x:c r="E239" s="23" t="n">
+        <x:f>'Prices'!H269/'Prices'!G269-1</x:f>
+        <x:v>-0.0768723193665456</x:v>
+      </x:c>
+      <x:c r="F239" s="21" t="n">
+        <x:f>D239*E239</x:f>
+        <x:v>-0.0041022611421324875</x:v>
+      </x:c>
+      <x:c r="G239" s="21" t="n">
+        <x:f>D239*(1+E239)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.051195142040718074</x:v>
+      </x:c>
+      <x:c r="H239" s="23" t="n">
+        <x:f>'Prices'!H269/'Prices'!I269-1</x:f>
+        <x:v>-0.3153902618057254</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="27" customHeight="1">
+      <x:c r="A240" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B240" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C240" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D240" s="20" t="n">
+        <x:f>G225</x:f>
+        <x:v>0.059580074194596454</x:v>
+      </x:c>
+      <x:c r="E240" s="22" t="n">
+        <x:f>'Prices'!H270/'Prices'!G270-1</x:f>
+        <x:v>-0.07960576194086422</x:v>
+      </x:c>
+      <x:c r="F240" s="20" t="n">
+        <x:f>D240*E240</x:f>
+        <x:v>-0.004742917202754072</x:v>
+      </x:c>
+      <x:c r="G240" s="20" t="n">
+        <x:f>D240*(1+E240)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.05698867908558656</x:v>
+      </x:c>
+      <x:c r="H240" s="22" t="n">
+        <x:f>'Prices'!H270/'Prices'!I270-1</x:f>
+        <x:v>-0.23791588198367852</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="27" customHeight="1">
+      <x:c r="A241" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B241" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C241" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D241" s="21" t="n">
+        <x:f>G226</x:f>
+        <x:v>0.07131605679994926</x:v>
+      </x:c>
+      <x:c r="E241" s="23" t="n">
+        <x:f>'Prices'!H271/'Prices'!G271-1</x:f>
+        <x:v>-0.03338578367654099</x:v>
+      </x:c>
+      <x:c r="F241" s="21" t="n">
+        <x:f>D241*E241</x:f>
+        <x:v>-0.0023809424449870165</x:v>
+      </x:c>
+      <x:c r="G241" s="21" t="n">
+        <x:f>D241*(1+E241)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.0716397662681084</x:v>
+      </x:c>
+      <x:c r="H241" s="23" t="n">
+        <x:f>'Prices'!H271/'Prices'!I271-1</x:f>
+        <x:v>-0.041993445587071965</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="27" customHeight="1">
+      <x:c r="A242" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B242" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C242" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D242" s="20" t="n">
+        <x:f>G227</x:f>
+        <x:v>0.07059391057596795</x:v>
+      </x:c>
+      <x:c r="E242" s="22" t="n">
+        <x:f>'Prices'!H272/'Prices'!G272-1</x:f>
+        <x:v>-0.04142455482661678</x:v>
+      </x:c>
+      <x:c r="F242" s="20" t="n">
+        <x:f>D242*E242</x:f>
+        <x:v>-0.002924321319079466</x:v>
+      </x:c>
+      <x:c r="G242" s="20" t="n">
+        <x:f>D242*(1+E242)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07032458861038246</x:v>
+      </x:c>
+      <x:c r="H242" s="22" t="n">
+        <x:f>'Prices'!H272/'Prices'!I272-1</x:f>
+        <x:v>-0.05958072820890026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="27" customHeight="1">
+      <x:c r="A243" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B243" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C243" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D243" s="21" t="n">
+        <x:f>G228</x:f>
+        <x:v>0.07291047791543871</x:v>
+      </x:c>
+      <x:c r="E243" s="23" t="n">
+        <x:f>'Prices'!H273/'Prices'!G273-1</x:f>
+        <x:v>-0.018856246905429974</x:v>
+      </x:c>
+      <x:c r="F243" s="21" t="n">
+        <x:f>D243*E243</x:f>
+        <x:v>-0.0013748179735664117</x:v>
+      </x:c>
+      <x:c r="G243" s="21" t="n">
+        <x:f>D243*(1+E243)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07434234360854022</x:v>
+      </x:c>
+      <x:c r="H243" s="23" t="n">
+        <x:f>'Prices'!H273/'Prices'!I273-1</x:f>
+        <x:v>-0.005853087503658205</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="27" customHeight="1">
+      <x:c r="A244" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B244" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C244" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D244" s="20" t="n">
+        <x:f>G229</x:f>
+        <x:v>0.06718191648901053</x:v>
+      </x:c>
+      <x:c r="E244" s="22" t="n">
+        <x:f>'Prices'!H274/'Prices'!G274-1</x:f>
+        <x:v>-0.044628099173553704</x:v>
+      </x:c>
+      <x:c r="F244" s="20" t="n">
+        <x:f>D244*E244</x:f>
+        <x:v>-0.0029982012317409648</x:v>
+      </x:c>
+      <x:c r="G244" s="20" t="n">
+        <x:f>D244*(1+E244)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.06670194721913338</x:v>
+      </x:c>
+      <x:c r="H244" s="22" t="n">
+        <x:f>'Prices'!H274/'Prices'!I274-1</x:f>
+        <x:v>-0.10802469135802473</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="27" customHeight="1">
+      <x:c r="A245" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B245" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C245" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D245" s="21" t="n">
+        <x:f>G230</x:f>
+        <x:v>0.07608442794504852</x:v>
+      </x:c>
+      <x:c r="E245" s="23" t="n">
+        <x:f>'Prices'!H275/'Prices'!G275-1</x:f>
+        <x:v>-0.02531041069723028</x:v>
+      </x:c>
+      <x:c r="F245" s="21" t="n">
+        <x:f>D245*E245</x:f>
+        <x:v>-0.0019257281189530024</x:v>
+      </x:c>
+      <x:c r="G245" s="21" t="n">
+        <x:f>D245*(1+E245)/(1+SUM($F$231:$F$245))</x:f>
+        <x:v>0.07706829780439557</x:v>
+      </x:c>
+      <x:c r="H245" s="23" t="n">
+        <x:f>'Prices'!H275/'Prices'!I275-1</x:f>
+        <x:v>0.030599878812361148</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -18103,7 +19259,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f5c3cbc5f21436d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra63f55e084b34900"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27982,6 +29138,654 @@
       </x:c>
       <x:c r="M260" s="14" t="str"/>
     </x:row>
+    <x:row r="261" ht="50" customHeight="1">
+      <x:c r="A261" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B261" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C261" s="33" t="n">
+        <x:v>5624</x:v>
+      </x:c>
+      <x:c r="D261" s="33" t="n">
+        <x:v>5624</x:v>
+      </x:c>
+      <x:c r="E261" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F261" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G261" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H261" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I261" s="32" t="str">
+        <x:f>IF(AND(G261=H261,C261&gt;0,ABS(C261-'Prices'!H261)&lt;=MAX(0.01,'Prices'!H261*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J261" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K261" s="16" t="str"/>
+      <x:c r="L261" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M261" s="16" t="str"/>
+    </x:row>
+    <x:row r="262" ht="50" customHeight="1">
+      <x:c r="A262" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B262" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C262" s="17" t="n">
+        <x:v>4033</x:v>
+      </x:c>
+      <x:c r="D262" s="17" t="n">
+        <x:v>4033</x:v>
+      </x:c>
+      <x:c r="E262" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F262" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G262" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H262" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I262" s="31" t="str">
+        <x:f>IF(AND(G262=H262,C262&gt;0,ABS(C262-'Prices'!H262)&lt;=MAX(0.01,'Prices'!H262*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J262" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K262" s="14" t="str"/>
+      <x:c r="L262" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M262" s="14" t="str"/>
+    </x:row>
+    <x:row r="263" ht="50" customHeight="1">
+      <x:c r="A263" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B263" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C263" s="33" t="n">
+        <x:v>26.53</x:v>
+      </x:c>
+      <x:c r="D263" s="33" t="n">
+        <x:v>26.53</x:v>
+      </x:c>
+      <x:c r="E263" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F263" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G263" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H263" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I263" s="32" t="str">
+        <x:f>IF(AND(G263=H263,C263&gt;0,ABS(C263-'Prices'!H263)&lt;=MAX(0.01,'Prices'!H263*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J263" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K263" s="16" t="str"/>
+      <x:c r="L263" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M263" s="16" t="str"/>
+    </x:row>
+    <x:row r="264" ht="50" customHeight="1">
+      <x:c r="A264" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B264" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C264" s="17" t="n">
+        <x:v>308.75</x:v>
+      </x:c>
+      <x:c r="D264" s="17" t="n">
+        <x:v>308.75</x:v>
+      </x:c>
+      <x:c r="E264" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F264" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G264" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H264" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I264" s="31" t="str">
+        <x:f>IF(AND(G264=H264,C264&gt;0,ABS(C264-'Prices'!H264)&lt;=MAX(0.01,'Prices'!H264*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J264" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K264" s="14" t="str"/>
+      <x:c r="L264" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M264" s="14" t="str"/>
+    </x:row>
+    <x:row r="265" ht="50" customHeight="1">
+      <x:c r="A265" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B265" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C265" s="33" t="n">
+        <x:v>4166</x:v>
+      </x:c>
+      <x:c r="D265" s="33" t="n">
+        <x:v>4166</x:v>
+      </x:c>
+      <x:c r="E265" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F265" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G265" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H265" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I265" s="32" t="str">
+        <x:f>IF(AND(G265=H265,C265&gt;0,ABS(C265-'Prices'!H265)&lt;=MAX(0.01,'Prices'!H265*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J265" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K265" s="16" t="str"/>
+      <x:c r="L265" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M265" s="16" t="str"/>
+    </x:row>
+    <x:row r="266" ht="50" customHeight="1">
+      <x:c r="A266" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B266" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C266" s="17" t="n">
+        <x:v>49.91</x:v>
+      </x:c>
+      <x:c r="D266" s="17" t="n">
+        <x:v>49.91</x:v>
+      </x:c>
+      <x:c r="E266" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F266" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G266" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H266" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I266" s="31" t="str">
+        <x:f>IF(AND(G266=H266,C266&gt;0,ABS(C266-'Prices'!H266)&lt;=MAX(0.01,'Prices'!H266*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J266" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K266" s="14" t="str"/>
+      <x:c r="L266" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M266" s="14" t="str"/>
+    </x:row>
+    <x:row r="267" ht="50" customHeight="1">
+      <x:c r="A267" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B267" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C267" s="33" t="n">
+        <x:v>80360</x:v>
+      </x:c>
+      <x:c r="D267" s="33" t="n">
+        <x:v>80360</x:v>
+      </x:c>
+      <x:c r="E267" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F267" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G267" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H267" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I267" s="32" t="str">
+        <x:f>IF(AND(G267=H267,C267&gt;0,ABS(C267-'Prices'!H267)&lt;=MAX(0.01,'Prices'!H267*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J267" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K267" s="16" t="str"/>
+      <x:c r="L267" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M267" s="16" t="str"/>
+    </x:row>
+    <x:row r="268" ht="50" customHeight="1">
+      <x:c r="A268" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B268" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C268" s="17" t="n">
+        <x:v>54.6</x:v>
+      </x:c>
+      <x:c r="D268" s="17" t="n">
+        <x:v>54.6</x:v>
+      </x:c>
+      <x:c r="E268" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F268" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G268" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H268" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I268" s="31" t="str">
+        <x:f>IF(AND(G268=H268,C268&gt;0,ABS(C268-'Prices'!H268)&lt;=MAX(0.01,'Prices'!H268*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J268" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K268" s="14" t="str"/>
+      <x:c r="L268" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M268" s="14" t="str"/>
+    </x:row>
+    <x:row r="269" ht="50" customHeight="1">
+      <x:c r="A269" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B269" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C269" s="33" t="n">
+        <x:v>27.98</x:v>
+      </x:c>
+      <x:c r="D269" s="33" t="n">
+        <x:v>27.98</x:v>
+      </x:c>
+      <x:c r="E269" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F269" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G269" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H269" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I269" s="32" t="str">
+        <x:f>IF(AND(OR(G269=H269,AND(B269="OUST",G269="XNAS",H269="XNYS",LEFT(M269,34)="ouster-marketstack-legacy-nyse-tag")),C269&gt;0,ABS(C269-'Prices'!H269)&lt;=MAX(0.01,'Prices'!H269*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J269" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K269" s="16" t="str"/>
+      <x:c r="L269" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M269" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="50" customHeight="1">
+      <x:c r="A270" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B270" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C270" s="17" t="n">
+        <x:v>12.14</x:v>
+      </x:c>
+      <x:c r="D270" s="17" t="n">
+        <x:v>12.14</x:v>
+      </x:c>
+      <x:c r="E270" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F270" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G270" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H270" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I270" s="31" t="str">
+        <x:f>IF(AND(G270=H270,C270&gt;0,ABS(C270-'Prices'!H270)&lt;=MAX(0.01,'Prices'!H270*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J270" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K270" s="14" t="str"/>
+      <x:c r="L270" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M270" s="14" t="str"/>
+    </x:row>
+    <x:row r="271" ht="50" customHeight="1">
+      <x:c r="A271" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B271" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C271" s="33" t="n">
+        <x:v>423.87</x:v>
+      </x:c>
+      <x:c r="D271" s="33" t="n">
+        <x:v>423.87</x:v>
+      </x:c>
+      <x:c r="E271" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F271" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G271" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H271" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I271" s="32" t="str">
+        <x:f>IF(AND(G271=H271,C271&gt;0,ABS(C271-'Prices'!H271)&lt;=MAX(0.01,'Prices'!H271*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J271" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K271" s="16" t="str"/>
+      <x:c r="L271" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M271" s="16" t="str"/>
+    </x:row>
+    <x:row r="272" ht="50" customHeight="1">
+      <x:c r="A272" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B272" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C272" s="17" t="n">
+        <x:v>255.7</x:v>
+      </x:c>
+      <x:c r="D272" s="17" t="n">
+        <x:v>255.7</x:v>
+      </x:c>
+      <x:c r="E272" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F272" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G272" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H272" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I272" s="31" t="str">
+        <x:f>IF(AND(G272=H272,C272&gt;0,ABS(C272-'Prices'!H272)&lt;=MAX(0.01,'Prices'!H272*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J272" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K272" s="14" t="str"/>
+      <x:c r="L272" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M272" s="14" t="str"/>
+    </x:row>
+    <x:row r="273" ht="50" customHeight="1">
+      <x:c r="A273" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B273" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C273" s="33" t="n">
+        <x:v>237.79</x:v>
+      </x:c>
+      <x:c r="D273" s="33" t="n">
+        <x:v>237.79</x:v>
+      </x:c>
+      <x:c r="E273" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F273" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G273" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H273" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I273" s="32" t="str">
+        <x:f>IF(AND(G273=H273,C273&gt;0,ABS(C273-'Prices'!H273)&lt;=MAX(0.01,'Prices'!H273*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J273" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K273" s="16" t="str"/>
+      <x:c r="L273" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M273" s="16" t="str"/>
+    </x:row>
+    <x:row r="274" ht="50" customHeight="1">
+      <x:c r="A274" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B274" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C274" s="17" t="n">
+        <x:v>5202</x:v>
+      </x:c>
+      <x:c r="D274" s="17" t="n">
+        <x:v>5202</x:v>
+      </x:c>
+      <x:c r="E274" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F274" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G274" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H274" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I274" s="31" t="str">
+        <x:f>IF(AND(G274=H274,C274&gt;0,ABS(C274-'Prices'!H274)&lt;=MAX(0.01,'Prices'!H274*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J274" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K274" s="14" t="str"/>
+      <x:c r="L274" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M274" s="14" t="str"/>
+    </x:row>
+    <x:row r="275" ht="50" customHeight="1">
+      <x:c r="A275" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B275" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C275" s="33" t="n">
+        <x:v>102.05</x:v>
+      </x:c>
+      <x:c r="D275" s="33" t="n">
+        <x:v>102.05</x:v>
+      </x:c>
+      <x:c r="E275" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F275" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G275" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H275" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I275" s="32" t="str">
+        <x:f>IF(AND(G275=H275,C275&gt;0,ABS(C275-'Prices'!H275)&lt;=MAX(0.01,'Prices'!H275*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J275" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K275" s="16" t="str"/>
+      <x:c r="L275" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M275" s="16" t="str"/>
+    </x:row>
+    <x:row r="276" ht="50" customHeight="1">
+      <x:c r="A276" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B276" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C276" s="17" t="n">
+        <x:v>7663.43</x:v>
+      </x:c>
+      <x:c r="D276" s="17" t="n">
+        <x:v>7663.43</x:v>
+      </x:c>
+      <x:c r="E276" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F276" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G276" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H276" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I276" s="31" t="str">
+        <x:f>IF(AND(G276=H276,C276&gt;0,ABS(C276-'Prices'!H276)&lt;=MAX(0.01,'Prices'!H276*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J276" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K276" s="14" t="str"/>
+      <x:c r="L276" s="38" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M276" s="14" t="str"/>
+    </x:row>
+    <x:row r="277" ht="50" customHeight="1">
+      <x:c r="A277" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B277" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C277" s="33" t="n">
+        <x:v>26008.8594</x:v>
+      </x:c>
+      <x:c r="D277" s="33" t="n">
+        <x:v>26008.8594</x:v>
+      </x:c>
+      <x:c r="E277" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F277" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G277" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H277" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I277" s="32" t="str">
+        <x:f>IF(AND(G277=H277,C277&gt;0,ABS(C277-'Prices'!H277)&lt;=MAX(0.01,'Prices'!H277*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J277" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-23T11-27-32-056Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K277" s="16" t="str"/>
+      <x:c r="L277" s="39" t="n">
+        <x:v>46318.47745435185</x:v>
+      </x:c>
+      <x:c r="M277" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -27989,7 +29793,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R667b5e536e664b29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af4806bb8ed4856"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35473,6 +37277,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="261" ht="27" customHeight="1">
+      <x:c r="A261" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B261" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C261" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D261" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E261" s="18" t="n">
+        <x:f>'Source Audit'!E261</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F261" s="41" t="n">
+        <x:f>'Source Audit'!F261</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G261" s="12" t="str">
+        <x:f>IF(AND(E261=0,F261=1,'Source Audit'!I261&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H261" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="27" customHeight="1">
+      <x:c r="A262" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B262" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C262" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D262" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E262" s="19" t="n">
+        <x:f>'Source Audit'!E262</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F262" s="40" t="n">
+        <x:f>'Source Audit'!F262</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G262" s="11" t="str">
+        <x:f>IF(AND(E262=0,F262=1,'Source Audit'!I262&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H262" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="27" customHeight="1">
+      <x:c r="A263" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B263" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C263" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D263" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E263" s="18" t="n">
+        <x:f>'Source Audit'!E263</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F263" s="41" t="n">
+        <x:f>'Source Audit'!F263</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G263" s="12" t="str">
+        <x:f>IF(AND(E263=0,F263=1,'Source Audit'!I263&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H263" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="27" customHeight="1">
+      <x:c r="A264" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B264" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C264" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D264" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E264" s="19" t="n">
+        <x:f>'Source Audit'!E264</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F264" s="40" t="n">
+        <x:f>'Source Audit'!F264</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G264" s="11" t="str">
+        <x:f>IF(AND(E264=0,F264=1,'Source Audit'!I264&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H264" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="27" customHeight="1">
+      <x:c r="A265" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B265" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C265" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D265" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E265" s="18" t="n">
+        <x:f>'Source Audit'!E265</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F265" s="41" t="n">
+        <x:f>'Source Audit'!F265</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G265" s="12" t="str">
+        <x:f>IF(AND(E265=0,F265=1,'Source Audit'!I265&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H265" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="27" customHeight="1">
+      <x:c r="A266" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B266" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C266" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D266" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E266" s="19" t="n">
+        <x:f>'Source Audit'!E266</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F266" s="40" t="n">
+        <x:f>'Source Audit'!F266</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G266" s="11" t="str">
+        <x:f>IF(AND(E266=0,F266=1,'Source Audit'!I266&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H266" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="27" customHeight="1">
+      <x:c r="A267" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B267" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C267" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D267" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E267" s="18" t="n">
+        <x:f>'Source Audit'!E267</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F267" s="41" t="n">
+        <x:f>'Source Audit'!F267</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G267" s="12" t="str">
+        <x:f>IF(AND(E267=0,F267=1,'Source Audit'!I267&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H267" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="27" customHeight="1">
+      <x:c r="A268" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B268" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C268" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D268" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E268" s="19" t="n">
+        <x:f>'Source Audit'!E268</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F268" s="40" t="n">
+        <x:f>'Source Audit'!F268</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G268" s="11" t="str">
+        <x:f>IF(AND(E268=0,F268=1,'Source Audit'!I268&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H268" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="44" customHeight="1">
+      <x:c r="A269" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B269" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C269" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D269" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E269" s="18" t="n">
+        <x:f>'Source Audit'!E269</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F269" s="41" t="n">
+        <x:f>'Source Audit'!F269</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G269" s="12" t="str">
+        <x:f>IF(AND(E269=0,F269=1,'Source Audit'!I269&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H269" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="27" customHeight="1">
+      <x:c r="A270" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B270" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C270" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D270" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E270" s="19" t="n">
+        <x:f>'Source Audit'!E270</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F270" s="40" t="n">
+        <x:f>'Source Audit'!F270</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G270" s="11" t="str">
+        <x:f>IF(AND(E270=0,F270=1,'Source Audit'!I270&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H270" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="27" customHeight="1">
+      <x:c r="A271" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B271" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C271" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D271" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E271" s="18" t="n">
+        <x:f>'Source Audit'!E271</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F271" s="41" t="n">
+        <x:f>'Source Audit'!F271</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G271" s="12" t="str">
+        <x:f>IF(AND(E271=0,F271=1,'Source Audit'!I271&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H271" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="27" customHeight="1">
+      <x:c r="A272" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B272" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C272" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D272" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E272" s="19" t="n">
+        <x:f>'Source Audit'!E272</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F272" s="40" t="n">
+        <x:f>'Source Audit'!F272</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G272" s="11" t="str">
+        <x:f>IF(AND(E272=0,F272=1,'Source Audit'!I272&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H272" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="27" customHeight="1">
+      <x:c r="A273" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B273" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C273" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D273" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E273" s="18" t="n">
+        <x:f>'Source Audit'!E273</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F273" s="41" t="n">
+        <x:f>'Source Audit'!F273</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G273" s="12" t="str">
+        <x:f>IF(AND(E273=0,F273=1,'Source Audit'!I273&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H273" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="27" customHeight="1">
+      <x:c r="A274" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B274" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C274" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D274" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E274" s="19" t="n">
+        <x:f>'Source Audit'!E274</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F274" s="40" t="n">
+        <x:f>'Source Audit'!F274</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G274" s="11" t="str">
+        <x:f>IF(AND(E274=0,F274=1,'Source Audit'!I274&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H274" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="27" customHeight="1">
+      <x:c r="A275" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B275" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C275" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D275" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E275" s="18" t="n">
+        <x:f>'Source Audit'!E275</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F275" s="41" t="n">
+        <x:f>'Source Audit'!F275</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G275" s="12" t="str">
+        <x:f>IF(AND(E275=0,F275=1,'Source Audit'!I275&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H275" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="27" customHeight="1">
+      <x:c r="A276" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B276" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C276" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D276" s="8" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E276" s="19" t="n">
+        <x:f>'Source Audit'!E276</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F276" s="40" t="n">
+        <x:f>'Source Audit'!F276</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G276" s="11" t="str">
+        <x:f>IF(AND(E276=0,F276=1,'Source Audit'!I276&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H276" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="27" customHeight="1">
+      <x:c r="A277" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="B277" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C277" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D277" s="9" t="n">
+        <x:v>46317</x:v>
+      </x:c>
+      <x:c r="E277" s="18" t="n">
+        <x:f>'Source Audit'!E277</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F277" s="41" t="n">
+        <x:f>'Source Audit'!F277</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G277" s="12" t="str">
+        <x:f>IF(AND(E277=0,F277=1,'Source Audit'!I277&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H277" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -35480,7 +37777,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3d5f6a12cce4bc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544a73e9ce3f47e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 23, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 257 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Shared-checkout build stopped on unrelated local
Insights taxonomy work; the exact main-based publication candidate
production build and article-preview checks passed. These results are
documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf0a6e9c376444121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R7fe7f3ed3dcf4d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R0e52e26b416045e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R39f702099641419e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Ra014eb96ff0049ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc7bed2ce2136496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rc24bab9c6b8f4740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R3955910673574566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Rd1b6391f339746e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rcd519c54707f461d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H245" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -1945,6 +1945,85 @@
         <x:v>-7.639059968904293</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="40" customHeight="1">
+      <x:c r="A22" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="n">
+        <x:f>B21*(1+SUM('Returns and Contributions'!F246:F260))</x:f>
+        <x:v>909.9828648645001</x:v>
+      </x:c>
+      <x:c r="C22" s="20" t="n">
+        <x:f>B22/B21-1</x:f>
+        <x:v>0.020728294288538063</x:v>
+      </x:c>
+      <x:c r="D22" s="20" t="n">
+        <x:f>B22/$B$6-1</x:f>
+        <x:v>-0.09001713513549991</x:v>
+      </x:c>
+      <x:c r="E22" s="19" t="n">
+        <x:f>1000*'Prices'!H293/'Prices'!I293</x:f>
+        <x:v>994.4211466845802</x:v>
+      </x:c>
+      <x:c r="F22" s="20" t="n">
+        <x:f>E22/E21-1</x:f>
+        <x:v>-0.005186972413136148</x:v>
+      </x:c>
+      <x:c r="G22" s="20" t="n">
+        <x:f>E22/1000-1</x:f>
+        <x:v>-0.005578853315419741</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="n">
+        <x:f>1000*'Prices'!H294/'Prices'!I294</x:f>
+        <x:v>965.902438015618</x:v>
+      </x:c>
+      <x:c r="I22" s="20" t="n">
+        <x:f>H22/H21-1</x:f>
+        <x:v>-0.002057744985156984</x:v>
+      </x:c>
+      <x:c r="J22" s="20" t="n">
+        <x:f>H22/1000-1</x:f>
+        <x:v>-0.03409756198438196</x:v>
+      </x:c>
+      <x:c r="K22" s="24" t="n">
+        <x:f>(C22-F22)*100</x:f>
+        <x:v>2.591526670167421</x:v>
+      </x:c>
+      <x:c r="L22" s="24" t="n">
+        <x:f>(C22-I22)*100</x:f>
+        <x:v>2.2786039273695047</x:v>
+      </x:c>
+      <x:c r="M22" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G246:G260)</x:f>
+        <x:v>0.9999999999999996</x:v>
+      </x:c>
+      <x:c r="N22" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F246:F260)-C22</x:f>
+        <x:v>3.469446951953614e-17</x:v>
+      </x:c>
+      <x:c r="O22" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P22" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I278:I294,"Mismatch")=0,IF(COUNTIF('Source Audit'!I278:I294,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q22" s="29" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="R22" s="28" t="n">
+        <x:f>B22-1000*('Prices'!H278/'Prices'!H6+'Prices'!H279/'Prices'!H7+'Prices'!H280/'Prices'!H8+'Prices'!H281/'Prices'!H9+'Prices'!H282/'Prices'!H10+'Prices'!H283/'Prices'!H11+'Prices'!H284/'Prices'!H12+'Prices'!H285/'Prices'!H13+'Prices'!H286/'Prices'!H14+'Prices'!H287/'Prices'!H15+'Prices'!H288/'Prices'!H16+'Prices'!H289/'Prices'!H17+'Prices'!H290/'Prices'!H18+'Prices'!H291/'Prices'!H19+'Prices'!H292/'Prices'!H20)/15</x:f>
+        <x:v>2.2737367544323206e-13</x:v>
+      </x:c>
+      <x:c r="S22" s="24" t="n">
+        <x:f>(D22-G22)*100</x:f>
+        <x:v>-8.443828182008017</x:v>
+      </x:c>
+      <x:c r="T22" s="24" t="n">
+        <x:f>(D22-J22)*100</x:f>
+        <x:v>-5.591957315111795</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -1952,7 +2031,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78569524b4a745d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9105081044214c7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11806,6 +11885,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="278" ht="27" customHeight="1">
+      <x:c r="A278" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B278" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C278" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D278" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E278" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F278" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G278" s="17" t="n">
+        <x:f>H261</x:f>
+        <x:v>5624</x:v>
+      </x:c>
+      <x:c r="H278" s="34" t="n">
+        <x:v>5587</x:v>
+      </x:c>
+      <x:c r="I278" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J278" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K278" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="27" customHeight="1">
+      <x:c r="A279" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B279" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C279" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D279" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E279" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F279" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G279" s="33" t="n">
+        <x:f>H262</x:f>
+        <x:v>4033</x:v>
+      </x:c>
+      <x:c r="H279" s="35" t="n">
+        <x:v>4022</x:v>
+      </x:c>
+      <x:c r="I279" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J279" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K279" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="27" customHeight="1">
+      <x:c r="A280" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B280" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C280" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D280" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E280" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F280" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G280" s="17" t="n">
+        <x:f>H263</x:f>
+        <x:v>26.53</x:v>
+      </x:c>
+      <x:c r="H280" s="34" t="n">
+        <x:v>29.18</x:v>
+      </x:c>
+      <x:c r="I280" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J280" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K280" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="27" customHeight="1">
+      <x:c r="A281" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B281" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C281" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D281" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E281" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F281" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G281" s="33" t="n">
+        <x:f>H264</x:f>
+        <x:v>308.75</x:v>
+      </x:c>
+      <x:c r="H281" s="35" t="n">
+        <x:v>308.85</x:v>
+      </x:c>
+      <x:c r="I281" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J281" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K281" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="27" customHeight="1">
+      <x:c r="A282" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B282" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C282" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D282" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E282" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F282" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G282" s="17" t="n">
+        <x:f>H265</x:f>
+        <x:v>4166</x:v>
+      </x:c>
+      <x:c r="H282" s="34" t="n">
+        <x:v>4118</x:v>
+      </x:c>
+      <x:c r="I282" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J282" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K282" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="27" customHeight="1">
+      <x:c r="A283" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B283" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C283" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D283" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E283" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F283" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G283" s="33" t="n">
+        <x:f>H266</x:f>
+        <x:v>49.91</x:v>
+      </x:c>
+      <x:c r="H283" s="35" t="n">
+        <x:v>53.5</x:v>
+      </x:c>
+      <x:c r="I283" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J283" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K283" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="27" customHeight="1">
+      <x:c r="A284" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B284" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C284" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D284" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E284" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F284" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G284" s="17" t="n">
+        <x:f>H267</x:f>
+        <x:v>80360</x:v>
+      </x:c>
+      <x:c r="H284" s="34" t="n">
+        <x:v>78380</x:v>
+      </x:c>
+      <x:c r="I284" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J284" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K284" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="27" customHeight="1">
+      <x:c r="A285" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B285" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C285" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D285" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E285" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F285" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G285" s="33" t="n">
+        <x:f>H268</x:f>
+        <x:v>54.6</x:v>
+      </x:c>
+      <x:c r="H285" s="35" t="n">
+        <x:v>55.55</x:v>
+      </x:c>
+      <x:c r="I285" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J285" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K285" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="27" customHeight="1">
+      <x:c r="A286" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B286" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C286" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D286" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E286" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F286" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G286" s="17" t="n">
+        <x:f>H269</x:f>
+        <x:v>27.98</x:v>
+      </x:c>
+      <x:c r="H286" s="34" t="n">
+        <x:v>29.69</x:v>
+      </x:c>
+      <x:c r="I286" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J286" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K286" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="27" customHeight="1">
+      <x:c r="A287" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B287" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C287" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D287" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E287" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F287" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G287" s="33" t="n">
+        <x:f>H270</x:f>
+        <x:v>12.14</x:v>
+      </x:c>
+      <x:c r="H287" s="35" t="n">
+        <x:v>13.13</x:v>
+      </x:c>
+      <x:c r="I287" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J287" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K287" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="27" customHeight="1">
+      <x:c r="A288" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B288" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C288" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D288" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E288" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F288" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G288" s="17" t="n">
+        <x:f>H271</x:f>
+        <x:v>423.87</x:v>
+      </x:c>
+      <x:c r="H288" s="34" t="n">
+        <x:v>426.11</x:v>
+      </x:c>
+      <x:c r="I288" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J288" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K288" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="289" ht="27" customHeight="1">
+      <x:c r="A289" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B289" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C289" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D289" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E289" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F289" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G289" s="33" t="n">
+        <x:f>H272</x:f>
+        <x:v>255.7</x:v>
+      </x:c>
+      <x:c r="H289" s="35" t="n">
+        <x:v>256.8</x:v>
+      </x:c>
+      <x:c r="I289" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J289" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K289" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="27" customHeight="1">
+      <x:c r="A290" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B290" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C290" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D290" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E290" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F290" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G290" s="17" t="n">
+        <x:f>H273</x:f>
+        <x:v>237.79</x:v>
+      </x:c>
+      <x:c r="H290" s="34" t="n">
+        <x:v>234.92</x:v>
+      </x:c>
+      <x:c r="I290" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J290" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K290" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="291" ht="27" customHeight="1">
+      <x:c r="A291" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B291" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C291" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D291" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E291" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F291" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G291" s="33" t="n">
+        <x:f>H274</x:f>
+        <x:v>5202</x:v>
+      </x:c>
+      <x:c r="H291" s="35" t="n">
+        <x:v>5199</x:v>
+      </x:c>
+      <x:c r="I291" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J291" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K291" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="27" customHeight="1">
+      <x:c r="A292" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B292" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C292" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D292" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E292" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F292" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G292" s="17" t="n">
+        <x:f>H275</x:f>
+        <x:v>102.05</x:v>
+      </x:c>
+      <x:c r="H292" s="34" t="n">
+        <x:v>106.05</x:v>
+      </x:c>
+      <x:c r="I292" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J292" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K292" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="27" customHeight="1">
+      <x:c r="A293" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B293" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C293" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D293" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E293" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F293" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G293" s="33" t="n">
+        <x:f>H276</x:f>
+        <x:v>7663.43</x:v>
+      </x:c>
+      <x:c r="H293" s="35" t="n">
+        <x:v>7623.68</x:v>
+      </x:c>
+      <x:c r="I293" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J293" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K293" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="27" customHeight="1">
+      <x:c r="A294" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B294" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C294" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D294" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E294" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F294" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G294" s="17" t="n">
+        <x:f>H277</x:f>
+        <x:v>26008.8594</x:v>
+      </x:c>
+      <x:c r="H294" s="34" t="n">
+        <x:v>25955.3398</x:v>
+      </x:c>
+      <x:c r="I294" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J294" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="K294" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -11813,7 +12504,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R152397450ee9406f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9c4bb53f444761"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19252,6 +19943,471 @@
         <x:v>0.030599878812361148</x:v>
       </x:c>
     </x:row>
+    <x:row r="246" ht="27" customHeight="1">
+      <x:c r="A246" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B246" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C246" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D246" s="20" t="n">
+        <x:f>G231</x:f>
+        <x:v>0.06864092249009104</x:v>
+      </x:c>
+      <x:c r="E246" s="22" t="n">
+        <x:f>'Prices'!H278/'Prices'!G278-1</x:f>
+        <x:v>-0.006578947368421018</x:v>
+      </x:c>
+      <x:c r="F246" s="20" t="n">
+        <x:f>D246*E246</x:f>
+        <x:v>-0.0004515850163821755</x:v>
+      </x:c>
+      <x:c r="G246" s="20" t="n">
+        <x:f>D246*(1+E246)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.06680459222621804</x:v>
+      </x:c>
+      <x:c r="H246" s="22" t="n">
+        <x:f>'Prices'!H278/'Prices'!I278-1</x:f>
+        <x:v>-0.08813448669822099</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="27" customHeight="1">
+      <x:c r="A247" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B247" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C247" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D247" s="21" t="n">
+        <x:f>G232</x:f>
+        <x:v>0.06310690355633457</x:v>
+      </x:c>
+      <x:c r="E247" s="23" t="n">
+        <x:f>'Prices'!H279/'Prices'!G279-1</x:f>
+        <x:v>-0.0027274981403421217</x:v>
+      </x:c>
+      <x:c r="F247" s="21" t="n">
+        <x:f>D247*E247</x:f>
+        <x:v>-0.00017212396209265215</x:v>
+      </x:c>
+      <x:c r="G247" s="21" t="n">
+        <x:f>D247*(1+E247)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.06165674053163025</x:v>
+      </x:c>
+      <x:c r="H247" s="23" t="n">
+        <x:f>'Prices'!H279/'Prices'!I279-1</x:f>
+        <x:v>-0.1584013391922996</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="27" customHeight="1">
+      <x:c r="A248" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B248" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C248" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D248" s="20" t="n">
+        <x:f>G233</x:f>
+        <x:v>0.07030171511412424</x:v>
+      </x:c>
+      <x:c r="E248" s="22" t="n">
+        <x:f>'Prices'!H280/'Prices'!G280-1</x:f>
+        <x:v>0.09988692046739533</x:v>
+      </x:c>
+      <x:c r="F248" s="20" t="n">
+        <x:f>D248*E248</x:f>
+        <x:v>0.007022221826326012</x:v>
+      </x:c>
+      <x:c r="G248" s="20" t="n">
+        <x:f>D248*(1+E248)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07575369211680971</x:v>
+      </x:c>
+      <x:c r="H248" s="22" t="n">
+        <x:f>'Prices'!H280/'Prices'!I280-1</x:f>
+        <x:v>0.03401842664776766</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="27" customHeight="1">
+      <x:c r="A249" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B249" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C249" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D249" s="21" t="n">
+        <x:f>G234</x:f>
+        <x:v>0.055528840625861685</x:v>
+      </x:c>
+      <x:c r="E249" s="23" t="n">
+        <x:f>'Prices'!H281/'Prices'!G281-1</x:f>
+        <x:v>0.00032388663967619635</x:v>
+      </x:c>
+      <x:c r="F249" s="21" t="n">
+        <x:f>D249*E249</x:f>
+        <x:v>0.000017985049595425397</x:v>
+      </x:c>
+      <x:c r="G249" s="21" t="n">
+        <x:f>D249*(1+E249)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.05441881643358777</x:v>
+      </x:c>
+      <x:c r="H249" s="23" t="n">
+        <x:f>'Prices'!H281/'Prices'!I281-1</x:f>
+        <x:v>-0.25719714278842687</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="27" customHeight="1">
+      <x:c r="A250" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B250" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C250" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D250" s="20" t="n">
+        <x:f>G235</x:f>
+        <x:v>0.06261982655508047</x:v>
+      </x:c>
+      <x:c r="E250" s="22" t="n">
+        <x:f>'Prices'!H282/'Prices'!G282-1</x:f>
+        <x:v>-0.011521843494959216</x:v>
+      </x:c>
+      <x:c r="F250" s="20" t="n">
+        <x:f>D250*E250</x:f>
+        <x:v>-0.0007214958412491284</x:v>
+      </x:c>
+      <x:c r="G250" s="20" t="n">
+        <x:f>D250*(1+E250)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.060641339189069256</x:v>
+      </x:c>
+      <x:c r="H250" s="22" t="n">
+        <x:f>'Prices'!H282/'Prices'!I282-1</x:f>
+        <x:v>-0.17226130653266336</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="27" customHeight="1">
+      <x:c r="A251" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B251" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C251" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D251" s="21" t="n">
+        <x:f>G236</x:f>
+        <x:v>0.07191274917622073</x:v>
+      </x:c>
+      <x:c r="E251" s="23" t="n">
+        <x:f>'Prices'!H283/'Prices'!G283-1</x:f>
+        <x:v>0.07192947305149278</x:v>
+      </x:c>
+      <x:c r="F251" s="21" t="n">
+        <x:f>D251*E251</x:f>
+        <x:v>0.005172646153929729</x:v>
+      </x:c>
+      <x:c r="G251" s="21" t="n">
+        <x:f>D251*(1+E251)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07551999465624695</x:v>
+      </x:c>
+      <x:c r="H251" s="23" t="n">
+        <x:f>'Prices'!H283/'Prices'!I283-1</x:f>
+        <x:v>0.030828516377649384</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="27" customHeight="1">
+      <x:c r="A252" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B252" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C252" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D252" s="20" t="n">
+        <x:f>G237</x:f>
+        <x:v>0.07400645111577114</x:v>
+      </x:c>
+      <x:c r="E252" s="22" t="n">
+        <x:f>'Prices'!H284/'Prices'!G284-1</x:f>
+        <x:v>-0.024639123942259866</x:v>
+      </x:c>
+      <x:c r="F252" s="20" t="n">
+        <x:f>D252*E252</x:f>
+        <x:v>-0.0018234541215682812</x:v>
+      </x:c>
+      <x:c r="G252" s="20" t="n">
+        <x:f>D252*(1+E252)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07071715107546364</x:v>
+      </x:c>
+      <x:c r="H252" s="22" t="n">
+        <x:f>'Prices'!H284/'Prices'!I284-1</x:f>
+        <x:v>-0.0347290640394089</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="27" customHeight="1">
+      <x:c r="A253" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B253" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C253" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D253" s="21" t="n">
+        <x:f>G238</x:f>
+        <x:v>0.06562182672965099</x:v>
+      </x:c>
+      <x:c r="E253" s="23" t="n">
+        <x:f>'Prices'!H285/'Prices'!G285-1</x:f>
+        <x:v>0.017399267399267337</x:v>
+      </x:c>
+      <x:c r="F253" s="21" t="n">
+        <x:f>D253*E253</x:f>
+        <x:v>0.0011417717104975863</x:v>
+      </x:c>
+      <x:c r="G253" s="21" t="n">
+        <x:f>D253*(1+E253)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.06540780618478274</x:v>
+      </x:c>
+      <x:c r="H253" s="23" t="n">
+        <x:f>'Prices'!H285/'Prices'!I285-1</x:f>
+        <x:v>-0.10720025715204118</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="27" customHeight="1">
+      <x:c r="A254" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B254" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C254" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D254" s="20" t="n">
+        <x:f>G239</x:f>
+        <x:v>0.051195142040718074</x:v>
+      </x:c>
+      <x:c r="E254" s="22" t="n">
+        <x:f>'Prices'!H286/'Prices'!G286-1</x:f>
+        <x:v>0.06111508220157269</x:v>
+      </x:c>
+      <x:c r="F254" s="20" t="n">
+        <x:f>D254*E254</x:f>
+        <x:v>0.003128795314139675</x:v>
+      </x:c>
+      <x:c r="G254" s="20" t="n">
+        <x:f>D254*(1+E254)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.053220761743184845</x:v>
+      </x:c>
+      <x:c r="H254" s="22" t="n">
+        <x:f>'Prices'!H286/'Prices'!I286-1</x:f>
+        <x:v>-0.27355028137998527</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="27" customHeight="1">
+      <x:c r="A255" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B255" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C255" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D255" s="21" t="n">
+        <x:f>G240</x:f>
+        <x:v>0.05698867908558656</x:v>
+      </x:c>
+      <x:c r="E255" s="23" t="n">
+        <x:f>'Prices'!H287/'Prices'!G287-1</x:f>
+        <x:v>0.08154859967051076</x:v>
+      </x:c>
+      <x:c r="F255" s="21" t="n">
+        <x:f>D255*E255</x:f>
+        <x:v>0.004647346976501708</x:v>
+      </x:c>
+      <x:c r="G255" s="21" t="n">
+        <x:f>D255*(1+E255)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.0603843612516389</x:v>
+      </x:c>
+      <x:c r="H255" s="23" t="n">
+        <x:f>'Prices'!H287/'Prices'!I287-1</x:f>
+        <x:v>-0.1757689893283113</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="27" customHeight="1">
+      <x:c r="A256" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B256" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C256" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D256" s="20" t="n">
+        <x:f>G241</x:f>
+        <x:v>0.0716397662681084</x:v>
+      </x:c>
+      <x:c r="E256" s="22" t="n">
+        <x:f>'Prices'!H288/'Prices'!G288-1</x:f>
+        <x:v>0.005284639158232407</x:v>
+      </x:c>
+      <x:c r="F256" s="20" t="n">
+        <x:f>D256*E256</x:f>
+        <x:v>0.0003785903141070628</x:v>
+      </x:c>
+      <x:c r="G256" s="20" t="n">
+        <x:f>D256*(1+E256)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07055585407516626</x:v>
+      </x:c>
+      <x:c r="H256" s="22" t="n">
+        <x:f>'Prices'!H288/'Prices'!I288-1</x:f>
+        <x:v>-0.03693072663577801</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="27" customHeight="1">
+      <x:c r="A257" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B257" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C257" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D257" s="21" t="n">
+        <x:f>G242</x:f>
+        <x:v>0.07032458861038246</x:v>
+      </x:c>
+      <x:c r="E257" s="23" t="n">
+        <x:f>'Prices'!H289/'Prices'!G289-1</x:f>
+        <x:v>0.00430191630817367</x:v>
+      </x:c>
+      <x:c r="F257" s="21" t="n">
+        <x:f>D257*E257</x:f>
+        <x:v>0.00030253049460860865</x:v>
+      </x:c>
+      <x:c r="G257" s="21" t="n">
+        <x:f>D257*(1+E257)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.06919286895463123</x:v>
+      </x:c>
+      <x:c r="H257" s="23" t="n">
+        <x:f>'Prices'!H289/'Prices'!I289-1</x:f>
+        <x:v>-0.05553512320706133</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="27" customHeight="1">
+      <x:c r="A258" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B258" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C258" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D258" s="20" t="n">
+        <x:f>G243</x:f>
+        <x:v>0.07434234360854022</x:v>
+      </x:c>
+      <x:c r="E258" s="22" t="n">
+        <x:f>'Prices'!H290/'Prices'!G290-1</x:f>
+        <x:v>-0.012069473064468705</x:v>
+      </x:c>
+      <x:c r="F258" s="20" t="n">
+        <x:f>D258*E258</x:f>
+        <x:v>-0.0008972729137327535</x:v>
+      </x:c>
+      <x:c r="G258" s="20" t="n">
+        <x:f>D258*(1+E258)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07195359539435489</x:v>
+      </x:c>
+      <x:c r="H258" s="22" t="n">
+        <x:f>'Prices'!H290/'Prices'!I290-1</x:f>
+        <x:v>-0.017851916886157504</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="27" customHeight="1">
+      <x:c r="A259" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B259" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C259" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D259" s="21" t="n">
+        <x:f>G244</x:f>
+        <x:v>0.06670194721913338</x:v>
+      </x:c>
+      <x:c r="E259" s="23" t="n">
+        <x:f>'Prices'!H291/'Prices'!G291-1</x:f>
+        <x:v>-0.0005767012687427631</x:v>
+      </x:c>
+      <x:c r="F259" s="21" t="n">
+        <x:f>D259*E259</x:f>
+        <x:v>-0.000038467097588887034</x:v>
+      </x:c>
+      <x:c r="G259" s="21" t="n">
+        <x:f>D259*(1+E259)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.06530972100465764</x:v>
+      </x:c>
+      <x:c r="H259" s="23" t="n">
+        <x:f>'Prices'!H291/'Prices'!I291-1</x:f>
+        <x:v>-0.10853909465020573</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="27" customHeight="1">
+      <x:c r="A260" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B260" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C260" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D260" s="20" t="n">
+        <x:f>G245</x:f>
+        <x:v>0.07706829780439557</x:v>
+      </x:c>
+      <x:c r="E260" s="22" t="n">
+        <x:f>'Prices'!H292/'Prices'!G292-1</x:f>
+        <x:v>0.03919647231749135</x:v>
+      </x:c>
+      <x:c r="F260" s="20" t="n">
+        <x:f>D260*E260</x:f>
+        <x:v>0.0030208054014461702</x:v>
+      </x:c>
+      <x:c r="G260" s="20" t="n">
+        <x:f>D260*(1+E260)/(1+SUM($F$246:$F$260))</x:f>
+        <x:v>0.07846270516255746</x:v>
+      </x:c>
+      <x:c r="H260" s="22" t="n">
+        <x:f>'Prices'!H292/'Prices'!I292-1</x:f>
+        <x:v>0.07099575843263994</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -19259,7 +20415,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra63f55e084b34900"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90b0f52b5e1b4f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29786,6 +30942,654 @@
       </x:c>
       <x:c r="M277" s="16" t="str"/>
     </x:row>
+    <x:row r="278" ht="50" customHeight="1">
+      <x:c r="A278" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B278" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C278" s="17" t="n">
+        <x:v>5587</x:v>
+      </x:c>
+      <x:c r="D278" s="17" t="n">
+        <x:v>5587</x:v>
+      </x:c>
+      <x:c r="E278" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F278" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G278" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H278" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I278" s="31" t="str">
+        <x:f>IF(AND(G278=H278,C278&gt;0,ABS(C278-'Prices'!H278)&lt;=MAX(0.01,'Prices'!H278*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J278" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K278" s="14" t="str"/>
+      <x:c r="L278" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M278" s="14" t="str"/>
+    </x:row>
+    <x:row r="279" ht="50" customHeight="1">
+      <x:c r="A279" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B279" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C279" s="33" t="n">
+        <x:v>4022</x:v>
+      </x:c>
+      <x:c r="D279" s="33" t="n">
+        <x:v>4022</x:v>
+      </x:c>
+      <x:c r="E279" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F279" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G279" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H279" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I279" s="32" t="str">
+        <x:f>IF(AND(G279=H279,C279&gt;0,ABS(C279-'Prices'!H279)&lt;=MAX(0.01,'Prices'!H279*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J279" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K279" s="16" t="str"/>
+      <x:c r="L279" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M279" s="16" t="str"/>
+    </x:row>
+    <x:row r="280" ht="50" customHeight="1">
+      <x:c r="A280" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B280" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C280" s="17" t="n">
+        <x:v>29.18</x:v>
+      </x:c>
+      <x:c r="D280" s="17" t="n">
+        <x:v>29.18</x:v>
+      </x:c>
+      <x:c r="E280" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F280" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G280" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H280" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I280" s="31" t="str">
+        <x:f>IF(AND(G280=H280,C280&gt;0,ABS(C280-'Prices'!H280)&lt;=MAX(0.01,'Prices'!H280*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J280" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K280" s="14" t="str"/>
+      <x:c r="L280" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M280" s="14" t="str"/>
+    </x:row>
+    <x:row r="281" ht="50" customHeight="1">
+      <x:c r="A281" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B281" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C281" s="33" t="n">
+        <x:v>308.85</x:v>
+      </x:c>
+      <x:c r="D281" s="33" t="n">
+        <x:v>308.85</x:v>
+      </x:c>
+      <x:c r="E281" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F281" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G281" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H281" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I281" s="32" t="str">
+        <x:f>IF(AND(G281=H281,C281&gt;0,ABS(C281-'Prices'!H281)&lt;=MAX(0.01,'Prices'!H281*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J281" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K281" s="16" t="str"/>
+      <x:c r="L281" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M281" s="16" t="str"/>
+    </x:row>
+    <x:row r="282" ht="50" customHeight="1">
+      <x:c r="A282" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B282" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C282" s="17" t="n">
+        <x:v>4118</x:v>
+      </x:c>
+      <x:c r="D282" s="17" t="n">
+        <x:v>4118</x:v>
+      </x:c>
+      <x:c r="E282" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F282" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G282" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H282" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I282" s="31" t="str">
+        <x:f>IF(AND(G282=H282,C282&gt;0,ABS(C282-'Prices'!H282)&lt;=MAX(0.01,'Prices'!H282*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J282" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K282" s="14" t="str"/>
+      <x:c r="L282" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M282" s="14" t="str"/>
+    </x:row>
+    <x:row r="283" ht="50" customHeight="1">
+      <x:c r="A283" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B283" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C283" s="33" t="n">
+        <x:v>53.5</x:v>
+      </x:c>
+      <x:c r="D283" s="33" t="n">
+        <x:v>53.5</x:v>
+      </x:c>
+      <x:c r="E283" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F283" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G283" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H283" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I283" s="32" t="str">
+        <x:f>IF(AND(G283=H283,C283&gt;0,ABS(C283-'Prices'!H283)&lt;=MAX(0.01,'Prices'!H283*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J283" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K283" s="16" t="str"/>
+      <x:c r="L283" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M283" s="16" t="str"/>
+    </x:row>
+    <x:row r="284" ht="50" customHeight="1">
+      <x:c r="A284" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B284" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C284" s="17" t="n">
+        <x:v>78380</x:v>
+      </x:c>
+      <x:c r="D284" s="17" t="n">
+        <x:v>78380</x:v>
+      </x:c>
+      <x:c r="E284" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F284" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G284" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H284" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I284" s="31" t="str">
+        <x:f>IF(AND(G284=H284,C284&gt;0,ABS(C284-'Prices'!H284)&lt;=MAX(0.01,'Prices'!H284*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J284" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K284" s="14" t="str"/>
+      <x:c r="L284" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M284" s="14" t="str"/>
+    </x:row>
+    <x:row r="285" ht="50" customHeight="1">
+      <x:c r="A285" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B285" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C285" s="33" t="n">
+        <x:v>55.55</x:v>
+      </x:c>
+      <x:c r="D285" s="33" t="n">
+        <x:v>55.55</x:v>
+      </x:c>
+      <x:c r="E285" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F285" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G285" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H285" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I285" s="32" t="str">
+        <x:f>IF(AND(G285=H285,C285&gt;0,ABS(C285-'Prices'!H285)&lt;=MAX(0.01,'Prices'!H285*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J285" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K285" s="16" t="str"/>
+      <x:c r="L285" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M285" s="16" t="str"/>
+    </x:row>
+    <x:row r="286" ht="50" customHeight="1">
+      <x:c r="A286" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B286" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C286" s="17" t="n">
+        <x:v>29.69</x:v>
+      </x:c>
+      <x:c r="D286" s="17" t="n">
+        <x:v>29.69</x:v>
+      </x:c>
+      <x:c r="E286" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F286" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G286" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H286" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I286" s="31" t="str">
+        <x:f>IF(AND(OR(G286=H286,AND(B286="OUST",G286="XNAS",H286="XNYS",LEFT(M286,34)="ouster-marketstack-legacy-nyse-tag")),C286&gt;0,ABS(C286-'Prices'!H286)&lt;=MAX(0.01,'Prices'!H286*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J286" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K286" s="14" t="str"/>
+      <x:c r="L286" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M286" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="50" customHeight="1">
+      <x:c r="A287" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B287" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C287" s="33" t="n">
+        <x:v>13.13</x:v>
+      </x:c>
+      <x:c r="D287" s="33" t="n">
+        <x:v>13.13</x:v>
+      </x:c>
+      <x:c r="E287" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F287" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G287" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H287" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I287" s="32" t="str">
+        <x:f>IF(AND(G287=H287,C287&gt;0,ABS(C287-'Prices'!H287)&lt;=MAX(0.01,'Prices'!H287*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J287" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K287" s="16" t="str"/>
+      <x:c r="L287" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M287" s="16" t="str"/>
+    </x:row>
+    <x:row r="288" ht="50" customHeight="1">
+      <x:c r="A288" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B288" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C288" s="17" t="n">
+        <x:v>426.11</x:v>
+      </x:c>
+      <x:c r="D288" s="17" t="n">
+        <x:v>426.11</x:v>
+      </x:c>
+      <x:c r="E288" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F288" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G288" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H288" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I288" s="31" t="str">
+        <x:f>IF(AND(G288=H288,C288&gt;0,ABS(C288-'Prices'!H288)&lt;=MAX(0.01,'Prices'!H288*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J288" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K288" s="14" t="str"/>
+      <x:c r="L288" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M288" s="14" t="str"/>
+    </x:row>
+    <x:row r="289" ht="50" customHeight="1">
+      <x:c r="A289" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B289" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C289" s="33" t="n">
+        <x:v>256.8</x:v>
+      </x:c>
+      <x:c r="D289" s="33" t="n">
+        <x:v>256.8</x:v>
+      </x:c>
+      <x:c r="E289" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F289" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G289" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H289" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I289" s="32" t="str">
+        <x:f>IF(AND(G289=H289,C289&gt;0,ABS(C289-'Prices'!H289)&lt;=MAX(0.01,'Prices'!H289*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J289" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K289" s="16" t="str"/>
+      <x:c r="L289" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M289" s="16" t="str"/>
+    </x:row>
+    <x:row r="290" ht="50" customHeight="1">
+      <x:c r="A290" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B290" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C290" s="17" t="n">
+        <x:v>234.92</x:v>
+      </x:c>
+      <x:c r="D290" s="17" t="n">
+        <x:v>234.92</x:v>
+      </x:c>
+      <x:c r="E290" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F290" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G290" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H290" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I290" s="31" t="str">
+        <x:f>IF(AND(G290=H290,C290&gt;0,ABS(C290-'Prices'!H290)&lt;=MAX(0.01,'Prices'!H290*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J290" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K290" s="14" t="str"/>
+      <x:c r="L290" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M290" s="14" t="str"/>
+    </x:row>
+    <x:row r="291" ht="50" customHeight="1">
+      <x:c r="A291" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B291" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C291" s="33" t="n">
+        <x:v>5199</x:v>
+      </x:c>
+      <x:c r="D291" s="33" t="n">
+        <x:v>5199</x:v>
+      </x:c>
+      <x:c r="E291" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F291" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G291" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H291" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I291" s="32" t="str">
+        <x:f>IF(AND(G291=H291,C291&gt;0,ABS(C291-'Prices'!H291)&lt;=MAX(0.01,'Prices'!H291*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J291" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K291" s="16" t="str"/>
+      <x:c r="L291" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M291" s="16" t="str"/>
+    </x:row>
+    <x:row r="292" ht="50" customHeight="1">
+      <x:c r="A292" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B292" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C292" s="17" t="n">
+        <x:v>106.05</x:v>
+      </x:c>
+      <x:c r="D292" s="17" t="n">
+        <x:v>106.05</x:v>
+      </x:c>
+      <x:c r="E292" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F292" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G292" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H292" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I292" s="31" t="str">
+        <x:f>IF(AND(G292=H292,C292&gt;0,ABS(C292-'Prices'!H292)&lt;=MAX(0.01,'Prices'!H292*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J292" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K292" s="14" t="str"/>
+      <x:c r="L292" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M292" s="14" t="str"/>
+    </x:row>
+    <x:row r="293" ht="50" customHeight="1">
+      <x:c r="A293" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B293" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C293" s="33" t="n">
+        <x:v>7623.68</x:v>
+      </x:c>
+      <x:c r="D293" s="33" t="n">
+        <x:v>7623.68</x:v>
+      </x:c>
+      <x:c r="E293" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F293" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G293" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H293" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I293" s="32" t="str">
+        <x:f>IF(AND(G293=H293,C293&gt;0,ABS(C293-'Prices'!H293)&lt;=MAX(0.01,'Prices'!H293*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J293" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K293" s="16" t="str"/>
+      <x:c r="L293" s="39" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M293" s="16" t="str"/>
+    </x:row>
+    <x:row r="294" ht="50" customHeight="1">
+      <x:c r="A294" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B294" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C294" s="17" t="n">
+        <x:v>25955.3398</x:v>
+      </x:c>
+      <x:c r="D294" s="17" t="n">
+        <x:v>25955.3398</x:v>
+      </x:c>
+      <x:c r="E294" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F294" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G294" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H294" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I294" s="31" t="str">
+        <x:f>IF(AND(G294=H294,C294&gt;0,ABS(C294-'Prices'!H294)&lt;=MAX(0.01,'Prices'!H294*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J294" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-24T11-29-06-564Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K294" s="14" t="str"/>
+      <x:c r="L294" s="38" t="n">
+        <x:v>46319.47854819444</x:v>
+      </x:c>
+      <x:c r="M294" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -29793,7 +31597,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af4806bb8ed4856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98066f6298c54dfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37770,6 +39574,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="278" ht="27" customHeight="1">
+      <x:c r="A278" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B278" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C278" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D278" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E278" s="19" t="n">
+        <x:f>'Source Audit'!E278</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F278" s="40" t="n">
+        <x:f>'Source Audit'!F278</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G278" s="11" t="str">
+        <x:f>IF(AND(E278=0,F278=1,'Source Audit'!I278&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H278" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="27" customHeight="1">
+      <x:c r="A279" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B279" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C279" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D279" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E279" s="18" t="n">
+        <x:f>'Source Audit'!E279</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F279" s="41" t="n">
+        <x:f>'Source Audit'!F279</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G279" s="12" t="str">
+        <x:f>IF(AND(E279=0,F279=1,'Source Audit'!I279&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H279" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="27" customHeight="1">
+      <x:c r="A280" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B280" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C280" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D280" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E280" s="19" t="n">
+        <x:f>'Source Audit'!E280</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F280" s="40" t="n">
+        <x:f>'Source Audit'!F280</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G280" s="11" t="str">
+        <x:f>IF(AND(E280=0,F280=1,'Source Audit'!I280&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H280" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="27" customHeight="1">
+      <x:c r="A281" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B281" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C281" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D281" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E281" s="18" t="n">
+        <x:f>'Source Audit'!E281</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F281" s="41" t="n">
+        <x:f>'Source Audit'!F281</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G281" s="12" t="str">
+        <x:f>IF(AND(E281=0,F281=1,'Source Audit'!I281&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H281" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="27" customHeight="1">
+      <x:c r="A282" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B282" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C282" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D282" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E282" s="19" t="n">
+        <x:f>'Source Audit'!E282</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F282" s="40" t="n">
+        <x:f>'Source Audit'!F282</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G282" s="11" t="str">
+        <x:f>IF(AND(E282=0,F282=1,'Source Audit'!I282&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H282" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="27" customHeight="1">
+      <x:c r="A283" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B283" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C283" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D283" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E283" s="18" t="n">
+        <x:f>'Source Audit'!E283</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F283" s="41" t="n">
+        <x:f>'Source Audit'!F283</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G283" s="12" t="str">
+        <x:f>IF(AND(E283=0,F283=1,'Source Audit'!I283&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H283" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="27" customHeight="1">
+      <x:c r="A284" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B284" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C284" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D284" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E284" s="19" t="n">
+        <x:f>'Source Audit'!E284</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F284" s="40" t="n">
+        <x:f>'Source Audit'!F284</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G284" s="11" t="str">
+        <x:f>IF(AND(E284=0,F284=1,'Source Audit'!I284&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H284" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="27" customHeight="1">
+      <x:c r="A285" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B285" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C285" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D285" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E285" s="18" t="n">
+        <x:f>'Source Audit'!E285</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F285" s="41" t="n">
+        <x:f>'Source Audit'!F285</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G285" s="12" t="str">
+        <x:f>IF(AND(E285=0,F285=1,'Source Audit'!I285&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H285" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="44" customHeight="1">
+      <x:c r="A286" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B286" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C286" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D286" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E286" s="19" t="n">
+        <x:f>'Source Audit'!E286</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F286" s="40" t="n">
+        <x:f>'Source Audit'!F286</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G286" s="11" t="str">
+        <x:f>IF(AND(E286=0,F286=1,'Source Audit'!I286&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H286" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="27" customHeight="1">
+      <x:c r="A287" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B287" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C287" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D287" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E287" s="18" t="n">
+        <x:f>'Source Audit'!E287</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F287" s="41" t="n">
+        <x:f>'Source Audit'!F287</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G287" s="12" t="str">
+        <x:f>IF(AND(E287=0,F287=1,'Source Audit'!I287&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H287" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="27" customHeight="1">
+      <x:c r="A288" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B288" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C288" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D288" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E288" s="19" t="n">
+        <x:f>'Source Audit'!E288</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F288" s="40" t="n">
+        <x:f>'Source Audit'!F288</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G288" s="11" t="str">
+        <x:f>IF(AND(E288=0,F288=1,'Source Audit'!I288&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H288" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="289" ht="27" customHeight="1">
+      <x:c r="A289" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B289" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C289" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D289" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E289" s="18" t="n">
+        <x:f>'Source Audit'!E289</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F289" s="41" t="n">
+        <x:f>'Source Audit'!F289</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G289" s="12" t="str">
+        <x:f>IF(AND(E289=0,F289=1,'Source Audit'!I289&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H289" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="27" customHeight="1">
+      <x:c r="A290" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B290" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C290" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D290" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E290" s="19" t="n">
+        <x:f>'Source Audit'!E290</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F290" s="40" t="n">
+        <x:f>'Source Audit'!F290</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G290" s="11" t="str">
+        <x:f>IF(AND(E290=0,F290=1,'Source Audit'!I290&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H290" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="291" ht="27" customHeight="1">
+      <x:c r="A291" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B291" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C291" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D291" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E291" s="18" t="n">
+        <x:f>'Source Audit'!E291</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F291" s="41" t="n">
+        <x:f>'Source Audit'!F291</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G291" s="12" t="str">
+        <x:f>IF(AND(E291=0,F291=1,'Source Audit'!I291&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H291" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="27" customHeight="1">
+      <x:c r="A292" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B292" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C292" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D292" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E292" s="19" t="n">
+        <x:f>'Source Audit'!E292</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F292" s="40" t="n">
+        <x:f>'Source Audit'!F292</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G292" s="11" t="str">
+        <x:f>IF(AND(E292=0,F292=1,'Source Audit'!I292&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H292" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="27" customHeight="1">
+      <x:c r="A293" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B293" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C293" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D293" s="9" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E293" s="18" t="n">
+        <x:f>'Source Audit'!E293</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F293" s="41" t="n">
+        <x:f>'Source Audit'!F293</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G293" s="12" t="str">
+        <x:f>IF(AND(E293=0,F293=1,'Source Audit'!I293&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H293" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="27" customHeight="1">
+      <x:c r="A294" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="B294" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C294" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D294" s="8" t="n">
+        <x:v>46318</x:v>
+      </x:c>
+      <x:c r="E294" s="19" t="n">
+        <x:f>'Source Audit'!E294</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F294" s="40" t="n">
+        <x:f>'Source Audit'!F294</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G294" s="11" t="str">
+        <x:f>IF(AND(E294=0,F294=1,'Source Audit'!I294&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H294" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -37777,7 +40074,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544a73e9ce3f47e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fa397610514ae2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 26, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 274 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Shared-checkout build stopped on unrelated local
Insights taxonomy work; the exact main-based publication candidate
production build and article-preview checks passed. These results are
documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc7bed2ce2136496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rc24bab9c6b8f4740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R3955910673574566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Rd1b6391f339746e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rcd519c54707f461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8437e955c5274fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Ree12527931bb481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Rf2422b7d20234e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R1d2f15a332e14d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rcdbb2266a93b4998"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H275" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H294" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -2024,6 +2024,85 @@
         <x:v>-5.591957315111795</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="40" customHeight="1">
+      <x:c r="A23" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B23" s="18" t="n">
+        <x:f>B22*(1+SUM('Returns and Contributions'!F261:F275))</x:f>
+        <x:v>923.7297152894076</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="n">
+        <x:f>B23/B22-1</x:f>
+        <x:v>0.015106713495044222</x:v>
+      </x:c>
+      <x:c r="D23" s="21" t="n">
+        <x:f>B23/$B$6-1</x:f>
+        <x:v>-0.07627028471059238</x:v>
+      </x:c>
+      <x:c r="E23" s="18" t="n">
+        <x:f>1000*'Prices'!H310/'Prices'!I310</x:f>
+        <x:v>1001.3461249991848</x:v>
+      </x:c>
+      <x:c r="F23" s="21" t="n">
+        <x:f>E23/E22-1</x:f>
+        <x:v>0.006963828492276836</x:v>
+      </x:c>
+      <x:c r="G23" s="21" t="n">
+        <x:f>E23/1000-1</x:f>
+        <x:v>0.00134612499918485</x:v>
+      </x:c>
+      <x:c r="H23" s="18" t="n">
+        <x:f>1000*'Prices'!H311/'Prices'!I311</x:f>
+        <x:v>973.8677669968068</x:v>
+      </x:c>
+      <x:c r="I23" s="21" t="n">
+        <x:f>H23/H22-1</x:f>
+        <x:v>0.008246515038882185</x:v>
+      </x:c>
+      <x:c r="J23" s="21" t="n">
+        <x:f>H23/1000-1</x:f>
+        <x:v>-0.026132233003193117</x:v>
+      </x:c>
+      <x:c r="K23" s="25" t="n">
+        <x:f>(C23-F23)*100</x:f>
+        <x:v>0.8142885002767386</x:v>
+      </x:c>
+      <x:c r="L23" s="25" t="n">
+        <x:f>(C23-I23)*100</x:f>
+        <x:v>0.6860198456162037</x:v>
+      </x:c>
+      <x:c r="M23" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G261:G275)</x:f>
+        <x:v>0.9999999999999996</x:v>
+      </x:c>
+      <x:c r="N23" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F261:F275)-C23</x:f>
+        <x:v>-7.979727989493313e-17</x:v>
+      </x:c>
+      <x:c r="O23" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P23" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I295:I311,"Mismatch")=0,IF(COUNTIF('Source Audit'!I295:I311,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q23" s="30" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="R23" s="27" t="n">
+        <x:f>B23-1000*('Prices'!H295/'Prices'!H6+'Prices'!H296/'Prices'!H7+'Prices'!H297/'Prices'!H8+'Prices'!H298/'Prices'!H9+'Prices'!H299/'Prices'!H10+'Prices'!H300/'Prices'!H11+'Prices'!H301/'Prices'!H12+'Prices'!H302/'Prices'!H13+'Prices'!H303/'Prices'!H14+'Prices'!H304/'Prices'!H15+'Prices'!H305/'Prices'!H16+'Prices'!H306/'Prices'!H17+'Prices'!H307/'Prices'!H18+'Prices'!H308/'Prices'!H19+'Prices'!H309/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S23" s="25" t="n">
+        <x:f>(D23-G23)*100</x:f>
+        <x:v>-7.761640970977723</x:v>
+      </x:c>
+      <x:c r="T23" s="25" t="n">
+        <x:f>(D23-J23)*100</x:f>
+        <x:v>-5.013805170739927</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -2031,7 +2110,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9105081044214c7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R611178679d4e46a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12497,6 +12576,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="295" ht="27" customHeight="1">
+      <x:c r="A295" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B295" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C295" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D295" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E295" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F295" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G295" s="33" t="n">
+        <x:f>H278</x:f>
+        <x:v>5587</x:v>
+      </x:c>
+      <x:c r="H295" s="35" t="n">
+        <x:v>5639</x:v>
+      </x:c>
+      <x:c r="I295" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J295" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K295" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="27" customHeight="1">
+      <x:c r="A296" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B296" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C296" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D296" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E296" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F296" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G296" s="17" t="n">
+        <x:f>H279</x:f>
+        <x:v>4022</x:v>
+      </x:c>
+      <x:c r="H296" s="34" t="n">
+        <x:v>3980</x:v>
+      </x:c>
+      <x:c r="I296" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J296" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K296" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="27" customHeight="1">
+      <x:c r="A297" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B297" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C297" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D297" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E297" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F297" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G297" s="33" t="n">
+        <x:f>H280</x:f>
+        <x:v>29.18</x:v>
+      </x:c>
+      <x:c r="H297" s="35" t="n">
+        <x:v>30.59</x:v>
+      </x:c>
+      <x:c r="I297" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J297" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K297" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="27" customHeight="1">
+      <x:c r="A298" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B298" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C298" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D298" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E298" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F298" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G298" s="17" t="n">
+        <x:f>H281</x:f>
+        <x:v>308.85</x:v>
+      </x:c>
+      <x:c r="H298" s="34" t="n">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="I298" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J298" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K298" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="27" customHeight="1">
+      <x:c r="A299" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B299" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C299" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D299" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E299" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F299" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G299" s="33" t="n">
+        <x:f>H282</x:f>
+        <x:v>4118</x:v>
+      </x:c>
+      <x:c r="H299" s="35" t="n">
+        <x:v>4140</x:v>
+      </x:c>
+      <x:c r="I299" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J299" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K299" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="27" customHeight="1">
+      <x:c r="A300" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B300" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C300" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D300" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E300" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F300" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G300" s="17" t="n">
+        <x:f>H283</x:f>
+        <x:v>53.5</x:v>
+      </x:c>
+      <x:c r="H300" s="34" t="n">
+        <x:v>55.25</x:v>
+      </x:c>
+      <x:c r="I300" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J300" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K300" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="27" customHeight="1">
+      <x:c r="A301" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B301" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C301" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D301" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E301" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F301" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G301" s="33" t="n">
+        <x:f>H284</x:f>
+        <x:v>78380</x:v>
+      </x:c>
+      <x:c r="H301" s="35" t="n">
+        <x:v>77270</x:v>
+      </x:c>
+      <x:c r="I301" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J301" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K301" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="27" customHeight="1">
+      <x:c r="A302" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B302" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C302" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D302" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E302" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F302" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G302" s="17" t="n">
+        <x:f>H285</x:f>
+        <x:v>55.55</x:v>
+      </x:c>
+      <x:c r="H302" s="34" t="n">
+        <x:v>55.63</x:v>
+      </x:c>
+      <x:c r="I302" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J302" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K302" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="27" customHeight="1">
+      <x:c r="A303" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B303" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C303" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D303" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E303" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F303" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G303" s="33" t="n">
+        <x:f>H286</x:f>
+        <x:v>29.69</x:v>
+      </x:c>
+      <x:c r="H303" s="35" t="n">
+        <x:v>29.71</x:v>
+      </x:c>
+      <x:c r="I303" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J303" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K303" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="27" customHeight="1">
+      <x:c r="A304" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B304" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C304" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D304" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E304" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F304" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G304" s="17" t="n">
+        <x:f>H287</x:f>
+        <x:v>13.13</x:v>
+      </x:c>
+      <x:c r="H304" s="34" t="n">
+        <x:v>13.69</x:v>
+      </x:c>
+      <x:c r="I304" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J304" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K304" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="27" customHeight="1">
+      <x:c r="A305" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B305" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C305" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D305" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E305" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F305" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G305" s="33" t="n">
+        <x:f>H288</x:f>
+        <x:v>426.11</x:v>
+      </x:c>
+      <x:c r="H305" s="35" t="n">
+        <x:v>429.89</x:v>
+      </x:c>
+      <x:c r="I305" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J305" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K305" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="27" customHeight="1">
+      <x:c r="A306" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B306" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C306" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D306" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E306" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F306" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G306" s="17" t="n">
+        <x:f>H289</x:f>
+        <x:v>256.8</x:v>
+      </x:c>
+      <x:c r="H306" s="34" t="n">
+        <x:v>261.4</x:v>
+      </x:c>
+      <x:c r="I306" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J306" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K306" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="27" customHeight="1">
+      <x:c r="A307" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B307" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C307" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D307" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E307" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F307" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G307" s="33" t="n">
+        <x:f>H290</x:f>
+        <x:v>234.92</x:v>
+      </x:c>
+      <x:c r="H307" s="35" t="n">
+        <x:v>245.83</x:v>
+      </x:c>
+      <x:c r="I307" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J307" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K307" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="27" customHeight="1">
+      <x:c r="A308" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B308" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C308" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D308" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E308" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F308" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G308" s="17" t="n">
+        <x:f>H291</x:f>
+        <x:v>5199</x:v>
+      </x:c>
+      <x:c r="H308" s="34" t="n">
+        <x:v>5137</x:v>
+      </x:c>
+      <x:c r="I308" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J308" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K308" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="27" customHeight="1">
+      <x:c r="A309" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B309" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C309" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D309" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E309" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F309" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G309" s="33" t="n">
+        <x:f>H292</x:f>
+        <x:v>106.05</x:v>
+      </x:c>
+      <x:c r="H309" s="35" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="I309" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J309" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K309" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="27" customHeight="1">
+      <x:c r="A310" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B310" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C310" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D310" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E310" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F310" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G310" s="17" t="n">
+        <x:f>H293</x:f>
+        <x:v>7623.68</x:v>
+      </x:c>
+      <x:c r="H310" s="34" t="n">
+        <x:v>7676.77</x:v>
+      </x:c>
+      <x:c r="I310" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J310" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K310" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="27" customHeight="1">
+      <x:c r="A311" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B311" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C311" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D311" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E311" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F311" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G311" s="33" t="n">
+        <x:f>H294</x:f>
+        <x:v>25955.3398</x:v>
+      </x:c>
+      <x:c r="H311" s="35" t="n">
+        <x:v>26169.3809</x:v>
+      </x:c>
+      <x:c r="I311" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J311" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="K311" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -12504,7 +13195,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9c4bb53f444761"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeef5d0423e34c1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20408,6 +21099,471 @@
         <x:v>0.07099575843263994</x:v>
       </x:c>
     </x:row>
+    <x:row r="261" ht="27" customHeight="1">
+      <x:c r="A261" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B261" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C261" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D261" s="21" t="n">
+        <x:f>G246</x:f>
+        <x:v>0.06680459222621804</x:v>
+      </x:c>
+      <x:c r="E261" s="23" t="n">
+        <x:f>'Prices'!H295/'Prices'!G295-1</x:f>
+        <x:v>0.009307320565598687</x:v>
+      </x:c>
+      <x:c r="F261" s="21" t="n">
+        <x:f>D261*E261</x:f>
+        <x:v>0.0006217717551035134</x:v>
+      </x:c>
+      <x:c r="G261" s="21" t="n">
+        <x:f>D261*(1+E261)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06642293178139909</x:v>
+      </x:c>
+      <x:c r="H261" s="23" t="n">
+        <x:f>'Prices'!H295/'Prices'!I295-1</x:f>
+        <x:v>-0.07964746205320716</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="27" customHeight="1">
+      <x:c r="A262" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B262" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C262" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D262" s="20" t="n">
+        <x:f>G247</x:f>
+        <x:v>0.06165674053163025</x:v>
+      </x:c>
+      <x:c r="E262" s="22" t="n">
+        <x:f>'Prices'!H296/'Prices'!G296-1</x:f>
+        <x:v>-0.01044256588761805</x:v>
+      </x:c>
+      <x:c r="F262" s="20" t="n">
+        <x:f>D262*E262</x:f>
+        <x:v>-0.0006438545754173192</x:v>
+      </x:c>
+      <x:c r="G262" s="20" t="n">
+        <x:f>D262*(1+E262)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06010489847529789</x:v>
+      </x:c>
+      <x:c r="H262" s="22" t="n">
+        <x:f>'Prices'!H296/'Prices'!I296-1</x:f>
+        <x:v>-0.16718978865871525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="27" customHeight="1">
+      <x:c r="A263" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B263" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C263" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D263" s="21" t="n">
+        <x:f>G248</x:f>
+        <x:v>0.07575369211680971</x:v>
+      </x:c>
+      <x:c r="E263" s="23" t="n">
+        <x:f>'Prices'!H297/'Prices'!G297-1</x:f>
+        <x:v>0.04832076764907467</x:v>
+      </x:c>
+      <x:c r="F263" s="21" t="n">
+        <x:f>D263*E263</x:f>
+        <x:v>0.0036604765553359016</x:v>
+      </x:c>
+      <x:c r="G263" s="21" t="n">
+        <x:f>D263*(1+E263)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.07823233519825727</x:v>
+      </x:c>
+      <x:c r="H263" s="23" t="n">
+        <x:f>'Prices'!H297/'Prices'!I297-1</x:f>
+        <x:v>0.08398299078667626</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="27" customHeight="1">
+      <x:c r="A264" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B264" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C264" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D264" s="20" t="n">
+        <x:f>G249</x:f>
+        <x:v>0.05441881643358777</x:v>
+      </x:c>
+      <x:c r="E264" s="22" t="n">
+        <x:f>'Prices'!H298/'Prices'!G298-1</x:f>
+        <x:v>0.00048567265662935455</x:v>
+      </x:c>
+      <x:c r="F264" s="20" t="n">
+        <x:f>D264*E264</x:f>
+        <x:v>0.00002642973114792575</x:v>
+      </x:c>
+      <x:c r="G264" s="20" t="n">
+        <x:f>D264*(1+E264)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.05363499762234752</x:v>
+      </x:c>
+      <x:c r="H264" s="22" t="n">
+        <x:f>'Prices'!H298/'Prices'!I298-1</x:f>
+        <x:v>-0.25683638375141304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="27" customHeight="1">
+      <x:c r="A265" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B265" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C265" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D265" s="21" t="n">
+        <x:f>G250</x:f>
+        <x:v>0.060641339189069256</x:v>
+      </x:c>
+      <x:c r="E265" s="23" t="n">
+        <x:f>'Prices'!H299/'Prices'!G299-1</x:f>
+        <x:v>0.005342399222923788</x:v>
+      </x:c>
+      <x:c r="F265" s="21" t="n">
+        <x:f>D265*E265</x:f>
+        <x:v>0.0003239702433607415</x:v>
+      </x:c>
+      <x:c r="G265" s="21" t="n">
+        <x:f>D265*(1+E265)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.060058029980438736</x:v>
+      </x:c>
+      <x:c r="H265" s="23" t="n">
+        <x:f>'Prices'!H299/'Prices'!I299-1</x:f>
+        <x:v>-0.1678391959798995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="27" customHeight="1">
+      <x:c r="A266" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B266" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C266" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D266" s="20" t="n">
+        <x:f>G251</x:f>
+        <x:v>0.07551999465624695</x:v>
+      </x:c>
+      <x:c r="E266" s="22" t="n">
+        <x:f>'Prices'!H300/'Prices'!G300-1</x:f>
+        <x:v>0.032710280373831724</x:v>
+      </x:c>
+      <x:c r="F266" s="20" t="n">
+        <x:f>D266*E266</x:f>
+        <x:v>0.0024702801990361114</x:v>
+      </x:c>
+      <x:c r="G266" s="20" t="n">
+        <x:f>D266*(1+E266)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.07682963162243318</x:v>
+      </x:c>
+      <x:c r="H266" s="22" t="n">
+        <x:f>'Prices'!H300/'Prices'!I300-1</x:f>
+        <x:v>0.06454720616570331</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="27" customHeight="1">
+      <x:c r="A267" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B267" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C267" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D267" s="21" t="n">
+        <x:f>G252</x:f>
+        <x:v>0.07071715107546364</x:v>
+      </x:c>
+      <x:c r="E267" s="23" t="n">
+        <x:f>'Prices'!H301/'Prices'!G301-1</x:f>
+        <x:v>-0.014161775963255963</x:v>
+      </x:c>
+      <x:c r="F267" s="21" t="n">
+        <x:f>D267*E267</x:f>
+        <x:v>-0.0010014804502904416</x:v>
+      </x:c>
+      <x:c r="G267" s="21" t="n">
+        <x:f>D267*(1+E267)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06867816919970902</x:v>
+      </x:c>
+      <x:c r="H267" s="23" t="n">
+        <x:f>'Prices'!H301/'Prices'!I301-1</x:f>
+        <x:v>-0.04839901477832509</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="27" customHeight="1">
+      <x:c r="A268" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B268" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C268" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D268" s="20" t="n">
+        <x:f>G253</x:f>
+        <x:v>0.06540780618478274</x:v>
+      </x:c>
+      <x:c r="E268" s="22" t="n">
+        <x:f>'Prices'!H302/'Prices'!G302-1</x:f>
+        <x:v>0.001440144014401623</x:v>
+      </x:c>
+      <x:c r="F268" s="20" t="n">
+        <x:f>D268*E268</x:f>
+        <x:v>0.00009419666057215633</x:v>
+      </x:c>
+      <x:c r="G268" s="20" t="n">
+        <x:f>D268*(1+E268)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06452720878953648</x:v>
+      </x:c>
+      <x:c r="H268" s="22" t="n">
+        <x:f>'Prices'!H302/'Prices'!I302-1</x:f>
+        <x:v>-0.10591449694631949</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="27" customHeight="1">
+      <x:c r="A269" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B269" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C269" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D269" s="21" t="n">
+        <x:f>G254</x:f>
+        <x:v>0.053220761743184845</x:v>
+      </x:c>
+      <x:c r="E269" s="23" t="n">
+        <x:f>'Prices'!H303/'Prices'!G303-1</x:f>
+        <x:v>0.000673627484001349</x:v>
+      </x:c>
+      <x:c r="F269" s="21" t="n">
+        <x:f>D269*E269</x:f>
+        <x:v>0.000035850967829696855</x:v>
+      </x:c>
+      <x:c r="G269" s="21" t="n">
+        <x:f>D269*(1+E269)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.052464053289186074</x:v>
+      </x:c>
+      <x:c r="H269" s="23" t="n">
+        <x:f>'Prices'!H303/'Prices'!I303-1</x:f>
+        <x:v>-0.27306092488377776</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="27" customHeight="1">
+      <x:c r="A270" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B270" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C270" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D270" s="20" t="n">
+        <x:f>G255</x:f>
+        <x:v>0.0603843612516389</x:v>
+      </x:c>
+      <x:c r="E270" s="22" t="n">
+        <x:f>'Prices'!H304/'Prices'!G304-1</x:f>
+        <x:v>0.04265041888804255</x:v>
+      </x:c>
+      <x:c r="F270" s="20" t="n">
+        <x:f>D270*E270</x:f>
+        <x:v>0.0025754183016692845</x:v>
+      </x:c>
+      <x:c r="G270" s="20" t="n">
+        <x:f>D270*(1+E270)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.062022818602524746</x:v>
+      </x:c>
+      <x:c r="H270" s="22" t="n">
+        <x:f>'Prices'!H304/'Prices'!I304-1</x:f>
+        <x:v>-0.14061519146264911</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="27" customHeight="1">
+      <x:c r="A271" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B271" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C271" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D271" s="21" t="n">
+        <x:f>G256</x:f>
+        <x:v>0.07055585407516626</x:v>
+      </x:c>
+      <x:c r="E271" s="23" t="n">
+        <x:f>'Prices'!H305/'Prices'!G305-1</x:f>
+        <x:v>0.008870948816033453</x:v>
+      </x:c>
+      <x:c r="F271" s="21" t="n">
+        <x:f>D271*E271</x:f>
+        <x:v>0.0006258973701723252</x:v>
+      </x:c>
+      <x:c r="G271" s="21" t="n">
+        <x:f>D271*(1+E271)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.07012243195620053</x:v>
+      </x:c>
+      <x:c r="H271" s="23" t="n">
+        <x:f>'Prices'!H305/'Prices'!I305-1</x:f>
+        <x:v>-0.028387388405469505</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="27" customHeight="1">
+      <x:c r="A272" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B272" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C272" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D272" s="20" t="n">
+        <x:f>G257</x:f>
+        <x:v>0.06919286895463123</x:v>
+      </x:c>
+      <x:c r="E272" s="22" t="n">
+        <x:f>'Prices'!H306/'Prices'!G306-1</x:f>
+        <x:v>0.01791277258566959</x:v>
+      </x:c>
+      <x:c r="F272" s="20" t="n">
+        <x:f>D272*E272</x:f>
+        <x:v>0.0012394361261343467</x:v>
+      </x:c>
+      <x:c r="G272" s="20" t="n">
+        <x:f>D272*(1+E272)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06938413877518841</x:v>
+      </x:c>
+      <x:c r="H272" s="22" t="n">
+        <x:f>'Prices'!H306/'Prices'!I306-1</x:f>
+        <x:v>-0.038617138653916916</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="27" customHeight="1">
+      <x:c r="A273" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B273" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C273" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D273" s="21" t="n">
+        <x:f>G258</x:f>
+        <x:v>0.07195359539435489</x:v>
+      </x:c>
+      <x:c r="E273" s="23" t="n">
+        <x:f>'Prices'!H307/'Prices'!G307-1</x:f>
+        <x:v>0.046441341733356234</x:v>
+      </x:c>
+      <x:c r="F273" s="21" t="n">
+        <x:f>D273*E273</x:f>
+        <x:v>0.0033416215126528827</x:v>
+      </x:c>
+      <x:c r="G273" s="21" t="n">
+        <x:f>D273*(1+E273)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.07417468124879598</x:v>
+      </x:c>
+      <x:c r="H273" s="23" t="n">
+        <x:f>'Prices'!H307/'Prices'!I307-1</x:f>
+        <x:v>0.027760357874493158</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="27" customHeight="1">
+      <x:c r="A274" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B274" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C274" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D274" s="20" t="n">
+        <x:f>G259</x:f>
+        <x:v>0.06530972100465764</x:v>
+      </x:c>
+      <x:c r="E274" s="22" t="n">
+        <x:f>'Prices'!H308/'Prices'!G308-1</x:f>
+        <x:v>-0.011925370263512258</x:v>
+      </x:c>
+      <x:c r="F274" s="20" t="n">
+        <x:f>D274*E274</x:f>
+        <x:v>-0.0007788426047872261</x:v>
+      </x:c>
+      <x:c r="G274" s="20" t="n">
+        <x:f>D274*(1+E274)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.06357053651796724</x:v>
+      </x:c>
+      <x:c r="H274" s="22" t="n">
+        <x:f>'Prices'!H308/'Prices'!I308-1</x:f>
+        <x:v>-0.11917009602194784</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="27" customHeight="1">
+      <x:c r="A275" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B275" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C275" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D275" s="21" t="n">
+        <x:f>G260</x:f>
+        <x:v>0.07846270516255746</x:v>
+      </x:c>
+      <x:c r="E275" s="23" t="n">
+        <x:f>'Prices'!H309/'Prices'!G309-1</x:f>
+        <x:v>0.03206034889203213</x:v>
+      </x:c>
+      <x:c r="F275" s="21" t="n">
+        <x:f>D275*E275</x:f>
+        <x:v>0.002515541702524243</x:v>
+      </x:c>
+      <x:c r="G275" s="21" t="n">
+        <x:f>D275*(1+E275)/(1+SUM($F$261:$F$275))</x:f>
+        <x:v>0.07977313694071736</x:v>
+      </x:c>
+      <x:c r="H275" s="23" t="n">
+        <x:f>'Prices'!H309/'Prices'!I309-1</x:f>
+        <x:v>0.10533225610987684</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -20415,7 +21571,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90b0f52b5e1b4f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c3949a75bb4701"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31590,6 +32746,654 @@
       </x:c>
       <x:c r="M294" s="14" t="str"/>
     </x:row>
+    <x:row r="295" ht="50" customHeight="1">
+      <x:c r="A295" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B295" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C295" s="33" t="n">
+        <x:v>5639</x:v>
+      </x:c>
+      <x:c r="D295" s="33" t="n">
+        <x:v>5639</x:v>
+      </x:c>
+      <x:c r="E295" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F295" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G295" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H295" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I295" s="32" t="str">
+        <x:f>IF(AND(G295=H295,C295&gt;0,ABS(C295-'Prices'!H295)&lt;=MAX(0.01,'Prices'!H295*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J295" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K295" s="16" t="str"/>
+      <x:c r="L295" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M295" s="16" t="str"/>
+    </x:row>
+    <x:row r="296" ht="50" customHeight="1">
+      <x:c r="A296" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B296" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C296" s="17" t="n">
+        <x:v>3980</x:v>
+      </x:c>
+      <x:c r="D296" s="17" t="n">
+        <x:v>3980</x:v>
+      </x:c>
+      <x:c r="E296" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F296" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G296" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H296" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I296" s="31" t="str">
+        <x:f>IF(AND(G296=H296,C296&gt;0,ABS(C296-'Prices'!H296)&lt;=MAX(0.01,'Prices'!H296*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J296" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K296" s="14" t="str"/>
+      <x:c r="L296" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M296" s="14" t="str"/>
+    </x:row>
+    <x:row r="297" ht="50" customHeight="1">
+      <x:c r="A297" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B297" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C297" s="33" t="n">
+        <x:v>30.59</x:v>
+      </x:c>
+      <x:c r="D297" s="33" t="n">
+        <x:v>30.59</x:v>
+      </x:c>
+      <x:c r="E297" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F297" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G297" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H297" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I297" s="32" t="str">
+        <x:f>IF(AND(G297=H297,C297&gt;0,ABS(C297-'Prices'!H297)&lt;=MAX(0.01,'Prices'!H297*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J297" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K297" s="16" t="str"/>
+      <x:c r="L297" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M297" s="16" t="str"/>
+    </x:row>
+    <x:row r="298" ht="50" customHeight="1">
+      <x:c r="A298" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B298" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C298" s="17" t="n">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="D298" s="17" t="n">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="E298" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F298" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G298" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H298" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I298" s="31" t="str">
+        <x:f>IF(AND(G298=H298,C298&gt;0,ABS(C298-'Prices'!H298)&lt;=MAX(0.01,'Prices'!H298*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J298" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K298" s="14" t="str"/>
+      <x:c r="L298" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M298" s="14" t="str"/>
+    </x:row>
+    <x:row r="299" ht="50" customHeight="1">
+      <x:c r="A299" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B299" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C299" s="33" t="n">
+        <x:v>4140</x:v>
+      </x:c>
+      <x:c r="D299" s="33" t="n">
+        <x:v>4140</x:v>
+      </x:c>
+      <x:c r="E299" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F299" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G299" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H299" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I299" s="32" t="str">
+        <x:f>IF(AND(G299=H299,C299&gt;0,ABS(C299-'Prices'!H299)&lt;=MAX(0.01,'Prices'!H299*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J299" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K299" s="16" t="str"/>
+      <x:c r="L299" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M299" s="16" t="str"/>
+    </x:row>
+    <x:row r="300" ht="50" customHeight="1">
+      <x:c r="A300" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B300" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C300" s="17" t="n">
+        <x:v>55.25</x:v>
+      </x:c>
+      <x:c r="D300" s="17" t="n">
+        <x:v>55.25</x:v>
+      </x:c>
+      <x:c r="E300" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F300" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G300" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H300" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I300" s="31" t="str">
+        <x:f>IF(AND(G300=H300,C300&gt;0,ABS(C300-'Prices'!H300)&lt;=MAX(0.01,'Prices'!H300*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J300" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K300" s="14" t="str"/>
+      <x:c r="L300" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M300" s="14" t="str"/>
+    </x:row>
+    <x:row r="301" ht="50" customHeight="1">
+      <x:c r="A301" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B301" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C301" s="33" t="n">
+        <x:v>77270</x:v>
+      </x:c>
+      <x:c r="D301" s="33" t="n">
+        <x:v>77270</x:v>
+      </x:c>
+      <x:c r="E301" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F301" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G301" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H301" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I301" s="32" t="str">
+        <x:f>IF(AND(G301=H301,C301&gt;0,ABS(C301-'Prices'!H301)&lt;=MAX(0.01,'Prices'!H301*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J301" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K301" s="16" t="str"/>
+      <x:c r="L301" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M301" s="16" t="str"/>
+    </x:row>
+    <x:row r="302" ht="50" customHeight="1">
+      <x:c r="A302" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B302" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C302" s="17" t="n">
+        <x:v>55.63</x:v>
+      </x:c>
+      <x:c r="D302" s="17" t="n">
+        <x:v>55.63</x:v>
+      </x:c>
+      <x:c r="E302" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F302" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G302" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H302" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I302" s="31" t="str">
+        <x:f>IF(AND(G302=H302,C302&gt;0,ABS(C302-'Prices'!H302)&lt;=MAX(0.01,'Prices'!H302*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J302" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K302" s="14" t="str"/>
+      <x:c r="L302" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M302" s="14" t="str"/>
+    </x:row>
+    <x:row r="303" ht="50" customHeight="1">
+      <x:c r="A303" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B303" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C303" s="33" t="n">
+        <x:v>29.71</x:v>
+      </x:c>
+      <x:c r="D303" s="33" t="n">
+        <x:v>29.71</x:v>
+      </x:c>
+      <x:c r="E303" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F303" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G303" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H303" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I303" s="32" t="str">
+        <x:f>IF(AND(OR(G303=H303,AND(B303="OUST",G303="XNAS",H303="XNYS",LEFT(M303,34)="ouster-marketstack-legacy-nyse-tag")),C303&gt;0,ABS(C303-'Prices'!H303)&lt;=MAX(0.01,'Prices'!H303*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J303" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K303" s="16" t="str"/>
+      <x:c r="L303" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M303" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="50" customHeight="1">
+      <x:c r="A304" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B304" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C304" s="17" t="n">
+        <x:v>13.69</x:v>
+      </x:c>
+      <x:c r="D304" s="17" t="n">
+        <x:v>13.69</x:v>
+      </x:c>
+      <x:c r="E304" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F304" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G304" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H304" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I304" s="31" t="str">
+        <x:f>IF(AND(G304=H304,C304&gt;0,ABS(C304-'Prices'!H304)&lt;=MAX(0.01,'Prices'!H304*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J304" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K304" s="14" t="str"/>
+      <x:c r="L304" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M304" s="14" t="str"/>
+    </x:row>
+    <x:row r="305" ht="50" customHeight="1">
+      <x:c r="A305" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B305" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C305" s="33" t="n">
+        <x:v>429.89</x:v>
+      </x:c>
+      <x:c r="D305" s="33" t="n">
+        <x:v>429.89</x:v>
+      </x:c>
+      <x:c r="E305" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F305" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G305" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H305" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I305" s="32" t="str">
+        <x:f>IF(AND(G305=H305,C305&gt;0,ABS(C305-'Prices'!H305)&lt;=MAX(0.01,'Prices'!H305*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J305" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K305" s="16" t="str"/>
+      <x:c r="L305" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M305" s="16" t="str"/>
+    </x:row>
+    <x:row r="306" ht="50" customHeight="1">
+      <x:c r="A306" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B306" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C306" s="17" t="n">
+        <x:v>261.4</x:v>
+      </x:c>
+      <x:c r="D306" s="17" t="n">
+        <x:v>261.4</x:v>
+      </x:c>
+      <x:c r="E306" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F306" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G306" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H306" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I306" s="31" t="str">
+        <x:f>IF(AND(G306=H306,C306&gt;0,ABS(C306-'Prices'!H306)&lt;=MAX(0.01,'Prices'!H306*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J306" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K306" s="14" t="str"/>
+      <x:c r="L306" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M306" s="14" t="str"/>
+    </x:row>
+    <x:row r="307" ht="50" customHeight="1">
+      <x:c r="A307" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B307" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C307" s="33" t="n">
+        <x:v>245.83</x:v>
+      </x:c>
+      <x:c r="D307" s="33" t="n">
+        <x:v>245.83</x:v>
+      </x:c>
+      <x:c r="E307" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F307" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G307" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H307" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I307" s="32" t="str">
+        <x:f>IF(AND(G307=H307,C307&gt;0,ABS(C307-'Prices'!H307)&lt;=MAX(0.01,'Prices'!H307*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J307" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K307" s="16" t="str"/>
+      <x:c r="L307" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M307" s="16" t="str"/>
+    </x:row>
+    <x:row r="308" ht="50" customHeight="1">
+      <x:c r="A308" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B308" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C308" s="17" t="n">
+        <x:v>5137</x:v>
+      </x:c>
+      <x:c r="D308" s="17" t="n">
+        <x:v>5137</x:v>
+      </x:c>
+      <x:c r="E308" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F308" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G308" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H308" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I308" s="31" t="str">
+        <x:f>IF(AND(G308=H308,C308&gt;0,ABS(C308-'Prices'!H308)&lt;=MAX(0.01,'Prices'!H308*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J308" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K308" s="14" t="str"/>
+      <x:c r="L308" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M308" s="14" t="str"/>
+    </x:row>
+    <x:row r="309" ht="50" customHeight="1">
+      <x:c r="A309" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B309" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C309" s="33" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="D309" s="33" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="E309" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F309" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G309" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H309" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I309" s="32" t="str">
+        <x:f>IF(AND(G309=H309,C309&gt;0,ABS(C309-'Prices'!H309)&lt;=MAX(0.01,'Prices'!H309*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J309" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K309" s="16" t="str"/>
+      <x:c r="L309" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M309" s="16" t="str"/>
+    </x:row>
+    <x:row r="310" ht="50" customHeight="1">
+      <x:c r="A310" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B310" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C310" s="17" t="n">
+        <x:v>7676.77</x:v>
+      </x:c>
+      <x:c r="D310" s="17" t="n">
+        <x:v>7676.77</x:v>
+      </x:c>
+      <x:c r="E310" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F310" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G310" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H310" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I310" s="31" t="str">
+        <x:f>IF(AND(G310=H310,C310&gt;0,ABS(C310-'Prices'!H310)&lt;=MAX(0.01,'Prices'!H310*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J310" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K310" s="14" t="str"/>
+      <x:c r="L310" s="38" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M310" s="14" t="str"/>
+    </x:row>
+    <x:row r="311" ht="50" customHeight="1">
+      <x:c r="A311" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B311" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C311" s="33" t="n">
+        <x:v>26169.3809</x:v>
+      </x:c>
+      <x:c r="D311" s="33" t="n">
+        <x:v>26169.3809</x:v>
+      </x:c>
+      <x:c r="E311" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F311" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G311" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H311" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I311" s="32" t="str">
+        <x:f>IF(AND(G311=H311,C311&gt;0,ABS(C311-'Prices'!H311)&lt;=MAX(0.01,'Prices'!H311*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J311" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-27T11-26-35-870Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K311" s="16" t="str"/>
+      <x:c r="L311" s="39" t="n">
+        <x:v>46322.47680405092</x:v>
+      </x:c>
+      <x:c r="M311" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -31597,7 +33401,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98066f6298c54dfd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7457bf2abf7a4fd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40067,6 +41871,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="295" ht="27" customHeight="1">
+      <x:c r="A295" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B295" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C295" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D295" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E295" s="18" t="n">
+        <x:f>'Source Audit'!E295</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F295" s="41" t="n">
+        <x:f>'Source Audit'!F295</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G295" s="12" t="str">
+        <x:f>IF(AND(E295=0,F295=1,'Source Audit'!I295&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H295" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="27" customHeight="1">
+      <x:c r="A296" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B296" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C296" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D296" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E296" s="19" t="n">
+        <x:f>'Source Audit'!E296</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F296" s="40" t="n">
+        <x:f>'Source Audit'!F296</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G296" s="11" t="str">
+        <x:f>IF(AND(E296=0,F296=1,'Source Audit'!I296&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H296" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="27" customHeight="1">
+      <x:c r="A297" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B297" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C297" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D297" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E297" s="18" t="n">
+        <x:f>'Source Audit'!E297</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F297" s="41" t="n">
+        <x:f>'Source Audit'!F297</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G297" s="12" t="str">
+        <x:f>IF(AND(E297=0,F297=1,'Source Audit'!I297&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H297" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="27" customHeight="1">
+      <x:c r="A298" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B298" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C298" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D298" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E298" s="19" t="n">
+        <x:f>'Source Audit'!E298</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F298" s="40" t="n">
+        <x:f>'Source Audit'!F298</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G298" s="11" t="str">
+        <x:f>IF(AND(E298=0,F298=1,'Source Audit'!I298&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H298" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="27" customHeight="1">
+      <x:c r="A299" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B299" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C299" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D299" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E299" s="18" t="n">
+        <x:f>'Source Audit'!E299</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F299" s="41" t="n">
+        <x:f>'Source Audit'!F299</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G299" s="12" t="str">
+        <x:f>IF(AND(E299=0,F299=1,'Source Audit'!I299&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H299" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="27" customHeight="1">
+      <x:c r="A300" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B300" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C300" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D300" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E300" s="19" t="n">
+        <x:f>'Source Audit'!E300</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F300" s="40" t="n">
+        <x:f>'Source Audit'!F300</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G300" s="11" t="str">
+        <x:f>IF(AND(E300=0,F300=1,'Source Audit'!I300&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H300" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="27" customHeight="1">
+      <x:c r="A301" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B301" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C301" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D301" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E301" s="18" t="n">
+        <x:f>'Source Audit'!E301</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F301" s="41" t="n">
+        <x:f>'Source Audit'!F301</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G301" s="12" t="str">
+        <x:f>IF(AND(E301=0,F301=1,'Source Audit'!I301&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H301" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="27" customHeight="1">
+      <x:c r="A302" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B302" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C302" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D302" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E302" s="19" t="n">
+        <x:f>'Source Audit'!E302</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F302" s="40" t="n">
+        <x:f>'Source Audit'!F302</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G302" s="11" t="str">
+        <x:f>IF(AND(E302=0,F302=1,'Source Audit'!I302&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H302" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="44" customHeight="1">
+      <x:c r="A303" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B303" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C303" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D303" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E303" s="18" t="n">
+        <x:f>'Source Audit'!E303</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F303" s="41" t="n">
+        <x:f>'Source Audit'!F303</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G303" s="12" t="str">
+        <x:f>IF(AND(E303=0,F303=1,'Source Audit'!I303&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H303" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="27" customHeight="1">
+      <x:c r="A304" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B304" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C304" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D304" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E304" s="19" t="n">
+        <x:f>'Source Audit'!E304</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F304" s="40" t="n">
+        <x:f>'Source Audit'!F304</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G304" s="11" t="str">
+        <x:f>IF(AND(E304=0,F304=1,'Source Audit'!I304&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H304" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="27" customHeight="1">
+      <x:c r="A305" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B305" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C305" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D305" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E305" s="18" t="n">
+        <x:f>'Source Audit'!E305</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F305" s="41" t="n">
+        <x:f>'Source Audit'!F305</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G305" s="12" t="str">
+        <x:f>IF(AND(E305=0,F305=1,'Source Audit'!I305&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H305" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="27" customHeight="1">
+      <x:c r="A306" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B306" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C306" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D306" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E306" s="19" t="n">
+        <x:f>'Source Audit'!E306</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F306" s="40" t="n">
+        <x:f>'Source Audit'!F306</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G306" s="11" t="str">
+        <x:f>IF(AND(E306=0,F306=1,'Source Audit'!I306&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H306" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="27" customHeight="1">
+      <x:c r="A307" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B307" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C307" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D307" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E307" s="18" t="n">
+        <x:f>'Source Audit'!E307</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F307" s="41" t="n">
+        <x:f>'Source Audit'!F307</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G307" s="12" t="str">
+        <x:f>IF(AND(E307=0,F307=1,'Source Audit'!I307&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H307" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="27" customHeight="1">
+      <x:c r="A308" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B308" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C308" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D308" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E308" s="19" t="n">
+        <x:f>'Source Audit'!E308</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F308" s="40" t="n">
+        <x:f>'Source Audit'!F308</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G308" s="11" t="str">
+        <x:f>IF(AND(E308=0,F308=1,'Source Audit'!I308&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H308" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="27" customHeight="1">
+      <x:c r="A309" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B309" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C309" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D309" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E309" s="18" t="n">
+        <x:f>'Source Audit'!E309</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F309" s="41" t="n">
+        <x:f>'Source Audit'!F309</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G309" s="12" t="str">
+        <x:f>IF(AND(E309=0,F309=1,'Source Audit'!I309&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H309" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="27" customHeight="1">
+      <x:c r="A310" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B310" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C310" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D310" s="8" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E310" s="19" t="n">
+        <x:f>'Source Audit'!E310</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F310" s="40" t="n">
+        <x:f>'Source Audit'!F310</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G310" s="11" t="str">
+        <x:f>IF(AND(E310=0,F310=1,'Source Audit'!I310&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H310" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="27" customHeight="1">
+      <x:c r="A311" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="B311" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C311" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D311" s="9" t="n">
+        <x:v>46321</x:v>
+      </x:c>
+      <x:c r="E311" s="18" t="n">
+        <x:f>'Source Audit'!E311</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F311" s="41" t="n">
+        <x:f>'Source Audit'!F311</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G311" s="12" t="str">
+        <x:f>IF(AND(E311=0,F311=1,'Source Audit'!I311&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H311" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -40074,7 +42371,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6fa397610514ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70571c29aa1d4e59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 27, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 291 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Both the shared-checkout and exact main-based
publication candidate production builds and article-preview checks passed.
These results are documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8437e955c5274fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Ree12527931bb481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Rf2422b7d20234e3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R1d2f15a332e14d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rcdbb2266a93b4998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R95f3db0ca9c244cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R4cbedd9c43b44ccd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R24dc70abf7bd48fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R345e558209b44efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R4fa0cdd4e8a349fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H275" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H290" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H311" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -2103,6 +2103,85 @@
         <x:v>-5.013805170739927</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="40" customHeight="1">
+      <x:c r="A24" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B24" s="19" t="n">
+        <x:f>B23*(1+SUM('Returns and Contributions'!F276:F290))</x:f>
+        <x:v>937.6004397134458</x:v>
+      </x:c>
+      <x:c r="C24" s="20" t="n">
+        <x:f>B24/B23-1</x:f>
+        <x:v>0.015015998938274322</x:v>
+      </x:c>
+      <x:c r="D24" s="20" t="n">
+        <x:f>B24/$B$6-1</x:f>
+        <x:v>-0.062399560286554245</x:v>
+      </x:c>
+      <x:c r="E24" s="19" t="n">
+        <x:f>1000*'Prices'!H327/'Prices'!I327</x:f>
+        <x:v>1007.3241200294791</x:v>
+      </x:c>
+      <x:c r="F24" s="20" t="n">
+        <x:f>E24/E23-1</x:f>
+        <x:v>0.005969958719617807</x:v>
+      </x:c>
+      <x:c r="G24" s="20" t="n">
+        <x:f>E24/1000-1</x:f>
+        <x:v>0.007324120029479131</x:v>
+      </x:c>
+      <x:c r="H24" s="19" t="n">
+        <x:f>1000*'Prices'!H328/'Prices'!I328</x:f>
+        <x:v>985.3456711541696</x:v>
+      </x:c>
+      <x:c r="I24" s="20" t="n">
+        <x:f>H24/H23-1</x:f>
+        <x:v>0.011785895936116786</x:v>
+      </x:c>
+      <x:c r="J24" s="20" t="n">
+        <x:f>H24/1000-1</x:f>
+        <x:v>-0.0146543288458304</x:v>
+      </x:c>
+      <x:c r="K24" s="24" t="n">
+        <x:f>(C24-F24)*100</x:f>
+        <x:v>0.9046040218656515</x:v>
+      </x:c>
+      <x:c r="L24" s="24" t="n">
+        <x:f>(C24-I24)*100</x:f>
+        <x:v>0.3230103002157536</x:v>
+      </x:c>
+      <x:c r="M24" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G276:G290)</x:f>
+        <x:v>0.9999999999999994</x:v>
+      </x:c>
+      <x:c r="N24" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F276:F290)-C24</x:f>
+        <x:v>1.9081958235744878e-17</x:v>
+      </x:c>
+      <x:c r="O24" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P24" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I312:I328,"Mismatch")=0,IF(COUNTIF('Source Audit'!I312:I328,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q24" s="29" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="R24" s="28" t="n">
+        <x:f>B24-1000*('Prices'!H312/'Prices'!H6+'Prices'!H313/'Prices'!H7+'Prices'!H314/'Prices'!H8+'Prices'!H315/'Prices'!H9+'Prices'!H316/'Prices'!H10+'Prices'!H317/'Prices'!H11+'Prices'!H318/'Prices'!H12+'Prices'!H319/'Prices'!H13+'Prices'!H320/'Prices'!H14+'Prices'!H321/'Prices'!H15+'Prices'!H322/'Prices'!H16+'Prices'!H323/'Prices'!H17+'Prices'!H324/'Prices'!H18+'Prices'!H325/'Prices'!H19+'Prices'!H326/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S24" s="24" t="n">
+        <x:f>(D24-G24)*100</x:f>
+        <x:v>-6.972368031603338</x:v>
+      </x:c>
+      <x:c r="T24" s="24" t="n">
+        <x:f>(D24-J24)*100</x:f>
+        <x:v>-4.7745231440723845</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -2110,7 +2189,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R611178679d4e46a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f71bd91509e4acb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13188,6 +13267,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="312" ht="27" customHeight="1">
+      <x:c r="A312" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B312" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C312" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D312" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E312" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F312" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G312" s="17" t="n">
+        <x:f>H295</x:f>
+        <x:v>5639</x:v>
+      </x:c>
+      <x:c r="H312" s="34" t="n">
+        <x:v>5820</x:v>
+      </x:c>
+      <x:c r="I312" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J312" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K312" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="27" customHeight="1">
+      <x:c r="A313" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B313" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C313" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D313" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E313" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F313" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G313" s="33" t="n">
+        <x:f>H296</x:f>
+        <x:v>3980</x:v>
+      </x:c>
+      <x:c r="H313" s="35" t="n">
+        <x:v>4090</x:v>
+      </x:c>
+      <x:c r="I313" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J313" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K313" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="27" customHeight="1">
+      <x:c r="A314" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B314" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C314" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D314" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E314" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F314" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G314" s="17" t="n">
+        <x:f>H297</x:f>
+        <x:v>30.59</x:v>
+      </x:c>
+      <x:c r="H314" s="34" t="n">
+        <x:v>28.45</x:v>
+      </x:c>
+      <x:c r="I314" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J314" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K314" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="27" customHeight="1">
+      <x:c r="A315" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B315" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C315" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D315" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E315" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F315" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G315" s="33" t="n">
+        <x:f>H298</x:f>
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="H315" s="35" t="n">
+        <x:v>323.68</x:v>
+      </x:c>
+      <x:c r="I315" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J315" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K315" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="27" customHeight="1">
+      <x:c r="A316" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B316" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C316" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D316" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E316" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F316" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G316" s="17" t="n">
+        <x:f>H299</x:f>
+        <x:v>4140</x:v>
+      </x:c>
+      <x:c r="H316" s="34" t="n">
+        <x:v>4285</x:v>
+      </x:c>
+      <x:c r="I316" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J316" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K316" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="27" customHeight="1">
+      <x:c r="A317" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B317" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C317" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D317" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E317" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F317" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G317" s="33" t="n">
+        <x:f>H300</x:f>
+        <x:v>55.25</x:v>
+      </x:c>
+      <x:c r="H317" s="35" t="n">
+        <x:v>53.31</x:v>
+      </x:c>
+      <x:c r="I317" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J317" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K317" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="27" customHeight="1">
+      <x:c r="A318" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B318" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C318" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D318" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E318" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F318" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G318" s="17" t="n">
+        <x:f>H301</x:f>
+        <x:v>77270</x:v>
+      </x:c>
+      <x:c r="H318" s="34" t="n">
+        <x:v>79080</x:v>
+      </x:c>
+      <x:c r="I318" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J318" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K318" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319" ht="27" customHeight="1">
+      <x:c r="A319" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B319" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C319" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D319" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E319" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F319" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G319" s="33" t="n">
+        <x:f>H302</x:f>
+        <x:v>55.63</x:v>
+      </x:c>
+      <x:c r="H319" s="35" t="n">
+        <x:v>58.22</x:v>
+      </x:c>
+      <x:c r="I319" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J319" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K319" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320" ht="27" customHeight="1">
+      <x:c r="A320" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B320" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C320" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D320" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E320" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F320" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G320" s="17" t="n">
+        <x:f>H303</x:f>
+        <x:v>29.71</x:v>
+      </x:c>
+      <x:c r="H320" s="34" t="n">
+        <x:v>32.79</x:v>
+      </x:c>
+      <x:c r="I320" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J320" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K320" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321" ht="27" customHeight="1">
+      <x:c r="A321" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B321" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C321" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D321" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E321" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F321" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G321" s="33" t="n">
+        <x:f>H304</x:f>
+        <x:v>13.69</x:v>
+      </x:c>
+      <x:c r="H321" s="35" t="n">
+        <x:v>13.35</x:v>
+      </x:c>
+      <x:c r="I321" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J321" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K321" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322" ht="27" customHeight="1">
+      <x:c r="A322" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B322" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C322" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D322" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E322" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F322" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G322" s="17" t="n">
+        <x:f>H305</x:f>
+        <x:v>429.89</x:v>
+      </x:c>
+      <x:c r="H322" s="34" t="n">
+        <x:v>439.2</x:v>
+      </x:c>
+      <x:c r="I322" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J322" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K322" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323" ht="27" customHeight="1">
+      <x:c r="A323" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B323" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C323" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D323" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E323" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F323" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G323" s="33" t="n">
+        <x:f>H306</x:f>
+        <x:v>261.4</x:v>
+      </x:c>
+      <x:c r="H323" s="35" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="I323" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J323" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K323" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324" ht="27" customHeight="1">
+      <x:c r="A324" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B324" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C324" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D324" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E324" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F324" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G324" s="17" t="n">
+        <x:f>H307</x:f>
+        <x:v>245.83</x:v>
+      </x:c>
+      <x:c r="H324" s="34" t="n">
+        <x:v>253.5</x:v>
+      </x:c>
+      <x:c r="I324" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J324" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K324" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325" ht="27" customHeight="1">
+      <x:c r="A325" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B325" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C325" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D325" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E325" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F325" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G325" s="33" t="n">
+        <x:f>H308</x:f>
+        <x:v>5137</x:v>
+      </x:c>
+      <x:c r="H325" s="35" t="n">
+        <x:v>5216</x:v>
+      </x:c>
+      <x:c r="I325" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J325" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K325" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326" ht="27" customHeight="1">
+      <x:c r="A326" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B326" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C326" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D326" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E326" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F326" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G326" s="17" t="n">
+        <x:f>H309</x:f>
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="H326" s="34" t="n">
+        <x:v>109.65</x:v>
+      </x:c>
+      <x:c r="I326" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J326" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K326" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="27" customHeight="1">
+      <x:c r="A327" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B327" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C327" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D327" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E327" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F327" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G327" s="33" t="n">
+        <x:f>H310</x:f>
+        <x:v>7676.77</x:v>
+      </x:c>
+      <x:c r="H327" s="35" t="n">
+        <x:v>7722.6</x:v>
+      </x:c>
+      <x:c r="I327" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J327" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K327" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="27" customHeight="1">
+      <x:c r="A328" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B328" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C328" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D328" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E328" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F328" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G328" s="17" t="n">
+        <x:f>H311</x:f>
+        <x:v>26169.3809</x:v>
+      </x:c>
+      <x:c r="H328" s="34" t="n">
+        <x:v>26477.8105</x:v>
+      </x:c>
+      <x:c r="I328" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J328" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="K328" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -13195,7 +13886,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeef5d0423e34c1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a98f5428dc34294"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21564,6 +22255,471 @@
         <x:v>0.10533225610987684</x:v>
       </x:c>
     </x:row>
+    <x:row r="276" ht="27" customHeight="1">
+      <x:c r="A276" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B276" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C276" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D276" s="20" t="n">
+        <x:f>G261</x:f>
+        <x:v>0.06642293178139909</x:v>
+      </x:c>
+      <x:c r="E276" s="22" t="n">
+        <x:f>'Prices'!H312/'Prices'!G312-1</x:f>
+        <x:v>0.032097889696754756</x:v>
+      </x:c>
+      <x:c r="F276" s="20" t="n">
+        <x:f>D276*E276</x:f>
+        <x:v>0.0021320359376544138</x:v>
+      </x:c>
+      <x:c r="G276" s="20" t="n">
+        <x:f>D276*(1+E276)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06754077550576866</x:v>
+      </x:c>
+      <x:c r="H276" s="22" t="n">
+        <x:f>'Prices'!H312/'Prices'!I312-1</x:f>
+        <x:v>-0.050106087808062694</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="27" customHeight="1">
+      <x:c r="A277" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B277" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C277" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D277" s="21" t="n">
+        <x:f>G262</x:f>
+        <x:v>0.06010489847529789</x:v>
+      </x:c>
+      <x:c r="E277" s="23" t="n">
+        <x:f>'Prices'!H313/'Prices'!G313-1</x:f>
+        <x:v>0.027638190954773822</x:v>
+      </x:c>
+      <x:c r="F277" s="21" t="n">
+        <x:f>D277*E277</x:f>
+        <x:v>0.001661190661377577</x:v>
+      </x:c>
+      <x:c r="G277" s="21" t="n">
+        <x:f>D277*(1+E277)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.060852330604920464</x:v>
+      </x:c>
+      <x:c r="H277" s="23" t="n">
+        <x:f>'Prices'!H313/'Prices'!I313-1</x:f>
+        <x:v>-0.1441724210085792</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" ht="27" customHeight="1">
+      <x:c r="A278" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B278" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C278" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D278" s="20" t="n">
+        <x:f>G263</x:f>
+        <x:v>0.07823233519825727</x:v>
+      </x:c>
+      <x:c r="E278" s="22" t="n">
+        <x:f>'Prices'!H314/'Prices'!G314-1</x:f>
+        <x:v>-0.06995750245178167</x:v>
+      </x:c>
+      <x:c r="F278" s="20" t="n">
+        <x:f>D278*E278</x:f>
+        <x:v>-0.005472938781440688</x:v>
+      </x:c>
+      <x:c r="G278" s="20" t="n">
+        <x:f>D278*(1+E278)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.07168300449739144</x:v>
+      </x:c>
+      <x:c r="H278" s="22" t="n">
+        <x:f>'Prices'!H314/'Prices'!I314-1</x:f>
+        <x:v>0.008150248051027598</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="27" customHeight="1">
+      <x:c r="A279" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B279" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C279" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D279" s="21" t="n">
+        <x:f>G264</x:f>
+        <x:v>0.05363499762234752</x:v>
+      </x:c>
+      <x:c r="E279" s="23" t="n">
+        <x:f>'Prices'!H315/'Prices'!G315-1</x:f>
+        <x:v>0.04750809061488681</x:v>
+      </x:c>
+      <x:c r="F279" s="21" t="n">
+        <x:f>D279*E279</x:f>
+        <x:v>0.0025480963271717243</x:v>
+      </x:c>
+      <x:c r="G279" s="21" t="n">
+        <x:f>D279*(1+E279)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.055351929435878654</x:v>
+      </x:c>
+      <x:c r="H279" s="23" t="n">
+        <x:f>'Prices'!H315/'Prices'!I315-1</x:f>
+        <x:v>-0.22153009932898826</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="27" customHeight="1">
+      <x:c r="A280" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B280" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C280" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D280" s="20" t="n">
+        <x:f>G265</x:f>
+        <x:v>0.060058029980438736</x:v>
+      </x:c>
+      <x:c r="E280" s="22" t="n">
+        <x:f>'Prices'!H316/'Prices'!G316-1</x:f>
+        <x:v>0.035024154589371914</x:v>
+      </x:c>
+      <x:c r="F280" s="20" t="n">
+        <x:f>D280*E280</x:f>
+        <x:v>0.0021034817263680195</x:v>
+      </x:c>
+      <x:c r="G280" s="20" t="n">
+        <x:f>D280*(1+E280)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06124190335110861</x:v>
+      </x:c>
+      <x:c r="H280" s="22" t="n">
+        <x:f>'Prices'!H316/'Prices'!I316-1</x:f>
+        <x:v>-0.13869346733668342</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="27" customHeight="1">
+      <x:c r="A281" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B281" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C281" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D281" s="21" t="n">
+        <x:f>G266</x:f>
+        <x:v>0.07682963162243318</x:v>
+      </x:c>
+      <x:c r="E281" s="23" t="n">
+        <x:f>'Prices'!H317/'Prices'!G317-1</x:f>
+        <x:v>-0.03511312217194562</x:v>
+      </x:c>
+      <x:c r="F281" s="21" t="n">
+        <x:f>D281*E281</x:f>
+        <x:v>-0.002697728241584073</x:v>
+      </x:c>
+      <x:c r="G281" s="21" t="n">
+        <x:f>D281*(1+E281)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.073035206793186</x:v>
+      </x:c>
+      <x:c r="H281" s="23" t="n">
+        <x:f>'Prices'!H317/'Prices'!I317-1</x:f>
+        <x:v>0.02716763005780365</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="27" customHeight="1">
+      <x:c r="A282" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B282" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C282" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D282" s="20" t="n">
+        <x:f>G267</x:f>
+        <x:v>0.06867816919970902</x:v>
+      </x:c>
+      <x:c r="E282" s="22" t="n">
+        <x:f>'Prices'!H318/'Prices'!G318-1</x:f>
+        <x:v>0.023424356153746606</x:v>
+      </x:c>
+      <x:c r="F282" s="20" t="n">
+        <x:f>D282*E282</x:f>
+        <x:v>0.0016087418953212548</x:v>
+      </x:c>
+      <x:c r="G282" s="20" t="n">
+        <x:f>D282*(1+E282)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06924709676355023</x:v>
+      </x:c>
+      <x:c r="H282" s="22" t="n">
+        <x:f>'Prices'!H318/'Prices'!I318-1</x:f>
+        <x:v>-0.02610837438423641</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="27" customHeight="1">
+      <x:c r="A283" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B283" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C283" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D283" s="21" t="n">
+        <x:f>G268</x:f>
+        <x:v>0.06452720878953648</x:v>
+      </x:c>
+      <x:c r="E283" s="23" t="n">
+        <x:f>'Prices'!H319/'Prices'!G319-1</x:f>
+        <x:v>0.0465576127988494</x:v>
+      </x:c>
+      <x:c r="F283" s="21" t="n">
+        <x:f>D283*E283</x:f>
+        <x:v>0.003004232801813751</x:v>
+      </x:c>
+      <x:c r="G283" s="21" t="n">
+        <x:f>D283*(1+E283)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06653239127460983</x:v>
+      </x:c>
+      <x:c r="H283" s="23" t="n">
+        <x:f>'Prices'!H319/'Prices'!I319-1</x:f>
+        <x:v>-0.06428801028608166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="27" customHeight="1">
+      <x:c r="A284" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B284" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C284" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D284" s="20" t="n">
+        <x:f>G269</x:f>
+        <x:v>0.052464053289186074</x:v>
+      </x:c>
+      <x:c r="E284" s="22" t="n">
+        <x:f>'Prices'!H320/'Prices'!G320-1</x:f>
+        <x:v>0.10366879838438225</x:v>
+      </x:c>
+      <x:c r="F284" s="20" t="n">
+        <x:f>D284*E284</x:f>
+        <x:v>0.005438885362864118</x:v>
+      </x:c>
+      <x:c r="G284" s="20" t="n">
+        <x:f>D284*(1+E284)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.057046331006228225</x:v>
+      </x:c>
+      <x:c r="H284" s="22" t="n">
+        <x:f>'Prices'!H320/'Prices'!I320-1</x:f>
+        <x:v>-0.19770002446782475</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="27" customHeight="1">
+      <x:c r="A285" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B285" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C285" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D285" s="21" t="n">
+        <x:f>G270</x:f>
+        <x:v>0.062022818602524746</x:v>
+      </x:c>
+      <x:c r="E285" s="23" t="n">
+        <x:f>'Prices'!H321/'Prices'!G321-1</x:f>
+        <x:v>-0.0248356464572681</x:v>
+      </x:c>
+      <x:c r="F285" s="21" t="n">
+        <x:f>D285*E285</x:f>
+        <x:v>-0.0015403767950955757</x:v>
+      </x:c>
+      <x:c r="G285" s="21" t="n">
+        <x:f>D285*(1+E285)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.05958767336740991</x:v>
+      </x:c>
+      <x:c r="H285" s="23" t="n">
+        <x:f>'Prices'!H321/'Prices'!I321-1</x:f>
+        <x:v>-0.16195856873822978</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="27" customHeight="1">
+      <x:c r="A286" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B286" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C286" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D286" s="20" t="n">
+        <x:f>G271</x:f>
+        <x:v>0.07012243195620053</x:v>
+      </x:c>
+      <x:c r="E286" s="22" t="n">
+        <x:f>'Prices'!H322/'Prices'!G322-1</x:f>
+        <x:v>0.02165670287748034</x:v>
+      </x:c>
+      <x:c r="F286" s="20" t="n">
+        <x:f>D286*E286</x:f>
+        <x:v>0.0015186206739217674</x:v>
+      </x:c>
+      <x:c r="G286" s="20" t="n">
+        <x:f>D286*(1+E286)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.07058120532588666</x:v>
+      </x:c>
+      <x:c r="H286" s="22" t="n">
+        <x:f>'Prices'!H322/'Prices'!I322-1</x:f>
+        <x:v>-0.007345462764154154</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="27" customHeight="1">
+      <x:c r="A287" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B287" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C287" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D287" s="21" t="n">
+        <x:f>G272</x:f>
+        <x:v>0.06938413877518841</x:v>
+      </x:c>
+      <x:c r="E287" s="23" t="n">
+        <x:f>'Prices'!H323/'Prices'!G323-1</x:f>
+        <x:v>0.018362662586075107</x:v>
+      </x:c>
+      <x:c r="F287" s="21" t="n">
+        <x:f>D287*E287</x:f>
+        <x:v>0.0012740775291541953</x:v>
+      </x:c>
+      <x:c r="G287" s="21" t="n">
+        <x:f>D287*(1+E287)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06961290893764474</x:v>
+      </x:c>
+      <x:c r="H287" s="23" t="n">
+        <x:f>'Prices'!H323/'Prices'!I323-1</x:f>
+        <x:v>-0.020963589554983453</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="27" customHeight="1">
+      <x:c r="A288" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B288" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C288" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D288" s="20" t="n">
+        <x:f>G273</x:f>
+        <x:v>0.07417468124879598</x:v>
+      </x:c>
+      <x:c r="E288" s="22" t="n">
+        <x:f>'Prices'!H324/'Prices'!G324-1</x:f>
+        <x:v>0.03120042305658366</x:v>
+      </x:c>
+      <x:c r="F288" s="20" t="n">
+        <x:f>D288*E288</x:f>
+        <x:v>0.0023142814350496778</x:v>
+      </x:c>
+      <x:c r="G288" s="20" t="n">
+        <x:f>D288*(1+E288)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.07535739610395752</x:v>
+      </x:c>
+      <x:c r="H288" s="22" t="n">
+        <x:f>'Prices'!H324/'Prices'!I324-1</x:f>
+        <x:v>0.059826915840963224</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="289" ht="27" customHeight="1">
+      <x:c r="A289" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B289" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C289" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D289" s="21" t="n">
+        <x:f>G274</x:f>
+        <x:v>0.06357053651796724</x:v>
+      </x:c>
+      <x:c r="E289" s="23" t="n">
+        <x:f>'Prices'!H325/'Prices'!G325-1</x:f>
+        <x:v>0.015378625656998324</x:v>
+      </x:c>
+      <x:c r="F289" s="21" t="n">
+        <x:f>D289*E289</x:f>
+        <x:v>0.0009776274839243598</x:v>
+      </x:c>
+      <x:c r="G289" s="21" t="n">
+        <x:f>D289*(1+E289)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.06359324785955116</x:v>
+      </x:c>
+      <x:c r="H289" s="23" t="n">
+        <x:f>'Prices'!H325/'Prices'!I325-1</x:f>
+        <x:v>-0.1056241426611797</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="27" customHeight="1">
+      <x:c r="A290" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B290" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C290" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D290" s="20" t="n">
+        <x:f>G275</x:f>
+        <x:v>0.07977313694071736</x:v>
+      </x:c>
+      <x:c r="E290" s="22" t="n">
+        <x:f>'Prices'!H326/'Prices'!G326-1</x:f>
+        <x:v>0.001827318410233092</x:v>
+      </x:c>
+      <x:c r="F290" s="20" t="n">
+        <x:f>D290*E290</x:f>
+        <x:v>0.0001457709217738184</x:v>
+      </x:c>
+      <x:c r="G290" s="20" t="n">
+        <x:f>D290*(1+E290)/(1+SUM($F$276:$F$290))</x:f>
+        <x:v>0.07873659917290747</x:v>
+      </x:c>
+      <x:c r="H290" s="22" t="n">
+        <x:f>'Prices'!H326/'Prices'!I326-1</x:f>
+        <x:v>0.10735205009089088</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -21571,7 +22727,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c3949a75bb4701"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08b3de111cc94505"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33394,6 +34550,654 @@
       </x:c>
       <x:c r="M311" s="16" t="str"/>
     </x:row>
+    <x:row r="312" ht="50" customHeight="1">
+      <x:c r="A312" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B312" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C312" s="17" t="n">
+        <x:v>5820</x:v>
+      </x:c>
+      <x:c r="D312" s="17" t="n">
+        <x:v>5820</x:v>
+      </x:c>
+      <x:c r="E312" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F312" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G312" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H312" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I312" s="31" t="str">
+        <x:f>IF(AND(G312=H312,C312&gt;0,ABS(C312-'Prices'!H312)&lt;=MAX(0.01,'Prices'!H312*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J312" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K312" s="14" t="str"/>
+      <x:c r="L312" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M312" s="14" t="str"/>
+    </x:row>
+    <x:row r="313" ht="50" customHeight="1">
+      <x:c r="A313" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B313" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C313" s="33" t="n">
+        <x:v>4090</x:v>
+      </x:c>
+      <x:c r="D313" s="33" t="n">
+        <x:v>4090</x:v>
+      </x:c>
+      <x:c r="E313" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F313" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G313" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H313" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I313" s="32" t="str">
+        <x:f>IF(AND(G313=H313,C313&gt;0,ABS(C313-'Prices'!H313)&lt;=MAX(0.01,'Prices'!H313*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J313" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K313" s="16" t="str"/>
+      <x:c r="L313" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M313" s="16" t="str"/>
+    </x:row>
+    <x:row r="314" ht="50" customHeight="1">
+      <x:c r="A314" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B314" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C314" s="17" t="n">
+        <x:v>28.45</x:v>
+      </x:c>
+      <x:c r="D314" s="17" t="n">
+        <x:v>28.45</x:v>
+      </x:c>
+      <x:c r="E314" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F314" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G314" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H314" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I314" s="31" t="str">
+        <x:f>IF(AND(G314=H314,C314&gt;0,ABS(C314-'Prices'!H314)&lt;=MAX(0.01,'Prices'!H314*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J314" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K314" s="14" t="str"/>
+      <x:c r="L314" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M314" s="14" t="str"/>
+    </x:row>
+    <x:row r="315" ht="50" customHeight="1">
+      <x:c r="A315" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B315" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C315" s="33" t="n">
+        <x:v>323.68</x:v>
+      </x:c>
+      <x:c r="D315" s="33" t="n">
+        <x:v>323.68</x:v>
+      </x:c>
+      <x:c r="E315" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F315" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G315" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H315" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I315" s="32" t="str">
+        <x:f>IF(AND(G315=H315,C315&gt;0,ABS(C315-'Prices'!H315)&lt;=MAX(0.01,'Prices'!H315*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J315" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K315" s="16" t="str"/>
+      <x:c r="L315" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M315" s="16" t="str"/>
+    </x:row>
+    <x:row r="316" ht="50" customHeight="1">
+      <x:c r="A316" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B316" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C316" s="17" t="n">
+        <x:v>4285</x:v>
+      </x:c>
+      <x:c r="D316" s="17" t="n">
+        <x:v>4285</x:v>
+      </x:c>
+      <x:c r="E316" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F316" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G316" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H316" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I316" s="31" t="str">
+        <x:f>IF(AND(G316=H316,C316&gt;0,ABS(C316-'Prices'!H316)&lt;=MAX(0.01,'Prices'!H316*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J316" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K316" s="14" t="str"/>
+      <x:c r="L316" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M316" s="14" t="str"/>
+    </x:row>
+    <x:row r="317" ht="50" customHeight="1">
+      <x:c r="A317" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B317" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C317" s="33" t="n">
+        <x:v>53.31</x:v>
+      </x:c>
+      <x:c r="D317" s="33" t="n">
+        <x:v>53.31</x:v>
+      </x:c>
+      <x:c r="E317" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F317" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G317" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H317" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I317" s="32" t="str">
+        <x:f>IF(AND(G317=H317,C317&gt;0,ABS(C317-'Prices'!H317)&lt;=MAX(0.01,'Prices'!H317*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J317" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K317" s="16" t="str"/>
+      <x:c r="L317" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M317" s="16" t="str"/>
+    </x:row>
+    <x:row r="318" ht="50" customHeight="1">
+      <x:c r="A318" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B318" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C318" s="17" t="n">
+        <x:v>79080</x:v>
+      </x:c>
+      <x:c r="D318" s="17" t="n">
+        <x:v>79080</x:v>
+      </x:c>
+      <x:c r="E318" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F318" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G318" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H318" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I318" s="31" t="str">
+        <x:f>IF(AND(G318=H318,C318&gt;0,ABS(C318-'Prices'!H318)&lt;=MAX(0.01,'Prices'!H318*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J318" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K318" s="14" t="str"/>
+      <x:c r="L318" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M318" s="14" t="str"/>
+    </x:row>
+    <x:row r="319" ht="50" customHeight="1">
+      <x:c r="A319" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B319" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C319" s="33" t="n">
+        <x:v>58.22</x:v>
+      </x:c>
+      <x:c r="D319" s="33" t="n">
+        <x:v>58.22</x:v>
+      </x:c>
+      <x:c r="E319" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F319" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G319" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H319" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I319" s="32" t="str">
+        <x:f>IF(AND(G319=H319,C319&gt;0,ABS(C319-'Prices'!H319)&lt;=MAX(0.01,'Prices'!H319*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J319" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K319" s="16" t="str"/>
+      <x:c r="L319" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M319" s="16" t="str"/>
+    </x:row>
+    <x:row r="320" ht="50" customHeight="1">
+      <x:c r="A320" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B320" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C320" s="17" t="n">
+        <x:v>32.79</x:v>
+      </x:c>
+      <x:c r="D320" s="17" t="n">
+        <x:v>32.79</x:v>
+      </x:c>
+      <x:c r="E320" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F320" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G320" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H320" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I320" s="31" t="str">
+        <x:f>IF(AND(OR(G320=H320,AND(B320="OUST",G320="XNAS",H320="XNYS",LEFT(M320,34)="ouster-marketstack-legacy-nyse-tag")),C320&gt;0,ABS(C320-'Prices'!H320)&lt;=MAX(0.01,'Prices'!H320*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J320" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K320" s="14" t="str"/>
+      <x:c r="L320" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M320" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321" ht="50" customHeight="1">
+      <x:c r="A321" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B321" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C321" s="33" t="n">
+        <x:v>13.35</x:v>
+      </x:c>
+      <x:c r="D321" s="33" t="n">
+        <x:v>13.35</x:v>
+      </x:c>
+      <x:c r="E321" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F321" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G321" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H321" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I321" s="32" t="str">
+        <x:f>IF(AND(G321=H321,C321&gt;0,ABS(C321-'Prices'!H321)&lt;=MAX(0.01,'Prices'!H321*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J321" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K321" s="16" t="str"/>
+      <x:c r="L321" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M321" s="16" t="str"/>
+    </x:row>
+    <x:row r="322" ht="50" customHeight="1">
+      <x:c r="A322" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B322" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C322" s="17" t="n">
+        <x:v>439.2</x:v>
+      </x:c>
+      <x:c r="D322" s="17" t="n">
+        <x:v>439.2</x:v>
+      </x:c>
+      <x:c r="E322" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F322" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G322" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H322" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I322" s="31" t="str">
+        <x:f>IF(AND(G322=H322,C322&gt;0,ABS(C322-'Prices'!H322)&lt;=MAX(0.01,'Prices'!H322*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J322" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K322" s="14" t="str"/>
+      <x:c r="L322" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M322" s="14" t="str"/>
+    </x:row>
+    <x:row r="323" ht="50" customHeight="1">
+      <x:c r="A323" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B323" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C323" s="33" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="D323" s="33" t="n">
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="E323" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F323" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G323" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H323" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I323" s="32" t="str">
+        <x:f>IF(AND(G323=H323,C323&gt;0,ABS(C323-'Prices'!H323)&lt;=MAX(0.01,'Prices'!H323*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J323" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K323" s="16" t="str"/>
+      <x:c r="L323" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M323" s="16" t="str"/>
+    </x:row>
+    <x:row r="324" ht="50" customHeight="1">
+      <x:c r="A324" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B324" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C324" s="17" t="n">
+        <x:v>253.5</x:v>
+      </x:c>
+      <x:c r="D324" s="17" t="n">
+        <x:v>253.5</x:v>
+      </x:c>
+      <x:c r="E324" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F324" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G324" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H324" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I324" s="31" t="str">
+        <x:f>IF(AND(G324=H324,C324&gt;0,ABS(C324-'Prices'!H324)&lt;=MAX(0.01,'Prices'!H324*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J324" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K324" s="14" t="str"/>
+      <x:c r="L324" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M324" s="14" t="str"/>
+    </x:row>
+    <x:row r="325" ht="50" customHeight="1">
+      <x:c r="A325" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B325" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C325" s="33" t="n">
+        <x:v>5216</x:v>
+      </x:c>
+      <x:c r="D325" s="33" t="n">
+        <x:v>5216</x:v>
+      </x:c>
+      <x:c r="E325" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F325" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G325" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H325" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I325" s="32" t="str">
+        <x:f>IF(AND(G325=H325,C325&gt;0,ABS(C325-'Prices'!H325)&lt;=MAX(0.01,'Prices'!H325*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J325" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K325" s="16" t="str"/>
+      <x:c r="L325" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M325" s="16" t="str"/>
+    </x:row>
+    <x:row r="326" ht="50" customHeight="1">
+      <x:c r="A326" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B326" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C326" s="17" t="n">
+        <x:v>109.65</x:v>
+      </x:c>
+      <x:c r="D326" s="17" t="n">
+        <x:v>109.65</x:v>
+      </x:c>
+      <x:c r="E326" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F326" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G326" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H326" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I326" s="31" t="str">
+        <x:f>IF(AND(G326=H326,C326&gt;0,ABS(C326-'Prices'!H326)&lt;=MAX(0.01,'Prices'!H326*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J326" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K326" s="14" t="str"/>
+      <x:c r="L326" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M326" s="14" t="str"/>
+    </x:row>
+    <x:row r="327" ht="50" customHeight="1">
+      <x:c r="A327" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B327" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C327" s="33" t="n">
+        <x:v>7722.6</x:v>
+      </x:c>
+      <x:c r="D327" s="33" t="n">
+        <x:v>7722.6</x:v>
+      </x:c>
+      <x:c r="E327" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F327" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G327" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H327" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I327" s="32" t="str">
+        <x:f>IF(AND(G327=H327,C327&gt;0,ABS(C327-'Prices'!H327)&lt;=MAX(0.01,'Prices'!H327*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J327" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K327" s="16" t="str"/>
+      <x:c r="L327" s="39" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M327" s="16" t="str"/>
+    </x:row>
+    <x:row r="328" ht="50" customHeight="1">
+      <x:c r="A328" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B328" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C328" s="17" t="n">
+        <x:v>26477.8105</x:v>
+      </x:c>
+      <x:c r="D328" s="17" t="n">
+        <x:v>26477.8105</x:v>
+      </x:c>
+      <x:c r="E328" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F328" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G328" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H328" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I328" s="31" t="str">
+        <x:f>IF(AND(G328=H328,C328&gt;0,ABS(C328-'Prices'!H328)&lt;=MAX(0.01,'Prices'!H328*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J328" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-28T11-29-17-918Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K328" s="14" t="str"/>
+      <x:c r="L328" s="38" t="n">
+        <x:v>46323.47867960648</x:v>
+      </x:c>
+      <x:c r="M328" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -33401,7 +35205,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7457bf2abf7a4fd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac79c4f628984bbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42364,6 +44168,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="312" ht="27" customHeight="1">
+      <x:c r="A312" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B312" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C312" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D312" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E312" s="19" t="n">
+        <x:f>'Source Audit'!E312</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F312" s="40" t="n">
+        <x:f>'Source Audit'!F312</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G312" s="11" t="str">
+        <x:f>IF(AND(E312=0,F312=1,'Source Audit'!I312&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H312" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="27" customHeight="1">
+      <x:c r="A313" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B313" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C313" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D313" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E313" s="18" t="n">
+        <x:f>'Source Audit'!E313</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F313" s="41" t="n">
+        <x:f>'Source Audit'!F313</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G313" s="12" t="str">
+        <x:f>IF(AND(E313=0,F313=1,'Source Audit'!I313&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H313" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="27" customHeight="1">
+      <x:c r="A314" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B314" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C314" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D314" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E314" s="19" t="n">
+        <x:f>'Source Audit'!E314</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F314" s="40" t="n">
+        <x:f>'Source Audit'!F314</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G314" s="11" t="str">
+        <x:f>IF(AND(E314=0,F314=1,'Source Audit'!I314&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H314" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="27" customHeight="1">
+      <x:c r="A315" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B315" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C315" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D315" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E315" s="18" t="n">
+        <x:f>'Source Audit'!E315</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F315" s="41" t="n">
+        <x:f>'Source Audit'!F315</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G315" s="12" t="str">
+        <x:f>IF(AND(E315=0,F315=1,'Source Audit'!I315&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H315" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="27" customHeight="1">
+      <x:c r="A316" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B316" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C316" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D316" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E316" s="19" t="n">
+        <x:f>'Source Audit'!E316</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F316" s="40" t="n">
+        <x:f>'Source Audit'!F316</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G316" s="11" t="str">
+        <x:f>IF(AND(E316=0,F316=1,'Source Audit'!I316&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H316" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="27" customHeight="1">
+      <x:c r="A317" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B317" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C317" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D317" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E317" s="18" t="n">
+        <x:f>'Source Audit'!E317</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F317" s="41" t="n">
+        <x:f>'Source Audit'!F317</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G317" s="12" t="str">
+        <x:f>IF(AND(E317=0,F317=1,'Source Audit'!I317&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H317" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="27" customHeight="1">
+      <x:c r="A318" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B318" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C318" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D318" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E318" s="19" t="n">
+        <x:f>'Source Audit'!E318</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F318" s="40" t="n">
+        <x:f>'Source Audit'!F318</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G318" s="11" t="str">
+        <x:f>IF(AND(E318=0,F318=1,'Source Audit'!I318&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H318" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319" ht="27" customHeight="1">
+      <x:c r="A319" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B319" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C319" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D319" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E319" s="18" t="n">
+        <x:f>'Source Audit'!E319</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F319" s="41" t="n">
+        <x:f>'Source Audit'!F319</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G319" s="12" t="str">
+        <x:f>IF(AND(E319=0,F319=1,'Source Audit'!I319&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H319" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320" ht="44" customHeight="1">
+      <x:c r="A320" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B320" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C320" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D320" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E320" s="19" t="n">
+        <x:f>'Source Audit'!E320</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F320" s="40" t="n">
+        <x:f>'Source Audit'!F320</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G320" s="11" t="str">
+        <x:f>IF(AND(E320=0,F320=1,'Source Audit'!I320&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H320" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321" ht="27" customHeight="1">
+      <x:c r="A321" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B321" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C321" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D321" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E321" s="18" t="n">
+        <x:f>'Source Audit'!E321</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F321" s="41" t="n">
+        <x:f>'Source Audit'!F321</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G321" s="12" t="str">
+        <x:f>IF(AND(E321=0,F321=1,'Source Audit'!I321&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H321" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322" ht="27" customHeight="1">
+      <x:c r="A322" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B322" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C322" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D322" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E322" s="19" t="n">
+        <x:f>'Source Audit'!E322</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F322" s="40" t="n">
+        <x:f>'Source Audit'!F322</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G322" s="11" t="str">
+        <x:f>IF(AND(E322=0,F322=1,'Source Audit'!I322&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H322" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323" ht="27" customHeight="1">
+      <x:c r="A323" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B323" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C323" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D323" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E323" s="18" t="n">
+        <x:f>'Source Audit'!E323</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F323" s="41" t="n">
+        <x:f>'Source Audit'!F323</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G323" s="12" t="str">
+        <x:f>IF(AND(E323=0,F323=1,'Source Audit'!I323&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H323" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324" ht="27" customHeight="1">
+      <x:c r="A324" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B324" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C324" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D324" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E324" s="19" t="n">
+        <x:f>'Source Audit'!E324</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F324" s="40" t="n">
+        <x:f>'Source Audit'!F324</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G324" s="11" t="str">
+        <x:f>IF(AND(E324=0,F324=1,'Source Audit'!I324&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H324" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325" ht="27" customHeight="1">
+      <x:c r="A325" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B325" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C325" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D325" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E325" s="18" t="n">
+        <x:f>'Source Audit'!E325</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F325" s="41" t="n">
+        <x:f>'Source Audit'!F325</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G325" s="12" t="str">
+        <x:f>IF(AND(E325=0,F325=1,'Source Audit'!I325&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H325" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326" ht="27" customHeight="1">
+      <x:c r="A326" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B326" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C326" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D326" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E326" s="19" t="n">
+        <x:f>'Source Audit'!E326</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F326" s="40" t="n">
+        <x:f>'Source Audit'!F326</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G326" s="11" t="str">
+        <x:f>IF(AND(E326=0,F326=1,'Source Audit'!I326&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H326" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="27" customHeight="1">
+      <x:c r="A327" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B327" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C327" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D327" s="9" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E327" s="18" t="n">
+        <x:f>'Source Audit'!E327</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F327" s="41" t="n">
+        <x:f>'Source Audit'!F327</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G327" s="12" t="str">
+        <x:f>IF(AND(E327=0,F327=1,'Source Audit'!I327&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H327" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="27" customHeight="1">
+      <x:c r="A328" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="B328" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C328" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D328" s="8" t="n">
+        <x:v>46322</x:v>
+      </x:c>
+      <x:c r="E328" s="19" t="n">
+        <x:f>'Source Audit'!E328</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F328" s="40" t="n">
+        <x:f>'Source Audit'!F328</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G328" s="11" t="str">
+        <x:f>IF(AND(E328=0,F328=1,'Source Audit'!I328&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H328" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -42371,7 +44668,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70571c29aa1d4e59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6479dd0b91864ef6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 28, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 308 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Both the shared-checkout and exact main-based
publication candidate production builds and article-preview checks passed.
These results are documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R95f3db0ca9c244cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R4cbedd9c43b44ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R24dc70abf7bd48fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R345e558209b44efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R4fa0cdd4e8a349fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0c6f7da7b3c74541"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R25e5422527154232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Ra40c58b1cb3d48c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Ra06f34215e75475e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R22af659891df4127"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H290" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H305" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H328" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -2182,6 +2182,85 @@
         <x:v>-4.7745231440723845</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="40" customHeight="1">
+      <x:c r="A25" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="n">
+        <x:f>B24*(1+SUM('Returns and Contributions'!F291:F305))</x:f>
+        <x:v>954.9187500693777</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="n">
+        <x:f>B25/B24-1</x:f>
+        <x:v>0.018470885488518718</x:v>
+      </x:c>
+      <x:c r="D25" s="21" t="n">
+        <x:f>B25/$B$6-1</x:f>
+        <x:v>-0.04508124993062235</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="n">
+        <x:f>1000*'Prices'!H344/'Prices'!I344</x:f>
+        <x:v>1010.1128944948445</x:v>
+      </x:c>
+      <x:c r="F25" s="21" t="n">
+        <x:f>E25/E24-1</x:f>
+        <x:v>0.0027684976562298846</x:v>
+      </x:c>
+      <x:c r="G25" s="21" t="n">
+        <x:f>E25/1000-1</x:f>
+        <x:v>0.010112894494844538</x:v>
+      </x:c>
+      <x:c r="H25" s="18" t="n">
+        <x:f>1000*'Prices'!H345/'Prices'!I345</x:f>
+        <x:v>988.0266098228026</x:v>
+      </x:c>
+      <x:c r="I25" s="21" t="n">
+        <x:f>H25/H24-1</x:f>
+        <x:v>0.0027208103177565057</x:v>
+      </x:c>
+      <x:c r="J25" s="21" t="n">
+        <x:f>H25/1000-1</x:f>
+        <x:v>-0.011973390177197452</x:v>
+      </x:c>
+      <x:c r="K25" s="25" t="n">
+        <x:f>(C25-F25)*100</x:f>
+        <x:v>1.5702387832288833</x:v>
+      </x:c>
+      <x:c r="L25" s="25" t="n">
+        <x:f>(C25-I25)*100</x:f>
+        <x:v>1.5750075170762212</x:v>
+      </x:c>
+      <x:c r="M25" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G291:G305)</x:f>
+        <x:v>0.9999999999999996</x:v>
+      </x:c>
+      <x:c r="N25" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F291:F305)-C25</x:f>
+        <x:v>-6.938893903907228e-18</x:v>
+      </x:c>
+      <x:c r="O25" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P25" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I329:I345,"Mismatch")=0,IF(COUNTIF('Source Audit'!I329:I345,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q25" s="30" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="R25" s="27" t="n">
+        <x:f>B25-1000*('Prices'!H329/'Prices'!H6+'Prices'!H330/'Prices'!H7+'Prices'!H331/'Prices'!H8+'Prices'!H332/'Prices'!H9+'Prices'!H333/'Prices'!H10+'Prices'!H334/'Prices'!H11+'Prices'!H335/'Prices'!H12+'Prices'!H336/'Prices'!H13+'Prices'!H337/'Prices'!H14+'Prices'!H338/'Prices'!H15+'Prices'!H339/'Prices'!H16+'Prices'!H340/'Prices'!H17+'Prices'!H341/'Prices'!H18+'Prices'!H342/'Prices'!H19+'Prices'!H343/'Prices'!H20)/15</x:f>
+        <x:v>4.547473508864641e-13</x:v>
+      </x:c>
+      <x:c r="S25" s="25" t="n">
+        <x:f>(D25-G25)*100</x:f>
+        <x:v>-5.5194144425466884</x:v>
+      </x:c>
+      <x:c r="T25" s="25" t="n">
+        <x:f>(D25-J25)*100</x:f>
+        <x:v>-3.3107859753424895</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -2189,7 +2268,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f71bd91509e4acb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39614baf2ad246d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13879,6 +13958,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="329" ht="27" customHeight="1">
+      <x:c r="A329" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B329" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C329" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D329" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E329" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F329" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G329" s="33" t="n">
+        <x:f>H312</x:f>
+        <x:v>5820</x:v>
+      </x:c>
+      <x:c r="H329" s="35" t="n">
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="I329" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J329" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K329" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="27" customHeight="1">
+      <x:c r="A330" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B330" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C330" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D330" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E330" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F330" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G330" s="17" t="n">
+        <x:f>H313</x:f>
+        <x:v>4090</x:v>
+      </x:c>
+      <x:c r="H330" s="34" t="n">
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="I330" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J330" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K330" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="27" customHeight="1">
+      <x:c r="A331" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B331" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C331" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D331" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E331" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F331" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G331" s="33" t="n">
+        <x:f>H314</x:f>
+        <x:v>28.45</x:v>
+      </x:c>
+      <x:c r="H331" s="35" t="n">
+        <x:v>30.14</x:v>
+      </x:c>
+      <x:c r="I331" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J331" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K331" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="27" customHeight="1">
+      <x:c r="A332" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B332" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C332" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D332" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E332" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F332" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G332" s="17" t="n">
+        <x:f>H315</x:f>
+        <x:v>323.68</x:v>
+      </x:c>
+      <x:c r="H332" s="34" t="n">
+        <x:v>313.24</x:v>
+      </x:c>
+      <x:c r="I332" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J332" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K332" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="27" customHeight="1">
+      <x:c r="A333" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B333" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C333" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D333" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E333" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F333" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G333" s="33" t="n">
+        <x:f>H316</x:f>
+        <x:v>4285</x:v>
+      </x:c>
+      <x:c r="H333" s="35" t="n">
+        <x:v>4420</x:v>
+      </x:c>
+      <x:c r="I333" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J333" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K333" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="27" customHeight="1">
+      <x:c r="A334" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B334" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C334" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D334" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E334" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F334" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G334" s="17" t="n">
+        <x:f>H317</x:f>
+        <x:v>53.31</x:v>
+      </x:c>
+      <x:c r="H334" s="34" t="n">
+        <x:v>56.16</x:v>
+      </x:c>
+      <x:c r="I334" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J334" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K334" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="27" customHeight="1">
+      <x:c r="A335" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B335" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C335" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D335" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E335" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F335" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G335" s="33" t="n">
+        <x:f>H318</x:f>
+        <x:v>79080</x:v>
+      </x:c>
+      <x:c r="H335" s="35" t="n">
+        <x:v>79190</x:v>
+      </x:c>
+      <x:c r="I335" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J335" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K335" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336" ht="27" customHeight="1">
+      <x:c r="A336" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B336" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C336" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D336" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E336" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F336" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G336" s="17" t="n">
+        <x:f>H319</x:f>
+        <x:v>58.22</x:v>
+      </x:c>
+      <x:c r="H336" s="34" t="n">
+        <x:v>58.43</x:v>
+      </x:c>
+      <x:c r="I336" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J336" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K336" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337" ht="27" customHeight="1">
+      <x:c r="A337" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B337" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C337" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D337" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E337" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F337" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G337" s="33" t="n">
+        <x:f>H320</x:f>
+        <x:v>32.79</x:v>
+      </x:c>
+      <x:c r="H337" s="35" t="n">
+        <x:v>33.61</x:v>
+      </x:c>
+      <x:c r="I337" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J337" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K337" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="27" customHeight="1">
+      <x:c r="A338" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B338" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C338" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D338" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E338" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F338" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G338" s="17" t="n">
+        <x:f>H321</x:f>
+        <x:v>13.35</x:v>
+      </x:c>
+      <x:c r="H338" s="34" t="n">
+        <x:v>13.83</x:v>
+      </x:c>
+      <x:c r="I338" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J338" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K338" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" ht="27" customHeight="1">
+      <x:c r="A339" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B339" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C339" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D339" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E339" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F339" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G339" s="33" t="n">
+        <x:f>H322</x:f>
+        <x:v>439.2</x:v>
+      </x:c>
+      <x:c r="H339" s="35" t="n">
+        <x:v>443.81</x:v>
+      </x:c>
+      <x:c r="I339" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J339" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K339" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340" ht="27" customHeight="1">
+      <x:c r="A340" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B340" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C340" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D340" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E340" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F340" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G340" s="17" t="n">
+        <x:f>H323</x:f>
+        <x:v>266.2</x:v>
+      </x:c>
+      <x:c r="H340" s="34" t="n">
+        <x:v>270.05</x:v>
+      </x:c>
+      <x:c r="I340" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J340" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K340" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341" ht="27" customHeight="1">
+      <x:c r="A341" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B341" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C341" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D341" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E341" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F341" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G341" s="33" t="n">
+        <x:f>H324</x:f>
+        <x:v>253.5</x:v>
+      </x:c>
+      <x:c r="H341" s="35" t="n">
+        <x:v>251.69</x:v>
+      </x:c>
+      <x:c r="I341" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J341" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K341" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342" ht="27" customHeight="1">
+      <x:c r="A342" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B342" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C342" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D342" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E342" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F342" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G342" s="17" t="n">
+        <x:f>H325</x:f>
+        <x:v>5216</x:v>
+      </x:c>
+      <x:c r="H342" s="34" t="n">
+        <x:v>5441</x:v>
+      </x:c>
+      <x:c r="I342" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J342" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K342" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343" ht="27" customHeight="1">
+      <x:c r="A343" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B343" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C343" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D343" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E343" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F343" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G343" s="33" t="n">
+        <x:f>H326</x:f>
+        <x:v>109.65</x:v>
+      </x:c>
+      <x:c r="H343" s="35" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="I343" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J343" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K343" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344" ht="27" customHeight="1">
+      <x:c r="A344" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B344" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C344" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D344" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E344" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F344" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G344" s="17" t="n">
+        <x:f>H327</x:f>
+        <x:v>7722.6</x:v>
+      </x:c>
+      <x:c r="H344" s="34" t="n">
+        <x:v>7743.98</x:v>
+      </x:c>
+      <x:c r="I344" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J344" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K344" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345" ht="27" customHeight="1">
+      <x:c r="A345" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B345" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C345" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D345" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E345" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F345" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G345" s="33" t="n">
+        <x:f>H328</x:f>
+        <x:v>26477.8105</x:v>
+      </x:c>
+      <x:c r="H345" s="35" t="n">
+        <x:v>26549.8516</x:v>
+      </x:c>
+      <x:c r="I345" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J345" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="K345" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -13886,7 +14577,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a98f5428dc34294"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re707c100ef7340ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22720,6 +23411,471 @@
         <x:v>0.10735205009089088</x:v>
       </x:c>
     </x:row>
+    <x:row r="291" ht="27" customHeight="1">
+      <x:c r="A291" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B291" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C291" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D291" s="21" t="n">
+        <x:f>G276</x:f>
+        <x:v>0.06754077550576866</x:v>
+      </x:c>
+      <x:c r="E291" s="23" t="n">
+        <x:f>'Prices'!H329/'Prices'!G329-1</x:f>
+        <x:v>0.015120274914089293</x:v>
+      </x:c>
+      <x:c r="F291" s="21" t="n">
+        <x:f>D291*E291</x:f>
+        <x:v>0.0010212350935580104</x:v>
+      </x:c>
+      <x:c r="G291" s="21" t="n">
+        <x:f>D291*(1+E291)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06731857687462542</x:v>
+      </x:c>
+      <x:c r="H291" s="23" t="n">
+        <x:f>'Prices'!H329/'Prices'!I329-1</x:f>
+        <x:v>-0.03574343071650077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="27" customHeight="1">
+      <x:c r="A292" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B292" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C292" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D292" s="20" t="n">
+        <x:f>G277</x:f>
+        <x:v>0.060852330604920464</x:v>
+      </x:c>
+      <x:c r="E292" s="22" t="n">
+        <x:f>'Prices'!H330/'Prices'!G330-1</x:f>
+        <x:v>0.02347188264058686</x:v>
+      </x:c>
+      <x:c r="F292" s="20" t="n">
+        <x:f>D292*E292</x:f>
+        <x:v>0.0014283187623648852</x:v>
+      </x:c>
+      <x:c r="G292" s="20" t="n">
+        <x:f>D292*(1+E292)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.061151133777782835</x:v>
+      </x:c>
+      <x:c r="H292" s="22" t="n">
+        <x:f>'Prices'!H330/'Prices'!I330-1</x:f>
+        <x:v>-0.12408453651391504</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="27" customHeight="1">
+      <x:c r="A293" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B293" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C293" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D293" s="21" t="n">
+        <x:f>G278</x:f>
+        <x:v>0.07168300449739144</x:v>
+      </x:c>
+      <x:c r="E293" s="23" t="n">
+        <x:f>'Prices'!H331/'Prices'!G331-1</x:f>
+        <x:v>0.059402460456942086</x:v>
+      </x:c>
+      <x:c r="F293" s="21" t="n">
+        <x:f>D293*E293</x:f>
+        <x:v>0.0042581468400910965</x:v>
+      </x:c>
+      <x:c r="G293" s="21" t="n">
+        <x:f>D293*(1+E293)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.07456389025893134</x:v>
+      </x:c>
+      <x:c r="H293" s="23" t="n">
+        <x:f>'Prices'!H331/'Prices'!I331-1</x:f>
+        <x:v>0.0680368532955351</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="27" customHeight="1">
+      <x:c r="A294" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B294" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C294" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D294" s="20" t="n">
+        <x:f>G279</x:f>
+        <x:v>0.055351929435878654</x:v>
+      </x:c>
+      <x:c r="E294" s="22" t="n">
+        <x:f>'Prices'!H332/'Prices'!G332-1</x:f>
+        <x:v>-0.03225407810182901</x:v>
+      </x:c>
+      <x:c r="F294" s="20" t="n">
+        <x:f>D294*E294</x:f>
+        <x:v>-0.0017853254551117583</x:v>
+      </x:c>
+      <x:c r="G294" s="20" t="n">
+        <x:f>D294*(1+E294)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.05259512544148299</x:v>
+      </x:c>
+      <x:c r="H294" s="22" t="n">
+        <x:f>'Prices'!H332/'Prices'!I332-1</x:f>
+        <x:v>-0.2466389283051541</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="295" ht="27" customHeight="1">
+      <x:c r="A295" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B295" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C295" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D295" s="21" t="n">
+        <x:f>G280</x:f>
+        <x:v>0.06124190335110861</x:v>
+      </x:c>
+      <x:c r="E295" s="23" t="n">
+        <x:f>'Prices'!H333/'Prices'!G333-1</x:f>
+        <x:v>0.031505250875145885</x:v>
+      </x:c>
+      <x:c r="F295" s="21" t="n">
+        <x:f>D295*E295</x:f>
+        <x:v>0.0019294415291481143</x:v>
+      </x:c>
+      <x:c r="G295" s="21" t="n">
+        <x:f>D295*(1+E295)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.062025675726563374</x:v>
+      </x:c>
+      <x:c r="H295" s="23" t="n">
+        <x:f>'Prices'!H333/'Prices'!I333-1</x:f>
+        <x:v>-0.11155778894472357</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="27" customHeight="1">
+      <x:c r="A296" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B296" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C296" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D296" s="20" t="n">
+        <x:f>G281</x:f>
+        <x:v>0.073035206793186</x:v>
+      </x:c>
+      <x:c r="E296" s="22" t="n">
+        <x:f>'Prices'!H334/'Prices'!G334-1</x:f>
+        <x:v>0.05346088913899827</x:v>
+      </x:c>
+      <x:c r="F296" s="20" t="n">
+        <x:f>D296*E296</x:f>
+        <x:v>0.00390452709361433</x:v>
+      </x:c>
+      <x:c r="G296" s="20" t="n">
+        <x:f>D296*(1+E296)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.075544362615624</x:v>
+      </x:c>
+      <x:c r="H296" s="22" t="n">
+        <x:f>'Prices'!H334/'Prices'!I334-1</x:f>
+        <x:v>0.08208092485549123</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="27" customHeight="1">
+      <x:c r="A297" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B297" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C297" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D297" s="21" t="n">
+        <x:f>G282</x:f>
+        <x:v>0.06924709676355023</x:v>
+      </x:c>
+      <x:c r="E297" s="23" t="n">
+        <x:f>'Prices'!H335/'Prices'!G335-1</x:f>
+        <x:v>0.001390996459281757</x:v>
+      </x:c>
+      <x:c r="F297" s="21" t="n">
+        <x:f>D297*E297</x:f>
+        <x:v>0.00009632246641363958</x:v>
+      </x:c>
+      <x:c r="G297" s="21" t="n">
+        <x:f>D297*(1+E297)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06808581395697205</x:v>
+      </x:c>
+      <x:c r="H297" s="23" t="n">
+        <x:f>'Prices'!H335/'Prices'!I335-1</x:f>
+        <x:v>-0.02475369458128074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="27" customHeight="1">
+      <x:c r="A298" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B298" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C298" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D298" s="20" t="n">
+        <x:f>G283</x:f>
+        <x:v>0.06653239127460983</x:v>
+      </x:c>
+      <x:c r="E298" s="22" t="n">
+        <x:f>'Prices'!H336/'Prices'!G336-1</x:f>
+        <x:v>0.0036070079010650513</x:v>
+      </x:c>
+      <x:c r="F298" s="20" t="n">
+        <x:f>D298*E298</x:f>
+        <x:v>0.00023998286100426915</x:v>
+      </x:c>
+      <x:c r="G298" s="20" t="n">
+        <x:f>D298*(1+E298)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06556139707772415</x:v>
+      </x:c>
+      <x:c r="H298" s="22" t="n">
+        <x:f>'Prices'!H336/'Prices'!I336-1</x:f>
+        <x:v>-0.06091288974606235</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="27" customHeight="1">
+      <x:c r="A299" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B299" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C299" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D299" s="21" t="n">
+        <x:f>G284</x:f>
+        <x:v>0.057046331006228225</x:v>
+      </x:c>
+      <x:c r="E299" s="23" t="n">
+        <x:f>'Prices'!H337/'Prices'!G337-1</x:f>
+        <x:v>0.025007624275693807</x:v>
+      </x:c>
+      <x:c r="F299" s="21" t="n">
+        <x:f>D299*E299</x:f>
+        <x:v>0.0014265932121106174</x:v>
+      </x:c>
+      <x:c r="G299" s="21" t="n">
+        <x:f>D299*(1+E299)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.057412465148958855</x:v>
+      </x:c>
+      <x:c r="H299" s="23" t="n">
+        <x:f>'Prices'!H337/'Prices'!I337-1</x:f>
+        <x:v>-0.17763640812331782</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="27" customHeight="1">
+      <x:c r="A300" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B300" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C300" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D300" s="20" t="n">
+        <x:f>G285</x:f>
+        <x:v>0.05958767336740991</x:v>
+      </x:c>
+      <x:c r="E300" s="22" t="n">
+        <x:f>'Prices'!H338/'Prices'!G338-1</x:f>
+        <x:v>0.035955056179775235</x:v>
+      </x:c>
+      <x:c r="F300" s="20" t="n">
+        <x:f>D300*E300</x:f>
+        <x:v>0.00214247814354732</x:v>
+      </x:c>
+      <x:c r="G300" s="20" t="n">
+        <x:f>D300*(1+E300)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06061061969517942</x:v>
+      </x:c>
+      <x:c r="H300" s="22" t="n">
+        <x:f>'Prices'!H338/'Prices'!I338-1</x:f>
+        <x:v>-0.13182674199623345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="27" customHeight="1">
+      <x:c r="A301" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B301" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C301" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D301" s="21" t="n">
+        <x:f>G286</x:f>
+        <x:v>0.07058120532588666</x:v>
+      </x:c>
+      <x:c r="E301" s="23" t="n">
+        <x:f>'Prices'!H339/'Prices'!G339-1</x:f>
+        <x:v>0.010496357012750535</x:v>
+      </x:c>
+      <x:c r="F301" s="21" t="n">
+        <x:f>D301*E301</x:f>
+        <x:v>0.0007408455294907558</x:v>
+      </x:c>
+      <x:c r="G301" s="21" t="n">
+        <x:f>D301*(1+E301)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.07002856131834063</x:v>
+      </x:c>
+      <x:c r="H301" s="23" t="n">
+        <x:f>'Prices'!H339/'Prices'!I339-1</x:f>
+        <x:v>0.0030737936489999562</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="27" customHeight="1">
+      <x:c r="A302" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B302" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C302" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D302" s="20" t="n">
+        <x:f>G287</x:f>
+        <x:v>0.06961290893764474</x:v>
+      </x:c>
+      <x:c r="E302" s="22" t="n">
+        <x:f>'Prices'!H340/'Prices'!G340-1</x:f>
+        <x:v>0.01446280991735538</x:v>
+      </x:c>
+      <x:c r="F302" s="20" t="n">
+        <x:f>D302*E302</x:f>
+        <x:v>0.0010067982697593253</x:v>
+      </x:c>
+      <x:c r="G302" s="20" t="n">
+        <x:f>D302*(1+E302)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06933895530408873</x:v>
+      </x:c>
+      <x:c r="H302" s="22" t="n">
+        <x:f>'Prices'!H340/'Prices'!I340-1</x:f>
+        <x:v>-0.006803972048547102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="27" customHeight="1">
+      <x:c r="A303" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B303" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C303" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D303" s="21" t="n">
+        <x:f>G288</x:f>
+        <x:v>0.07535739610395752</x:v>
+      </x:c>
+      <x:c r="E303" s="23" t="n">
+        <x:f>'Prices'!H341/'Prices'!G341-1</x:f>
+        <x:v>-0.007140039447731783</x:v>
+      </x:c>
+      <x:c r="F303" s="21" t="n">
+        <x:f>D303*E303</x:f>
+        <x:v>-0.000538054780860606</x:v>
+      </x:c>
+      <x:c r="G303" s="21" t="n">
+        <x:f>D303*(1+E303)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.07346242527807668</x:v>
+      </x:c>
+      <x:c r="H303" s="23" t="n">
+        <x:f>'Prices'!H341/'Prices'!I341-1</x:f>
+        <x:v>0.0522597098540909</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="27" customHeight="1">
+      <x:c r="A304" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B304" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C304" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D304" s="20" t="n">
+        <x:f>G289</x:f>
+        <x:v>0.06359324785955116</x:v>
+      </x:c>
+      <x:c r="E304" s="22" t="n">
+        <x:f>'Prices'!H342/'Prices'!G342-1</x:f>
+        <x:v>0.04313650306748462</x:v>
+      </x:c>
+      <x:c r="F304" s="20" t="n">
+        <x:f>D304*E304</x:f>
+        <x:v>0.0027431903313648383</x:v>
+      </x:c>
+      <x:c r="G304" s="20" t="n">
+        <x:f>D304*(1+E304)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.06513336722345002</x:v>
+      </x:c>
+      <x:c r="H304" s="22" t="n">
+        <x:f>'Prices'!H342/'Prices'!I342-1</x:f>
+        <x:v>-0.0670438957475995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="27" customHeight="1">
+      <x:c r="A305" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B305" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C305" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D305" s="21" t="n">
+        <x:f>G290</x:f>
+        <x:v>0.07873659917290747</x:v>
+      </x:c>
+      <x:c r="E305" s="23" t="n">
+        <x:f>'Prices'!H343/'Prices'!G343-1</x:f>
+        <x:v>-0.0018239854081167906</x:v>
+      </x:c>
+      <x:c r="F305" s="21" t="n">
+        <x:f>D305*E305</x:f>
+        <x:v>-0.00014361440797612377</x:v>
+      </x:c>
+      <x:c r="G305" s="21" t="n">
+        <x:f>D305*(1+E305)/(1+SUM($F$291:$F$305))</x:f>
+        <x:v>0.07716763030219907</x:v>
+      </x:c>
+      <x:c r="H305" s="23" t="n">
+        <x:f>'Prices'!H343/'Prices'!I343-1</x:f>
+        <x:v>0.10533225610987684</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -22727,7 +23883,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08b3de111cc94505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae68bcb6acd044f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35198,6 +36354,654 @@
       </x:c>
       <x:c r="M328" s="14" t="str"/>
     </x:row>
+    <x:row r="329" ht="50" customHeight="1">
+      <x:c r="A329" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B329" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C329" s="33" t="n">
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="D329" s="33" t="n">
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="E329" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F329" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G329" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H329" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I329" s="32" t="str">
+        <x:f>IF(AND(G329=H329,C329&gt;0,ABS(C329-'Prices'!H329)&lt;=MAX(0.01,'Prices'!H329*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J329" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K329" s="16" t="str"/>
+      <x:c r="L329" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M329" s="16" t="str"/>
+    </x:row>
+    <x:row r="330" ht="50" customHeight="1">
+      <x:c r="A330" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B330" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C330" s="17" t="n">
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="D330" s="17" t="n">
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="E330" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F330" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G330" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H330" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I330" s="31" t="str">
+        <x:f>IF(AND(G330=H330,C330&gt;0,ABS(C330-'Prices'!H330)&lt;=MAX(0.01,'Prices'!H330*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J330" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K330" s="14" t="str"/>
+      <x:c r="L330" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M330" s="14" t="str"/>
+    </x:row>
+    <x:row r="331" ht="50" customHeight="1">
+      <x:c r="A331" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B331" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C331" s="33" t="n">
+        <x:v>30.14</x:v>
+      </x:c>
+      <x:c r="D331" s="33" t="n">
+        <x:v>30.14</x:v>
+      </x:c>
+      <x:c r="E331" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F331" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G331" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H331" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I331" s="32" t="str">
+        <x:f>IF(AND(G331=H331,C331&gt;0,ABS(C331-'Prices'!H331)&lt;=MAX(0.01,'Prices'!H331*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J331" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K331" s="16" t="str"/>
+      <x:c r="L331" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M331" s="16" t="str"/>
+    </x:row>
+    <x:row r="332" ht="50" customHeight="1">
+      <x:c r="A332" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B332" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C332" s="17" t="n">
+        <x:v>313.24</x:v>
+      </x:c>
+      <x:c r="D332" s="17" t="n">
+        <x:v>313.24</x:v>
+      </x:c>
+      <x:c r="E332" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F332" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G332" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H332" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I332" s="31" t="str">
+        <x:f>IF(AND(G332=H332,C332&gt;0,ABS(C332-'Prices'!H332)&lt;=MAX(0.01,'Prices'!H332*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J332" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K332" s="14" t="str"/>
+      <x:c r="L332" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M332" s="14" t="str"/>
+    </x:row>
+    <x:row r="333" ht="50" customHeight="1">
+      <x:c r="A333" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B333" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C333" s="33" t="n">
+        <x:v>4420</x:v>
+      </x:c>
+      <x:c r="D333" s="33" t="n">
+        <x:v>4420</x:v>
+      </x:c>
+      <x:c r="E333" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F333" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G333" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H333" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I333" s="32" t="str">
+        <x:f>IF(AND(G333=H333,C333&gt;0,ABS(C333-'Prices'!H333)&lt;=MAX(0.01,'Prices'!H333*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J333" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K333" s="16" t="str"/>
+      <x:c r="L333" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M333" s="16" t="str"/>
+    </x:row>
+    <x:row r="334" ht="50" customHeight="1">
+      <x:c r="A334" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B334" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C334" s="17" t="n">
+        <x:v>56.16</x:v>
+      </x:c>
+      <x:c r="D334" s="17" t="n">
+        <x:v>56.16</x:v>
+      </x:c>
+      <x:c r="E334" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F334" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G334" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H334" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I334" s="31" t="str">
+        <x:f>IF(AND(G334=H334,C334&gt;0,ABS(C334-'Prices'!H334)&lt;=MAX(0.01,'Prices'!H334*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J334" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K334" s="14" t="str"/>
+      <x:c r="L334" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M334" s="14" t="str"/>
+    </x:row>
+    <x:row r="335" ht="50" customHeight="1">
+      <x:c r="A335" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B335" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C335" s="33" t="n">
+        <x:v>79190</x:v>
+      </x:c>
+      <x:c r="D335" s="33" t="n">
+        <x:v>79190</x:v>
+      </x:c>
+      <x:c r="E335" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F335" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G335" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H335" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I335" s="32" t="str">
+        <x:f>IF(AND(G335=H335,C335&gt;0,ABS(C335-'Prices'!H335)&lt;=MAX(0.01,'Prices'!H335*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J335" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K335" s="16" t="str"/>
+      <x:c r="L335" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M335" s="16" t="str"/>
+    </x:row>
+    <x:row r="336" ht="50" customHeight="1">
+      <x:c r="A336" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B336" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C336" s="17" t="n">
+        <x:v>58.43</x:v>
+      </x:c>
+      <x:c r="D336" s="17" t="n">
+        <x:v>58.43</x:v>
+      </x:c>
+      <x:c r="E336" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F336" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G336" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H336" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I336" s="31" t="str">
+        <x:f>IF(AND(G336=H336,C336&gt;0,ABS(C336-'Prices'!H336)&lt;=MAX(0.01,'Prices'!H336*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J336" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K336" s="14" t="str"/>
+      <x:c r="L336" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M336" s="14" t="str"/>
+    </x:row>
+    <x:row r="337" ht="50" customHeight="1">
+      <x:c r="A337" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B337" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C337" s="33" t="n">
+        <x:v>33.61</x:v>
+      </x:c>
+      <x:c r="D337" s="33" t="n">
+        <x:v>33.61</x:v>
+      </x:c>
+      <x:c r="E337" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F337" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G337" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H337" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I337" s="32" t="str">
+        <x:f>IF(AND(OR(G337=H337,AND(B337="OUST",G337="XNAS",H337="XNYS",LEFT(M337,34)="ouster-marketstack-legacy-nyse-tag")),C337&gt;0,ABS(C337-'Prices'!H337)&lt;=MAX(0.01,'Prices'!H337*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J337" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K337" s="16" t="str"/>
+      <x:c r="L337" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M337" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="50" customHeight="1">
+      <x:c r="A338" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B338" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C338" s="17" t="n">
+        <x:v>13.83</x:v>
+      </x:c>
+      <x:c r="D338" s="17" t="n">
+        <x:v>13.83</x:v>
+      </x:c>
+      <x:c r="E338" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F338" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G338" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H338" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I338" s="31" t="str">
+        <x:f>IF(AND(G338=H338,C338&gt;0,ABS(C338-'Prices'!H338)&lt;=MAX(0.01,'Prices'!H338*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J338" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K338" s="14" t="str"/>
+      <x:c r="L338" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M338" s="14" t="str"/>
+    </x:row>
+    <x:row r="339" ht="50" customHeight="1">
+      <x:c r="A339" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B339" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C339" s="33" t="n">
+        <x:v>443.81</x:v>
+      </x:c>
+      <x:c r="D339" s="33" t="n">
+        <x:v>443.81</x:v>
+      </x:c>
+      <x:c r="E339" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F339" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G339" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H339" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I339" s="32" t="str">
+        <x:f>IF(AND(G339=H339,C339&gt;0,ABS(C339-'Prices'!H339)&lt;=MAX(0.01,'Prices'!H339*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J339" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K339" s="16" t="str"/>
+      <x:c r="L339" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M339" s="16" t="str"/>
+    </x:row>
+    <x:row r="340" ht="50" customHeight="1">
+      <x:c r="A340" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B340" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C340" s="17" t="n">
+        <x:v>270.05</x:v>
+      </x:c>
+      <x:c r="D340" s="17" t="n">
+        <x:v>270.05</x:v>
+      </x:c>
+      <x:c r="E340" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F340" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G340" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H340" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I340" s="31" t="str">
+        <x:f>IF(AND(G340=H340,C340&gt;0,ABS(C340-'Prices'!H340)&lt;=MAX(0.01,'Prices'!H340*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J340" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K340" s="14" t="str"/>
+      <x:c r="L340" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M340" s="14" t="str"/>
+    </x:row>
+    <x:row r="341" ht="50" customHeight="1">
+      <x:c r="A341" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B341" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C341" s="33" t="n">
+        <x:v>251.69</x:v>
+      </x:c>
+      <x:c r="D341" s="33" t="n">
+        <x:v>251.69</x:v>
+      </x:c>
+      <x:c r="E341" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F341" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G341" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H341" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I341" s="32" t="str">
+        <x:f>IF(AND(G341=H341,C341&gt;0,ABS(C341-'Prices'!H341)&lt;=MAX(0.01,'Prices'!H341*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J341" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K341" s="16" t="str"/>
+      <x:c r="L341" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M341" s="16" t="str"/>
+    </x:row>
+    <x:row r="342" ht="50" customHeight="1">
+      <x:c r="A342" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B342" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C342" s="17" t="n">
+        <x:v>5441</x:v>
+      </x:c>
+      <x:c r="D342" s="17" t="n">
+        <x:v>5441</x:v>
+      </x:c>
+      <x:c r="E342" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F342" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G342" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H342" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I342" s="31" t="str">
+        <x:f>IF(AND(G342=H342,C342&gt;0,ABS(C342-'Prices'!H342)&lt;=MAX(0.01,'Prices'!H342*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J342" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K342" s="14" t="str"/>
+      <x:c r="L342" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M342" s="14" t="str"/>
+    </x:row>
+    <x:row r="343" ht="50" customHeight="1">
+      <x:c r="A343" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B343" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C343" s="33" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="D343" s="33" t="n">
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="E343" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F343" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G343" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H343" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I343" s="32" t="str">
+        <x:f>IF(AND(G343=H343,C343&gt;0,ABS(C343-'Prices'!H343)&lt;=MAX(0.01,'Prices'!H343*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J343" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K343" s="16" t="str"/>
+      <x:c r="L343" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M343" s="16" t="str"/>
+    </x:row>
+    <x:row r="344" ht="50" customHeight="1">
+      <x:c r="A344" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B344" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C344" s="17" t="n">
+        <x:v>7743.98</x:v>
+      </x:c>
+      <x:c r="D344" s="17" t="n">
+        <x:v>7743.98</x:v>
+      </x:c>
+      <x:c r="E344" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F344" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G344" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H344" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I344" s="31" t="str">
+        <x:f>IF(AND(G344=H344,C344&gt;0,ABS(C344-'Prices'!H344)&lt;=MAX(0.01,'Prices'!H344*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J344" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K344" s="14" t="str"/>
+      <x:c r="L344" s="38" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M344" s="14" t="str"/>
+    </x:row>
+    <x:row r="345" ht="50" customHeight="1">
+      <x:c r="A345" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B345" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C345" s="33" t="n">
+        <x:v>26549.8516</x:v>
+      </x:c>
+      <x:c r="D345" s="33" t="n">
+        <x:v>26549.8516</x:v>
+      </x:c>
+      <x:c r="E345" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F345" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G345" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H345" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I345" s="32" t="str">
+        <x:f>IF(AND(G345=H345,C345&gt;0,ABS(C345-'Prices'!H345)&lt;=MAX(0.01,'Prices'!H345*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J345" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-29T11-28-29-199Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K345" s="16" t="str"/>
+      <x:c r="L345" s="39" t="n">
+        <x:v>46324.478115729165</x:v>
+      </x:c>
+      <x:c r="M345" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -35205,7 +37009,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac79c4f628984bbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc758ba6c7546e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44661,6 +46465,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="329" ht="27" customHeight="1">
+      <x:c r="A329" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B329" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C329" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D329" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E329" s="18" t="n">
+        <x:f>'Source Audit'!E329</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F329" s="41" t="n">
+        <x:f>'Source Audit'!F329</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G329" s="12" t="str">
+        <x:f>IF(AND(E329=0,F329=1,'Source Audit'!I329&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H329" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="27" customHeight="1">
+      <x:c r="A330" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B330" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C330" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D330" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E330" s="19" t="n">
+        <x:f>'Source Audit'!E330</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F330" s="40" t="n">
+        <x:f>'Source Audit'!F330</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G330" s="11" t="str">
+        <x:f>IF(AND(E330=0,F330=1,'Source Audit'!I330&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H330" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="27" customHeight="1">
+      <x:c r="A331" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B331" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C331" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D331" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E331" s="18" t="n">
+        <x:f>'Source Audit'!E331</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F331" s="41" t="n">
+        <x:f>'Source Audit'!F331</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G331" s="12" t="str">
+        <x:f>IF(AND(E331=0,F331=1,'Source Audit'!I331&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H331" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="27" customHeight="1">
+      <x:c r="A332" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B332" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C332" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D332" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E332" s="19" t="n">
+        <x:f>'Source Audit'!E332</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F332" s="40" t="n">
+        <x:f>'Source Audit'!F332</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G332" s="11" t="str">
+        <x:f>IF(AND(E332=0,F332=1,'Source Audit'!I332&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H332" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="27" customHeight="1">
+      <x:c r="A333" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B333" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C333" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D333" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E333" s="18" t="n">
+        <x:f>'Source Audit'!E333</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F333" s="41" t="n">
+        <x:f>'Source Audit'!F333</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G333" s="12" t="str">
+        <x:f>IF(AND(E333=0,F333=1,'Source Audit'!I333&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H333" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="27" customHeight="1">
+      <x:c r="A334" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B334" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C334" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D334" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E334" s="19" t="n">
+        <x:f>'Source Audit'!E334</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F334" s="40" t="n">
+        <x:f>'Source Audit'!F334</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G334" s="11" t="str">
+        <x:f>IF(AND(E334=0,F334=1,'Source Audit'!I334&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H334" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="27" customHeight="1">
+      <x:c r="A335" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B335" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C335" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D335" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E335" s="18" t="n">
+        <x:f>'Source Audit'!E335</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F335" s="41" t="n">
+        <x:f>'Source Audit'!F335</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G335" s="12" t="str">
+        <x:f>IF(AND(E335=0,F335=1,'Source Audit'!I335&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H335" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336" ht="27" customHeight="1">
+      <x:c r="A336" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B336" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C336" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D336" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E336" s="19" t="n">
+        <x:f>'Source Audit'!E336</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F336" s="40" t="n">
+        <x:f>'Source Audit'!F336</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G336" s="11" t="str">
+        <x:f>IF(AND(E336=0,F336=1,'Source Audit'!I336&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H336" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337" ht="44" customHeight="1">
+      <x:c r="A337" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B337" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C337" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D337" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E337" s="18" t="n">
+        <x:f>'Source Audit'!E337</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F337" s="41" t="n">
+        <x:f>'Source Audit'!F337</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G337" s="12" t="str">
+        <x:f>IF(AND(E337=0,F337=1,'Source Audit'!I337&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H337" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="27" customHeight="1">
+      <x:c r="A338" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B338" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C338" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D338" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E338" s="19" t="n">
+        <x:f>'Source Audit'!E338</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F338" s="40" t="n">
+        <x:f>'Source Audit'!F338</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G338" s="11" t="str">
+        <x:f>IF(AND(E338=0,F338=1,'Source Audit'!I338&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H338" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" ht="27" customHeight="1">
+      <x:c r="A339" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B339" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C339" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D339" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E339" s="18" t="n">
+        <x:f>'Source Audit'!E339</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F339" s="41" t="n">
+        <x:f>'Source Audit'!F339</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G339" s="12" t="str">
+        <x:f>IF(AND(E339=0,F339=1,'Source Audit'!I339&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H339" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340" ht="27" customHeight="1">
+      <x:c r="A340" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B340" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C340" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D340" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E340" s="19" t="n">
+        <x:f>'Source Audit'!E340</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F340" s="40" t="n">
+        <x:f>'Source Audit'!F340</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G340" s="11" t="str">
+        <x:f>IF(AND(E340=0,F340=1,'Source Audit'!I340&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H340" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341" ht="27" customHeight="1">
+      <x:c r="A341" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B341" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C341" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D341" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E341" s="18" t="n">
+        <x:f>'Source Audit'!E341</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F341" s="41" t="n">
+        <x:f>'Source Audit'!F341</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G341" s="12" t="str">
+        <x:f>IF(AND(E341=0,F341=1,'Source Audit'!I341&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H341" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342" ht="27" customHeight="1">
+      <x:c r="A342" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B342" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C342" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D342" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E342" s="19" t="n">
+        <x:f>'Source Audit'!E342</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F342" s="40" t="n">
+        <x:f>'Source Audit'!F342</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G342" s="11" t="str">
+        <x:f>IF(AND(E342=0,F342=1,'Source Audit'!I342&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H342" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343" ht="27" customHeight="1">
+      <x:c r="A343" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B343" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C343" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D343" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E343" s="18" t="n">
+        <x:f>'Source Audit'!E343</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F343" s="41" t="n">
+        <x:f>'Source Audit'!F343</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G343" s="12" t="str">
+        <x:f>IF(AND(E343=0,F343=1,'Source Audit'!I343&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H343" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344" ht="27" customHeight="1">
+      <x:c r="A344" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B344" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C344" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D344" s="8" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E344" s="19" t="n">
+        <x:f>'Source Audit'!E344</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F344" s="40" t="n">
+        <x:f>'Source Audit'!F344</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G344" s="11" t="str">
+        <x:f>IF(AND(E344=0,F344=1,'Source Audit'!I344&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H344" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345" ht="27" customHeight="1">
+      <x:c r="A345" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="B345" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C345" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D345" s="9" t="n">
+        <x:v>46323</x:v>
+      </x:c>
+      <x:c r="E345" s="18" t="n">
+        <x:f>'Source Audit'!E345</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F345" s="41" t="n">
+        <x:f>'Source Audit'!F345</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G345" s="12" t="str">
+        <x:f>IF(AND(E345=0,F345=1,'Source Audit'!I345&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H345" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -44668,7 +46965,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6479dd0b91864ef6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a0ac8ad6f454596"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 29, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.
Retain the official notices for the upcoming Keyence 5-for-1 split and
document the future ex-date and split-calculation validation gate.

Validation: 17 requested prices, 325 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Both the shared-checkout and exact main-based
publication candidate production builds and article-preview checks passed.
These results are documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0c6f7da7b3c74541"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="R25e5422527154232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="Ra40c58b1cb3d48c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="Ra06f34215e75475e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="R22af659891df4127"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R944c648a01784b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rcf56e2d583eb449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R7096512c37574475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R34c211b0c18441ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Re069f6d8566340ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H305" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H320" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H345" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -2261,6 +2261,85 @@
         <x:v>-3.3107859753424895</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="40" customHeight="1">
+      <x:c r="A26" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="n">
+        <x:f>B25*(1+SUM('Returns and Contributions'!F306:F320))</x:f>
+        <x:v>944.6321286880909</x:v>
+      </x:c>
+      <x:c r="C26" s="20" t="n">
+        <x:f>B26/B25-1</x:f>
+        <x:v>-0.010772247775571953</x:v>
+      </x:c>
+      <x:c r="D26" s="20" t="n">
+        <x:f>B26/$B$6-1</x:f>
+        <x:v>-0.05536787131190912</x:v>
+      </x:c>
+      <x:c r="E26" s="19" t="n">
+        <x:f>1000*'Prices'!H361/'Prices'!I361</x:f>
+        <x:v>1007.0358510131808</x:v>
+      </x:c>
+      <x:c r="F26" s="20" t="n">
+        <x:f>E26/E25-1</x:f>
+        <x:v>-0.003046237206191127</x:v>
+      </x:c>
+      <x:c r="G26" s="20" t="n">
+        <x:f>E26/1000-1</x:f>
+        <x:v>0.007035851013180938</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="n">
+        <x:f>1000*'Prices'!H362/'Prices'!I362</x:f>
+        <x:v>974.4387676984884</x:v>
+      </x:c>
+      <x:c r="I26" s="20" t="n">
+        <x:f>H26/H25-1</x:f>
+        <x:v>-0.013752506247530216</x:v>
+      </x:c>
+      <x:c r="J26" s="20" t="n">
+        <x:f>H26/1000-1</x:f>
+        <x:v>-0.02556123230151164</x:v>
+      </x:c>
+      <x:c r="K26" s="24" t="n">
+        <x:f>(C26-F26)*100</x:f>
+        <x:v>-0.7726010569380826</x:v>
+      </x:c>
+      <x:c r="L26" s="24" t="n">
+        <x:f>(C26-I26)*100</x:f>
+        <x:v>0.29802584719582637</x:v>
+      </x:c>
+      <x:c r="M26" s="22" t="n">
+        <x:f>SUM('Returns and Contributions'!G306:G320)</x:f>
+        <x:v>0.9999999999999998</x:v>
+      </x:c>
+      <x:c r="N26" s="28" t="n">
+        <x:f>SUM('Returns and Contributions'!F306:F320)-C26</x:f>
+        <x:v>4.85722573273506e-17</x:v>
+      </x:c>
+      <x:c r="O26" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P26" s="31" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I346:I362,"Mismatch")=0,IF(COUNTIF('Source Audit'!I346:I362,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q26" s="29" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="R26" s="28" t="n">
+        <x:f>B26-1000*('Prices'!H346/'Prices'!H6+'Prices'!H347/'Prices'!H7+'Prices'!H348/'Prices'!H8+'Prices'!H349/'Prices'!H9+'Prices'!H350/'Prices'!H10+'Prices'!H351/'Prices'!H11+'Prices'!H352/'Prices'!H12+'Prices'!H353/'Prices'!H13+'Prices'!H354/'Prices'!H14+'Prices'!H355/'Prices'!H15+'Prices'!H356/'Prices'!H16+'Prices'!H357/'Prices'!H17+'Prices'!H358/'Prices'!H18+'Prices'!H359/'Prices'!H19+'Prices'!H360/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S26" s="24" t="n">
+        <x:f>(D26-G26)*100</x:f>
+        <x:v>-6.2403722325090065</x:v>
+      </x:c>
+      <x:c r="T26" s="24" t="n">
+        <x:f>(D26-J26)*100</x:f>
+        <x:v>-2.9806639010397484</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -2268,7 +2347,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39614baf2ad246d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d54feeb29d4705"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14570,6 +14649,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="346" ht="27" customHeight="1">
+      <x:c r="A346" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B346" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C346" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D346" s="2" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E346" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F346" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G346" s="17" t="n">
+        <x:f>H329</x:f>
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="H346" s="34" t="n">
+        <x:v>5795</x:v>
+      </x:c>
+      <x:c r="I346" s="34" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J346" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K346" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347" ht="27" customHeight="1">
+      <x:c r="A347" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B347" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C347" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D347" s="10" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E347" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F347" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G347" s="33" t="n">
+        <x:f>H330</x:f>
+        <x:v>4186</x:v>
+      </x:c>
+      <x:c r="H347" s="35" t="n">
+        <x:v>4159</x:v>
+      </x:c>
+      <x:c r="I347" s="35" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J347" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K347" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348" ht="27" customHeight="1">
+      <x:c r="A348" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B348" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C348" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D348" s="2" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E348" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F348" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G348" s="17" t="n">
+        <x:f>H331</x:f>
+        <x:v>30.14</x:v>
+      </x:c>
+      <x:c r="H348" s="34" t="n">
+        <x:v>28.4</x:v>
+      </x:c>
+      <x:c r="I348" s="34" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J348" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K348" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349" ht="27" customHeight="1">
+      <x:c r="A349" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B349" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C349" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D349" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E349" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F349" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G349" s="33" t="n">
+        <x:f>H332</x:f>
+        <x:v>313.24</x:v>
+      </x:c>
+      <x:c r="H349" s="35" t="n">
+        <x:v>296.23</x:v>
+      </x:c>
+      <x:c r="I349" s="35" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J349" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K349" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350" ht="27" customHeight="1">
+      <x:c r="A350" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B350" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C350" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D350" s="2" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E350" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F350" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G350" s="17" t="n">
+        <x:f>H333</x:f>
+        <x:v>4420</x:v>
+      </x:c>
+      <x:c r="H350" s="34" t="n">
+        <x:v>4384</x:v>
+      </x:c>
+      <x:c r="I350" s="34" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J350" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K350" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351" ht="27" customHeight="1">
+      <x:c r="A351" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B351" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C351" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D351" s="10" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E351" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F351" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G351" s="33" t="n">
+        <x:f>H334</x:f>
+        <x:v>56.16</x:v>
+      </x:c>
+      <x:c r="H351" s="35" t="n">
+        <x:v>56.78</x:v>
+      </x:c>
+      <x:c r="I351" s="35" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J351" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K351" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352" ht="27" customHeight="1">
+      <x:c r="A352" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B352" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C352" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D352" s="2" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E352" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F352" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G352" s="17" t="n">
+        <x:f>H335</x:f>
+        <x:v>79190</x:v>
+      </x:c>
+      <x:c r="H352" s="34" t="n">
+        <x:v>76360</x:v>
+      </x:c>
+      <x:c r="I352" s="34" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J352" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K352" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353" ht="27" customHeight="1">
+      <x:c r="A353" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B353" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C353" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D353" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E353" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F353" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G353" s="33" t="n">
+        <x:f>H336</x:f>
+        <x:v>58.43</x:v>
+      </x:c>
+      <x:c r="H353" s="35" t="n">
+        <x:v>58.97</x:v>
+      </x:c>
+      <x:c r="I353" s="35" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J353" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K353" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354" ht="27" customHeight="1">
+      <x:c r="A354" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B354" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C354" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D354" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E354" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F354" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G354" s="17" t="n">
+        <x:f>H337</x:f>
+        <x:v>33.61</x:v>
+      </x:c>
+      <x:c r="H354" s="34" t="n">
+        <x:v>32.14</x:v>
+      </x:c>
+      <x:c r="I354" s="34" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J354" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K354" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="27" customHeight="1">
+      <x:c r="A355" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B355" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C355" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D355" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E355" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F355" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G355" s="33" t="n">
+        <x:f>H338</x:f>
+        <x:v>13.83</x:v>
+      </x:c>
+      <x:c r="H355" s="35" t="n">
+        <x:v>12.97</x:v>
+      </x:c>
+      <x:c r="I355" s="35" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J355" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K355" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="27" customHeight="1">
+      <x:c r="A356" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B356" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C356" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D356" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E356" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F356" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G356" s="17" t="n">
+        <x:f>H339</x:f>
+        <x:v>443.81</x:v>
+      </x:c>
+      <x:c r="H356" s="34" t="n">
+        <x:v>451.4</x:v>
+      </x:c>
+      <x:c r="I356" s="34" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J356" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K356" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357" ht="27" customHeight="1">
+      <x:c r="A357" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B357" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C357" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D357" s="10" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E357" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F357" s="10" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G357" s="33" t="n">
+        <x:f>H340</x:f>
+        <x:v>270.05</x:v>
+      </x:c>
+      <x:c r="H357" s="35" t="n">
+        <x:v>273.75</x:v>
+      </x:c>
+      <x:c r="I357" s="35" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J357" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K357" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="27" customHeight="1">
+      <x:c r="A358" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B358" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C358" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D358" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E358" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F358" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G358" s="17" t="n">
+        <x:f>H341</x:f>
+        <x:v>251.69</x:v>
+      </x:c>
+      <x:c r="H358" s="34" t="n">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="I358" s="34" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J358" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K358" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="27" customHeight="1">
+      <x:c r="A359" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B359" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C359" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D359" s="10" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E359" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F359" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G359" s="33" t="n">
+        <x:f>H342</x:f>
+        <x:v>5441</x:v>
+      </x:c>
+      <x:c r="H359" s="35" t="n">
+        <x:v>5363</x:v>
+      </x:c>
+      <x:c r="I359" s="35" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J359" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K359" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="27" customHeight="1">
+      <x:c r="A360" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B360" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C360" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D360" s="2" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E360" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F360" s="2" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G360" s="17" t="n">
+        <x:f>H343</x:f>
+        <x:v>109.45</x:v>
+      </x:c>
+      <x:c r="H360" s="34" t="n">
+        <x:v>110.1</x:v>
+      </x:c>
+      <x:c r="I360" s="34" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J360" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K360" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="27" customHeight="1">
+      <x:c r="A361" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B361" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C361" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D361" s="10" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E361" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F361" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G361" s="33" t="n">
+        <x:f>H344</x:f>
+        <x:v>7743.98</x:v>
+      </x:c>
+      <x:c r="H361" s="35" t="n">
+        <x:v>7720.39</x:v>
+      </x:c>
+      <x:c r="I361" s="35" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J361" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K361" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="27" customHeight="1">
+      <x:c r="A362" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B362" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C362" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D362" s="2" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E362" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F362" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G362" s="17" t="n">
+        <x:f>H345</x:f>
+        <x:v>26549.8516</x:v>
+      </x:c>
+      <x:c r="H362" s="34" t="n">
+        <x:v>26184.7246</x:v>
+      </x:c>
+      <x:c r="I362" s="34" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J362" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="K362" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -14577,7 +15268,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re707c100ef7340ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46cb2231a0b940ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23876,6 +24567,471 @@
         <x:v>0.10533225610987684</x:v>
       </x:c>
     </x:row>
+    <x:row r="306" ht="27" customHeight="1">
+      <x:c r="A306" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B306" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C306" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D306" s="20" t="n">
+        <x:f>G291</x:f>
+        <x:v>0.06731857687462542</x:v>
+      </x:c>
+      <x:c r="E306" s="22" t="n">
+        <x:f>'Prices'!H346/'Prices'!G346-1</x:f>
+        <x:v>-0.01912660798916721</x:v>
+      </x:c>
+      <x:c r="F306" s="20" t="n">
+        <x:f>D306*E306</x:f>
+        <x:v>-0.0012875760302695776</x:v>
+      </x:c>
+      <x:c r="G306" s="20" t="n">
+        <x:f>D306*(1+E306)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.06675004891024859</x:v>
+      </x:c>
+      <x:c r="H306" s="22" t="n">
+        <x:f>'Prices'!H346/'Prices'!I346-1</x:f>
+        <x:v>-0.05418638811816545</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="27" customHeight="1">
+      <x:c r="A307" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B307" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C307" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D307" s="21" t="n">
+        <x:f>G292</x:f>
+        <x:v>0.061151133777782835</x:v>
+      </x:c>
+      <x:c r="E307" s="23" t="n">
+        <x:f>'Prices'!H347/'Prices'!G347-1</x:f>
+        <x:v>-0.00645007166746292</x:v>
+      </x:c>
+      <x:c r="F307" s="21" t="n">
+        <x:f>D307*E307</x:f>
+        <x:v>-0.0003944291954133118</x:v>
+      </x:c>
+      <x:c r="G307" s="21" t="n">
+        <x:f>D307*(1+E307)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.061418317920973096</x:v>
+      </x:c>
+      <x:c r="H307" s="23" t="n">
+        <x:f>'Prices'!H347/'Prices'!I347-1</x:f>
+        <x:v>-0.1297342540280393</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="27" customHeight="1">
+      <x:c r="A308" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B308" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C308" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D308" s="20" t="n">
+        <x:f>G293</x:f>
+        <x:v>0.07456389025893134</x:v>
+      </x:c>
+      <x:c r="E308" s="22" t="n">
+        <x:f>'Prices'!H348/'Prices'!G348-1</x:f>
+        <x:v>-0.05773059057730601</x:v>
+      </x:c>
+      <x:c r="F308" s="20" t="n">
+        <x:f>D308*E308</x:f>
+        <x:v>-0.004304617420389541</x:v>
+      </x:c>
+      <x:c r="G308" s="20" t="n">
+        <x:f>D308*(1+E308)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07102436489529657</x:v>
+      </x:c>
+      <x:c r="H308" s="22" t="n">
+        <x:f>'Prices'!H348/'Prices'!I348-1</x:f>
+        <x:v>0.006378454996456506</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="27" customHeight="1">
+      <x:c r="A309" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B309" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C309" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D309" s="21" t="n">
+        <x:f>G294</x:f>
+        <x:v>0.05259512544148299</x:v>
+      </x:c>
+      <x:c r="E309" s="23" t="n">
+        <x:f>'Prices'!H349/'Prices'!G349-1</x:f>
+        <x:v>-0.0543034095262418</x:v>
+      </x:c>
+      <x:c r="F309" s="21" t="n">
+        <x:f>D309*E309</x:f>
+        <x:v>-0.0028560946359329096</x:v>
+      </x:c>
+      <x:c r="G309" s="21" t="n">
+        <x:f>D309*(1+E309)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.05028066660453506</x:v>
+      </x:c>
+      <x:c r="H309" s="23" t="n">
+        <x:f>'Prices'!H349/'Prices'!I349-1</x:f>
+        <x:v>-0.28754900310252773</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="27" customHeight="1">
+      <x:c r="A310" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B310" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C310" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D310" s="20" t="n">
+        <x:f>G295</x:f>
+        <x:v>0.062025675726563374</x:v>
+      </x:c>
+      <x:c r="E310" s="22" t="n">
+        <x:f>'Prices'!H350/'Prices'!G350-1</x:f>
+        <x:v>-0.008144796380090469</x:v>
+      </x:c>
+      <x:c r="F310" s="20" t="n">
+        <x:f>D310*E310</x:f>
+        <x:v>-0.0005051864991303787</x:v>
+      </x:c>
+      <x:c r="G310" s="20" t="n">
+        <x:f>D310*(1+E310)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.06219041983920778</x:v>
+      </x:c>
+      <x:c r="H310" s="22" t="n">
+        <x:f>'Prices'!H350/'Prices'!I350-1</x:f>
+        <x:v>-0.11879396984924628</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="27" customHeight="1">
+      <x:c r="A311" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B311" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C311" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D311" s="21" t="n">
+        <x:f>G296</x:f>
+        <x:v>0.075544362615624</x:v>
+      </x:c>
+      <x:c r="E311" s="23" t="n">
+        <x:f>'Prices'!H351/'Prices'!G351-1</x:f>
+        <x:v>0.011039886039886149</x:v>
+      </x:c>
+      <x:c r="F311" s="21" t="n">
+        <x:f>D311*E311</x:f>
+        <x:v>0.0008340011542323244</x:v>
+      </x:c>
+      <x:c r="G311" s="21" t="n">
+        <x:f>D311*(1+E311)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07721008999000284</x:v>
+      </x:c>
+      <x:c r="H311" s="23" t="n">
+        <x:f>'Prices'!H351/'Prices'!I351-1</x:f>
+        <x:v>0.09402697495183054</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="312" ht="27" customHeight="1">
+      <x:c r="A312" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B312" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C312" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D312" s="20" t="n">
+        <x:f>G297</x:f>
+        <x:v>0.06808581395697205</x:v>
+      </x:c>
+      <x:c r="E312" s="22" t="n">
+        <x:f>'Prices'!H352/'Prices'!G352-1</x:f>
+        <x:v>-0.03573683545902262</x:v>
+      </x:c>
+      <x:c r="F312" s="20" t="n">
+        <x:f>D312*E312</x:f>
+        <x:v>-0.002433171530473936</x:v>
+      </x:c>
+      <x:c r="G312" s="20" t="n">
+        <x:f>D312*(1+E312)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.06636757033844656</x:v>
+      </x:c>
+      <x:c r="H312" s="22" t="n">
+        <x:f>'Prices'!H352/'Prices'!I352-1</x:f>
+        <x:v>-0.05960591133004922</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="27" customHeight="1">
+      <x:c r="A313" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B313" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C313" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D313" s="21" t="n">
+        <x:f>G298</x:f>
+        <x:v>0.06556139707772415</x:v>
+      </x:c>
+      <x:c r="E313" s="23" t="n">
+        <x:f>'Prices'!H353/'Prices'!G353-1</x:f>
+        <x:v>0.009241827828170512</x:v>
+      </x:c>
+      <x:c r="F313" s="21" t="n">
+        <x:f>D313*E313</x:f>
+        <x:v>0.000605907143966648</x:v>
+      </x:c>
+      <x:c r="G313" s="21" t="n">
+        <x:f>D313*(1+E313)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.06688783657039911</x:v>
+      </x:c>
+      <x:c r="H313" s="23" t="n">
+        <x:f>'Prices'!H353/'Prices'!I353-1</x:f>
+        <x:v>-0.0522340083574413</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="27" customHeight="1">
+      <x:c r="A314" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B314" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C314" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D314" s="20" t="n">
+        <x:f>G299</x:f>
+        <x:v>0.057412465148958855</x:v>
+      </x:c>
+      <x:c r="E314" s="22" t="n">
+        <x:f>'Prices'!H354/'Prices'!G354-1</x:f>
+        <x:v>-0.04373698304076168</x:v>
+      </x:c>
+      <x:c r="F314" s="20" t="n">
+        <x:f>D314*E314</x:f>
+        <x:v>-0.0025110480145483344</x:v>
+      </x:c>
+      <x:c r="G314" s="20" t="n">
+        <x:f>D314*(1+E314)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.05549926901156623</x:v>
+      </x:c>
+      <x:c r="H314" s="22" t="n">
+        <x:f>'Prices'!H354/'Prices'!I354-1</x:f>
+        <x:v>-0.21360411059456808</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="27" customHeight="1">
+      <x:c r="A315" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B315" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C315" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D315" s="21" t="n">
+        <x:f>G300</x:f>
+        <x:v>0.06061061969517942</x:v>
+      </x:c>
+      <x:c r="E315" s="23" t="n">
+        <x:f>'Prices'!H355/'Prices'!G355-1</x:f>
+        <x:v>-0.062183658712942846</x:v>
+      </x:c>
+      <x:c r="F315" s="21" t="n">
+        <x:f>D315*E315</x:f>
+        <x:v>-0.003768990089505009</x:v>
+      </x:c>
+      <x:c r="G315" s="21" t="n">
+        <x:f>D315*(1+E315)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.05746060952885462</x:v>
+      </x:c>
+      <x:c r="H315" s="23" t="n">
+        <x:f>'Prices'!H355/'Prices'!I355-1</x:f>
+        <x:v>-0.18581293157564338</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="27" customHeight="1">
+      <x:c r="A316" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B316" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C316" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D316" s="20" t="n">
+        <x:f>G301</x:f>
+        <x:v>0.07002856131834063</x:v>
+      </x:c>
+      <x:c r="E316" s="22" t="n">
+        <x:f>'Prices'!H356/'Prices'!G356-1</x:f>
+        <x:v>0.0171019129807799</x:v>
+      </x:c>
+      <x:c r="F316" s="20" t="n">
+        <x:f>D316*E316</x:f>
+        <x:v>0.0011976223618354708</x:v>
+      </x:c>
+      <x:c r="G316" s="20" t="n">
+        <x:f>D316*(1+E316)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07200180496353167</x:v>
+      </x:c>
+      <x:c r="H316" s="22" t="n">
+        <x:f>'Prices'!H356/'Prices'!I356-1</x:f>
+        <x:v>0.02022827438128605</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="27" customHeight="1">
+      <x:c r="A317" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B317" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C317" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D317" s="21" t="n">
+        <x:f>G302</x:f>
+        <x:v>0.06933895530408873</x:v>
+      </x:c>
+      <x:c r="E317" s="23" t="n">
+        <x:f>'Prices'!H357/'Prices'!G357-1</x:f>
+        <x:v>0.01370116645065722</x:v>
+      </x:c>
+      <x:c r="F317" s="21" t="n">
+        <x:f>D317*E317</x:f>
+        <x:v>0.0009500245681360011</x:v>
+      </x:c>
+      <x:c r="G317" s="21" t="n">
+        <x:f>D317*(1+E317)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07105439542528942</x:v>
+      </x:c>
+      <x:c r="H317" s="23" t="n">
+        <x:f>'Prices'!H357/'Prices'!I357-1</x:f>
+        <x:v>0.006803972048547324</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="27" customHeight="1">
+      <x:c r="A318" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B318" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C318" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D318" s="20" t="n">
+        <x:f>G303</x:f>
+        <x:v>0.07346242527807668</x:v>
+      </x:c>
+      <x:c r="E318" s="22" t="n">
+        <x:f>'Prices'!H358/'Prices'!G358-1</x:f>
+        <x:v>0.05685565576701501</x:v>
+      </x:c>
+      <x:c r="F318" s="20" t="n">
+        <x:f>D318*E318</x:f>
+        <x:v>0.00417675436342039</x:v>
+      </x:c>
+      <x:c r="G318" s="20" t="n">
+        <x:f>D318*(1+E318)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07848463558256798</x:v>
+      </x:c>
+      <x:c r="H318" s="22" t="n">
+        <x:f>'Prices'!H358/'Prices'!I358-1</x:f>
+        <x:v>0.11208662569505412</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319" ht="27" customHeight="1">
+      <x:c r="A319" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B319" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C319" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D319" s="21" t="n">
+        <x:f>G304</x:f>
+        <x:v>0.06513336722345002</x:v>
+      </x:c>
+      <x:c r="E319" s="23" t="n">
+        <x:f>'Prices'!H359/'Prices'!G359-1</x:f>
+        <x:v>-0.014335600073515864</x:v>
+      </x:c>
+      <x:c r="F319" s="21" t="n">
+        <x:f>D319*E319</x:f>
+        <x:v>-0.0009337259039568259</x:v>
+      </x:c>
+      <x:c r="G319" s="21" t="n">
+        <x:f>D319*(1+E319)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.06489874669926173</x:v>
+      </x:c>
+      <x:c r="H319" s="23" t="n">
+        <x:f>'Prices'!H359/'Prices'!I359-1</x:f>
+        <x:v>-0.08041838134430723</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320" ht="27" customHeight="1">
+      <x:c r="A320" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B320" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C320" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D320" s="20" t="n">
+        <x:f>G305</x:f>
+        <x:v>0.07716763030219907</x:v>
+      </x:c>
+      <x:c r="E320" s="22" t="n">
+        <x:f>'Prices'!H360/'Prices'!G360-1</x:f>
+        <x:v>0.005938784833257049</x:v>
+      </x:c>
+      <x:c r="F320" s="20" t="n">
+        <x:f>D320*E320</x:f>
+        <x:v>0.00045828195245708694</x:v>
+      </x:c>
+      <x:c r="G320" s="20" t="n">
+        <x:f>D320*(1+E320)/(1+SUM($F$306:$F$320))</x:f>
+        <x:v>0.07847122371981839</x:v>
+      </x:c>
+      <x:c r="H320" s="22" t="n">
+        <x:f>'Prices'!H360/'Prices'!I360-1</x:f>
+        <x:v>0.11189658654817203</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -23883,7 +25039,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae68bcb6acd044f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43d6650d4c52470c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37002,6 +38158,654 @@
       </x:c>
       <x:c r="M345" s="16" t="str"/>
     </x:row>
+    <x:row r="346" ht="50" customHeight="1">
+      <x:c r="A346" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B346" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C346" s="17" t="n">
+        <x:v>5795</x:v>
+      </x:c>
+      <x:c r="D346" s="17" t="n">
+        <x:v>5795</x:v>
+      </x:c>
+      <x:c r="E346" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F346" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G346" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H346" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I346" s="31" t="str">
+        <x:f>IF(AND(G346=H346,C346&gt;0,ABS(C346-'Prices'!H346)&lt;=MAX(0.01,'Prices'!H346*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J346" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K346" s="14" t="str"/>
+      <x:c r="L346" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M346" s="14" t="str"/>
+    </x:row>
+    <x:row r="347" ht="50" customHeight="1">
+      <x:c r="A347" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B347" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C347" s="33" t="n">
+        <x:v>4159</x:v>
+      </x:c>
+      <x:c r="D347" s="33" t="n">
+        <x:v>4159</x:v>
+      </x:c>
+      <x:c r="E347" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F347" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G347" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H347" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I347" s="32" t="str">
+        <x:f>IF(AND(G347=H347,C347&gt;0,ABS(C347-'Prices'!H347)&lt;=MAX(0.01,'Prices'!H347*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J347" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K347" s="16" t="str"/>
+      <x:c r="L347" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M347" s="16" t="str"/>
+    </x:row>
+    <x:row r="348" ht="50" customHeight="1">
+      <x:c r="A348" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B348" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C348" s="17" t="n">
+        <x:v>28.4</x:v>
+      </x:c>
+      <x:c r="D348" s="17" t="n">
+        <x:v>28.4</x:v>
+      </x:c>
+      <x:c r="E348" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F348" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G348" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H348" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I348" s="31" t="str">
+        <x:f>IF(AND(G348=H348,C348&gt;0,ABS(C348-'Prices'!H348)&lt;=MAX(0.01,'Prices'!H348*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J348" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K348" s="14" t="str"/>
+      <x:c r="L348" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M348" s="14" t="str"/>
+    </x:row>
+    <x:row r="349" ht="50" customHeight="1">
+      <x:c r="A349" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B349" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C349" s="33" t="n">
+        <x:v>296.23</x:v>
+      </x:c>
+      <x:c r="D349" s="33" t="n">
+        <x:v>296.23</x:v>
+      </x:c>
+      <x:c r="E349" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F349" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G349" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H349" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I349" s="32" t="str">
+        <x:f>IF(AND(G349=H349,C349&gt;0,ABS(C349-'Prices'!H349)&lt;=MAX(0.01,'Prices'!H349*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J349" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K349" s="16" t="str"/>
+      <x:c r="L349" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M349" s="16" t="str"/>
+    </x:row>
+    <x:row r="350" ht="50" customHeight="1">
+      <x:c r="A350" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B350" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C350" s="17" t="n">
+        <x:v>4384</x:v>
+      </x:c>
+      <x:c r="D350" s="17" t="n">
+        <x:v>4384</x:v>
+      </x:c>
+      <x:c r="E350" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F350" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G350" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H350" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I350" s="31" t="str">
+        <x:f>IF(AND(G350=H350,C350&gt;0,ABS(C350-'Prices'!H350)&lt;=MAX(0.01,'Prices'!H350*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J350" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K350" s="14" t="str"/>
+      <x:c r="L350" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M350" s="14" t="str"/>
+    </x:row>
+    <x:row r="351" ht="50" customHeight="1">
+      <x:c r="A351" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B351" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C351" s="33" t="n">
+        <x:v>56.78</x:v>
+      </x:c>
+      <x:c r="D351" s="33" t="n">
+        <x:v>56.78</x:v>
+      </x:c>
+      <x:c r="E351" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F351" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G351" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H351" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I351" s="32" t="str">
+        <x:f>IF(AND(G351=H351,C351&gt;0,ABS(C351-'Prices'!H351)&lt;=MAX(0.01,'Prices'!H351*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J351" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K351" s="16" t="str"/>
+      <x:c r="L351" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M351" s="16" t="str"/>
+    </x:row>
+    <x:row r="352" ht="50" customHeight="1">
+      <x:c r="A352" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B352" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C352" s="17" t="n">
+        <x:v>76360</x:v>
+      </x:c>
+      <x:c r="D352" s="17" t="n">
+        <x:v>76360</x:v>
+      </x:c>
+      <x:c r="E352" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F352" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G352" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H352" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I352" s="31" t="str">
+        <x:f>IF(AND(G352=H352,C352&gt;0,ABS(C352-'Prices'!H352)&lt;=MAX(0.01,'Prices'!H352*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J352" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K352" s="14" t="str"/>
+      <x:c r="L352" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M352" s="14" t="str"/>
+    </x:row>
+    <x:row r="353" ht="50" customHeight="1">
+      <x:c r="A353" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B353" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C353" s="33" t="n">
+        <x:v>58.97</x:v>
+      </x:c>
+      <x:c r="D353" s="33" t="n">
+        <x:v>58.97</x:v>
+      </x:c>
+      <x:c r="E353" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F353" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G353" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H353" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I353" s="32" t="str">
+        <x:f>IF(AND(G353=H353,C353&gt;0,ABS(C353-'Prices'!H353)&lt;=MAX(0.01,'Prices'!H353*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J353" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K353" s="16" t="str"/>
+      <x:c r="L353" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M353" s="16" t="str"/>
+    </x:row>
+    <x:row r="354" ht="50" customHeight="1">
+      <x:c r="A354" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B354" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C354" s="17" t="n">
+        <x:v>32.14</x:v>
+      </x:c>
+      <x:c r="D354" s="17" t="n">
+        <x:v>32.14</x:v>
+      </x:c>
+      <x:c r="E354" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F354" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G354" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H354" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I354" s="31" t="str">
+        <x:f>IF(AND(OR(G354=H354,AND(B354="OUST",G354="XNAS",H354="XNYS",LEFT(M354,34)="ouster-marketstack-legacy-nyse-tag")),C354&gt;0,ABS(C354-'Prices'!H354)&lt;=MAX(0.01,'Prices'!H354*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J354" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K354" s="14" t="str"/>
+      <x:c r="L354" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M354" s="14" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="50" customHeight="1">
+      <x:c r="A355" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B355" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C355" s="33" t="n">
+        <x:v>12.97</x:v>
+      </x:c>
+      <x:c r="D355" s="33" t="n">
+        <x:v>12.97</x:v>
+      </x:c>
+      <x:c r="E355" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F355" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G355" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H355" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I355" s="32" t="str">
+        <x:f>IF(AND(G355=H355,C355&gt;0,ABS(C355-'Prices'!H355)&lt;=MAX(0.01,'Prices'!H355*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J355" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K355" s="16" t="str"/>
+      <x:c r="L355" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M355" s="16" t="str"/>
+    </x:row>
+    <x:row r="356" ht="50" customHeight="1">
+      <x:c r="A356" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B356" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C356" s="17" t="n">
+        <x:v>451.4</x:v>
+      </x:c>
+      <x:c r="D356" s="17" t="n">
+        <x:v>451.4</x:v>
+      </x:c>
+      <x:c r="E356" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F356" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G356" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H356" s="2" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I356" s="31" t="str">
+        <x:f>IF(AND(G356=H356,C356&gt;0,ABS(C356-'Prices'!H356)&lt;=MAX(0.01,'Prices'!H356*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J356" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K356" s="14" t="str"/>
+      <x:c r="L356" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M356" s="14" t="str"/>
+    </x:row>
+    <x:row r="357" ht="50" customHeight="1">
+      <x:c r="A357" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B357" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C357" s="33" t="n">
+        <x:v>273.75</x:v>
+      </x:c>
+      <x:c r="D357" s="33" t="n">
+        <x:v>273.75</x:v>
+      </x:c>
+      <x:c r="E357" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F357" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G357" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H357" s="10" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I357" s="32" t="str">
+        <x:f>IF(AND(G357=H357,C357&gt;0,ABS(C357-'Prices'!H357)&lt;=MAX(0.01,'Prices'!H357*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J357" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K357" s="16" t="str"/>
+      <x:c r="L357" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M357" s="16" t="str"/>
+    </x:row>
+    <x:row r="358" ht="50" customHeight="1">
+      <x:c r="A358" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B358" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C358" s="17" t="n">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="D358" s="17" t="n">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="E358" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F358" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G358" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H358" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I358" s="31" t="str">
+        <x:f>IF(AND(G358=H358,C358&gt;0,ABS(C358-'Prices'!H358)&lt;=MAX(0.01,'Prices'!H358*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J358" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K358" s="14" t="str"/>
+      <x:c r="L358" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M358" s="14" t="str"/>
+    </x:row>
+    <x:row r="359" ht="50" customHeight="1">
+      <x:c r="A359" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B359" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C359" s="33" t="n">
+        <x:v>5363</x:v>
+      </x:c>
+      <x:c r="D359" s="33" t="n">
+        <x:v>5363</x:v>
+      </x:c>
+      <x:c r="E359" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F359" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G359" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H359" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I359" s="32" t="str">
+        <x:f>IF(AND(G359=H359,C359&gt;0,ABS(C359-'Prices'!H359)&lt;=MAX(0.01,'Prices'!H359*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J359" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K359" s="16" t="str"/>
+      <x:c r="L359" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M359" s="16" t="str"/>
+    </x:row>
+    <x:row r="360" ht="50" customHeight="1">
+      <x:c r="A360" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B360" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C360" s="17" t="n">
+        <x:v>110.1</x:v>
+      </x:c>
+      <x:c r="D360" s="17" t="n">
+        <x:v>110.1</x:v>
+      </x:c>
+      <x:c r="E360" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F360" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G360" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H360" s="2" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I360" s="31" t="str">
+        <x:f>IF(AND(G360=H360,C360&gt;0,ABS(C360-'Prices'!H360)&lt;=MAX(0.01,'Prices'!H360*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J360" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K360" s="14" t="str"/>
+      <x:c r="L360" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M360" s="14" t="str"/>
+    </x:row>
+    <x:row r="361" ht="50" customHeight="1">
+      <x:c r="A361" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B361" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C361" s="33" t="n">
+        <x:v>7720.39</x:v>
+      </x:c>
+      <x:c r="D361" s="33" t="n">
+        <x:v>7720.39</x:v>
+      </x:c>
+      <x:c r="E361" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F361" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G361" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H361" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I361" s="32" t="str">
+        <x:f>IF(AND(G361=H361,C361&gt;0,ABS(C361-'Prices'!H361)&lt;=MAX(0.01,'Prices'!H361*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J361" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K361" s="16" t="str"/>
+      <x:c r="L361" s="39" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M361" s="16" t="str"/>
+    </x:row>
+    <x:row r="362" ht="50" customHeight="1">
+      <x:c r="A362" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B362" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C362" s="17" t="n">
+        <x:v>26184.7246</x:v>
+      </x:c>
+      <x:c r="D362" s="17" t="n">
+        <x:v>26184.7246</x:v>
+      </x:c>
+      <x:c r="E362" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F362" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G362" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H362" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I362" s="31" t="str">
+        <x:f>IF(AND(G362=H362,C362&gt;0,ABS(C362-'Prices'!H362)&lt;=MAX(0.01,'Prices'!H362*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J362" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-30T11-33-49-817Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K362" s="14" t="str"/>
+      <x:c r="L362" s="38" t="n">
+        <x:v>46325.481826585645</x:v>
+      </x:c>
+      <x:c r="M362" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -37009,7 +38813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc758ba6c7546e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d6c6f350b214026"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46958,6 +48762,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="346" ht="27" customHeight="1">
+      <x:c r="A346" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B346" s="2" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C346" s="2" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D346" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E346" s="19" t="n">
+        <x:f>'Source Audit'!E346</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F346" s="40" t="n">
+        <x:f>'Source Audit'!F346</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G346" s="11" t="str">
+        <x:f>IF(AND(E346=0,F346=1,'Source Audit'!I346&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H346" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347" ht="27" customHeight="1">
+      <x:c r="A347" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B347" s="10" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C347" s="10" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D347" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E347" s="18" t="n">
+        <x:f>'Source Audit'!E347</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F347" s="41" t="n">
+        <x:f>'Source Audit'!F347</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G347" s="12" t="str">
+        <x:f>IF(AND(E347=0,F347=1,'Source Audit'!I347&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H347" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348" ht="27" customHeight="1">
+      <x:c r="A348" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B348" s="2" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C348" s="13" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D348" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E348" s="19" t="n">
+        <x:f>'Source Audit'!E348</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F348" s="40" t="n">
+        <x:f>'Source Audit'!F348</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G348" s="11" t="str">
+        <x:f>IF(AND(E348=0,F348=1,'Source Audit'!I348&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H348" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349" ht="27" customHeight="1">
+      <x:c r="A349" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B349" s="10" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C349" s="10" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D349" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E349" s="18" t="n">
+        <x:f>'Source Audit'!E349</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F349" s="41" t="n">
+        <x:f>'Source Audit'!F349</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G349" s="12" t="str">
+        <x:f>IF(AND(E349=0,F349=1,'Source Audit'!I349&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H349" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350" ht="27" customHeight="1">
+      <x:c r="A350" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B350" s="2" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C350" s="2" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D350" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E350" s="19" t="n">
+        <x:f>'Source Audit'!E350</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F350" s="40" t="n">
+        <x:f>'Source Audit'!F350</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G350" s="11" t="str">
+        <x:f>IF(AND(E350=0,F350=1,'Source Audit'!I350&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H350" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351" ht="27" customHeight="1">
+      <x:c r="A351" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B351" s="10" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C351" s="10" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D351" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E351" s="18" t="n">
+        <x:f>'Source Audit'!E351</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F351" s="41" t="n">
+        <x:f>'Source Audit'!F351</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G351" s="12" t="str">
+        <x:f>IF(AND(E351=0,F351=1,'Source Audit'!I351&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H351" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352" ht="27" customHeight="1">
+      <x:c r="A352" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B352" s="2" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C352" s="2" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D352" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E352" s="19" t="n">
+        <x:f>'Source Audit'!E352</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F352" s="40" t="n">
+        <x:f>'Source Audit'!F352</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G352" s="11" t="str">
+        <x:f>IF(AND(E352=0,F352=1,'Source Audit'!I352&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H352" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353" ht="27" customHeight="1">
+      <x:c r="A353" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B353" s="10" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C353" s="10" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D353" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E353" s="18" t="n">
+        <x:f>'Source Audit'!E353</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F353" s="41" t="n">
+        <x:f>'Source Audit'!F353</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G353" s="12" t="str">
+        <x:f>IF(AND(E353=0,F353=1,'Source Audit'!I353&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H353" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354" ht="44" customHeight="1">
+      <x:c r="A354" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B354" s="2" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C354" s="2" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D354" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E354" s="19" t="n">
+        <x:f>'Source Audit'!E354</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F354" s="40" t="n">
+        <x:f>'Source Audit'!F354</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G354" s="11" t="str">
+        <x:f>IF(AND(E354=0,F354=1,'Source Audit'!I354&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H354" s="14" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="27" customHeight="1">
+      <x:c r="A355" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B355" s="10" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C355" s="10" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D355" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E355" s="18" t="n">
+        <x:f>'Source Audit'!E355</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F355" s="41" t="n">
+        <x:f>'Source Audit'!F355</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G355" s="12" t="str">
+        <x:f>IF(AND(E355=0,F355=1,'Source Audit'!I355&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H355" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="27" customHeight="1">
+      <x:c r="A356" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B356" s="2" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C356" s="2" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D356" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E356" s="19" t="n">
+        <x:f>'Source Audit'!E356</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F356" s="40" t="n">
+        <x:f>'Source Audit'!F356</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G356" s="11" t="str">
+        <x:f>IF(AND(E356=0,F356=1,'Source Audit'!I356&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H356" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357" ht="27" customHeight="1">
+      <x:c r="A357" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B357" s="10" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C357" s="10" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D357" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E357" s="18" t="n">
+        <x:f>'Source Audit'!E357</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F357" s="41" t="n">
+        <x:f>'Source Audit'!F357</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G357" s="12" t="str">
+        <x:f>IF(AND(E357=0,F357=1,'Source Audit'!I357&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H357" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="27" customHeight="1">
+      <x:c r="A358" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B358" s="2" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C358" s="2" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D358" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E358" s="19" t="n">
+        <x:f>'Source Audit'!E358</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F358" s="40" t="n">
+        <x:f>'Source Audit'!F358</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G358" s="11" t="str">
+        <x:f>IF(AND(E358=0,F358=1,'Source Audit'!I358&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H358" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="27" customHeight="1">
+      <x:c r="A359" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B359" s="10" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C359" s="10" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D359" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E359" s="18" t="n">
+        <x:f>'Source Audit'!E359</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F359" s="41" t="n">
+        <x:f>'Source Audit'!F359</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G359" s="12" t="str">
+        <x:f>IF(AND(E359=0,F359=1,'Source Audit'!I359&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H359" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="27" customHeight="1">
+      <x:c r="A360" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B360" s="2" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C360" s="2" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D360" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E360" s="19" t="n">
+        <x:f>'Source Audit'!E360</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F360" s="40" t="n">
+        <x:f>'Source Audit'!F360</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G360" s="11" t="str">
+        <x:f>IF(AND(E360=0,F360=1,'Source Audit'!I360&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H360" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="27" customHeight="1">
+      <x:c r="A361" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B361" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C361" s="10" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D361" s="9" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E361" s="18" t="n">
+        <x:f>'Source Audit'!E361</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F361" s="41" t="n">
+        <x:f>'Source Audit'!F361</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G361" s="12" t="str">
+        <x:f>IF(AND(E361=0,F361=1,'Source Audit'!I361&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H361" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="27" customHeight="1">
+      <x:c r="A362" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="B362" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C362" s="2" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D362" s="8" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="E362" s="19" t="n">
+        <x:f>'Source Audit'!E362</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F362" s="40" t="n">
+        <x:f>'Source Audit'!F362</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G362" s="11" t="str">
+        <x:f>IF(AND(E362=0,F362=1,'Source Audit'!I362&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H362" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -46965,7 +49262,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a0ac8ad6f454596"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b99d3baab24f4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update BSPI15 for October 30, 2026
Append the complete audited closing-price row and update the cumulative
five-sheet review workbook, preserved source history and website data.

Validation: 17 requested prices, 342 historical closes, both index
calculations, weights and contributions, workbook recalculation, typecheck,
production builds, targeted BSPI15 lint, desktop/mobile rendering, eight
responsive sizes and holdings CSV passed. Preserve the approved OUST
provider-MIC exception. Repository lint reports 13 unrelated output-script
errors and 9 warnings. Both the shared-checkout and exact main-based
publication candidate production builds and article-preview checks passed.
These results are documented in the dated status report.
</commit_message>
<xml_diff>
--- a/outputs/bspi15-daily-review.xlsx
+++ b/outputs/bspi15-daily-review.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R944c648a01784b21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rcf56e2d583eb449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R7096512c37574475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R34c211b0c18441ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Re069f6d8566340ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfa69787172494cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="2" r:id="Rf7d11f67011b4561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Contributions" sheetId="3" r:id="R00467ecc521047e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Audit" sheetId="4" r:id="R7a7307434dcf4f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporate Actions" sheetId="5" r:id="Rc8b00c38dcba4a3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryHistory" displayName="SummaryHistory" ref="A5:T27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="20">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="BSPI15 level"/>
@@ -254,7 +254,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PricesHistory" displayName="PricesHistory" ref="A5:K379" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -273,7 +273,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H320" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReturnsandContributionsHistory" displayName="ReturnsandContributionsHistory" ref="A5:H335" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceAuditHistory" displayName="SourceAuditHistory" ref="A5:M379" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Ticker"/>
@@ -310,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H362" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CorporateActionsHistory" displayName="CorporateActionsHistory" ref="A5:H379" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Company"/>
@@ -2340,6 +2340,85 @@
         <x:v>-2.9806639010397484</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="40" customHeight="1">
+      <x:c r="A27" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B27" s="18" t="n">
+        <x:f>B26*(1+SUM('Returns and Contributions'!F321:F335))</x:f>
+        <x:v>919.8620937836546</x:v>
+      </x:c>
+      <x:c r="C27" s="21" t="n">
+        <x:f>B27/B26-1</x:f>
+        <x:v>-0.026221884850388344</x:v>
+      </x:c>
+      <x:c r="D27" s="21" t="n">
+        <x:f>B27/$B$6-1</x:f>
+        <x:v>-0.08013790621634542</x:v>
+      </x:c>
+      <x:c r="E27" s="18" t="n">
+        <x:f>1000*'Prices'!H378/'Prices'!I378</x:f>
+        <x:v>988.7327250552734</x:v>
+      </x:c>
+      <x:c r="F27" s="21" t="n">
+        <x:f>E27/E26-1</x:f>
+        <x:v>-0.018175247623500868</x:v>
+      </x:c>
+      <x:c r="G27" s="21" t="n">
+        <x:f>E27/1000-1</x:f>
+        <x:v>-0.01126727494472668</x:v>
+      </x:c>
+      <x:c r="H27" s="18" t="n">
+        <x:f>1000*'Prices'!H379/'Prices'!I379</x:f>
+        <x:v>946.6129322569407</x:v>
+      </x:c>
+      <x:c r="I27" s="21" t="n">
+        <x:f>H27/H26-1</x:f>
+        <x:v>-0.02855575574776148</x:v>
+      </x:c>
+      <x:c r="J27" s="21" t="n">
+        <x:f>H27/1000-1</x:f>
+        <x:v>-0.05338706774305935</x:v>
+      </x:c>
+      <x:c r="K27" s="25" t="n">
+        <x:f>(C27-F27)*100</x:f>
+        <x:v>-0.8046637226887476</x:v>
+      </x:c>
+      <x:c r="L27" s="25" t="n">
+        <x:f>(C27-I27)*100</x:f>
+        <x:v>0.2333870897373136</x:v>
+      </x:c>
+      <x:c r="M27" s="23" t="n">
+        <x:f>SUM('Returns and Contributions'!G321:G335)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N27" s="27" t="n">
+        <x:f>SUM('Returns and Contributions'!F321:F335)-C27</x:f>
+        <x:v>4.5102810375396984e-17</x:v>
+      </x:c>
+      <x:c r="O27" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P27" s="32" t="str">
+        <x:f>IF(COUNTIF('Source Audit'!I363:I379,"Mismatch")=0,IF(COUNTIF('Source Audit'!I363:I379,"Approved MIC exception")&gt;0,"Passed / exception","Passed"),"Failed")</x:f>
+        <x:v>Passed / exception</x:v>
+      </x:c>
+      <x:c r="Q27" s="30" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="R27" s="27" t="n">
+        <x:f>B27-1000*('Prices'!H363/'Prices'!H6+'Prices'!H364/'Prices'!H7+'Prices'!H365/'Prices'!H8+'Prices'!H366/'Prices'!H9+'Prices'!H367/'Prices'!H10+'Prices'!H368/'Prices'!H11+'Prices'!H369/'Prices'!H12+'Prices'!H370/'Prices'!H13+'Prices'!H371/'Prices'!H14+'Prices'!H372/'Prices'!H15+'Prices'!H373/'Prices'!H16+'Prices'!H374/'Prices'!H17+'Prices'!H375/'Prices'!H18+'Prices'!H376/'Prices'!H19+'Prices'!H377/'Prices'!H20)/15</x:f>
+        <x:v>3.410605131648481e-13</x:v>
+      </x:c>
+      <x:c r="S27" s="25" t="n">
+        <x:f>(D27-G27)*100</x:f>
+        <x:v>-6.887063127161874</x:v>
+      </x:c>
+      <x:c r="T27" s="25" t="n">
+        <x:f>(D27-J27)*100</x:f>
+        <x:v>-2.6750838473286076</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -2347,7 +2426,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d54feeb29d4705"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40fc0376a0ce4404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15261,6 +15340,618 @@
         <x:v>Open</x:v>
       </x:c>
     </x:row>
+    <x:row r="363" ht="27" customHeight="1">
+      <x:c r="A363" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B363" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C363" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D363" s="10" t="str">
+        <x:v>6954.T</x:v>
+      </x:c>
+      <x:c r="E363" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F363" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G363" s="33" t="n">
+        <x:f>H346</x:f>
+        <x:v>5795</x:v>
+      </x:c>
+      <x:c r="H363" s="35" t="n">
+        <x:v>5704</x:v>
+      </x:c>
+      <x:c r="I363" s="35" t="n">
+        <x:v>6127</x:v>
+      </x:c>
+      <x:c r="J363" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K363" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="27" customHeight="1">
+      <x:c r="A364" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B364" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C364" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D364" s="2" t="str">
+        <x:v>6506.T</x:v>
+      </x:c>
+      <x:c r="E364" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F364" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G364" s="17" t="n">
+        <x:f>H347</x:f>
+        <x:v>4159</x:v>
+      </x:c>
+      <x:c r="H364" s="34" t="n">
+        <x:v>3992</x:v>
+      </x:c>
+      <x:c r="I364" s="34" t="n">
+        <x:v>4779</x:v>
+      </x:c>
+      <x:c r="J364" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K364" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365" ht="27" customHeight="1">
+      <x:c r="A365" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B365" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C365" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D365" s="10" t="str">
+        <x:v>002747.SZ</x:v>
+      </x:c>
+      <x:c r="E365" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F365" s="10" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G365" s="33" t="n">
+        <x:f>H348</x:f>
+        <x:v>28.4</x:v>
+      </x:c>
+      <x:c r="H365" s="35" t="n">
+        <x:v>29.24</x:v>
+      </x:c>
+      <x:c r="I365" s="35" t="n">
+        <x:v>28.22</x:v>
+      </x:c>
+      <x:c r="J365" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K365" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366" ht="27" customHeight="1">
+      <x:c r="A366" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B366" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C366" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D366" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="E366" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F366" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G366" s="17" t="n">
+        <x:f>H349</x:f>
+        <x:v>296.23</x:v>
+      </x:c>
+      <x:c r="H366" s="34" t="n">
+        <x:v>274.37</x:v>
+      </x:c>
+      <x:c r="I366" s="34" t="n">
+        <x:v>415.79</x:v>
+      </x:c>
+      <x:c r="J366" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K366" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367" ht="27" customHeight="1">
+      <x:c r="A367" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B367" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C367" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D367" s="10" t="str">
+        <x:v>6268.T</x:v>
+      </x:c>
+      <x:c r="E367" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F367" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G367" s="33" t="n">
+        <x:f>H350</x:f>
+        <x:v>4384</x:v>
+      </x:c>
+      <x:c r="H367" s="35" t="n">
+        <x:v>4311</x:v>
+      </x:c>
+      <x:c r="I367" s="35" t="n">
+        <x:v>4975</x:v>
+      </x:c>
+      <x:c r="J367" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K367" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368" ht="27" customHeight="1">
+      <x:c r="A368" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B368" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C368" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D368" s="2" t="str">
+        <x:v>300124.SZ</x:v>
+      </x:c>
+      <x:c r="E368" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="F368" s="2" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G368" s="17" t="n">
+        <x:f>H351</x:f>
+        <x:v>56.78</x:v>
+      </x:c>
+      <x:c r="H368" s="34" t="n">
+        <x:v>55.39</x:v>
+      </x:c>
+      <x:c r="I368" s="34" t="n">
+        <x:v>51.9</x:v>
+      </x:c>
+      <x:c r="J368" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K368" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369" ht="27" customHeight="1">
+      <x:c r="A369" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B369" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C369" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D369" s="10" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="E369" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F369" s="10" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G369" s="33" t="n">
+        <x:f>H352</x:f>
+        <x:v>76360</x:v>
+      </x:c>
+      <x:c r="H369" s="35" t="n">
+        <x:v>78000</x:v>
+      </x:c>
+      <x:c r="I369" s="35" t="n">
+        <x:v>81200</x:v>
+      </x:c>
+      <x:c r="J369" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K369" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370" ht="27" customHeight="1">
+      <x:c r="A370" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B370" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C370" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D370" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="E370" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F370" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G370" s="17" t="n">
+        <x:f>H353</x:f>
+        <x:v>58.97</x:v>
+      </x:c>
+      <x:c r="H370" s="34" t="n">
+        <x:v>56.15</x:v>
+      </x:c>
+      <x:c r="I370" s="34" t="n">
+        <x:v>62.22</x:v>
+      </x:c>
+      <x:c r="J370" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K370" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="27" customHeight="1">
+      <x:c r="A371" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B371" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C371" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D371" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="E371" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F371" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G371" s="33" t="n">
+        <x:f>H354</x:f>
+        <x:v>32.14</x:v>
+      </x:c>
+      <x:c r="H371" s="35" t="n">
+        <x:v>29.74</x:v>
+      </x:c>
+      <x:c r="I371" s="35" t="n">
+        <x:v>40.87</x:v>
+      </x:c>
+      <x:c r="J371" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K371" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="27" customHeight="1">
+      <x:c r="A372" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B372" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C372" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D372" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="E372" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F372" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G372" s="17" t="n">
+        <x:f>H355</x:f>
+        <x:v>12.97</x:v>
+      </x:c>
+      <x:c r="H372" s="34" t="n">
+        <x:v>12.18</x:v>
+      </x:c>
+      <x:c r="I372" s="34" t="n">
+        <x:v>15.93</x:v>
+      </x:c>
+      <x:c r="J372" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K372" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373" ht="27" customHeight="1">
+      <x:c r="A373" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B373" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C373" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D373" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="E373" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="F373" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G373" s="33" t="n">
+        <x:f>H356</x:f>
+        <x:v>451.4</x:v>
+      </x:c>
+      <x:c r="H373" s="35" t="n">
+        <x:v>436.2</x:v>
+      </x:c>
+      <x:c r="I373" s="35" t="n">
+        <x:v>442.45</x:v>
+      </x:c>
+      <x:c r="J373" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K373" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374" ht="27" customHeight="1">
+      <x:c r="A374" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B374" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C374" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D374" s="2" t="str">
+        <x:v>SIE.DE</x:v>
+      </x:c>
+      <x:c r="E374" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="F374" s="2" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G374" s="17" t="n">
+        <x:f>H357</x:f>
+        <x:v>273.75</x:v>
+      </x:c>
+      <x:c r="H374" s="34" t="n">
+        <x:v>265.65</x:v>
+      </x:c>
+      <x:c r="I374" s="34" t="n">
+        <x:v>271.9</x:v>
+      </x:c>
+      <x:c r="J374" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K374" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375" ht="27" customHeight="1">
+      <x:c r="A375" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B375" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C375" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D375" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="E375" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="F375" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G375" s="33" t="n">
+        <x:f>H358</x:f>
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="H375" s="35" t="n">
+        <x:v>259.61</x:v>
+      </x:c>
+      <x:c r="I375" s="35" t="n">
+        <x:v>239.19</x:v>
+      </x:c>
+      <x:c r="J375" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K375" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376" ht="27" customHeight="1">
+      <x:c r="A376" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B376" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C376" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D376" s="2" t="str">
+        <x:v>6383.T</x:v>
+      </x:c>
+      <x:c r="E376" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="F376" s="2" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="G376" s="17" t="n">
+        <x:f>H359</x:f>
+        <x:v>5363</x:v>
+      </x:c>
+      <x:c r="H376" s="34" t="n">
+        <x:v>5193</x:v>
+      </x:c>
+      <x:c r="I376" s="34" t="n">
+        <x:v>5832</x:v>
+      </x:c>
+      <x:c r="J376" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K376" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377" ht="27" customHeight="1">
+      <x:c r="A377" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B377" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C377" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D377" s="10" t="str">
+        <x:v>HEXA-B.ST</x:v>
+      </x:c>
+      <x:c r="E377" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="F377" s="10" t="str">
+        <x:v>SEK</x:v>
+      </x:c>
+      <x:c r="G377" s="33" t="n">
+        <x:f>H360</x:f>
+        <x:v>110.1</x:v>
+      </x:c>
+      <x:c r="H377" s="35" t="n">
+        <x:v>109.7</x:v>
+      </x:c>
+      <x:c r="I377" s="35" t="n">
+        <x:v>99.02</x:v>
+      </x:c>
+      <x:c r="J377" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K377" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378" ht="27" customHeight="1">
+      <x:c r="A378" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B378" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C378" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D378" s="2" t="str">
+        <x:v>GSPC.INDX</x:v>
+      </x:c>
+      <x:c r="E378" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F378" s="2" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G378" s="17" t="n">
+        <x:f>H361</x:f>
+        <x:v>7720.39</x:v>
+      </x:c>
+      <x:c r="H378" s="34" t="n">
+        <x:v>7580.07</x:v>
+      </x:c>
+      <x:c r="I378" s="34" t="n">
+        <x:v>7666.45</x:v>
+      </x:c>
+      <x:c r="J378" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K378" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379" ht="27" customHeight="1">
+      <x:c r="A379" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B379" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C379" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D379" s="10" t="str">
+        <x:v>IXIC.INDX</x:v>
+      </x:c>
+      <x:c r="E379" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="F379" s="10" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G379" s="33" t="n">
+        <x:f>H362</x:f>
+        <x:v>26184.7246</x:v>
+      </x:c>
+      <x:c r="H379" s="35" t="n">
+        <x:v>25437</x:v>
+      </x:c>
+      <x:c r="I379" s="35" t="n">
+        <x:v>26871.5957</x:v>
+      </x:c>
+      <x:c r="J379" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="K379" s="10" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -15268,7 +15959,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46cb2231a0b940ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra891e89159cd4e3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25032,6 +25723,471 @@
         <x:v>0.11189658654817203</x:v>
       </x:c>
     </x:row>
+    <x:row r="321" ht="27" customHeight="1">
+      <x:c r="A321" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B321" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C321" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D321" s="21" t="n">
+        <x:f>G306</x:f>
+        <x:v>0.06675004891024859</x:v>
+      </x:c>
+      <x:c r="E321" s="23" t="n">
+        <x:f>'Prices'!H363/'Prices'!G363-1</x:f>
+        <x:v>-0.0157031924072476</x:v>
+      </x:c>
+      <x:c r="F321" s="21" t="n">
+        <x:f>D321*E321</x:f>
+        <x:v>-0.0010481888612308217</x:v>
+      </x:c>
+      <x:c r="G321" s="21" t="n">
+        <x:f>D321*(1+E321)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.06747107891095222</x:v>
+      </x:c>
+      <x:c r="H321" s="23" t="n">
+        <x:f>'Prices'!H363/'Prices'!I363-1</x:f>
+        <x:v>-0.06903868124693979</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322" ht="27" customHeight="1">
+      <x:c r="A322" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B322" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C322" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D322" s="20" t="n">
+        <x:f>G307</x:f>
+        <x:v>0.061418317920973096</x:v>
+      </x:c>
+      <x:c r="E322" s="22" t="n">
+        <x:f>'Prices'!H364/'Prices'!G364-1</x:f>
+        <x:v>-0.0401538831449868</x:v>
+      </x:c>
+      <x:c r="F322" s="20" t="n">
+        <x:f>D322*E322</x:f>
+        <x:v>-0.0024661839607604025</x:v>
+      </x:c>
+      <x:c r="G322" s="20" t="n">
+        <x:f>D322*(1+E322)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.06053959628283006</x:v>
+      </x:c>
+      <x:c r="H322" s="22" t="n">
+        <x:f>'Prices'!H364/'Prices'!I364-1</x:f>
+        <x:v>-0.1646788030968822</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323" ht="27" customHeight="1">
+      <x:c r="A323" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B323" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C323" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D323" s="21" t="n">
+        <x:f>G308</x:f>
+        <x:v>0.07102436489529657</x:v>
+      </x:c>
+      <x:c r="E323" s="23" t="n">
+        <x:f>'Prices'!H365/'Prices'!G365-1</x:f>
+        <x:v>0.029577464788732355</x:v>
+      </x:c>
+      <x:c r="F323" s="21" t="n">
+        <x:f>D323*E323</x:f>
+        <x:v>0.0021007206518327127</x:v>
+      </x:c>
+      <x:c r="G323" s="21" t="n">
+        <x:f>D323*(1+E323)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.07509419693201291</x:v>
+      </x:c>
+      <x:c r="H323" s="23" t="n">
+        <x:f>'Prices'!H365/'Prices'!I365-1</x:f>
+        <x:v>0.03614457831325302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324" ht="27" customHeight="1">
+      <x:c r="A324" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B324" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C324" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D324" s="20" t="n">
+        <x:f>G309</x:f>
+        <x:v>0.05028066660453506</x:v>
+      </x:c>
+      <x:c r="E324" s="22" t="n">
+        <x:f>'Prices'!H366/'Prices'!G366-1</x:f>
+        <x:v>-0.07379401141005304</x:v>
+      </x:c>
+      <x:c r="F324" s="20" t="n">
+        <x:f>D324*E324</x:f>
+        <x:v>-0.0037104120851201333</x:v>
+      </x:c>
+      <x:c r="G324" s="20" t="n">
+        <x:f>D324*(1+E324)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.047824297748014034</x:v>
+      </x:c>
+      <x:c r="H324" s="22" t="n">
+        <x:f>'Prices'!H366/'Prices'!I366-1</x:f>
+        <x:v>-0.3401236200966834</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325" ht="27" customHeight="1">
+      <x:c r="A325" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B325" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C325" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D325" s="21" t="n">
+        <x:f>G310</x:f>
+        <x:v>0.06219041983920778</x:v>
+      </x:c>
+      <x:c r="E325" s="23" t="n">
+        <x:f>'Prices'!H367/'Prices'!G367-1</x:f>
+        <x:v>-0.016651459854014616</x:v>
+      </x:c>
+      <x:c r="F325" s="21" t="n">
+        <x:f>D325*E325</x:f>
+        <x:v>-0.0010355612792568825</x:v>
+      </x:c>
+      <x:c r="G325" s="21" t="n">
+        <x:f>D325*(1+E325)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.06280163582291541</x:v>
+      </x:c>
+      <x:c r="H325" s="23" t="n">
+        <x:f>'Prices'!H367/'Prices'!I367-1</x:f>
+        <x:v>-0.13346733668341704</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326" ht="27" customHeight="1">
+      <x:c r="A326" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B326" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C326" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D326" s="20" t="n">
+        <x:f>G311</x:f>
+        <x:v>0.07721008999000284</x:v>
+      </x:c>
+      <x:c r="E326" s="22" t="n">
+        <x:f>'Prices'!H368/'Prices'!G368-1</x:f>
+        <x:v>-0.024480450862979897</x:v>
+      </x:c>
+      <x:c r="F326" s="20" t="n">
+        <x:f>D326*E326</x:f>
+        <x:v>-0.0018901378141265204</x:v>
+      </x:c>
+      <x:c r="G326" s="20" t="n">
+        <x:f>D326*(1+E326)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.07734816690176297</x:v>
+      </x:c>
+      <x:c r="H326" s="22" t="n">
+        <x:f>'Prices'!H368/'Prices'!I368-1</x:f>
+        <x:v>0.0672447013487476</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="27" customHeight="1">
+      <x:c r="A327" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B327" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C327" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D327" s="21" t="n">
+        <x:f>G312</x:f>
+        <x:v>0.06636757033844656</x:v>
+      </x:c>
+      <x:c r="E327" s="23" t="n">
+        <x:f>'Prices'!H369/'Prices'!G369-1</x:f>
+        <x:v>0.021477213200628675</x:v>
+      </x:c>
+      <x:c r="F327" s="21" t="n">
+        <x:f>D327*E327</x:f>
+        <x:v>0.0014253904577665366</x:v>
+      </x:c>
+      <x:c r="G327" s="21" t="n">
+        <x:f>D327*(1+E327)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.06961848879279584</x:v>
+      </x:c>
+      <x:c r="H327" s="23" t="n">
+        <x:f>'Prices'!H369/'Prices'!I369-1</x:f>
+        <x:v>-0.039408866995073843</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="27" customHeight="1">
+      <x:c r="A328" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B328" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C328" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D328" s="20" t="n">
+        <x:f>G313</x:f>
+        <x:v>0.06688783657039911</x:v>
+      </x:c>
+      <x:c r="E328" s="22" t="n">
+        <x:f>'Prices'!H370/'Prices'!G370-1</x:f>
+        <x:v>-0.04782092589452269</x:v>
+      </x:c>
+      <x:c r="F328" s="20" t="n">
+        <x:f>D328*E328</x:f>
+        <x:v>-0.0031986382758780007</x:v>
+      </x:c>
+      <x:c r="G328" s="20" t="n">
+        <x:f>D328*(1+E328)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.06540422022601716</x:v>
+      </x:c>
+      <x:c r="H328" s="22" t="n">
+        <x:f>'Prices'!H370/'Prices'!I370-1</x:f>
+        <x:v>-0.09755705560912886</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329" ht="27" customHeight="1">
+      <x:c r="A329" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B329" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C329" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D329" s="21" t="n">
+        <x:f>G314</x:f>
+        <x:v>0.05549926901156623</x:v>
+      </x:c>
+      <x:c r="E329" s="23" t="n">
+        <x:f>'Prices'!H371/'Prices'!G371-1</x:f>
+        <x:v>-0.0746733042937151</x:v>
+      </x:c>
+      <x:c r="F329" s="21" t="n">
+        <x:f>D329*E329</x:f>
+        <x:v>-0.004144313802979438</x:v>
+      </x:c>
+      <x:c r="G329" s="21" t="n">
+        <x:f>D329*(1+E329)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.05273784079722987</x:v>
+      </x:c>
+      <x:c r="H329" s="23" t="n">
+        <x:f>'Prices'!H371/'Prices'!I371-1</x:f>
+        <x:v>-0.27232689013946665</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="27" customHeight="1">
+      <x:c r="A330" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B330" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C330" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D330" s="20" t="n">
+        <x:f>G315</x:f>
+        <x:v>0.05746060952885462</x:v>
+      </x:c>
+      <x:c r="E330" s="22" t="n">
+        <x:f>'Prices'!H372/'Prices'!G372-1</x:f>
+        <x:v>-0.060909791827293835</x:v>
+      </x:c>
+      <x:c r="F330" s="20" t="n">
+        <x:f>D330*E330</x:f>
+        <x:v>-0.0034999137646719515</x:v>
+      </x:c>
+      <x:c r="G330" s="20" t="n">
+        <x:f>D330*(1+E330)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.05541374870176881</x:v>
+      </x:c>
+      <x:c r="H330" s="22" t="n">
+        <x:f>'Prices'!H372/'Prices'!I372-1</x:f>
+        <x:v>-0.2354048964218456</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="27" customHeight="1">
+      <x:c r="A331" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B331" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C331" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D331" s="21" t="n">
+        <x:f>G316</x:f>
+        <x:v>0.07200180496353167</x:v>
+      </x:c>
+      <x:c r="E331" s="23" t="n">
+        <x:f>'Prices'!H373/'Prices'!G373-1</x:f>
+        <x:v>-0.03367301727957461</x:v>
+      </x:c>
+      <x:c r="F331" s="21" t="n">
+        <x:f>D331*E331</x:f>
+        <x:v>-0.002424518022697563</x:v>
+      </x:c>
+      <x:c r="G331" s="21" t="n">
+        <x:f>D331*(1+E331)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.07145086324942128</x:v>
+      </x:c>
+      <x:c r="H331" s="23" t="n">
+        <x:f>'Prices'!H373/'Prices'!I373-1</x:f>
+        <x:v>-0.014125889931065672</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="27" customHeight="1">
+      <x:c r="A332" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B332" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C332" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D332" s="20" t="n">
+        <x:f>G317</x:f>
+        <x:v>0.07105439542528942</x:v>
+      </x:c>
+      <x:c r="E332" s="22" t="n">
+        <x:f>'Prices'!H374/'Prices'!G374-1</x:f>
+        <x:v>-0.029589041095890445</x:v>
+      </x:c>
+      <x:c r="F332" s="20" t="n">
+        <x:f>D332*E332</x:f>
+        <x:v>-0.002102431426282539</x:v>
+      </x:c>
+      <x:c r="G332" s="20" t="n">
+        <x:f>D332*(1+E332)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.07080870161927297</x:v>
+      </x:c>
+      <x:c r="H332" s="22" t="n">
+        <x:f>'Prices'!H374/'Prices'!I374-1</x:f>
+        <x:v>-0.022986392055902916</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="27" customHeight="1">
+      <x:c r="A333" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B333" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C333" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D333" s="21" t="n">
+        <x:f>G318</x:f>
+        <x:v>0.07848463558256798</x:v>
+      </x:c>
+      <x:c r="E333" s="23" t="n">
+        <x:f>'Prices'!H375/'Prices'!G375-1</x:f>
+        <x:v>-0.02402255639097739</x:v>
+      </x:c>
+      <x:c r="F333" s="21" t="n">
+        <x:f>D333*E333</x:f>
+        <x:v>-0.0018854015841075497</x:v>
+      </x:c>
+      <x:c r="G333" s="21" t="n">
+        <x:f>D333*(1+E333)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.07866189720919298</x:v>
+      </x:c>
+      <x:c r="H333" s="23" t="n">
+        <x:f>'Prices'!H375/'Prices'!I375-1</x:f>
+        <x:v>0.0853714620176429</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="27" customHeight="1">
+      <x:c r="A334" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B334" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C334" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D334" s="20" t="n">
+        <x:f>G319</x:f>
+        <x:v>0.06489874669926173</x:v>
+      </x:c>
+      <x:c r="E334" s="22" t="n">
+        <x:f>'Prices'!H376/'Prices'!G376-1</x:f>
+        <x:v>-0.031698676114115254</x:v>
+      </x:c>
+      <x:c r="F334" s="20" t="n">
+        <x:f>D334*E334</x:f>
+        <x:v>-0.002057204351831904</x:v>
+      </x:c>
+      <x:c r="G334" s="20" t="n">
+        <x:f>D334*(1+E334)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.0645337386102324</x:v>
+      </x:c>
+      <x:c r="H334" s="22" t="n">
+        <x:f>'Prices'!H376/'Prices'!I376-1</x:f>
+        <x:v>-0.10956790123456794</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="27" customHeight="1">
+      <x:c r="A335" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B335" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C335" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D335" s="21" t="n">
+        <x:f>G320</x:f>
+        <x:v>0.07847122371981839</x:v>
+      </x:c>
+      <x:c r="E335" s="23" t="n">
+        <x:f>'Prices'!H377/'Prices'!G377-1</x:f>
+        <x:v>-0.0036330608537692433</x:v>
+      </x:c>
+      <x:c r="F335" s="21" t="n">
+        <x:f>D335*E335</x:f>
+        <x:v>-0.0002850907310438407</x:v>
+      </x:c>
+      <x:c r="G335" s="21" t="n">
+        <x:f>D335*(1+E335)/(1+SUM($F$321:$F$335))</x:f>
+        <x:v>0.08029152819558079</x:v>
+      </x:c>
+      <x:c r="H335" s="23" t="n">
+        <x:f>'Prices'!H377/'Prices'!I377-1</x:f>
+        <x:v>0.10785699858614439</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -25039,7 +26195,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43d6650d4c52470c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf68c7362b4034069"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38806,6 +39962,654 @@
       </x:c>
       <x:c r="M362" s="14" t="str"/>
     </x:row>
+    <x:row r="363" ht="50" customHeight="1">
+      <x:c r="A363" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B363" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="C363" s="33" t="n">
+        <x:v>5704</x:v>
+      </x:c>
+      <x:c r="D363" s="33" t="n">
+        <x:v>5704</x:v>
+      </x:c>
+      <x:c r="E363" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F363" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G363" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H363" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I363" s="32" t="str">
+        <x:f>IF(AND(G363=H363,C363&gt;0,ABS(C363-'Prices'!H363)&lt;=MAX(0.01,'Prices'!H363*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J363" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K363" s="16" t="str"/>
+      <x:c r="L363" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M363" s="16" t="str"/>
+    </x:row>
+    <x:row r="364" ht="50" customHeight="1">
+      <x:c r="A364" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B364" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="C364" s="17" t="n">
+        <x:v>3992</x:v>
+      </x:c>
+      <x:c r="D364" s="17" t="n">
+        <x:v>3992</x:v>
+      </x:c>
+      <x:c r="E364" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F364" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G364" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H364" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I364" s="31" t="str">
+        <x:f>IF(AND(G364=H364,C364&gt;0,ABS(C364-'Prices'!H364)&lt;=MAX(0.01,'Prices'!H364*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J364" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K364" s="14" t="str"/>
+      <x:c r="L364" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M364" s="14" t="str"/>
+    </x:row>
+    <x:row r="365" ht="50" customHeight="1">
+      <x:c r="A365" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B365" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="C365" s="33" t="n">
+        <x:v>29.24</x:v>
+      </x:c>
+      <x:c r="D365" s="33" t="n">
+        <x:v>29.24</x:v>
+      </x:c>
+      <x:c r="E365" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F365" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G365" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H365" s="10" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I365" s="32" t="str">
+        <x:f>IF(AND(G365=H365,C365&gt;0,ABS(C365-'Prices'!H365)&lt;=MAX(0.01,'Prices'!H365*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J365" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K365" s="16" t="str"/>
+      <x:c r="L365" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M365" s="16" t="str"/>
+    </x:row>
+    <x:row r="366" ht="50" customHeight="1">
+      <x:c r="A366" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B366" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="C366" s="17" t="n">
+        <x:v>274.37</x:v>
+      </x:c>
+      <x:c r="D366" s="17" t="n">
+        <x:v>274.37</x:v>
+      </x:c>
+      <x:c r="E366" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F366" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G366" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H366" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I366" s="31" t="str">
+        <x:f>IF(AND(G366=H366,C366&gt;0,ABS(C366-'Prices'!H366)&lt;=MAX(0.01,'Prices'!H366*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J366" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K366" s="14" t="str"/>
+      <x:c r="L366" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M366" s="14" t="str"/>
+    </x:row>
+    <x:row r="367" ht="50" customHeight="1">
+      <x:c r="A367" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B367" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="C367" s="33" t="n">
+        <x:v>4311</x:v>
+      </x:c>
+      <x:c r="D367" s="33" t="n">
+        <x:v>4311</x:v>
+      </x:c>
+      <x:c r="E367" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F367" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G367" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H367" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I367" s="32" t="str">
+        <x:f>IF(AND(G367=H367,C367&gt;0,ABS(C367-'Prices'!H367)&lt;=MAX(0.01,'Prices'!H367*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J367" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K367" s="16" t="str"/>
+      <x:c r="L367" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M367" s="16" t="str"/>
+    </x:row>
+    <x:row r="368" ht="50" customHeight="1">
+      <x:c r="A368" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B368" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="C368" s="17" t="n">
+        <x:v>55.39</x:v>
+      </x:c>
+      <x:c r="D368" s="17" t="n">
+        <x:v>55.39</x:v>
+      </x:c>
+      <x:c r="E368" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F368" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G368" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="H368" s="2" t="str">
+        <x:v>XSHE</x:v>
+      </x:c>
+      <x:c r="I368" s="31" t="str">
+        <x:f>IF(AND(G368=H368,C368&gt;0,ABS(C368-'Prices'!H368)&lt;=MAX(0.01,'Prices'!H368*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J368" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K368" s="14" t="str"/>
+      <x:c r="L368" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M368" s="14" t="str"/>
+    </x:row>
+    <x:row r="369" ht="50" customHeight="1">
+      <x:c r="A369" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B369" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="C369" s="33" t="n">
+        <x:v>78000</x:v>
+      </x:c>
+      <x:c r="D369" s="33" t="n">
+        <x:v>78000</x:v>
+      </x:c>
+      <x:c r="E369" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F369" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G369" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H369" s="10" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I369" s="32" t="str">
+        <x:f>IF(AND(G369=H369,C369&gt;0,ABS(C369-'Prices'!H369)&lt;=MAX(0.01,'Prices'!H369*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J369" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K369" s="16" t="str"/>
+      <x:c r="L369" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M369" s="16" t="str"/>
+    </x:row>
+    <x:row r="370" ht="50" customHeight="1">
+      <x:c r="A370" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B370" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="C370" s="17" t="n">
+        <x:v>56.15</x:v>
+      </x:c>
+      <x:c r="D370" s="17" t="n">
+        <x:v>56.15</x:v>
+      </x:c>
+      <x:c r="E370" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F370" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G370" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H370" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I370" s="31" t="str">
+        <x:f>IF(AND(G370=H370,C370&gt;0,ABS(C370-'Prices'!H370)&lt;=MAX(0.01,'Prices'!H370*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J370" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K370" s="14" t="str"/>
+      <x:c r="L370" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M370" s="14" t="str"/>
+    </x:row>
+    <x:row r="371" ht="50" customHeight="1">
+      <x:c r="A371" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B371" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="C371" s="33" t="n">
+        <x:v>29.74</x:v>
+      </x:c>
+      <x:c r="D371" s="33" t="n">
+        <x:v>29.74</x:v>
+      </x:c>
+      <x:c r="E371" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F371" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G371" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H371" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I371" s="32" t="str">
+        <x:f>IF(AND(OR(G371=H371,AND(B371="OUST",G371="XNAS",H371="XNYS",LEFT(M371,34)="ouster-marketstack-legacy-nyse-tag")),C371&gt;0,ABS(C371-'Prices'!H371)&lt;=MAX(0.01,'Prices'!H371*0.000001)),"Approved MIC exception","Mismatch")</x:f>
+        <x:v>Approved MIC exception</x:v>
+      </x:c>
+      <x:c r="J371" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K371" s="16" t="str"/>
+      <x:c r="L371" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M371" s="16" t="str">
+        <x:v>ouster-marketstack-legacy-nyse-tag; approved 2026-10-14; data/bspi15/provider-mic-exceptions.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="50" customHeight="1">
+      <x:c r="A372" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B372" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="C372" s="17" t="n">
+        <x:v>12.18</x:v>
+      </x:c>
+      <x:c r="D372" s="17" t="n">
+        <x:v>12.18</x:v>
+      </x:c>
+      <x:c r="E372" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F372" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G372" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H372" s="2" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I372" s="31" t="str">
+        <x:f>IF(AND(G372=H372,C372&gt;0,ABS(C372-'Prices'!H372)&lt;=MAX(0.01,'Prices'!H372*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J372" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K372" s="14" t="str"/>
+      <x:c r="L372" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M372" s="14" t="str"/>
+    </x:row>
+    <x:row r="373" ht="50" customHeight="1">
+      <x:c r="A373" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B373" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C373" s="33" t="n">
+        <x:v>436.2</x:v>
+      </x:c>
+      <x:c r="D373" s="33" t="n">
+        <x:v>436.2</x:v>
+      </x:c>
+      <x:c r="E373" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F373" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G373" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="H373" s="10" t="str">
+        <x:v>XNYS</x:v>
+      </x:c>
+      <x:c r="I373" s="32" t="str">
+        <x:f>IF(AND(G373=H373,C373&gt;0,ABS(C373-'Prices'!H373)&lt;=MAX(0.01,'Prices'!H373*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J373" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K373" s="16" t="str"/>
+      <x:c r="L373" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M373" s="16" t="str"/>
+    </x:row>
+    <x:row r="374" ht="50" customHeight="1">
+      <x:c r="A374" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B374" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="C374" s="17" t="n">
+        <x:v>265.65</x:v>
+      </x:c>
+      <x:c r="D374" s="17" t="n">
+        <x:v>265.65</x:v>
+      </x:c>
+      <x:c r="E374" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F374" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G374" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="H374" s="2" t="str">
+        <x:v>XETR</x:v>
+      </x:c>
+      <x:c r="I374" s="31" t="str">
+        <x:f>IF(AND(G374=H374,C374&gt;0,ABS(C374-'Prices'!H374)&lt;=MAX(0.01,'Prices'!H374*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J374" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K374" s="14" t="str"/>
+      <x:c r="L374" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M374" s="14" t="str"/>
+    </x:row>
+    <x:row r="375" ht="50" customHeight="1">
+      <x:c r="A375" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B375" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="C375" s="33" t="n">
+        <x:v>259.61</x:v>
+      </x:c>
+      <x:c r="D375" s="33" t="n">
+        <x:v>259.61</x:v>
+      </x:c>
+      <x:c r="E375" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F375" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G375" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="H375" s="10" t="str">
+        <x:v>XNAS</x:v>
+      </x:c>
+      <x:c r="I375" s="32" t="str">
+        <x:f>IF(AND(G375=H375,C375&gt;0,ABS(C375-'Prices'!H375)&lt;=MAX(0.01,'Prices'!H375*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J375" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K375" s="16" t="str"/>
+      <x:c r="L375" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M375" s="16" t="str"/>
+    </x:row>
+    <x:row r="376" ht="50" customHeight="1">
+      <x:c r="A376" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B376" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="C376" s="17" t="n">
+        <x:v>5193</x:v>
+      </x:c>
+      <x:c r="D376" s="17" t="n">
+        <x:v>5193</x:v>
+      </x:c>
+      <x:c r="E376" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F376" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G376" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="H376" s="2" t="str">
+        <x:v>XJPX</x:v>
+      </x:c>
+      <x:c r="I376" s="31" t="str">
+        <x:f>IF(AND(G376=H376,C376&gt;0,ABS(C376-'Prices'!H376)&lt;=MAX(0.01,'Prices'!H376*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J376" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K376" s="14" t="str"/>
+      <x:c r="L376" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M376" s="14" t="str"/>
+    </x:row>
+    <x:row r="377" ht="50" customHeight="1">
+      <x:c r="A377" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B377" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="C377" s="33" t="n">
+        <x:v>109.7</x:v>
+      </x:c>
+      <x:c r="D377" s="33" t="n">
+        <x:v>109.7</x:v>
+      </x:c>
+      <x:c r="E377" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F377" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G377" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="H377" s="10" t="str">
+        <x:v>XSTO</x:v>
+      </x:c>
+      <x:c r="I377" s="32" t="str">
+        <x:f>IF(AND(G377=H377,C377&gt;0,ABS(C377-'Prices'!H377)&lt;=MAX(0.01,'Prices'!H377*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J377" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/constituents-v2.json</x:v>
+      </x:c>
+      <x:c r="K377" s="16" t="str"/>
+      <x:c r="L377" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M377" s="16" t="str"/>
+    </x:row>
+    <x:row r="378" ht="50" customHeight="1">
+      <x:c r="A378" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B378" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C378" s="17" t="n">
+        <x:v>7580.07</x:v>
+      </x:c>
+      <x:c r="D378" s="17" t="n">
+        <x:v>7580.07</x:v>
+      </x:c>
+      <x:c r="E378" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F378" s="36" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G378" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H378" s="2" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I378" s="31" t="str">
+        <x:f>IF(AND(G378=H378,C378&gt;0,ABS(C378-'Prices'!H378)&lt;=MAX(0.01,'Prices'!H378*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J378" s="14" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K378" s="14" t="str"/>
+      <x:c r="L378" s="38" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M378" s="14" t="str"/>
+    </x:row>
+    <x:row r="379" ht="50" customHeight="1">
+      <x:c r="A379" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B379" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C379" s="33" t="n">
+        <x:v>25437</x:v>
+      </x:c>
+      <x:c r="D379" s="33" t="n">
+        <x:v>25437</x:v>
+      </x:c>
+      <x:c r="E379" s="33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F379" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G379" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="H379" s="10" t="str">
+        <x:v>INDX</x:v>
+      </x:c>
+      <x:c r="I379" s="32" t="str">
+        <x:f>IF(AND(G379=H379,C379&gt;0,ABS(C379-'Prices'!H379)&lt;=MAX(0.01,'Prices'!H379*0.000001)),"Match","Mismatch")</x:f>
+        <x:v>Match</x:v>
+      </x:c>
+      <x:c r="J379" s="16" t="str">
+        <x:v>data/bspi15/raw/marketstack/2026-10-31T11-30-36-527Z/benchmarks-v1.json</x:v>
+      </x:c>
+      <x:c r="K379" s="16" t="str"/>
+      <x:c r="L379" s="39" t="n">
+        <x:v>46326.47958943287</x:v>
+      </x:c>
+      <x:c r="M379" s="16" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -38813,7 +40617,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d6c6f350b214026"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf53847e8a1874d26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49255,6 +51059,499 @@
         <x:v>No continuity adjustment</x:v>
       </x:c>
     </x:row>
+    <x:row r="363" ht="27" customHeight="1">
+      <x:c r="A363" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B363" s="10" t="str">
+        <x:v>FANUC</x:v>
+      </x:c>
+      <x:c r="C363" s="10" t="str">
+        <x:v>6954</x:v>
+      </x:c>
+      <x:c r="D363" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E363" s="18" t="n">
+        <x:f>'Source Audit'!E363</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F363" s="41" t="n">
+        <x:f>'Source Audit'!F363</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G363" s="12" t="str">
+        <x:f>IF(AND(E363=0,F363=1,'Source Audit'!I363&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H363" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="27" customHeight="1">
+      <x:c r="A364" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B364" s="2" t="str">
+        <x:v>Yaskawa Electric</x:v>
+      </x:c>
+      <x:c r="C364" s="2" t="str">
+        <x:v>6506</x:v>
+      </x:c>
+      <x:c r="D364" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E364" s="19" t="n">
+        <x:f>'Source Audit'!E364</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F364" s="40" t="n">
+        <x:f>'Source Audit'!F364</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G364" s="11" t="str">
+        <x:f>IF(AND(E364=0,F364=1,'Source Audit'!I364&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H364" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365" ht="27" customHeight="1">
+      <x:c r="A365" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B365" s="10" t="str">
+        <x:v>Estun Automation</x:v>
+      </x:c>
+      <x:c r="C365" s="15" t="str">
+        <x:v>002747</x:v>
+      </x:c>
+      <x:c r="D365" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E365" s="18" t="n">
+        <x:f>'Source Audit'!E365</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F365" s="41" t="n">
+        <x:f>'Source Audit'!F365</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G365" s="12" t="str">
+        <x:f>IF(AND(E365=0,F365=1,'Source Audit'!I365&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H365" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366" ht="27" customHeight="1">
+      <x:c r="A366" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B366" s="2" t="str">
+        <x:v>Teradyne</x:v>
+      </x:c>
+      <x:c r="C366" s="2" t="str">
+        <x:v>TER</x:v>
+      </x:c>
+      <x:c r="D366" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E366" s="19" t="n">
+        <x:f>'Source Audit'!E366</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F366" s="40" t="n">
+        <x:f>'Source Audit'!F366</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G366" s="11" t="str">
+        <x:f>IF(AND(E366=0,F366=1,'Source Audit'!I366&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H366" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367" ht="27" customHeight="1">
+      <x:c r="A367" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B367" s="10" t="str">
+        <x:v>Nabtesco</x:v>
+      </x:c>
+      <x:c r="C367" s="10" t="str">
+        <x:v>6268</x:v>
+      </x:c>
+      <x:c r="D367" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E367" s="18" t="n">
+        <x:f>'Source Audit'!E367</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F367" s="41" t="n">
+        <x:f>'Source Audit'!F367</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G367" s="12" t="str">
+        <x:f>IF(AND(E367=0,F367=1,'Source Audit'!I367&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H367" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368" ht="27" customHeight="1">
+      <x:c r="A368" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B368" s="2" t="str">
+        <x:v>Inovance</x:v>
+      </x:c>
+      <x:c r="C368" s="2" t="str">
+        <x:v>300124</x:v>
+      </x:c>
+      <x:c r="D368" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E368" s="19" t="n">
+        <x:f>'Source Audit'!E368</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F368" s="40" t="n">
+        <x:f>'Source Audit'!F368</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G368" s="11" t="str">
+        <x:f>IF(AND(E368=0,F368=1,'Source Audit'!I368&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H368" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369" ht="27" customHeight="1">
+      <x:c r="A369" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B369" s="10" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C369" s="10" t="str">
+        <x:v>6861</x:v>
+      </x:c>
+      <x:c r="D369" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E369" s="18" t="n">
+        <x:f>'Source Audit'!E369</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F369" s="41" t="n">
+        <x:f>'Source Audit'!F369</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G369" s="12" t="str">
+        <x:f>IF(AND(E369=0,F369=1,'Source Audit'!I369&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H369" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370" ht="27" customHeight="1">
+      <x:c r="A370" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B370" s="2" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C370" s="2" t="str">
+        <x:v>CGNX</x:v>
+      </x:c>
+      <x:c r="D370" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E370" s="19" t="n">
+        <x:f>'Source Audit'!E370</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F370" s="40" t="n">
+        <x:f>'Source Audit'!F370</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G370" s="11" t="str">
+        <x:f>IF(AND(E370=0,F370=1,'Source Audit'!I370&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H370" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="44" customHeight="1">
+      <x:c r="A371" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B371" s="10" t="str">
+        <x:v>Ouster</x:v>
+      </x:c>
+      <x:c r="C371" s="10" t="str">
+        <x:v>OUST</x:v>
+      </x:c>
+      <x:c r="D371" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E371" s="18" t="n">
+        <x:f>'Source Audit'!E371</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F371" s="41" t="n">
+        <x:f>'Source Audit'!F371</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G371" s="12" t="str">
+        <x:f>IF(AND(E371=0,F371=1,'Source Audit'!I371&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H371" s="16" t="str">
+        <x:v>Approved provider MIC exception; no price adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="27" customHeight="1">
+      <x:c r="A372" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B372" s="2" t="str">
+        <x:v>Hesai</x:v>
+      </x:c>
+      <x:c r="C372" s="2" t="str">
+        <x:v>HSAI</x:v>
+      </x:c>
+      <x:c r="D372" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E372" s="19" t="n">
+        <x:f>'Source Audit'!E372</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F372" s="40" t="n">
+        <x:f>'Source Audit'!F372</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G372" s="11" t="str">
+        <x:f>IF(AND(E372=0,F372=1,'Source Audit'!I372&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H372" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373" ht="27" customHeight="1">
+      <x:c r="A373" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B373" s="10" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C373" s="10" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="D373" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E373" s="18" t="n">
+        <x:f>'Source Audit'!E373</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F373" s="41" t="n">
+        <x:f>'Source Audit'!F373</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G373" s="12" t="str">
+        <x:f>IF(AND(E373=0,F373=1,'Source Audit'!I373&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H373" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374" ht="27" customHeight="1">
+      <x:c r="A374" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B374" s="2" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C374" s="2" t="str">
+        <x:v>SIE</x:v>
+      </x:c>
+      <x:c r="D374" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E374" s="19" t="n">
+        <x:f>'Source Audit'!E374</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F374" s="40" t="n">
+        <x:f>'Source Audit'!F374</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G374" s="11" t="str">
+        <x:f>IF(AND(E374=0,F374=1,'Source Audit'!I374&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H374" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375" ht="27" customHeight="1">
+      <x:c r="A375" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B375" s="10" t="str">
+        <x:v>NXP Semiconductors</x:v>
+      </x:c>
+      <x:c r="C375" s="10" t="str">
+        <x:v>NXPI</x:v>
+      </x:c>
+      <x:c r="D375" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E375" s="18" t="n">
+        <x:f>'Source Audit'!E375</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F375" s="41" t="n">
+        <x:f>'Source Audit'!F375</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G375" s="12" t="str">
+        <x:f>IF(AND(E375=0,F375=1,'Source Audit'!I375&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H375" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376" ht="27" customHeight="1">
+      <x:c r="A376" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B376" s="2" t="str">
+        <x:v>Daifuku</x:v>
+      </x:c>
+      <x:c r="C376" s="2" t="str">
+        <x:v>6383</x:v>
+      </x:c>
+      <x:c r="D376" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E376" s="19" t="n">
+        <x:f>'Source Audit'!E376</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F376" s="40" t="n">
+        <x:f>'Source Audit'!F376</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G376" s="11" t="str">
+        <x:f>IF(AND(E376=0,F376=1,'Source Audit'!I376&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H376" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377" ht="27" customHeight="1">
+      <x:c r="A377" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B377" s="10" t="str">
+        <x:v>Hexagon</x:v>
+      </x:c>
+      <x:c r="C377" s="10" t="str">
+        <x:v>HEXA B</x:v>
+      </x:c>
+      <x:c r="D377" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E377" s="18" t="n">
+        <x:f>'Source Audit'!E377</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F377" s="41" t="n">
+        <x:f>'Source Audit'!F377</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G377" s="12" t="str">
+        <x:f>IF(AND(E377=0,F377=1,'Source Audit'!I377&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H377" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378" ht="27" customHeight="1">
+      <x:c r="A378" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B378" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="C378" s="2" t="str">
+        <x:v>S&amp;P 500</x:v>
+      </x:c>
+      <x:c r="D378" s="8" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E378" s="19" t="n">
+        <x:f>'Source Audit'!E378</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F378" s="40" t="n">
+        <x:f>'Source Audit'!F378</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G378" s="11" t="str">
+        <x:f>IF(AND(E378=0,F378=1,'Source Audit'!I378&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H378" s="2" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379" ht="27" customHeight="1">
+      <x:c r="A379" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="B379" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="C379" s="10" t="str">
+        <x:v>Nasdaq Composite</x:v>
+      </x:c>
+      <x:c r="D379" s="9" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="E379" s="18" t="n">
+        <x:f>'Source Audit'!E379</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F379" s="41" t="n">
+        <x:f>'Source Audit'!F379</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G379" s="12" t="str">
+        <x:f>IF(AND(E379=0,F379=1,'Source Audit'!I379&lt;&gt;"Mismatch"),"No provider flag","Review required")</x:f>
+        <x:v>No provider flag</x:v>
+      </x:c>
+      <x:c r="H379" s="10" t="str">
+        <x:v>No continuity adjustment</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
@@ -49262,7 +51559,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72b99d3baab24f4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99c4874c8a264d1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>